<commit_message>
Save SQL practice, Python dictionary handoff and study hours
</commit_message>
<xml_diff>
--- a/outputs/study-tracker/study-hours.xlsx
+++ b/outputs/study-tracker/study-hours.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="Rf9c22f18cdc14588"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="R48ec36fb3f954678"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="R3fe13398cb1b4a98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="R554b80bc1bf34e9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="Ra7b7af1ebfd14894"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="Rd6e101ea294d4502"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -362,7 +362,7 @@
       </x:c>
       <x:c r="E4" s="6" t="n">
         <x:f>SUM(E15:E130)</x:f>
-        <x:v>0</x:v>
+        <x:v>1.9563888888899998</x:v>
       </x:c>
       <x:c r="F4" s="1"/>
       <x:c r="G4" s="1"/>
@@ -442,7 +442,7 @@
       </x:c>
       <x:c r="E8" s="6" t="n">
         <x:f>MAX(SUMIFS(D15:D130,A15:A130,B4)-SUMIFS(E15:E130,A15:A130,B4),0)</x:f>
-        <x:v>6</x:v>
+        <x:v>4.04361111111</x:v>
       </x:c>
       <x:c r="F8" s="1"/>
       <x:c r="G8" s="1"/>
@@ -564,8 +564,8 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E15" s="6" t="n">
-        <x:f>IF(A15&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A15,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
-        <x:v>0</x:v>
+        <x:f>IF(A15&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A15,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:v>1.9563888888899998</x:v>
       </x:c>
       <x:c r="F15" s="6" t="str">
         <x:f>IF(A15&gt;=$B$4,"",MAX(D15-E15,0))</x:f>
@@ -578,10 +578,10 @@
       </x:c>
       <x:c r="I15" s="6" t="n">
         <x:f>IF(A15&gt;$B$4,"",SUM($E$15:E15))</x:f>
-        <x:v>0</x:v>
+        <x:v>1.9563888888899998</x:v>
       </x:c>
       <x:c r="J15" s="1" t="str">
-        <x:f>IF(A15&gt;$B$4,"Future",IF(A15=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A15,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E15=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A15&gt;$B$4,"Future",IF(A15=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A15,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E15=0,"No confirmed time","Logged"))))</x:f>
         <x:v>In progress</x:v>
       </x:c>
     </x:row>
@@ -601,7 +601,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E16" s="6" t="str">
-        <x:f>IF(A16&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A16,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A16&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A16,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F16" s="6" t="str">
         <x:f>IF(A16&gt;=$B$4,"",MAX(D16-E16,0))</x:f>
@@ -616,7 +616,7 @@
         <x:f>IF(A16&gt;$B$4,"",SUM($E$15:E16))</x:f>
       </x:c>
       <x:c r="J16" s="1" t="str">
-        <x:f>IF(A16&gt;$B$4,"Future",IF(A16=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A16,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E16=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A16&gt;$B$4,"Future",IF(A16=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A16,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E16=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -636,7 +636,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E17" s="6" t="str">
-        <x:f>IF(A17&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A17,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A17&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A17,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F17" s="6" t="str">
         <x:f>IF(A17&gt;=$B$4,"",MAX(D17-E17,0))</x:f>
@@ -651,7 +651,7 @@
         <x:f>IF(A17&gt;$B$4,"",SUM($E$15:E17))</x:f>
       </x:c>
       <x:c r="J17" s="1" t="str">
-        <x:f>IF(A17&gt;$B$4,"Future",IF(A17=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A17,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E17=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A17&gt;$B$4,"Future",IF(A17=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A17,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E17=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -671,7 +671,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E18" s="6" t="str">
-        <x:f>IF(A18&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A18,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A18&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A18,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F18" s="6" t="str">
         <x:f>IF(A18&gt;=$B$4,"",MAX(D18-E18,0))</x:f>
@@ -686,7 +686,7 @@
         <x:f>IF(A18&gt;$B$4,"",SUM($E$15:E18))</x:f>
       </x:c>
       <x:c r="J18" s="1" t="str">
-        <x:f>IF(A18&gt;$B$4,"Future",IF(A18=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A18,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E18=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A18&gt;$B$4,"Future",IF(A18=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A18,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E18=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -706,7 +706,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E19" s="6" t="str">
-        <x:f>IF(A19&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A19,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A19&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A19,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F19" s="6" t="str">
         <x:f>IF(A19&gt;=$B$4,"",MAX(D19-E19,0))</x:f>
@@ -721,7 +721,7 @@
         <x:f>IF(A19&gt;$B$4,"",SUM($E$15:E19))</x:f>
       </x:c>
       <x:c r="J19" s="1" t="str">
-        <x:f>IF(A19&gt;$B$4,"Future",IF(A19=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A19,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E19=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A19&gt;$B$4,"Future",IF(A19=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A19,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E19=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -741,7 +741,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E20" s="6" t="str">
-        <x:f>IF(A20&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A20,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A20&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A20,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F20" s="6" t="str">
         <x:f>IF(A20&gt;=$B$4,"",MAX(D20-E20,0))</x:f>
@@ -756,7 +756,7 @@
         <x:f>IF(A20&gt;$B$4,"",SUM($E$15:E20))</x:f>
       </x:c>
       <x:c r="J20" s="1" t="str">
-        <x:f>IF(A20&gt;$B$4,"Future",IF(A20=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A20,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E20=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A20&gt;$B$4,"Future",IF(A20=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A20,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E20=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -776,7 +776,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E21" s="6" t="str">
-        <x:f>IF(A21&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A21,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A21&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A21,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F21" s="6" t="str">
         <x:f>IF(A21&gt;=$B$4,"",MAX(D21-E21,0))</x:f>
@@ -791,7 +791,7 @@
         <x:f>IF(A21&gt;$B$4,"",SUM($E$15:E21))</x:f>
       </x:c>
       <x:c r="J21" s="1" t="str">
-        <x:f>IF(A21&gt;$B$4,"Future",IF(A21=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A21,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E21=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A21&gt;$B$4,"Future",IF(A21=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A21,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E21=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -811,7 +811,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E22" s="6" t="str">
-        <x:f>IF(A22&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A22,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A22&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A22,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F22" s="6" t="str">
         <x:f>IF(A22&gt;=$B$4,"",MAX(D22-E22,0))</x:f>
@@ -826,7 +826,7 @@
         <x:f>IF(A22&gt;$B$4,"",SUM($E$15:E22))</x:f>
       </x:c>
       <x:c r="J22" s="1" t="str">
-        <x:f>IF(A22&gt;$B$4,"Future",IF(A22=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A22,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E22=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A22&gt;$B$4,"Future",IF(A22=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A22,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E22=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -846,7 +846,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E23" s="6" t="str">
-        <x:f>IF(A23&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A23,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A23&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A23,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F23" s="6" t="str">
         <x:f>IF(A23&gt;=$B$4,"",MAX(D23-E23,0))</x:f>
@@ -861,7 +861,7 @@
         <x:f>IF(A23&gt;$B$4,"",SUM($E$15:E23))</x:f>
       </x:c>
       <x:c r="J23" s="1" t="str">
-        <x:f>IF(A23&gt;$B$4,"Future",IF(A23=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A23,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E23=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A23&gt;$B$4,"Future",IF(A23=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A23,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E23=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -881,7 +881,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E24" s="6" t="str">
-        <x:f>IF(A24&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A24,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A24&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A24,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F24" s="6" t="str">
         <x:f>IF(A24&gt;=$B$4,"",MAX(D24-E24,0))</x:f>
@@ -896,7 +896,7 @@
         <x:f>IF(A24&gt;$B$4,"",SUM($E$15:E24))</x:f>
       </x:c>
       <x:c r="J24" s="1" t="str">
-        <x:f>IF(A24&gt;$B$4,"Future",IF(A24=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A24,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E24=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A24&gt;$B$4,"Future",IF(A24=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A24,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E24=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -916,7 +916,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E25" s="6" t="str">
-        <x:f>IF(A25&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A25,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A25&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A25,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F25" s="6" t="str">
         <x:f>IF(A25&gt;=$B$4,"",MAX(D25-E25,0))</x:f>
@@ -931,7 +931,7 @@
         <x:f>IF(A25&gt;$B$4,"",SUM($E$15:E25))</x:f>
       </x:c>
       <x:c r="J25" s="1" t="str">
-        <x:f>IF(A25&gt;$B$4,"Future",IF(A25=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A25,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E25=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A25&gt;$B$4,"Future",IF(A25=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A25,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E25=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -951,7 +951,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E26" s="6" t="str">
-        <x:f>IF(A26&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A26,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A26&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A26,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F26" s="6" t="str">
         <x:f>IF(A26&gt;=$B$4,"",MAX(D26-E26,0))</x:f>
@@ -966,7 +966,7 @@
         <x:f>IF(A26&gt;$B$4,"",SUM($E$15:E26))</x:f>
       </x:c>
       <x:c r="J26" s="1" t="str">
-        <x:f>IF(A26&gt;$B$4,"Future",IF(A26=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A26,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E26=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A26&gt;$B$4,"Future",IF(A26=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A26,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E26=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -986,7 +986,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E27" s="6" t="str">
-        <x:f>IF(A27&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A27,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A27&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A27,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F27" s="6" t="str">
         <x:f>IF(A27&gt;=$B$4,"",MAX(D27-E27,0))</x:f>
@@ -1001,7 +1001,7 @@
         <x:f>IF(A27&gt;$B$4,"",SUM($E$15:E27))</x:f>
       </x:c>
       <x:c r="J27" s="1" t="str">
-        <x:f>IF(A27&gt;$B$4,"Future",IF(A27=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A27,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E27=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A27&gt;$B$4,"Future",IF(A27=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A27,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E27=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1021,7 +1021,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E28" s="6" t="str">
-        <x:f>IF(A28&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A28,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A28&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A28,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F28" s="6" t="str">
         <x:f>IF(A28&gt;=$B$4,"",MAX(D28-E28,0))</x:f>
@@ -1036,7 +1036,7 @@
         <x:f>IF(A28&gt;$B$4,"",SUM($E$15:E28))</x:f>
       </x:c>
       <x:c r="J28" s="1" t="str">
-        <x:f>IF(A28&gt;$B$4,"Future",IF(A28=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A28,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E28=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A28&gt;$B$4,"Future",IF(A28=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A28,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E28=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1056,7 +1056,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E29" s="6" t="str">
-        <x:f>IF(A29&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A29,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A29&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A29,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F29" s="6" t="str">
         <x:f>IF(A29&gt;=$B$4,"",MAX(D29-E29,0))</x:f>
@@ -1071,7 +1071,7 @@
         <x:f>IF(A29&gt;$B$4,"",SUM($E$15:E29))</x:f>
       </x:c>
       <x:c r="J29" s="1" t="str">
-        <x:f>IF(A29&gt;$B$4,"Future",IF(A29=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A29,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E29=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A29&gt;$B$4,"Future",IF(A29=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A29,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E29=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1091,7 +1091,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E30" s="6" t="str">
-        <x:f>IF(A30&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A30,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A30&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A30,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F30" s="6" t="str">
         <x:f>IF(A30&gt;=$B$4,"",MAX(D30-E30,0))</x:f>
@@ -1106,7 +1106,7 @@
         <x:f>IF(A30&gt;$B$4,"",SUM($E$15:E30))</x:f>
       </x:c>
       <x:c r="J30" s="1" t="str">
-        <x:f>IF(A30&gt;$B$4,"Future",IF(A30=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A30,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E30=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A30&gt;$B$4,"Future",IF(A30=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A30,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E30=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1126,7 +1126,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E31" s="6" t="str">
-        <x:f>IF(A31&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A31,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A31&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A31,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F31" s="6" t="str">
         <x:f>IF(A31&gt;=$B$4,"",MAX(D31-E31,0))</x:f>
@@ -1141,7 +1141,7 @@
         <x:f>IF(A31&gt;$B$4,"",SUM($E$15:E31))</x:f>
       </x:c>
       <x:c r="J31" s="1" t="str">
-        <x:f>IF(A31&gt;$B$4,"Future",IF(A31=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A31,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E31=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A31&gt;$B$4,"Future",IF(A31=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A31,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E31=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1161,7 +1161,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E32" s="6" t="str">
-        <x:f>IF(A32&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A32,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A32&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A32,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F32" s="6" t="str">
         <x:f>IF(A32&gt;=$B$4,"",MAX(D32-E32,0))</x:f>
@@ -1176,7 +1176,7 @@
         <x:f>IF(A32&gt;$B$4,"",SUM($E$15:E32))</x:f>
       </x:c>
       <x:c r="J32" s="1" t="str">
-        <x:f>IF(A32&gt;$B$4,"Future",IF(A32=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A32,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E32=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A32&gt;$B$4,"Future",IF(A32=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A32,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E32=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1196,7 +1196,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E33" s="6" t="str">
-        <x:f>IF(A33&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A33,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A33&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A33,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F33" s="6" t="str">
         <x:f>IF(A33&gt;=$B$4,"",MAX(D33-E33,0))</x:f>
@@ -1211,7 +1211,7 @@
         <x:f>IF(A33&gt;$B$4,"",SUM($E$15:E33))</x:f>
       </x:c>
       <x:c r="J33" s="1" t="str">
-        <x:f>IF(A33&gt;$B$4,"Future",IF(A33=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A33,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E33=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A33&gt;$B$4,"Future",IF(A33=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A33,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E33=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1231,7 +1231,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E34" s="6" t="str">
-        <x:f>IF(A34&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A34,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A34&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A34,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F34" s="6" t="str">
         <x:f>IF(A34&gt;=$B$4,"",MAX(D34-E34,0))</x:f>
@@ -1246,7 +1246,7 @@
         <x:f>IF(A34&gt;$B$4,"",SUM($E$15:E34))</x:f>
       </x:c>
       <x:c r="J34" s="1" t="str">
-        <x:f>IF(A34&gt;$B$4,"Future",IF(A34=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A34,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E34=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A34&gt;$B$4,"Future",IF(A34=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A34,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E34=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1266,7 +1266,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E35" s="6" t="str">
-        <x:f>IF(A35&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A35,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A35&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A35,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F35" s="6" t="str">
         <x:f>IF(A35&gt;=$B$4,"",MAX(D35-E35,0))</x:f>
@@ -1281,7 +1281,7 @@
         <x:f>IF(A35&gt;$B$4,"",SUM($E$15:E35))</x:f>
       </x:c>
       <x:c r="J35" s="1" t="str">
-        <x:f>IF(A35&gt;$B$4,"Future",IF(A35=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A35,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E35=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A35&gt;$B$4,"Future",IF(A35=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A35,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E35=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1301,7 +1301,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E36" s="6" t="str">
-        <x:f>IF(A36&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A36,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A36&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A36,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F36" s="6" t="str">
         <x:f>IF(A36&gt;=$B$4,"",MAX(D36-E36,0))</x:f>
@@ -1316,7 +1316,7 @@
         <x:f>IF(A36&gt;$B$4,"",SUM($E$15:E36))</x:f>
       </x:c>
       <x:c r="J36" s="1" t="str">
-        <x:f>IF(A36&gt;$B$4,"Future",IF(A36=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A36,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E36=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A36&gt;$B$4,"Future",IF(A36=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A36,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E36=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1336,7 +1336,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E37" s="6" t="str">
-        <x:f>IF(A37&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A37,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A37&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A37,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F37" s="6" t="str">
         <x:f>IF(A37&gt;=$B$4,"",MAX(D37-E37,0))</x:f>
@@ -1351,7 +1351,7 @@
         <x:f>IF(A37&gt;$B$4,"",SUM($E$15:E37))</x:f>
       </x:c>
       <x:c r="J37" s="1" t="str">
-        <x:f>IF(A37&gt;$B$4,"Future",IF(A37=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A37,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E37=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A37&gt;$B$4,"Future",IF(A37=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A37,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E37=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1371,7 +1371,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E38" s="6" t="str">
-        <x:f>IF(A38&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A38,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A38&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A38,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F38" s="6" t="str">
         <x:f>IF(A38&gt;=$B$4,"",MAX(D38-E38,0))</x:f>
@@ -1386,7 +1386,7 @@
         <x:f>IF(A38&gt;$B$4,"",SUM($E$15:E38))</x:f>
       </x:c>
       <x:c r="J38" s="1" t="str">
-        <x:f>IF(A38&gt;$B$4,"Future",IF(A38=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A38,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E38=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A38&gt;$B$4,"Future",IF(A38=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A38,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E38=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1406,7 +1406,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E39" s="6" t="str">
-        <x:f>IF(A39&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A39,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A39&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A39,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F39" s="6" t="str">
         <x:f>IF(A39&gt;=$B$4,"",MAX(D39-E39,0))</x:f>
@@ -1421,7 +1421,7 @@
         <x:f>IF(A39&gt;$B$4,"",SUM($E$15:E39))</x:f>
       </x:c>
       <x:c r="J39" s="1" t="str">
-        <x:f>IF(A39&gt;$B$4,"Future",IF(A39=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A39,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E39=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A39&gt;$B$4,"Future",IF(A39=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A39,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E39=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1441,7 +1441,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E40" s="6" t="str">
-        <x:f>IF(A40&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A40,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A40&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A40,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F40" s="6" t="str">
         <x:f>IF(A40&gt;=$B$4,"",MAX(D40-E40,0))</x:f>
@@ -1456,7 +1456,7 @@
         <x:f>IF(A40&gt;$B$4,"",SUM($E$15:E40))</x:f>
       </x:c>
       <x:c r="J40" s="1" t="str">
-        <x:f>IF(A40&gt;$B$4,"Future",IF(A40=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A40,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E40=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A40&gt;$B$4,"Future",IF(A40=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A40,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E40=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1476,7 +1476,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E41" s="6" t="str">
-        <x:f>IF(A41&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A41,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A41&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A41,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F41" s="6" t="str">
         <x:f>IF(A41&gt;=$B$4,"",MAX(D41-E41,0))</x:f>
@@ -1491,7 +1491,7 @@
         <x:f>IF(A41&gt;$B$4,"",SUM($E$15:E41))</x:f>
       </x:c>
       <x:c r="J41" s="1" t="str">
-        <x:f>IF(A41&gt;$B$4,"Future",IF(A41=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A41,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E41=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A41&gt;$B$4,"Future",IF(A41=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A41,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E41=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1511,7 +1511,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E42" s="6" t="str">
-        <x:f>IF(A42&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A42,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A42&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A42,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F42" s="6" t="str">
         <x:f>IF(A42&gt;=$B$4,"",MAX(D42-E42,0))</x:f>
@@ -1526,7 +1526,7 @@
         <x:f>IF(A42&gt;$B$4,"",SUM($E$15:E42))</x:f>
       </x:c>
       <x:c r="J42" s="1" t="str">
-        <x:f>IF(A42&gt;$B$4,"Future",IF(A42=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A42,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E42=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A42&gt;$B$4,"Future",IF(A42=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A42,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E42=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1546,7 +1546,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E43" s="6" t="str">
-        <x:f>IF(A43&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A43,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A43&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A43,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F43" s="6" t="str">
         <x:f>IF(A43&gt;=$B$4,"",MAX(D43-E43,0))</x:f>
@@ -1561,7 +1561,7 @@
         <x:f>IF(A43&gt;$B$4,"",SUM($E$15:E43))</x:f>
       </x:c>
       <x:c r="J43" s="1" t="str">
-        <x:f>IF(A43&gt;$B$4,"Future",IF(A43=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A43,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E43=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A43&gt;$B$4,"Future",IF(A43=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A43,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E43=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1581,7 +1581,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E44" s="6" t="str">
-        <x:f>IF(A44&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A44,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A44&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A44,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F44" s="6" t="str">
         <x:f>IF(A44&gt;=$B$4,"",MAX(D44-E44,0))</x:f>
@@ -1596,7 +1596,7 @@
         <x:f>IF(A44&gt;$B$4,"",SUM($E$15:E44))</x:f>
       </x:c>
       <x:c r="J44" s="1" t="str">
-        <x:f>IF(A44&gt;$B$4,"Future",IF(A44=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A44,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E44=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A44&gt;$B$4,"Future",IF(A44=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A44,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E44=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1616,7 +1616,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E45" s="6" t="str">
-        <x:f>IF(A45&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A45,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A45&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A45,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F45" s="6" t="str">
         <x:f>IF(A45&gt;=$B$4,"",MAX(D45-E45,0))</x:f>
@@ -1631,7 +1631,7 @@
         <x:f>IF(A45&gt;$B$4,"",SUM($E$15:E45))</x:f>
       </x:c>
       <x:c r="J45" s="1" t="str">
-        <x:f>IF(A45&gt;$B$4,"Future",IF(A45=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A45,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E45=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A45&gt;$B$4,"Future",IF(A45=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A45,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E45=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1651,7 +1651,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E46" s="6" t="str">
-        <x:f>IF(A46&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A46,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A46&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A46,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F46" s="6" t="str">
         <x:f>IF(A46&gt;=$B$4,"",MAX(D46-E46,0))</x:f>
@@ -1666,7 +1666,7 @@
         <x:f>IF(A46&gt;$B$4,"",SUM($E$15:E46))</x:f>
       </x:c>
       <x:c r="J46" s="1" t="str">
-        <x:f>IF(A46&gt;$B$4,"Future",IF(A46=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A46,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E46=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A46&gt;$B$4,"Future",IF(A46=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A46,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E46=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1686,7 +1686,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E47" s="6" t="str">
-        <x:f>IF(A47&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A47,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A47&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A47,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F47" s="6" t="str">
         <x:f>IF(A47&gt;=$B$4,"",MAX(D47-E47,0))</x:f>
@@ -1701,7 +1701,7 @@
         <x:f>IF(A47&gt;$B$4,"",SUM($E$15:E47))</x:f>
       </x:c>
       <x:c r="J47" s="1" t="str">
-        <x:f>IF(A47&gt;$B$4,"Future",IF(A47=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A47,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E47=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A47&gt;$B$4,"Future",IF(A47=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A47,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E47=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1721,7 +1721,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E48" s="6" t="str">
-        <x:f>IF(A48&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A48,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A48&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A48,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F48" s="6" t="str">
         <x:f>IF(A48&gt;=$B$4,"",MAX(D48-E48,0))</x:f>
@@ -1736,7 +1736,7 @@
         <x:f>IF(A48&gt;$B$4,"",SUM($E$15:E48))</x:f>
       </x:c>
       <x:c r="J48" s="1" t="str">
-        <x:f>IF(A48&gt;$B$4,"Future",IF(A48=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A48,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E48=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A48&gt;$B$4,"Future",IF(A48=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A48,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E48=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1756,7 +1756,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E49" s="6" t="str">
-        <x:f>IF(A49&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A49,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A49&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A49,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F49" s="6" t="str">
         <x:f>IF(A49&gt;=$B$4,"",MAX(D49-E49,0))</x:f>
@@ -1771,7 +1771,7 @@
         <x:f>IF(A49&gt;$B$4,"",SUM($E$15:E49))</x:f>
       </x:c>
       <x:c r="J49" s="1" t="str">
-        <x:f>IF(A49&gt;$B$4,"Future",IF(A49=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A49,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E49=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A49&gt;$B$4,"Future",IF(A49=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A49,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E49=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1791,7 +1791,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E50" s="6" t="str">
-        <x:f>IF(A50&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A50,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A50&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A50,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F50" s="6" t="str">
         <x:f>IF(A50&gt;=$B$4,"",MAX(D50-E50,0))</x:f>
@@ -1806,7 +1806,7 @@
         <x:f>IF(A50&gt;$B$4,"",SUM($E$15:E50))</x:f>
       </x:c>
       <x:c r="J50" s="1" t="str">
-        <x:f>IF(A50&gt;$B$4,"Future",IF(A50=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A50,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E50=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A50&gt;$B$4,"Future",IF(A50=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A50,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E50=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1826,7 +1826,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E51" s="6" t="str">
-        <x:f>IF(A51&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A51,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A51&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A51,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F51" s="6" t="str">
         <x:f>IF(A51&gt;=$B$4,"",MAX(D51-E51,0))</x:f>
@@ -1841,7 +1841,7 @@
         <x:f>IF(A51&gt;$B$4,"",SUM($E$15:E51))</x:f>
       </x:c>
       <x:c r="J51" s="1" t="str">
-        <x:f>IF(A51&gt;$B$4,"Future",IF(A51=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A51,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E51=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A51&gt;$B$4,"Future",IF(A51=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A51,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E51=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1861,7 +1861,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E52" s="6" t="str">
-        <x:f>IF(A52&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A52,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A52&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A52,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F52" s="6" t="str">
         <x:f>IF(A52&gt;=$B$4,"",MAX(D52-E52,0))</x:f>
@@ -1876,7 +1876,7 @@
         <x:f>IF(A52&gt;$B$4,"",SUM($E$15:E52))</x:f>
       </x:c>
       <x:c r="J52" s="1" t="str">
-        <x:f>IF(A52&gt;$B$4,"Future",IF(A52=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A52,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E52=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A52&gt;$B$4,"Future",IF(A52=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A52,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E52=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1896,7 +1896,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E53" s="6" t="str">
-        <x:f>IF(A53&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A53,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A53&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A53,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F53" s="6" t="str">
         <x:f>IF(A53&gt;=$B$4,"",MAX(D53-E53,0))</x:f>
@@ -1911,7 +1911,7 @@
         <x:f>IF(A53&gt;$B$4,"",SUM($E$15:E53))</x:f>
       </x:c>
       <x:c r="J53" s="1" t="str">
-        <x:f>IF(A53&gt;$B$4,"Future",IF(A53=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A53,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E53=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A53&gt;$B$4,"Future",IF(A53=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A53,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E53=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1931,7 +1931,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E54" s="6" t="str">
-        <x:f>IF(A54&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A54,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A54&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A54,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F54" s="6" t="str">
         <x:f>IF(A54&gt;=$B$4,"",MAX(D54-E54,0))</x:f>
@@ -1946,7 +1946,7 @@
         <x:f>IF(A54&gt;$B$4,"",SUM($E$15:E54))</x:f>
       </x:c>
       <x:c r="J54" s="1" t="str">
-        <x:f>IF(A54&gt;$B$4,"Future",IF(A54=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A54,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E54=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A54&gt;$B$4,"Future",IF(A54=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A54,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E54=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1966,7 +1966,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E55" s="6" t="str">
-        <x:f>IF(A55&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A55,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A55&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A55,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F55" s="6" t="str">
         <x:f>IF(A55&gt;=$B$4,"",MAX(D55-E55,0))</x:f>
@@ -1981,7 +1981,7 @@
         <x:f>IF(A55&gt;$B$4,"",SUM($E$15:E55))</x:f>
       </x:c>
       <x:c r="J55" s="1" t="str">
-        <x:f>IF(A55&gt;$B$4,"Future",IF(A55=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A55,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E55=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A55&gt;$B$4,"Future",IF(A55=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A55,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E55=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2001,7 +2001,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E56" s="6" t="str">
-        <x:f>IF(A56&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A56,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A56&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A56,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F56" s="6" t="str">
         <x:f>IF(A56&gt;=$B$4,"",MAX(D56-E56,0))</x:f>
@@ -2016,7 +2016,7 @@
         <x:f>IF(A56&gt;$B$4,"",SUM($E$15:E56))</x:f>
       </x:c>
       <x:c r="J56" s="1" t="str">
-        <x:f>IF(A56&gt;$B$4,"Future",IF(A56=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A56,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E56=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A56&gt;$B$4,"Future",IF(A56=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A56,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E56=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2036,7 +2036,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E57" s="6" t="str">
-        <x:f>IF(A57&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A57,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A57&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A57,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F57" s="6" t="str">
         <x:f>IF(A57&gt;=$B$4,"",MAX(D57-E57,0))</x:f>
@@ -2051,7 +2051,7 @@
         <x:f>IF(A57&gt;$B$4,"",SUM($E$15:E57))</x:f>
       </x:c>
       <x:c r="J57" s="1" t="str">
-        <x:f>IF(A57&gt;$B$4,"Future",IF(A57=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A57,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E57=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A57&gt;$B$4,"Future",IF(A57=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A57,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E57=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2071,7 +2071,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E58" s="6" t="str">
-        <x:f>IF(A58&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A58,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A58&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A58,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F58" s="6" t="str">
         <x:f>IF(A58&gt;=$B$4,"",MAX(D58-E58,0))</x:f>
@@ -2086,7 +2086,7 @@
         <x:f>IF(A58&gt;$B$4,"",SUM($E$15:E58))</x:f>
       </x:c>
       <x:c r="J58" s="1" t="str">
-        <x:f>IF(A58&gt;$B$4,"Future",IF(A58=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A58,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E58=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A58&gt;$B$4,"Future",IF(A58=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A58,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E58=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2106,7 +2106,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E59" s="6" t="str">
-        <x:f>IF(A59&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A59,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A59&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A59,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F59" s="6" t="str">
         <x:f>IF(A59&gt;=$B$4,"",MAX(D59-E59,0))</x:f>
@@ -2121,7 +2121,7 @@
         <x:f>IF(A59&gt;$B$4,"",SUM($E$15:E59))</x:f>
       </x:c>
       <x:c r="J59" s="1" t="str">
-        <x:f>IF(A59&gt;$B$4,"Future",IF(A59=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A59,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E59=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A59&gt;$B$4,"Future",IF(A59=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A59,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E59=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2141,7 +2141,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E60" s="6" t="str">
-        <x:f>IF(A60&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A60,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A60&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A60,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F60" s="6" t="str">
         <x:f>IF(A60&gt;=$B$4,"",MAX(D60-E60,0))</x:f>
@@ -2156,7 +2156,7 @@
         <x:f>IF(A60&gt;$B$4,"",SUM($E$15:E60))</x:f>
       </x:c>
       <x:c r="J60" s="1" t="str">
-        <x:f>IF(A60&gt;$B$4,"Future",IF(A60=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A60,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E60=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A60&gt;$B$4,"Future",IF(A60=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A60,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E60=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2176,7 +2176,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E61" s="6" t="str">
-        <x:f>IF(A61&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A61,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A61&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A61,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F61" s="6" t="str">
         <x:f>IF(A61&gt;=$B$4,"",MAX(D61-E61,0))</x:f>
@@ -2191,7 +2191,7 @@
         <x:f>IF(A61&gt;$B$4,"",SUM($E$15:E61))</x:f>
       </x:c>
       <x:c r="J61" s="1" t="str">
-        <x:f>IF(A61&gt;$B$4,"Future",IF(A61=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A61,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E61=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A61&gt;$B$4,"Future",IF(A61=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A61,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E61=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2211,7 +2211,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E62" s="6" t="str">
-        <x:f>IF(A62&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A62,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A62&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A62,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F62" s="6" t="str">
         <x:f>IF(A62&gt;=$B$4,"",MAX(D62-E62,0))</x:f>
@@ -2226,7 +2226,7 @@
         <x:f>IF(A62&gt;$B$4,"",SUM($E$15:E62))</x:f>
       </x:c>
       <x:c r="J62" s="1" t="str">
-        <x:f>IF(A62&gt;$B$4,"Future",IF(A62=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A62,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E62=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A62&gt;$B$4,"Future",IF(A62=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A62,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E62=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2246,7 +2246,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E63" s="6" t="str">
-        <x:f>IF(A63&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A63,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A63&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A63,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F63" s="6" t="str">
         <x:f>IF(A63&gt;=$B$4,"",MAX(D63-E63,0))</x:f>
@@ -2261,7 +2261,7 @@
         <x:f>IF(A63&gt;$B$4,"",SUM($E$15:E63))</x:f>
       </x:c>
       <x:c r="J63" s="1" t="str">
-        <x:f>IF(A63&gt;$B$4,"Future",IF(A63=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A63,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E63=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A63&gt;$B$4,"Future",IF(A63=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A63,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E63=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2281,7 +2281,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E64" s="6" t="str">
-        <x:f>IF(A64&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A64,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A64&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A64,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F64" s="6" t="str">
         <x:f>IF(A64&gt;=$B$4,"",MAX(D64-E64,0))</x:f>
@@ -2296,7 +2296,7 @@
         <x:f>IF(A64&gt;$B$4,"",SUM($E$15:E64))</x:f>
       </x:c>
       <x:c r="J64" s="1" t="str">
-        <x:f>IF(A64&gt;$B$4,"Future",IF(A64=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A64,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E64=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A64&gt;$B$4,"Future",IF(A64=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A64,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E64=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2316,7 +2316,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E65" s="6" t="str">
-        <x:f>IF(A65&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A65,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A65&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A65,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F65" s="6" t="str">
         <x:f>IF(A65&gt;=$B$4,"",MAX(D65-E65,0))</x:f>
@@ -2331,7 +2331,7 @@
         <x:f>IF(A65&gt;$B$4,"",SUM($E$15:E65))</x:f>
       </x:c>
       <x:c r="J65" s="1" t="str">
-        <x:f>IF(A65&gt;$B$4,"Future",IF(A65=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A65,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E65=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A65&gt;$B$4,"Future",IF(A65=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A65,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E65=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2351,7 +2351,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E66" s="6" t="str">
-        <x:f>IF(A66&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A66,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A66&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A66,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F66" s="6" t="str">
         <x:f>IF(A66&gt;=$B$4,"",MAX(D66-E66,0))</x:f>
@@ -2366,7 +2366,7 @@
         <x:f>IF(A66&gt;$B$4,"",SUM($E$15:E66))</x:f>
       </x:c>
       <x:c r="J66" s="1" t="str">
-        <x:f>IF(A66&gt;$B$4,"Future",IF(A66=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A66,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E66=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A66&gt;$B$4,"Future",IF(A66=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A66,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E66=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2386,7 +2386,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E67" s="6" t="str">
-        <x:f>IF(A67&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A67,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A67&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A67,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F67" s="6" t="str">
         <x:f>IF(A67&gt;=$B$4,"",MAX(D67-E67,0))</x:f>
@@ -2401,7 +2401,7 @@
         <x:f>IF(A67&gt;$B$4,"",SUM($E$15:E67))</x:f>
       </x:c>
       <x:c r="J67" s="1" t="str">
-        <x:f>IF(A67&gt;$B$4,"Future",IF(A67=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A67,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E67=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A67&gt;$B$4,"Future",IF(A67=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A67,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E67=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2421,7 +2421,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E68" s="6" t="str">
-        <x:f>IF(A68&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A68,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A68&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A68,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F68" s="6" t="str">
         <x:f>IF(A68&gt;=$B$4,"",MAX(D68-E68,0))</x:f>
@@ -2436,7 +2436,7 @@
         <x:f>IF(A68&gt;$B$4,"",SUM($E$15:E68))</x:f>
       </x:c>
       <x:c r="J68" s="1" t="str">
-        <x:f>IF(A68&gt;$B$4,"Future",IF(A68=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A68,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E68=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A68&gt;$B$4,"Future",IF(A68=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A68,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E68=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2456,7 +2456,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E69" s="6" t="str">
-        <x:f>IF(A69&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A69,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A69&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A69,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F69" s="6" t="str">
         <x:f>IF(A69&gt;=$B$4,"",MAX(D69-E69,0))</x:f>
@@ -2471,7 +2471,7 @@
         <x:f>IF(A69&gt;$B$4,"",SUM($E$15:E69))</x:f>
       </x:c>
       <x:c r="J69" s="1" t="str">
-        <x:f>IF(A69&gt;$B$4,"Future",IF(A69=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A69,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E69=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A69&gt;$B$4,"Future",IF(A69=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A69,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E69=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2491,7 +2491,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E70" s="6" t="str">
-        <x:f>IF(A70&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A70,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A70&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A70,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F70" s="6" t="str">
         <x:f>IF(A70&gt;=$B$4,"",MAX(D70-E70,0))</x:f>
@@ -2506,7 +2506,7 @@
         <x:f>IF(A70&gt;$B$4,"",SUM($E$15:E70))</x:f>
       </x:c>
       <x:c r="J70" s="1" t="str">
-        <x:f>IF(A70&gt;$B$4,"Future",IF(A70=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A70,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E70=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A70&gt;$B$4,"Future",IF(A70=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A70,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E70=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2526,7 +2526,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E71" s="6" t="str">
-        <x:f>IF(A71&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A71,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A71&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A71,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F71" s="6" t="str">
         <x:f>IF(A71&gt;=$B$4,"",MAX(D71-E71,0))</x:f>
@@ -2541,7 +2541,7 @@
         <x:f>IF(A71&gt;$B$4,"",SUM($E$15:E71))</x:f>
       </x:c>
       <x:c r="J71" s="1" t="str">
-        <x:f>IF(A71&gt;$B$4,"Future",IF(A71=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A71,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E71=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A71&gt;$B$4,"Future",IF(A71=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A71,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E71=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2561,7 +2561,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E72" s="6" t="str">
-        <x:f>IF(A72&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A72,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A72&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A72,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F72" s="6" t="str">
         <x:f>IF(A72&gt;=$B$4,"",MAX(D72-E72,0))</x:f>
@@ -2576,7 +2576,7 @@
         <x:f>IF(A72&gt;$B$4,"",SUM($E$15:E72))</x:f>
       </x:c>
       <x:c r="J72" s="1" t="str">
-        <x:f>IF(A72&gt;$B$4,"Future",IF(A72=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A72,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E72=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A72&gt;$B$4,"Future",IF(A72=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A72,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E72=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2596,7 +2596,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E73" s="6" t="str">
-        <x:f>IF(A73&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A73,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A73&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A73,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F73" s="6" t="str">
         <x:f>IF(A73&gt;=$B$4,"",MAX(D73-E73,0))</x:f>
@@ -2611,7 +2611,7 @@
         <x:f>IF(A73&gt;$B$4,"",SUM($E$15:E73))</x:f>
       </x:c>
       <x:c r="J73" s="1" t="str">
-        <x:f>IF(A73&gt;$B$4,"Future",IF(A73=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A73,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E73=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A73&gt;$B$4,"Future",IF(A73=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A73,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E73=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2631,7 +2631,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E74" s="6" t="str">
-        <x:f>IF(A74&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A74,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A74&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A74,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F74" s="6" t="str">
         <x:f>IF(A74&gt;=$B$4,"",MAX(D74-E74,0))</x:f>
@@ -2646,7 +2646,7 @@
         <x:f>IF(A74&gt;$B$4,"",SUM($E$15:E74))</x:f>
       </x:c>
       <x:c r="J74" s="1" t="str">
-        <x:f>IF(A74&gt;$B$4,"Future",IF(A74=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A74,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E74=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A74&gt;$B$4,"Future",IF(A74=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A74,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E74=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2666,7 +2666,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E75" s="6" t="str">
-        <x:f>IF(A75&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A75,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A75&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A75,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F75" s="6" t="str">
         <x:f>IF(A75&gt;=$B$4,"",MAX(D75-E75,0))</x:f>
@@ -2681,7 +2681,7 @@
         <x:f>IF(A75&gt;$B$4,"",SUM($E$15:E75))</x:f>
       </x:c>
       <x:c r="J75" s="1" t="str">
-        <x:f>IF(A75&gt;$B$4,"Future",IF(A75=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A75,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E75=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A75&gt;$B$4,"Future",IF(A75=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A75,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E75=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2701,7 +2701,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E76" s="6" t="str">
-        <x:f>IF(A76&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A76,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A76&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A76,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F76" s="6" t="str">
         <x:f>IF(A76&gt;=$B$4,"",MAX(D76-E76,0))</x:f>
@@ -2716,7 +2716,7 @@
         <x:f>IF(A76&gt;$B$4,"",SUM($E$15:E76))</x:f>
       </x:c>
       <x:c r="J76" s="1" t="str">
-        <x:f>IF(A76&gt;$B$4,"Future",IF(A76=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A76,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E76=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A76&gt;$B$4,"Future",IF(A76=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A76,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E76=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2736,7 +2736,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E77" s="6" t="str">
-        <x:f>IF(A77&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A77,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A77&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A77,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F77" s="6" t="str">
         <x:f>IF(A77&gt;=$B$4,"",MAX(D77-E77,0))</x:f>
@@ -2751,7 +2751,7 @@
         <x:f>IF(A77&gt;$B$4,"",SUM($E$15:E77))</x:f>
       </x:c>
       <x:c r="J77" s="1" t="str">
-        <x:f>IF(A77&gt;$B$4,"Future",IF(A77=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A77,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E77=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A77&gt;$B$4,"Future",IF(A77=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A77,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E77=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2771,7 +2771,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E78" s="6" t="str">
-        <x:f>IF(A78&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A78,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A78&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A78,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F78" s="6" t="str">
         <x:f>IF(A78&gt;=$B$4,"",MAX(D78-E78,0))</x:f>
@@ -2786,7 +2786,7 @@
         <x:f>IF(A78&gt;$B$4,"",SUM($E$15:E78))</x:f>
       </x:c>
       <x:c r="J78" s="1" t="str">
-        <x:f>IF(A78&gt;$B$4,"Future",IF(A78=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A78,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E78=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A78&gt;$B$4,"Future",IF(A78=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A78,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E78=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2806,7 +2806,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E79" s="6" t="str">
-        <x:f>IF(A79&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A79,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A79&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A79,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F79" s="6" t="str">
         <x:f>IF(A79&gt;=$B$4,"",MAX(D79-E79,0))</x:f>
@@ -2821,7 +2821,7 @@
         <x:f>IF(A79&gt;$B$4,"",SUM($E$15:E79))</x:f>
       </x:c>
       <x:c r="J79" s="1" t="str">
-        <x:f>IF(A79&gt;$B$4,"Future",IF(A79=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A79,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E79=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A79&gt;$B$4,"Future",IF(A79=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A79,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E79=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2841,7 +2841,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E80" s="6" t="str">
-        <x:f>IF(A80&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A80,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A80&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A80,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F80" s="6" t="str">
         <x:f>IF(A80&gt;=$B$4,"",MAX(D80-E80,0))</x:f>
@@ -2856,7 +2856,7 @@
         <x:f>IF(A80&gt;$B$4,"",SUM($E$15:E80))</x:f>
       </x:c>
       <x:c r="J80" s="1" t="str">
-        <x:f>IF(A80&gt;$B$4,"Future",IF(A80=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A80,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E80=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A80&gt;$B$4,"Future",IF(A80=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A80,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E80=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2876,7 +2876,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E81" s="6" t="str">
-        <x:f>IF(A81&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A81,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A81&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A81,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F81" s="6" t="str">
         <x:f>IF(A81&gt;=$B$4,"",MAX(D81-E81,0))</x:f>
@@ -2891,7 +2891,7 @@
         <x:f>IF(A81&gt;$B$4,"",SUM($E$15:E81))</x:f>
       </x:c>
       <x:c r="J81" s="1" t="str">
-        <x:f>IF(A81&gt;$B$4,"Future",IF(A81=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A81,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E81=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A81&gt;$B$4,"Future",IF(A81=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A81,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E81=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2911,7 +2911,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E82" s="6" t="str">
-        <x:f>IF(A82&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A82,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A82&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A82,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F82" s="6" t="str">
         <x:f>IF(A82&gt;=$B$4,"",MAX(D82-E82,0))</x:f>
@@ -2926,7 +2926,7 @@
         <x:f>IF(A82&gt;$B$4,"",SUM($E$15:E82))</x:f>
       </x:c>
       <x:c r="J82" s="1" t="str">
-        <x:f>IF(A82&gt;$B$4,"Future",IF(A82=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A82,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E82=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A82&gt;$B$4,"Future",IF(A82=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A82,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E82=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2946,7 +2946,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E83" s="6" t="str">
-        <x:f>IF(A83&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A83,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A83&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A83,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F83" s="6" t="str">
         <x:f>IF(A83&gt;=$B$4,"",MAX(D83-E83,0))</x:f>
@@ -2961,7 +2961,7 @@
         <x:f>IF(A83&gt;$B$4,"",SUM($E$15:E83))</x:f>
       </x:c>
       <x:c r="J83" s="1" t="str">
-        <x:f>IF(A83&gt;$B$4,"Future",IF(A83=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A83,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E83=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A83&gt;$B$4,"Future",IF(A83=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A83,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E83=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2981,7 +2981,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E84" s="6" t="str">
-        <x:f>IF(A84&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A84,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A84&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A84,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F84" s="6" t="str">
         <x:f>IF(A84&gt;=$B$4,"",MAX(D84-E84,0))</x:f>
@@ -2996,7 +2996,7 @@
         <x:f>IF(A84&gt;$B$4,"",SUM($E$15:E84))</x:f>
       </x:c>
       <x:c r="J84" s="1" t="str">
-        <x:f>IF(A84&gt;$B$4,"Future",IF(A84=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A84,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E84=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A84&gt;$B$4,"Future",IF(A84=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A84,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E84=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3016,7 +3016,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E85" s="6" t="str">
-        <x:f>IF(A85&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A85,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A85&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A85,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F85" s="6" t="str">
         <x:f>IF(A85&gt;=$B$4,"",MAX(D85-E85,0))</x:f>
@@ -3031,7 +3031,7 @@
         <x:f>IF(A85&gt;$B$4,"",SUM($E$15:E85))</x:f>
       </x:c>
       <x:c r="J85" s="1" t="str">
-        <x:f>IF(A85&gt;$B$4,"Future",IF(A85=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A85,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E85=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A85&gt;$B$4,"Future",IF(A85=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A85,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E85=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3051,7 +3051,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E86" s="6" t="str">
-        <x:f>IF(A86&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A86,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A86&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A86,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F86" s="6" t="str">
         <x:f>IF(A86&gt;=$B$4,"",MAX(D86-E86,0))</x:f>
@@ -3066,7 +3066,7 @@
         <x:f>IF(A86&gt;$B$4,"",SUM($E$15:E86))</x:f>
       </x:c>
       <x:c r="J86" s="1" t="str">
-        <x:f>IF(A86&gt;$B$4,"Future",IF(A86=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A86,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E86=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A86&gt;$B$4,"Future",IF(A86=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A86,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E86=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3086,7 +3086,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E87" s="6" t="str">
-        <x:f>IF(A87&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A87,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A87&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A87,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F87" s="6" t="str">
         <x:f>IF(A87&gt;=$B$4,"",MAX(D87-E87,0))</x:f>
@@ -3101,7 +3101,7 @@
         <x:f>IF(A87&gt;$B$4,"",SUM($E$15:E87))</x:f>
       </x:c>
       <x:c r="J87" s="1" t="str">
-        <x:f>IF(A87&gt;$B$4,"Future",IF(A87=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A87,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E87=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A87&gt;$B$4,"Future",IF(A87=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A87,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E87=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3121,7 +3121,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E88" s="6" t="str">
-        <x:f>IF(A88&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A88,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A88&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A88,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F88" s="6" t="str">
         <x:f>IF(A88&gt;=$B$4,"",MAX(D88-E88,0))</x:f>
@@ -3136,7 +3136,7 @@
         <x:f>IF(A88&gt;$B$4,"",SUM($E$15:E88))</x:f>
       </x:c>
       <x:c r="J88" s="1" t="str">
-        <x:f>IF(A88&gt;$B$4,"Future",IF(A88=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A88,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E88=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A88&gt;$B$4,"Future",IF(A88=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A88,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E88=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3156,7 +3156,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E89" s="6" t="str">
-        <x:f>IF(A89&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A89,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A89&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A89,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F89" s="6" t="str">
         <x:f>IF(A89&gt;=$B$4,"",MAX(D89-E89,0))</x:f>
@@ -3171,7 +3171,7 @@
         <x:f>IF(A89&gt;$B$4,"",SUM($E$15:E89))</x:f>
       </x:c>
       <x:c r="J89" s="1" t="str">
-        <x:f>IF(A89&gt;$B$4,"Future",IF(A89=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A89,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E89=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A89&gt;$B$4,"Future",IF(A89=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A89,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E89=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3191,7 +3191,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E90" s="6" t="str">
-        <x:f>IF(A90&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A90,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A90&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A90,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F90" s="6" t="str">
         <x:f>IF(A90&gt;=$B$4,"",MAX(D90-E90,0))</x:f>
@@ -3206,7 +3206,7 @@
         <x:f>IF(A90&gt;$B$4,"",SUM($E$15:E90))</x:f>
       </x:c>
       <x:c r="J90" s="1" t="str">
-        <x:f>IF(A90&gt;$B$4,"Future",IF(A90=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A90,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E90=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A90&gt;$B$4,"Future",IF(A90=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A90,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E90=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3226,7 +3226,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E91" s="6" t="str">
-        <x:f>IF(A91&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A91,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A91&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A91,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F91" s="6" t="str">
         <x:f>IF(A91&gt;=$B$4,"",MAX(D91-E91,0))</x:f>
@@ -3241,7 +3241,7 @@
         <x:f>IF(A91&gt;$B$4,"",SUM($E$15:E91))</x:f>
       </x:c>
       <x:c r="J91" s="1" t="str">
-        <x:f>IF(A91&gt;$B$4,"Future",IF(A91=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A91,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E91=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A91&gt;$B$4,"Future",IF(A91=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A91,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E91=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3261,7 +3261,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E92" s="6" t="str">
-        <x:f>IF(A92&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A92,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A92&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A92,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F92" s="6" t="str">
         <x:f>IF(A92&gt;=$B$4,"",MAX(D92-E92,0))</x:f>
@@ -3276,7 +3276,7 @@
         <x:f>IF(A92&gt;$B$4,"",SUM($E$15:E92))</x:f>
       </x:c>
       <x:c r="J92" s="1" t="str">
-        <x:f>IF(A92&gt;$B$4,"Future",IF(A92=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A92,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E92=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A92&gt;$B$4,"Future",IF(A92=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A92,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E92=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3296,7 +3296,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E93" s="6" t="str">
-        <x:f>IF(A93&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A93,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A93&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A93,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F93" s="6" t="str">
         <x:f>IF(A93&gt;=$B$4,"",MAX(D93-E93,0))</x:f>
@@ -3311,7 +3311,7 @@
         <x:f>IF(A93&gt;$B$4,"",SUM($E$15:E93))</x:f>
       </x:c>
       <x:c r="J93" s="1" t="str">
-        <x:f>IF(A93&gt;$B$4,"Future",IF(A93=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A93,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E93=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A93&gt;$B$4,"Future",IF(A93=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A93,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E93=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3331,7 +3331,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E94" s="6" t="str">
-        <x:f>IF(A94&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A94,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A94&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A94,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F94" s="6" t="str">
         <x:f>IF(A94&gt;=$B$4,"",MAX(D94-E94,0))</x:f>
@@ -3346,7 +3346,7 @@
         <x:f>IF(A94&gt;$B$4,"",SUM($E$15:E94))</x:f>
       </x:c>
       <x:c r="J94" s="1" t="str">
-        <x:f>IF(A94&gt;$B$4,"Future",IF(A94=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A94,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E94=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A94&gt;$B$4,"Future",IF(A94=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A94,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E94=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3366,7 +3366,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E95" s="6" t="str">
-        <x:f>IF(A95&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A95,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A95&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A95,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F95" s="6" t="str">
         <x:f>IF(A95&gt;=$B$4,"",MAX(D95-E95,0))</x:f>
@@ -3381,7 +3381,7 @@
         <x:f>IF(A95&gt;$B$4,"",SUM($E$15:E95))</x:f>
       </x:c>
       <x:c r="J95" s="1" t="str">
-        <x:f>IF(A95&gt;$B$4,"Future",IF(A95=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A95,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E95=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A95&gt;$B$4,"Future",IF(A95=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A95,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E95=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3401,7 +3401,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E96" s="6" t="str">
-        <x:f>IF(A96&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A96,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A96&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A96,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F96" s="6" t="str">
         <x:f>IF(A96&gt;=$B$4,"",MAX(D96-E96,0))</x:f>
@@ -3416,7 +3416,7 @@
         <x:f>IF(A96&gt;$B$4,"",SUM($E$15:E96))</x:f>
       </x:c>
       <x:c r="J96" s="1" t="str">
-        <x:f>IF(A96&gt;$B$4,"Future",IF(A96=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A96,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E96=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A96&gt;$B$4,"Future",IF(A96=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A96,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E96=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3436,7 +3436,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E97" s="6" t="str">
-        <x:f>IF(A97&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A97,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A97&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A97,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F97" s="6" t="str">
         <x:f>IF(A97&gt;=$B$4,"",MAX(D97-E97,0))</x:f>
@@ -3451,7 +3451,7 @@
         <x:f>IF(A97&gt;$B$4,"",SUM($E$15:E97))</x:f>
       </x:c>
       <x:c r="J97" s="1" t="str">
-        <x:f>IF(A97&gt;$B$4,"Future",IF(A97=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A97,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E97=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A97&gt;$B$4,"Future",IF(A97=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A97,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E97=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3471,7 +3471,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E98" s="6" t="str">
-        <x:f>IF(A98&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A98,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A98&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A98,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F98" s="6" t="str">
         <x:f>IF(A98&gt;=$B$4,"",MAX(D98-E98,0))</x:f>
@@ -3486,7 +3486,7 @@
         <x:f>IF(A98&gt;$B$4,"",SUM($E$15:E98))</x:f>
       </x:c>
       <x:c r="J98" s="1" t="str">
-        <x:f>IF(A98&gt;$B$4,"Future",IF(A98=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A98,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E98=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A98&gt;$B$4,"Future",IF(A98=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A98,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E98=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3506,7 +3506,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E99" s="6" t="str">
-        <x:f>IF(A99&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A99,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A99&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A99,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F99" s="6" t="str">
         <x:f>IF(A99&gt;=$B$4,"",MAX(D99-E99,0))</x:f>
@@ -3521,7 +3521,7 @@
         <x:f>IF(A99&gt;$B$4,"",SUM($E$15:E99))</x:f>
       </x:c>
       <x:c r="J99" s="1" t="str">
-        <x:f>IF(A99&gt;$B$4,"Future",IF(A99=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A99,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E99=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A99&gt;$B$4,"Future",IF(A99=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A99,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E99=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3541,7 +3541,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E100" s="6" t="str">
-        <x:f>IF(A100&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A100,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A100&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A100,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F100" s="6" t="str">
         <x:f>IF(A100&gt;=$B$4,"",MAX(D100-E100,0))</x:f>
@@ -3556,7 +3556,7 @@
         <x:f>IF(A100&gt;$B$4,"",SUM($E$15:E100))</x:f>
       </x:c>
       <x:c r="J100" s="1" t="str">
-        <x:f>IF(A100&gt;$B$4,"Future",IF(A100=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A100,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E100=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A100&gt;$B$4,"Future",IF(A100=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A100,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E100=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3576,7 +3576,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E101" s="6" t="str">
-        <x:f>IF(A101&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A101,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A101&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A101,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F101" s="6" t="str">
         <x:f>IF(A101&gt;=$B$4,"",MAX(D101-E101,0))</x:f>
@@ -3591,7 +3591,7 @@
         <x:f>IF(A101&gt;$B$4,"",SUM($E$15:E101))</x:f>
       </x:c>
       <x:c r="J101" s="1" t="str">
-        <x:f>IF(A101&gt;$B$4,"Future",IF(A101=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A101,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E101=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A101&gt;$B$4,"Future",IF(A101=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A101,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E101=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3611,7 +3611,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E102" s="6" t="str">
-        <x:f>IF(A102&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A102,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A102&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A102,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F102" s="6" t="str">
         <x:f>IF(A102&gt;=$B$4,"",MAX(D102-E102,0))</x:f>
@@ -3626,7 +3626,7 @@
         <x:f>IF(A102&gt;$B$4,"",SUM($E$15:E102))</x:f>
       </x:c>
       <x:c r="J102" s="1" t="str">
-        <x:f>IF(A102&gt;$B$4,"Future",IF(A102=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A102,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E102=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A102&gt;$B$4,"Future",IF(A102=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A102,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E102=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3646,7 +3646,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E103" s="6" t="str">
-        <x:f>IF(A103&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A103,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A103&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A103,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F103" s="6" t="str">
         <x:f>IF(A103&gt;=$B$4,"",MAX(D103-E103,0))</x:f>
@@ -3661,7 +3661,7 @@
         <x:f>IF(A103&gt;$B$4,"",SUM($E$15:E103))</x:f>
       </x:c>
       <x:c r="J103" s="1" t="str">
-        <x:f>IF(A103&gt;$B$4,"Future",IF(A103=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A103,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E103=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A103&gt;$B$4,"Future",IF(A103=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A103,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E103=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3681,7 +3681,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E104" s="6" t="str">
-        <x:f>IF(A104&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A104,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A104&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A104,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F104" s="6" t="str">
         <x:f>IF(A104&gt;=$B$4,"",MAX(D104-E104,0))</x:f>
@@ -3696,7 +3696,7 @@
         <x:f>IF(A104&gt;$B$4,"",SUM($E$15:E104))</x:f>
       </x:c>
       <x:c r="J104" s="1" t="str">
-        <x:f>IF(A104&gt;$B$4,"Future",IF(A104=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A104,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E104=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A104&gt;$B$4,"Future",IF(A104=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A104,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E104=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3716,7 +3716,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E105" s="6" t="str">
-        <x:f>IF(A105&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A105,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A105&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A105,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F105" s="6" t="str">
         <x:f>IF(A105&gt;=$B$4,"",MAX(D105-E105,0))</x:f>
@@ -3731,7 +3731,7 @@
         <x:f>IF(A105&gt;$B$4,"",SUM($E$15:E105))</x:f>
       </x:c>
       <x:c r="J105" s="1" t="str">
-        <x:f>IF(A105&gt;$B$4,"Future",IF(A105=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A105,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E105=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A105&gt;$B$4,"Future",IF(A105=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A105,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E105=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3751,7 +3751,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E106" s="6" t="str">
-        <x:f>IF(A106&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A106,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A106&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A106,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F106" s="6" t="str">
         <x:f>IF(A106&gt;=$B$4,"",MAX(D106-E106,0))</x:f>
@@ -3766,7 +3766,7 @@
         <x:f>IF(A106&gt;$B$4,"",SUM($E$15:E106))</x:f>
       </x:c>
       <x:c r="J106" s="1" t="str">
-        <x:f>IF(A106&gt;$B$4,"Future",IF(A106=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A106,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E106=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A106&gt;$B$4,"Future",IF(A106=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A106,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E106=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3786,7 +3786,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E107" s="6" t="str">
-        <x:f>IF(A107&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A107,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A107&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A107,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F107" s="6" t="str">
         <x:f>IF(A107&gt;=$B$4,"",MAX(D107-E107,0))</x:f>
@@ -3801,7 +3801,7 @@
         <x:f>IF(A107&gt;$B$4,"",SUM($E$15:E107))</x:f>
       </x:c>
       <x:c r="J107" s="1" t="str">
-        <x:f>IF(A107&gt;$B$4,"Future",IF(A107=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A107,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E107=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A107&gt;$B$4,"Future",IF(A107=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A107,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E107=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3821,7 +3821,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E108" s="6" t="str">
-        <x:f>IF(A108&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A108,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A108&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A108,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F108" s="6" t="str">
         <x:f>IF(A108&gt;=$B$4,"",MAX(D108-E108,0))</x:f>
@@ -3836,7 +3836,7 @@
         <x:f>IF(A108&gt;$B$4,"",SUM($E$15:E108))</x:f>
       </x:c>
       <x:c r="J108" s="1" t="str">
-        <x:f>IF(A108&gt;$B$4,"Future",IF(A108=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A108,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E108=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A108&gt;$B$4,"Future",IF(A108=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A108,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E108=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3856,7 +3856,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E109" s="6" t="str">
-        <x:f>IF(A109&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A109,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A109&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A109,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F109" s="6" t="str">
         <x:f>IF(A109&gt;=$B$4,"",MAX(D109-E109,0))</x:f>
@@ -3871,7 +3871,7 @@
         <x:f>IF(A109&gt;$B$4,"",SUM($E$15:E109))</x:f>
       </x:c>
       <x:c r="J109" s="1" t="str">
-        <x:f>IF(A109&gt;$B$4,"Future",IF(A109=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A109,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E109=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A109&gt;$B$4,"Future",IF(A109=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A109,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E109=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3891,7 +3891,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E110" s="6" t="str">
-        <x:f>IF(A110&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A110,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A110&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A110,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F110" s="6" t="str">
         <x:f>IF(A110&gt;=$B$4,"",MAX(D110-E110,0))</x:f>
@@ -3906,7 +3906,7 @@
         <x:f>IF(A110&gt;$B$4,"",SUM($E$15:E110))</x:f>
       </x:c>
       <x:c r="J110" s="1" t="str">
-        <x:f>IF(A110&gt;$B$4,"Future",IF(A110=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A110,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E110=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A110&gt;$B$4,"Future",IF(A110=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A110,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E110=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3926,7 +3926,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E111" s="6" t="str">
-        <x:f>IF(A111&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A111,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A111&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A111,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F111" s="6" t="str">
         <x:f>IF(A111&gt;=$B$4,"",MAX(D111-E111,0))</x:f>
@@ -3941,7 +3941,7 @@
         <x:f>IF(A111&gt;$B$4,"",SUM($E$15:E111))</x:f>
       </x:c>
       <x:c r="J111" s="1" t="str">
-        <x:f>IF(A111&gt;$B$4,"Future",IF(A111=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A111,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E111=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A111&gt;$B$4,"Future",IF(A111=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A111,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E111=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3961,7 +3961,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E112" s="6" t="str">
-        <x:f>IF(A112&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A112,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A112&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A112,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F112" s="6" t="str">
         <x:f>IF(A112&gt;=$B$4,"",MAX(D112-E112,0))</x:f>
@@ -3976,7 +3976,7 @@
         <x:f>IF(A112&gt;$B$4,"",SUM($E$15:E112))</x:f>
       </x:c>
       <x:c r="J112" s="1" t="str">
-        <x:f>IF(A112&gt;$B$4,"Future",IF(A112=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A112,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E112=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A112&gt;$B$4,"Future",IF(A112=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A112,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E112=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3996,7 +3996,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E113" s="6" t="str">
-        <x:f>IF(A113&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A113,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A113&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A113,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F113" s="6" t="str">
         <x:f>IF(A113&gt;=$B$4,"",MAX(D113-E113,0))</x:f>
@@ -4011,7 +4011,7 @@
         <x:f>IF(A113&gt;$B$4,"",SUM($E$15:E113))</x:f>
       </x:c>
       <x:c r="J113" s="1" t="str">
-        <x:f>IF(A113&gt;$B$4,"Future",IF(A113=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A113,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E113=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A113&gt;$B$4,"Future",IF(A113=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A113,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E113=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4031,7 +4031,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E114" s="6" t="str">
-        <x:f>IF(A114&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A114,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A114&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A114,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F114" s="6" t="str">
         <x:f>IF(A114&gt;=$B$4,"",MAX(D114-E114,0))</x:f>
@@ -4046,7 +4046,7 @@
         <x:f>IF(A114&gt;$B$4,"",SUM($E$15:E114))</x:f>
       </x:c>
       <x:c r="J114" s="1" t="str">
-        <x:f>IF(A114&gt;$B$4,"Future",IF(A114=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A114,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E114=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A114&gt;$B$4,"Future",IF(A114=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A114,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E114=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4066,7 +4066,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E115" s="6" t="str">
-        <x:f>IF(A115&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A115,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A115&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A115,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F115" s="6" t="str">
         <x:f>IF(A115&gt;=$B$4,"",MAX(D115-E115,0))</x:f>
@@ -4081,7 +4081,7 @@
         <x:f>IF(A115&gt;$B$4,"",SUM($E$15:E115))</x:f>
       </x:c>
       <x:c r="J115" s="1" t="str">
-        <x:f>IF(A115&gt;$B$4,"Future",IF(A115=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A115,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E115=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A115&gt;$B$4,"Future",IF(A115=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A115,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E115=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4101,7 +4101,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E116" s="6" t="str">
-        <x:f>IF(A116&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A116,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A116&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A116,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F116" s="6" t="str">
         <x:f>IF(A116&gt;=$B$4,"",MAX(D116-E116,0))</x:f>
@@ -4116,7 +4116,7 @@
         <x:f>IF(A116&gt;$B$4,"",SUM($E$15:E116))</x:f>
       </x:c>
       <x:c r="J116" s="1" t="str">
-        <x:f>IF(A116&gt;$B$4,"Future",IF(A116=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A116,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E116=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A116&gt;$B$4,"Future",IF(A116=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A116,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E116=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4136,7 +4136,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E117" s="6" t="str">
-        <x:f>IF(A117&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A117,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A117&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A117,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F117" s="6" t="str">
         <x:f>IF(A117&gt;=$B$4,"",MAX(D117-E117,0))</x:f>
@@ -4151,7 +4151,7 @@
         <x:f>IF(A117&gt;$B$4,"",SUM($E$15:E117))</x:f>
       </x:c>
       <x:c r="J117" s="1" t="str">
-        <x:f>IF(A117&gt;$B$4,"Future",IF(A117=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A117,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E117=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A117&gt;$B$4,"Future",IF(A117=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A117,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E117=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4171,7 +4171,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E118" s="6" t="str">
-        <x:f>IF(A118&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A118,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A118&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A118,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F118" s="6" t="str">
         <x:f>IF(A118&gt;=$B$4,"",MAX(D118-E118,0))</x:f>
@@ -4186,7 +4186,7 @@
         <x:f>IF(A118&gt;$B$4,"",SUM($E$15:E118))</x:f>
       </x:c>
       <x:c r="J118" s="1" t="str">
-        <x:f>IF(A118&gt;$B$4,"Future",IF(A118=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A118,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E118=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A118&gt;$B$4,"Future",IF(A118=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A118,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E118=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4206,7 +4206,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E119" s="6" t="str">
-        <x:f>IF(A119&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A119,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A119&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A119,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F119" s="6" t="str">
         <x:f>IF(A119&gt;=$B$4,"",MAX(D119-E119,0))</x:f>
@@ -4221,7 +4221,7 @@
         <x:f>IF(A119&gt;$B$4,"",SUM($E$15:E119))</x:f>
       </x:c>
       <x:c r="J119" s="1" t="str">
-        <x:f>IF(A119&gt;$B$4,"Future",IF(A119=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A119,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E119=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A119&gt;$B$4,"Future",IF(A119=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A119,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E119=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4241,7 +4241,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E120" s="6" t="str">
-        <x:f>IF(A120&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A120,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A120&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A120,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F120" s="6" t="str">
         <x:f>IF(A120&gt;=$B$4,"",MAX(D120-E120,0))</x:f>
@@ -4256,7 +4256,7 @@
         <x:f>IF(A120&gt;$B$4,"",SUM($E$15:E120))</x:f>
       </x:c>
       <x:c r="J120" s="1" t="str">
-        <x:f>IF(A120&gt;$B$4,"Future",IF(A120=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A120,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E120=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A120&gt;$B$4,"Future",IF(A120=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A120,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E120=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4276,7 +4276,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E121" s="6" t="str">
-        <x:f>IF(A121&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A121,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A121&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A121,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F121" s="6" t="str">
         <x:f>IF(A121&gt;=$B$4,"",MAX(D121-E121,0))</x:f>
@@ -4291,7 +4291,7 @@
         <x:f>IF(A121&gt;$B$4,"",SUM($E$15:E121))</x:f>
       </x:c>
       <x:c r="J121" s="1" t="str">
-        <x:f>IF(A121&gt;$B$4,"Future",IF(A121=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A121,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E121=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A121&gt;$B$4,"Future",IF(A121=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A121,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E121=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4311,7 +4311,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E122" s="6" t="str">
-        <x:f>IF(A122&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A122,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A122&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A122,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F122" s="6" t="str">
         <x:f>IF(A122&gt;=$B$4,"",MAX(D122-E122,0))</x:f>
@@ -4326,7 +4326,7 @@
         <x:f>IF(A122&gt;$B$4,"",SUM($E$15:E122))</x:f>
       </x:c>
       <x:c r="J122" s="1" t="str">
-        <x:f>IF(A122&gt;$B$4,"Future",IF(A122=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A122,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E122=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A122&gt;$B$4,"Future",IF(A122=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A122,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E122=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4346,7 +4346,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E123" s="6" t="str">
-        <x:f>IF(A123&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A123,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A123&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A123,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F123" s="6" t="str">
         <x:f>IF(A123&gt;=$B$4,"",MAX(D123-E123,0))</x:f>
@@ -4361,7 +4361,7 @@
         <x:f>IF(A123&gt;$B$4,"",SUM($E$15:E123))</x:f>
       </x:c>
       <x:c r="J123" s="1" t="str">
-        <x:f>IF(A123&gt;$B$4,"Future",IF(A123=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A123,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E123=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A123&gt;$B$4,"Future",IF(A123=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A123,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E123=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4381,7 +4381,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E124" s="6" t="str">
-        <x:f>IF(A124&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A124,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A124&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A124,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F124" s="6" t="str">
         <x:f>IF(A124&gt;=$B$4,"",MAX(D124-E124,0))</x:f>
@@ -4396,7 +4396,7 @@
         <x:f>IF(A124&gt;$B$4,"",SUM($E$15:E124))</x:f>
       </x:c>
       <x:c r="J124" s="1" t="str">
-        <x:f>IF(A124&gt;$B$4,"Future",IF(A124=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A124,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E124=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A124&gt;$B$4,"Future",IF(A124=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A124,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E124=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4416,7 +4416,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E125" s="6" t="str">
-        <x:f>IF(A125&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A125,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A125&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A125,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F125" s="6" t="str">
         <x:f>IF(A125&gt;=$B$4,"",MAX(D125-E125,0))</x:f>
@@ -4431,7 +4431,7 @@
         <x:f>IF(A125&gt;$B$4,"",SUM($E$15:E125))</x:f>
       </x:c>
       <x:c r="J125" s="1" t="str">
-        <x:f>IF(A125&gt;$B$4,"Future",IF(A125=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A125,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E125=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A125&gt;$B$4,"Future",IF(A125=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A125,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E125=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4451,7 +4451,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E126" s="6" t="str">
-        <x:f>IF(A126&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A126,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A126&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A126,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F126" s="6" t="str">
         <x:f>IF(A126&gt;=$B$4,"",MAX(D126-E126,0))</x:f>
@@ -4466,7 +4466,7 @@
         <x:f>IF(A126&gt;$B$4,"",SUM($E$15:E126))</x:f>
       </x:c>
       <x:c r="J126" s="1" t="str">
-        <x:f>IF(A126&gt;$B$4,"Future",IF(A126=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A126,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E126=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A126&gt;$B$4,"Future",IF(A126=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A126,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E126=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4486,7 +4486,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E127" s="6" t="str">
-        <x:f>IF(A127&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A127,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A127&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A127,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F127" s="6" t="str">
         <x:f>IF(A127&gt;=$B$4,"",MAX(D127-E127,0))</x:f>
@@ -4501,7 +4501,7 @@
         <x:f>IF(A127&gt;$B$4,"",SUM($E$15:E127))</x:f>
       </x:c>
       <x:c r="J127" s="1" t="str">
-        <x:f>IF(A127&gt;$B$4,"Future",IF(A127=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A127,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E127=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A127&gt;$B$4,"Future",IF(A127=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A127,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E127=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4521,7 +4521,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E128" s="6" t="str">
-        <x:f>IF(A128&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A128,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A128&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A128,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F128" s="6" t="str">
         <x:f>IF(A128&gt;=$B$4,"",MAX(D128-E128,0))</x:f>
@@ -4536,7 +4536,7 @@
         <x:f>IF(A128&gt;$B$4,"",SUM($E$15:E128))</x:f>
       </x:c>
       <x:c r="J128" s="1" t="str">
-        <x:f>IF(A128&gt;$B$4,"Future",IF(A128=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A128,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E128=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A128&gt;$B$4,"Future",IF(A128=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A128,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E128=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4556,7 +4556,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E129" s="6" t="str">
-        <x:f>IF(A129&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A129,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A129&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A129,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F129" s="6" t="str">
         <x:f>IF(A129&gt;=$B$4,"",MAX(D129-E129,0))</x:f>
@@ -4571,7 +4571,7 @@
         <x:f>IF(A129&gt;$B$4,"",SUM($E$15:E129))</x:f>
       </x:c>
       <x:c r="J129" s="1" t="str">
-        <x:f>IF(A129&gt;$B$4,"Future",IF(A129=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A129,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E129=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A129&gt;$B$4,"Future",IF(A129=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A129,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E129=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4591,7 +4591,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E130" s="6" t="str">
-        <x:f>IF(A130&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$2,'Sessions'!$B$2:$B$2,A130,'Sessions'!$G$2:$G$2,"completed")/60)</x:f>
+        <x:f>IF(A130&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A130,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
       </x:c>
       <x:c r="F130" s="6" t="str">
         <x:f>IF(A130&gt;=$B$4,"",MAX(D130-E130,0))</x:f>
@@ -4606,7 +4606,7 @@
         <x:f>IF(A130&gt;$B$4,"",SUM($E$15:E130))</x:f>
       </x:c>
       <x:c r="J130" s="1" t="str">
-        <x:f>IF(A130&gt;$B$4,"Future",IF(A130=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$2,A130,'Sessions'!$G$2:$G$2,"needs_confirmation")&gt;0,"Uncertain time",IF(E130=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A130&gt;$B$4,"Future",IF(A130=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A130,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E130=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4730,7 +4730,7 @@
       </x:c>
       <x:c r="D8" s="6" t="n">
         <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A8)</x:f>
-        <x:v>0</x:v>
+        <x:v>1.9563888888899998</x:v>
       </x:c>
       <x:c r="E8" s="6" t="n">
         <x:f>MAX(C8-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A8,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
@@ -4742,11 +4742,11 @@
       </x:c>
       <x:c r="G8" s="6" t="n">
         <x:f>MAX(B8-D8,0)</x:f>
-        <x:v>32</x:v>
+        <x:v>30.04361111111</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
         <x:f>IF(B8=0,0,D8/B8)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.061137152777812495</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
@@ -5349,6 +5349,162 @@
         <x:v>Learner explicitly said lets start; initial lesson and prediction task; Migrated during platform setup; actual stop time needed; no duration assumed</x:v>
       </x:c>
     </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="A3" s="1" t="str">
+        <x:v>SQL-20261015T093101</x:v>
+      </x:c>
+      <x:c r="B3" s="7" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="C3" s="1" t="str">
+        <x:v>SQL: LEFT JOIN and unmatched rows</x:v>
+      </x:c>
+      <x:c r="D3" s="1" t="str">
+        <x:v>IST 2026-10-15 09:31:01</x:v>
+      </x:c>
+      <x:c r="E3" s="1" t="str">
+        <x:v>IST 2026-10-15 09:32:05</x:v>
+      </x:c>
+      <x:c r="F3" s="1" t="n">
+        <x:v>1.0666666667</x:v>
+      </x:c>
+      <x:c r="G3" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H3" s="1" t="str">
+        <x:v>Explicit start and pause; clock timestamps; 1 minute 4 seconds; prediction not answered; earlier uncertain interval excluded</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="1" t="str">
+        <x:v>SQL-20261015T100201</x:v>
+      </x:c>
+      <x:c r="B4" s="7" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="C4" s="1" t="str">
+        <x:v>SQL: LEFT JOIN and unmatched rows</x:v>
+      </x:c>
+      <x:c r="D4" s="1" t="str">
+        <x:v>IST 2026-10-15 10:02:01</x:v>
+      </x:c>
+      <x:c r="E4" s="1" t="str">
+        <x:v>IST 2026-10-15 10:21:23</x:v>
+      </x:c>
+      <x:c r="F4" s="1" t="n">
+        <x:v>19.3666666667</x:v>
+      </x:c>
+      <x:c r="G4" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H4" s="1" t="str">
+        <x:v>Explicit start and puase interpreted as pause; clock timestamps; 19 minutes 22 seconds; SQL attempts preserved; actual PostgreSQL output pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="1" t="str">
+        <x:v>SQL-20261015T103328</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="C5" s="1" t="str">
+        <x:v>SQL: joins counting grouping and SUM setup</x:v>
+      </x:c>
+      <x:c r="D5" s="1" t="str">
+        <x:v>IST 2026-10-15 10:33:28</x:v>
+      </x:c>
+      <x:c r="E5" s="1" t="str">
+        <x:v>IST 2026-10-15 11:43:58</x:v>
+      </x:c>
+      <x:c r="F5" s="1" t="n">
+        <x:v>70.5</x:v>
+      </x:c>
+      <x:c r="G5" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H5" s="1" t="str">
+        <x:v>Explicit pause sql and start python; clock timestamp; SQL-003 setup remains pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" s="1" t="str">
+        <x:v>PY-20261015T114358</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="C6" s="1" t="str">
+        <x:v>Python: dictionary records baseline</x:v>
+      </x:c>
+      <x:c r="D6" s="1" t="str">
+        <x:v>IST 2026-10-15 11:43:58</x:v>
+      </x:c>
+      <x:c r="E6" s="1" t="str">
+        <x:v>IST 2026-10-15 11:56:38</x:v>
+      </x:c>
+      <x:c r="F6" s="1" t="n">
+        <x:v>12.6666666667</x:v>
+      </x:c>
+      <x:c r="G6" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H6" s="1" t="str">
+        <x:v>Explicit pause; clock timestamps; 12 minutes 40 seconds; partial local attempt preserved and not yet reviewed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="A7" s="1" t="str">
+        <x:v>PY-20261015T121152</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="C7" s="1" t="str">
+        <x:v>Python: record cleaning</x:v>
+      </x:c>
+      <x:c r="D7" s="1" t="str">
+        <x:v>IST 2026-10-15 12:11:52</x:v>
+      </x:c>
+      <x:c r="E7" s="1" t="str">
+        <x:v>IST 2026-10-15 12:18:28</x:v>
+      </x:c>
+      <x:c r="F7" s="1" t="n">
+        <x:v>6.6</x:v>
+      </x:c>
+      <x:c r="G7" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H7" s="1" t="str">
+        <x:v>Explicit pause; clock timestamps; 6 minutes 36 seconds; review hints and revised draft saved at boundary</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="22" customHeight="1">
+      <x:c r="A8" s="1" t="str">
+        <x:v>PY-20261015T124142</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="C8" s="1" t="str">
+        <x:v>Python: record cleaning</x:v>
+      </x:c>
+      <x:c r="D8" s="1" t="str">
+        <x:v>IST 2026-10-15 12:41:42</x:v>
+      </x:c>
+      <x:c r="E8" s="1" t="str">
+        <x:v>IST 2026-10-15 12:48:53</x:v>
+      </x:c>
+      <x:c r="F8" s="1" t="n">
+        <x:v>7.1833333333</x:v>
+      </x:c>
+      <x:c r="G8" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H8" s="1" t="str">
+        <x:v>Explicit pause at first request; clock timestamp; 7 minutes 11 seconds; learner requested dictionary foundations; repeated pause does not extend interval</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Save dictionary practice and updated study checkpoint
</commit_message>
<xml_diff>
--- a/outputs/study-tracker/study-hours.xlsx
+++ b/outputs/study-tracker/study-hours.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="R554b80bc1bf34e9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="Ra7b7af1ebfd14894"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="Rd6e101ea294d4502"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="R5b131d87a3eb4221"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="R6125572898c64ece"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="Rc300a46b03f14ebd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -362,7 +362,7 @@
       </x:c>
       <x:c r="E4" s="6" t="n">
         <x:f>SUM(E15:E130)</x:f>
-        <x:v>1.9563888888899998</x:v>
+        <x:v>2.8094444444449995</x:v>
       </x:c>
       <x:c r="F4" s="1"/>
       <x:c r="G4" s="1"/>
@@ -442,7 +442,7 @@
       </x:c>
       <x:c r="E8" s="6" t="n">
         <x:f>MAX(SUMIFS(D15:D130,A15:A130,B4)-SUMIFS(E15:E130,A15:A130,B4),0)</x:f>
-        <x:v>4.04361111111</x:v>
+        <x:v>3.1905555555550005</x:v>
       </x:c>
       <x:c r="F8" s="1"/>
       <x:c r="G8" s="1"/>
@@ -564,8 +564,8 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E15" s="6" t="n">
-        <x:f>IF(A15&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A15,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
-        <x:v>1.9563888888899998</x:v>
+        <x:f>IF(A15&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A15,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:v>2.8094444444449995</x:v>
       </x:c>
       <x:c r="F15" s="6" t="str">
         <x:f>IF(A15&gt;=$B$4,"",MAX(D15-E15,0))</x:f>
@@ -578,10 +578,10 @@
       </x:c>
       <x:c r="I15" s="6" t="n">
         <x:f>IF(A15&gt;$B$4,"",SUM($E$15:E15))</x:f>
-        <x:v>1.9563888888899998</x:v>
+        <x:v>2.8094444444449995</x:v>
       </x:c>
       <x:c r="J15" s="1" t="str">
-        <x:f>IF(A15&gt;$B$4,"Future",IF(A15=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A15,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E15=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A15&gt;$B$4,"Future",IF(A15=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A15,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E15=0,"No confirmed time","Logged"))))</x:f>
         <x:v>In progress</x:v>
       </x:c>
     </x:row>
@@ -601,7 +601,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E16" s="6" t="str">
-        <x:f>IF(A16&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A16,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A16&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A16,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F16" s="6" t="str">
         <x:f>IF(A16&gt;=$B$4,"",MAX(D16-E16,0))</x:f>
@@ -616,7 +616,7 @@
         <x:f>IF(A16&gt;$B$4,"",SUM($E$15:E16))</x:f>
       </x:c>
       <x:c r="J16" s="1" t="str">
-        <x:f>IF(A16&gt;$B$4,"Future",IF(A16=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A16,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E16=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A16&gt;$B$4,"Future",IF(A16=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A16,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E16=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -636,7 +636,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E17" s="6" t="str">
-        <x:f>IF(A17&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A17,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A17&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A17,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F17" s="6" t="str">
         <x:f>IF(A17&gt;=$B$4,"",MAX(D17-E17,0))</x:f>
@@ -651,7 +651,7 @@
         <x:f>IF(A17&gt;$B$4,"",SUM($E$15:E17))</x:f>
       </x:c>
       <x:c r="J17" s="1" t="str">
-        <x:f>IF(A17&gt;$B$4,"Future",IF(A17=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A17,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E17=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A17&gt;$B$4,"Future",IF(A17=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A17,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E17=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -671,7 +671,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E18" s="6" t="str">
-        <x:f>IF(A18&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A18,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A18&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A18,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F18" s="6" t="str">
         <x:f>IF(A18&gt;=$B$4,"",MAX(D18-E18,0))</x:f>
@@ -686,7 +686,7 @@
         <x:f>IF(A18&gt;$B$4,"",SUM($E$15:E18))</x:f>
       </x:c>
       <x:c r="J18" s="1" t="str">
-        <x:f>IF(A18&gt;$B$4,"Future",IF(A18=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A18,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E18=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A18&gt;$B$4,"Future",IF(A18=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A18,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E18=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -706,7 +706,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E19" s="6" t="str">
-        <x:f>IF(A19&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A19,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A19&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A19,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F19" s="6" t="str">
         <x:f>IF(A19&gt;=$B$4,"",MAX(D19-E19,0))</x:f>
@@ -721,7 +721,7 @@
         <x:f>IF(A19&gt;$B$4,"",SUM($E$15:E19))</x:f>
       </x:c>
       <x:c r="J19" s="1" t="str">
-        <x:f>IF(A19&gt;$B$4,"Future",IF(A19=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A19,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E19=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A19&gt;$B$4,"Future",IF(A19=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A19,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E19=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -741,7 +741,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E20" s="6" t="str">
-        <x:f>IF(A20&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A20,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A20&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A20,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F20" s="6" t="str">
         <x:f>IF(A20&gt;=$B$4,"",MAX(D20-E20,0))</x:f>
@@ -756,7 +756,7 @@
         <x:f>IF(A20&gt;$B$4,"",SUM($E$15:E20))</x:f>
       </x:c>
       <x:c r="J20" s="1" t="str">
-        <x:f>IF(A20&gt;$B$4,"Future",IF(A20=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A20,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E20=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A20&gt;$B$4,"Future",IF(A20=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A20,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E20=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -776,7 +776,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E21" s="6" t="str">
-        <x:f>IF(A21&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A21,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A21&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A21,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F21" s="6" t="str">
         <x:f>IF(A21&gt;=$B$4,"",MAX(D21-E21,0))</x:f>
@@ -791,7 +791,7 @@
         <x:f>IF(A21&gt;$B$4,"",SUM($E$15:E21))</x:f>
       </x:c>
       <x:c r="J21" s="1" t="str">
-        <x:f>IF(A21&gt;$B$4,"Future",IF(A21=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A21,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E21=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A21&gt;$B$4,"Future",IF(A21=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A21,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E21=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -811,7 +811,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E22" s="6" t="str">
-        <x:f>IF(A22&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A22,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A22&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A22,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F22" s="6" t="str">
         <x:f>IF(A22&gt;=$B$4,"",MAX(D22-E22,0))</x:f>
@@ -826,7 +826,7 @@
         <x:f>IF(A22&gt;$B$4,"",SUM($E$15:E22))</x:f>
       </x:c>
       <x:c r="J22" s="1" t="str">
-        <x:f>IF(A22&gt;$B$4,"Future",IF(A22=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A22,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E22=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A22&gt;$B$4,"Future",IF(A22=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A22,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E22=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -846,7 +846,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E23" s="6" t="str">
-        <x:f>IF(A23&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A23,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A23&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A23,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F23" s="6" t="str">
         <x:f>IF(A23&gt;=$B$4,"",MAX(D23-E23,0))</x:f>
@@ -861,7 +861,7 @@
         <x:f>IF(A23&gt;$B$4,"",SUM($E$15:E23))</x:f>
       </x:c>
       <x:c r="J23" s="1" t="str">
-        <x:f>IF(A23&gt;$B$4,"Future",IF(A23=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A23,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E23=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A23&gt;$B$4,"Future",IF(A23=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A23,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E23=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -881,7 +881,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E24" s="6" t="str">
-        <x:f>IF(A24&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A24,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A24&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A24,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F24" s="6" t="str">
         <x:f>IF(A24&gt;=$B$4,"",MAX(D24-E24,0))</x:f>
@@ -896,7 +896,7 @@
         <x:f>IF(A24&gt;$B$4,"",SUM($E$15:E24))</x:f>
       </x:c>
       <x:c r="J24" s="1" t="str">
-        <x:f>IF(A24&gt;$B$4,"Future",IF(A24=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A24,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E24=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A24&gt;$B$4,"Future",IF(A24=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A24,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E24=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -916,7 +916,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E25" s="6" t="str">
-        <x:f>IF(A25&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A25,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A25&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A25,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F25" s="6" t="str">
         <x:f>IF(A25&gt;=$B$4,"",MAX(D25-E25,0))</x:f>
@@ -931,7 +931,7 @@
         <x:f>IF(A25&gt;$B$4,"",SUM($E$15:E25))</x:f>
       </x:c>
       <x:c r="J25" s="1" t="str">
-        <x:f>IF(A25&gt;$B$4,"Future",IF(A25=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A25,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E25=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A25&gt;$B$4,"Future",IF(A25=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A25,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E25=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -951,7 +951,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E26" s="6" t="str">
-        <x:f>IF(A26&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A26,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A26&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A26,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F26" s="6" t="str">
         <x:f>IF(A26&gt;=$B$4,"",MAX(D26-E26,0))</x:f>
@@ -966,7 +966,7 @@
         <x:f>IF(A26&gt;$B$4,"",SUM($E$15:E26))</x:f>
       </x:c>
       <x:c r="J26" s="1" t="str">
-        <x:f>IF(A26&gt;$B$4,"Future",IF(A26=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A26,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E26=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A26&gt;$B$4,"Future",IF(A26=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A26,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E26=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -986,7 +986,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E27" s="6" t="str">
-        <x:f>IF(A27&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A27,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A27&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A27,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F27" s="6" t="str">
         <x:f>IF(A27&gt;=$B$4,"",MAX(D27-E27,0))</x:f>
@@ -1001,7 +1001,7 @@
         <x:f>IF(A27&gt;$B$4,"",SUM($E$15:E27))</x:f>
       </x:c>
       <x:c r="J27" s="1" t="str">
-        <x:f>IF(A27&gt;$B$4,"Future",IF(A27=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A27,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E27=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A27&gt;$B$4,"Future",IF(A27=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A27,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E27=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1021,7 +1021,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E28" s="6" t="str">
-        <x:f>IF(A28&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A28,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A28&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A28,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F28" s="6" t="str">
         <x:f>IF(A28&gt;=$B$4,"",MAX(D28-E28,0))</x:f>
@@ -1036,7 +1036,7 @@
         <x:f>IF(A28&gt;$B$4,"",SUM($E$15:E28))</x:f>
       </x:c>
       <x:c r="J28" s="1" t="str">
-        <x:f>IF(A28&gt;$B$4,"Future",IF(A28=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A28,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E28=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A28&gt;$B$4,"Future",IF(A28=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A28,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E28=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1056,7 +1056,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E29" s="6" t="str">
-        <x:f>IF(A29&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A29,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A29&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A29,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F29" s="6" t="str">
         <x:f>IF(A29&gt;=$B$4,"",MAX(D29-E29,0))</x:f>
@@ -1071,7 +1071,7 @@
         <x:f>IF(A29&gt;$B$4,"",SUM($E$15:E29))</x:f>
       </x:c>
       <x:c r="J29" s="1" t="str">
-        <x:f>IF(A29&gt;$B$4,"Future",IF(A29=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A29,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E29=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A29&gt;$B$4,"Future",IF(A29=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A29,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E29=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1091,7 +1091,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E30" s="6" t="str">
-        <x:f>IF(A30&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A30,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A30&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A30,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F30" s="6" t="str">
         <x:f>IF(A30&gt;=$B$4,"",MAX(D30-E30,0))</x:f>
@@ -1106,7 +1106,7 @@
         <x:f>IF(A30&gt;$B$4,"",SUM($E$15:E30))</x:f>
       </x:c>
       <x:c r="J30" s="1" t="str">
-        <x:f>IF(A30&gt;$B$4,"Future",IF(A30=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A30,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E30=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A30&gt;$B$4,"Future",IF(A30=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A30,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E30=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1126,7 +1126,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E31" s="6" t="str">
-        <x:f>IF(A31&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A31,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A31&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A31,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F31" s="6" t="str">
         <x:f>IF(A31&gt;=$B$4,"",MAX(D31-E31,0))</x:f>
@@ -1141,7 +1141,7 @@
         <x:f>IF(A31&gt;$B$4,"",SUM($E$15:E31))</x:f>
       </x:c>
       <x:c r="J31" s="1" t="str">
-        <x:f>IF(A31&gt;$B$4,"Future",IF(A31=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A31,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E31=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A31&gt;$B$4,"Future",IF(A31=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A31,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E31=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1161,7 +1161,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E32" s="6" t="str">
-        <x:f>IF(A32&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A32,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A32&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A32,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F32" s="6" t="str">
         <x:f>IF(A32&gt;=$B$4,"",MAX(D32-E32,0))</x:f>
@@ -1176,7 +1176,7 @@
         <x:f>IF(A32&gt;$B$4,"",SUM($E$15:E32))</x:f>
       </x:c>
       <x:c r="J32" s="1" t="str">
-        <x:f>IF(A32&gt;$B$4,"Future",IF(A32=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A32,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E32=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A32&gt;$B$4,"Future",IF(A32=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A32,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E32=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1196,7 +1196,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E33" s="6" t="str">
-        <x:f>IF(A33&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A33,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A33&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A33,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F33" s="6" t="str">
         <x:f>IF(A33&gt;=$B$4,"",MAX(D33-E33,0))</x:f>
@@ -1211,7 +1211,7 @@
         <x:f>IF(A33&gt;$B$4,"",SUM($E$15:E33))</x:f>
       </x:c>
       <x:c r="J33" s="1" t="str">
-        <x:f>IF(A33&gt;$B$4,"Future",IF(A33=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A33,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E33=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A33&gt;$B$4,"Future",IF(A33=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A33,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E33=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1231,7 +1231,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E34" s="6" t="str">
-        <x:f>IF(A34&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A34,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A34&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A34,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F34" s="6" t="str">
         <x:f>IF(A34&gt;=$B$4,"",MAX(D34-E34,0))</x:f>
@@ -1246,7 +1246,7 @@
         <x:f>IF(A34&gt;$B$4,"",SUM($E$15:E34))</x:f>
       </x:c>
       <x:c r="J34" s="1" t="str">
-        <x:f>IF(A34&gt;$B$4,"Future",IF(A34=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A34,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E34=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A34&gt;$B$4,"Future",IF(A34=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A34,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E34=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1266,7 +1266,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E35" s="6" t="str">
-        <x:f>IF(A35&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A35,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A35&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A35,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F35" s="6" t="str">
         <x:f>IF(A35&gt;=$B$4,"",MAX(D35-E35,0))</x:f>
@@ -1281,7 +1281,7 @@
         <x:f>IF(A35&gt;$B$4,"",SUM($E$15:E35))</x:f>
       </x:c>
       <x:c r="J35" s="1" t="str">
-        <x:f>IF(A35&gt;$B$4,"Future",IF(A35=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A35,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E35=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A35&gt;$B$4,"Future",IF(A35=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A35,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E35=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1301,7 +1301,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E36" s="6" t="str">
-        <x:f>IF(A36&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A36,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A36&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A36,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F36" s="6" t="str">
         <x:f>IF(A36&gt;=$B$4,"",MAX(D36-E36,0))</x:f>
@@ -1316,7 +1316,7 @@
         <x:f>IF(A36&gt;$B$4,"",SUM($E$15:E36))</x:f>
       </x:c>
       <x:c r="J36" s="1" t="str">
-        <x:f>IF(A36&gt;$B$4,"Future",IF(A36=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A36,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E36=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A36&gt;$B$4,"Future",IF(A36=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A36,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E36=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1336,7 +1336,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E37" s="6" t="str">
-        <x:f>IF(A37&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A37,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A37&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A37,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F37" s="6" t="str">
         <x:f>IF(A37&gt;=$B$4,"",MAX(D37-E37,0))</x:f>
@@ -1351,7 +1351,7 @@
         <x:f>IF(A37&gt;$B$4,"",SUM($E$15:E37))</x:f>
       </x:c>
       <x:c r="J37" s="1" t="str">
-        <x:f>IF(A37&gt;$B$4,"Future",IF(A37=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A37,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E37=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A37&gt;$B$4,"Future",IF(A37=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A37,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E37=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1371,7 +1371,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E38" s="6" t="str">
-        <x:f>IF(A38&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A38,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A38&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A38,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F38" s="6" t="str">
         <x:f>IF(A38&gt;=$B$4,"",MAX(D38-E38,0))</x:f>
@@ -1386,7 +1386,7 @@
         <x:f>IF(A38&gt;$B$4,"",SUM($E$15:E38))</x:f>
       </x:c>
       <x:c r="J38" s="1" t="str">
-        <x:f>IF(A38&gt;$B$4,"Future",IF(A38=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A38,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E38=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A38&gt;$B$4,"Future",IF(A38=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A38,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E38=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1406,7 +1406,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E39" s="6" t="str">
-        <x:f>IF(A39&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A39,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A39&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A39,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F39" s="6" t="str">
         <x:f>IF(A39&gt;=$B$4,"",MAX(D39-E39,0))</x:f>
@@ -1421,7 +1421,7 @@
         <x:f>IF(A39&gt;$B$4,"",SUM($E$15:E39))</x:f>
       </x:c>
       <x:c r="J39" s="1" t="str">
-        <x:f>IF(A39&gt;$B$4,"Future",IF(A39=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A39,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E39=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A39&gt;$B$4,"Future",IF(A39=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A39,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E39=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1441,7 +1441,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E40" s="6" t="str">
-        <x:f>IF(A40&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A40,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A40&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A40,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F40" s="6" t="str">
         <x:f>IF(A40&gt;=$B$4,"",MAX(D40-E40,0))</x:f>
@@ -1456,7 +1456,7 @@
         <x:f>IF(A40&gt;$B$4,"",SUM($E$15:E40))</x:f>
       </x:c>
       <x:c r="J40" s="1" t="str">
-        <x:f>IF(A40&gt;$B$4,"Future",IF(A40=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A40,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E40=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A40&gt;$B$4,"Future",IF(A40=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A40,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E40=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1476,7 +1476,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E41" s="6" t="str">
-        <x:f>IF(A41&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A41,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A41&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A41,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F41" s="6" t="str">
         <x:f>IF(A41&gt;=$B$4,"",MAX(D41-E41,0))</x:f>
@@ -1491,7 +1491,7 @@
         <x:f>IF(A41&gt;$B$4,"",SUM($E$15:E41))</x:f>
       </x:c>
       <x:c r="J41" s="1" t="str">
-        <x:f>IF(A41&gt;$B$4,"Future",IF(A41=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A41,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E41=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A41&gt;$B$4,"Future",IF(A41=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A41,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E41=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1511,7 +1511,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E42" s="6" t="str">
-        <x:f>IF(A42&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A42,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A42&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A42,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F42" s="6" t="str">
         <x:f>IF(A42&gt;=$B$4,"",MAX(D42-E42,0))</x:f>
@@ -1526,7 +1526,7 @@
         <x:f>IF(A42&gt;$B$4,"",SUM($E$15:E42))</x:f>
       </x:c>
       <x:c r="J42" s="1" t="str">
-        <x:f>IF(A42&gt;$B$4,"Future",IF(A42=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A42,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E42=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A42&gt;$B$4,"Future",IF(A42=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A42,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E42=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1546,7 +1546,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E43" s="6" t="str">
-        <x:f>IF(A43&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A43,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A43&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A43,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F43" s="6" t="str">
         <x:f>IF(A43&gt;=$B$4,"",MAX(D43-E43,0))</x:f>
@@ -1561,7 +1561,7 @@
         <x:f>IF(A43&gt;$B$4,"",SUM($E$15:E43))</x:f>
       </x:c>
       <x:c r="J43" s="1" t="str">
-        <x:f>IF(A43&gt;$B$4,"Future",IF(A43=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A43,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E43=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A43&gt;$B$4,"Future",IF(A43=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A43,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E43=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1581,7 +1581,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E44" s="6" t="str">
-        <x:f>IF(A44&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A44,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A44&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A44,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F44" s="6" t="str">
         <x:f>IF(A44&gt;=$B$4,"",MAX(D44-E44,0))</x:f>
@@ -1596,7 +1596,7 @@
         <x:f>IF(A44&gt;$B$4,"",SUM($E$15:E44))</x:f>
       </x:c>
       <x:c r="J44" s="1" t="str">
-        <x:f>IF(A44&gt;$B$4,"Future",IF(A44=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A44,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E44=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A44&gt;$B$4,"Future",IF(A44=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A44,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E44=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1616,7 +1616,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E45" s="6" t="str">
-        <x:f>IF(A45&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A45,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A45&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A45,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F45" s="6" t="str">
         <x:f>IF(A45&gt;=$B$4,"",MAX(D45-E45,0))</x:f>
@@ -1631,7 +1631,7 @@
         <x:f>IF(A45&gt;$B$4,"",SUM($E$15:E45))</x:f>
       </x:c>
       <x:c r="J45" s="1" t="str">
-        <x:f>IF(A45&gt;$B$4,"Future",IF(A45=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A45,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E45=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A45&gt;$B$4,"Future",IF(A45=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A45,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E45=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1651,7 +1651,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E46" s="6" t="str">
-        <x:f>IF(A46&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A46,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A46&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A46,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F46" s="6" t="str">
         <x:f>IF(A46&gt;=$B$4,"",MAX(D46-E46,0))</x:f>
@@ -1666,7 +1666,7 @@
         <x:f>IF(A46&gt;$B$4,"",SUM($E$15:E46))</x:f>
       </x:c>
       <x:c r="J46" s="1" t="str">
-        <x:f>IF(A46&gt;$B$4,"Future",IF(A46=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A46,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E46=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A46&gt;$B$4,"Future",IF(A46=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A46,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E46=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1686,7 +1686,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E47" s="6" t="str">
-        <x:f>IF(A47&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A47,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A47&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A47,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F47" s="6" t="str">
         <x:f>IF(A47&gt;=$B$4,"",MAX(D47-E47,0))</x:f>
@@ -1701,7 +1701,7 @@
         <x:f>IF(A47&gt;$B$4,"",SUM($E$15:E47))</x:f>
       </x:c>
       <x:c r="J47" s="1" t="str">
-        <x:f>IF(A47&gt;$B$4,"Future",IF(A47=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A47,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E47=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A47&gt;$B$4,"Future",IF(A47=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A47,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E47=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1721,7 +1721,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E48" s="6" t="str">
-        <x:f>IF(A48&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A48,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A48&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A48,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F48" s="6" t="str">
         <x:f>IF(A48&gt;=$B$4,"",MAX(D48-E48,0))</x:f>
@@ -1736,7 +1736,7 @@
         <x:f>IF(A48&gt;$B$4,"",SUM($E$15:E48))</x:f>
       </x:c>
       <x:c r="J48" s="1" t="str">
-        <x:f>IF(A48&gt;$B$4,"Future",IF(A48=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A48,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E48=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A48&gt;$B$4,"Future",IF(A48=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A48,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E48=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1756,7 +1756,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E49" s="6" t="str">
-        <x:f>IF(A49&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A49,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A49&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A49,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F49" s="6" t="str">
         <x:f>IF(A49&gt;=$B$4,"",MAX(D49-E49,0))</x:f>
@@ -1771,7 +1771,7 @@
         <x:f>IF(A49&gt;$B$4,"",SUM($E$15:E49))</x:f>
       </x:c>
       <x:c r="J49" s="1" t="str">
-        <x:f>IF(A49&gt;$B$4,"Future",IF(A49=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A49,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E49=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A49&gt;$B$4,"Future",IF(A49=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A49,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E49=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1791,7 +1791,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E50" s="6" t="str">
-        <x:f>IF(A50&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A50,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A50&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A50,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F50" s="6" t="str">
         <x:f>IF(A50&gt;=$B$4,"",MAX(D50-E50,0))</x:f>
@@ -1806,7 +1806,7 @@
         <x:f>IF(A50&gt;$B$4,"",SUM($E$15:E50))</x:f>
       </x:c>
       <x:c r="J50" s="1" t="str">
-        <x:f>IF(A50&gt;$B$4,"Future",IF(A50=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A50,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E50=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A50&gt;$B$4,"Future",IF(A50=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A50,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E50=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1826,7 +1826,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E51" s="6" t="str">
-        <x:f>IF(A51&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A51,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A51&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A51,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F51" s="6" t="str">
         <x:f>IF(A51&gt;=$B$4,"",MAX(D51-E51,0))</x:f>
@@ -1841,7 +1841,7 @@
         <x:f>IF(A51&gt;$B$4,"",SUM($E$15:E51))</x:f>
       </x:c>
       <x:c r="J51" s="1" t="str">
-        <x:f>IF(A51&gt;$B$4,"Future",IF(A51=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A51,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E51=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A51&gt;$B$4,"Future",IF(A51=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A51,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E51=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1861,7 +1861,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E52" s="6" t="str">
-        <x:f>IF(A52&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A52,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A52&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A52,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F52" s="6" t="str">
         <x:f>IF(A52&gt;=$B$4,"",MAX(D52-E52,0))</x:f>
@@ -1876,7 +1876,7 @@
         <x:f>IF(A52&gt;$B$4,"",SUM($E$15:E52))</x:f>
       </x:c>
       <x:c r="J52" s="1" t="str">
-        <x:f>IF(A52&gt;$B$4,"Future",IF(A52=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A52,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E52=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A52&gt;$B$4,"Future",IF(A52=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A52,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E52=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1896,7 +1896,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E53" s="6" t="str">
-        <x:f>IF(A53&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A53,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A53&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A53,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F53" s="6" t="str">
         <x:f>IF(A53&gt;=$B$4,"",MAX(D53-E53,0))</x:f>
@@ -1911,7 +1911,7 @@
         <x:f>IF(A53&gt;$B$4,"",SUM($E$15:E53))</x:f>
       </x:c>
       <x:c r="J53" s="1" t="str">
-        <x:f>IF(A53&gt;$B$4,"Future",IF(A53=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A53,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E53=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A53&gt;$B$4,"Future",IF(A53=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A53,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E53=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1931,7 +1931,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E54" s="6" t="str">
-        <x:f>IF(A54&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A54,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A54&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A54,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F54" s="6" t="str">
         <x:f>IF(A54&gt;=$B$4,"",MAX(D54-E54,0))</x:f>
@@ -1946,7 +1946,7 @@
         <x:f>IF(A54&gt;$B$4,"",SUM($E$15:E54))</x:f>
       </x:c>
       <x:c r="J54" s="1" t="str">
-        <x:f>IF(A54&gt;$B$4,"Future",IF(A54=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A54,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E54=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A54&gt;$B$4,"Future",IF(A54=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A54,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E54=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1966,7 +1966,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E55" s="6" t="str">
-        <x:f>IF(A55&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A55,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A55&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A55,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F55" s="6" t="str">
         <x:f>IF(A55&gt;=$B$4,"",MAX(D55-E55,0))</x:f>
@@ -1981,7 +1981,7 @@
         <x:f>IF(A55&gt;$B$4,"",SUM($E$15:E55))</x:f>
       </x:c>
       <x:c r="J55" s="1" t="str">
-        <x:f>IF(A55&gt;$B$4,"Future",IF(A55=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A55,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E55=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A55&gt;$B$4,"Future",IF(A55=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A55,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E55=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2001,7 +2001,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E56" s="6" t="str">
-        <x:f>IF(A56&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A56,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A56&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A56,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F56" s="6" t="str">
         <x:f>IF(A56&gt;=$B$4,"",MAX(D56-E56,0))</x:f>
@@ -2016,7 +2016,7 @@
         <x:f>IF(A56&gt;$B$4,"",SUM($E$15:E56))</x:f>
       </x:c>
       <x:c r="J56" s="1" t="str">
-        <x:f>IF(A56&gt;$B$4,"Future",IF(A56=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A56,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E56=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A56&gt;$B$4,"Future",IF(A56=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A56,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E56=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2036,7 +2036,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E57" s="6" t="str">
-        <x:f>IF(A57&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A57,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A57&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A57,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F57" s="6" t="str">
         <x:f>IF(A57&gt;=$B$4,"",MAX(D57-E57,0))</x:f>
@@ -2051,7 +2051,7 @@
         <x:f>IF(A57&gt;$B$4,"",SUM($E$15:E57))</x:f>
       </x:c>
       <x:c r="J57" s="1" t="str">
-        <x:f>IF(A57&gt;$B$4,"Future",IF(A57=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A57,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E57=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A57&gt;$B$4,"Future",IF(A57=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A57,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E57=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2071,7 +2071,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E58" s="6" t="str">
-        <x:f>IF(A58&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A58,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A58&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A58,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F58" s="6" t="str">
         <x:f>IF(A58&gt;=$B$4,"",MAX(D58-E58,0))</x:f>
@@ -2086,7 +2086,7 @@
         <x:f>IF(A58&gt;$B$4,"",SUM($E$15:E58))</x:f>
       </x:c>
       <x:c r="J58" s="1" t="str">
-        <x:f>IF(A58&gt;$B$4,"Future",IF(A58=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A58,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E58=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A58&gt;$B$4,"Future",IF(A58=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A58,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E58=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2106,7 +2106,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E59" s="6" t="str">
-        <x:f>IF(A59&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A59,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A59&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A59,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F59" s="6" t="str">
         <x:f>IF(A59&gt;=$B$4,"",MAX(D59-E59,0))</x:f>
@@ -2121,7 +2121,7 @@
         <x:f>IF(A59&gt;$B$4,"",SUM($E$15:E59))</x:f>
       </x:c>
       <x:c r="J59" s="1" t="str">
-        <x:f>IF(A59&gt;$B$4,"Future",IF(A59=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A59,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E59=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A59&gt;$B$4,"Future",IF(A59=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A59,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E59=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2141,7 +2141,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E60" s="6" t="str">
-        <x:f>IF(A60&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A60,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A60&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A60,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F60" s="6" t="str">
         <x:f>IF(A60&gt;=$B$4,"",MAX(D60-E60,0))</x:f>
@@ -2156,7 +2156,7 @@
         <x:f>IF(A60&gt;$B$4,"",SUM($E$15:E60))</x:f>
       </x:c>
       <x:c r="J60" s="1" t="str">
-        <x:f>IF(A60&gt;$B$4,"Future",IF(A60=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A60,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E60=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A60&gt;$B$4,"Future",IF(A60=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A60,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E60=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2176,7 +2176,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E61" s="6" t="str">
-        <x:f>IF(A61&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A61,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A61&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A61,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F61" s="6" t="str">
         <x:f>IF(A61&gt;=$B$4,"",MAX(D61-E61,0))</x:f>
@@ -2191,7 +2191,7 @@
         <x:f>IF(A61&gt;$B$4,"",SUM($E$15:E61))</x:f>
       </x:c>
       <x:c r="J61" s="1" t="str">
-        <x:f>IF(A61&gt;$B$4,"Future",IF(A61=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A61,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E61=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A61&gt;$B$4,"Future",IF(A61=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A61,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E61=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2211,7 +2211,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E62" s="6" t="str">
-        <x:f>IF(A62&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A62,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A62&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A62,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F62" s="6" t="str">
         <x:f>IF(A62&gt;=$B$4,"",MAX(D62-E62,0))</x:f>
@@ -2226,7 +2226,7 @@
         <x:f>IF(A62&gt;$B$4,"",SUM($E$15:E62))</x:f>
       </x:c>
       <x:c r="J62" s="1" t="str">
-        <x:f>IF(A62&gt;$B$4,"Future",IF(A62=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A62,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E62=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A62&gt;$B$4,"Future",IF(A62=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A62,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E62=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2246,7 +2246,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E63" s="6" t="str">
-        <x:f>IF(A63&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A63,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A63&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A63,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F63" s="6" t="str">
         <x:f>IF(A63&gt;=$B$4,"",MAX(D63-E63,0))</x:f>
@@ -2261,7 +2261,7 @@
         <x:f>IF(A63&gt;$B$4,"",SUM($E$15:E63))</x:f>
       </x:c>
       <x:c r="J63" s="1" t="str">
-        <x:f>IF(A63&gt;$B$4,"Future",IF(A63=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A63,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E63=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A63&gt;$B$4,"Future",IF(A63=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A63,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E63=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2281,7 +2281,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E64" s="6" t="str">
-        <x:f>IF(A64&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A64,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A64&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A64,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F64" s="6" t="str">
         <x:f>IF(A64&gt;=$B$4,"",MAX(D64-E64,0))</x:f>
@@ -2296,7 +2296,7 @@
         <x:f>IF(A64&gt;$B$4,"",SUM($E$15:E64))</x:f>
       </x:c>
       <x:c r="J64" s="1" t="str">
-        <x:f>IF(A64&gt;$B$4,"Future",IF(A64=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A64,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E64=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A64&gt;$B$4,"Future",IF(A64=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A64,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E64=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2316,7 +2316,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E65" s="6" t="str">
-        <x:f>IF(A65&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A65,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A65&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A65,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F65" s="6" t="str">
         <x:f>IF(A65&gt;=$B$4,"",MAX(D65-E65,0))</x:f>
@@ -2331,7 +2331,7 @@
         <x:f>IF(A65&gt;$B$4,"",SUM($E$15:E65))</x:f>
       </x:c>
       <x:c r="J65" s="1" t="str">
-        <x:f>IF(A65&gt;$B$4,"Future",IF(A65=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A65,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E65=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A65&gt;$B$4,"Future",IF(A65=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A65,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E65=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2351,7 +2351,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E66" s="6" t="str">
-        <x:f>IF(A66&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A66,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A66&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A66,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F66" s="6" t="str">
         <x:f>IF(A66&gt;=$B$4,"",MAX(D66-E66,0))</x:f>
@@ -2366,7 +2366,7 @@
         <x:f>IF(A66&gt;$B$4,"",SUM($E$15:E66))</x:f>
       </x:c>
       <x:c r="J66" s="1" t="str">
-        <x:f>IF(A66&gt;$B$4,"Future",IF(A66=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A66,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E66=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A66&gt;$B$4,"Future",IF(A66=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A66,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E66=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2386,7 +2386,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E67" s="6" t="str">
-        <x:f>IF(A67&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A67,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A67&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A67,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F67" s="6" t="str">
         <x:f>IF(A67&gt;=$B$4,"",MAX(D67-E67,0))</x:f>
@@ -2401,7 +2401,7 @@
         <x:f>IF(A67&gt;$B$4,"",SUM($E$15:E67))</x:f>
       </x:c>
       <x:c r="J67" s="1" t="str">
-        <x:f>IF(A67&gt;$B$4,"Future",IF(A67=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A67,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E67=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A67&gt;$B$4,"Future",IF(A67=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A67,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E67=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2421,7 +2421,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E68" s="6" t="str">
-        <x:f>IF(A68&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A68,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A68&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A68,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F68" s="6" t="str">
         <x:f>IF(A68&gt;=$B$4,"",MAX(D68-E68,0))</x:f>
@@ -2436,7 +2436,7 @@
         <x:f>IF(A68&gt;$B$4,"",SUM($E$15:E68))</x:f>
       </x:c>
       <x:c r="J68" s="1" t="str">
-        <x:f>IF(A68&gt;$B$4,"Future",IF(A68=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A68,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E68=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A68&gt;$B$4,"Future",IF(A68=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A68,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E68=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2456,7 +2456,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E69" s="6" t="str">
-        <x:f>IF(A69&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A69,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A69&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A69,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F69" s="6" t="str">
         <x:f>IF(A69&gt;=$B$4,"",MAX(D69-E69,0))</x:f>
@@ -2471,7 +2471,7 @@
         <x:f>IF(A69&gt;$B$4,"",SUM($E$15:E69))</x:f>
       </x:c>
       <x:c r="J69" s="1" t="str">
-        <x:f>IF(A69&gt;$B$4,"Future",IF(A69=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A69,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E69=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A69&gt;$B$4,"Future",IF(A69=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A69,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E69=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2491,7 +2491,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E70" s="6" t="str">
-        <x:f>IF(A70&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A70,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A70&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A70,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F70" s="6" t="str">
         <x:f>IF(A70&gt;=$B$4,"",MAX(D70-E70,0))</x:f>
@@ -2506,7 +2506,7 @@
         <x:f>IF(A70&gt;$B$4,"",SUM($E$15:E70))</x:f>
       </x:c>
       <x:c r="J70" s="1" t="str">
-        <x:f>IF(A70&gt;$B$4,"Future",IF(A70=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A70,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E70=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A70&gt;$B$4,"Future",IF(A70=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A70,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E70=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2526,7 +2526,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E71" s="6" t="str">
-        <x:f>IF(A71&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A71,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A71&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A71,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F71" s="6" t="str">
         <x:f>IF(A71&gt;=$B$4,"",MAX(D71-E71,0))</x:f>
@@ -2541,7 +2541,7 @@
         <x:f>IF(A71&gt;$B$4,"",SUM($E$15:E71))</x:f>
       </x:c>
       <x:c r="J71" s="1" t="str">
-        <x:f>IF(A71&gt;$B$4,"Future",IF(A71=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A71,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E71=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A71&gt;$B$4,"Future",IF(A71=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A71,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E71=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2561,7 +2561,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E72" s="6" t="str">
-        <x:f>IF(A72&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A72,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A72&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A72,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F72" s="6" t="str">
         <x:f>IF(A72&gt;=$B$4,"",MAX(D72-E72,0))</x:f>
@@ -2576,7 +2576,7 @@
         <x:f>IF(A72&gt;$B$4,"",SUM($E$15:E72))</x:f>
       </x:c>
       <x:c r="J72" s="1" t="str">
-        <x:f>IF(A72&gt;$B$4,"Future",IF(A72=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A72,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E72=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A72&gt;$B$4,"Future",IF(A72=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A72,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E72=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2596,7 +2596,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E73" s="6" t="str">
-        <x:f>IF(A73&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A73,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A73&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A73,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F73" s="6" t="str">
         <x:f>IF(A73&gt;=$B$4,"",MAX(D73-E73,0))</x:f>
@@ -2611,7 +2611,7 @@
         <x:f>IF(A73&gt;$B$4,"",SUM($E$15:E73))</x:f>
       </x:c>
       <x:c r="J73" s="1" t="str">
-        <x:f>IF(A73&gt;$B$4,"Future",IF(A73=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A73,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E73=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A73&gt;$B$4,"Future",IF(A73=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A73,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E73=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2631,7 +2631,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E74" s="6" t="str">
-        <x:f>IF(A74&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A74,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A74&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A74,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F74" s="6" t="str">
         <x:f>IF(A74&gt;=$B$4,"",MAX(D74-E74,0))</x:f>
@@ -2646,7 +2646,7 @@
         <x:f>IF(A74&gt;$B$4,"",SUM($E$15:E74))</x:f>
       </x:c>
       <x:c r="J74" s="1" t="str">
-        <x:f>IF(A74&gt;$B$4,"Future",IF(A74=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A74,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E74=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A74&gt;$B$4,"Future",IF(A74=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A74,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E74=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2666,7 +2666,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E75" s="6" t="str">
-        <x:f>IF(A75&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A75,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A75&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A75,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F75" s="6" t="str">
         <x:f>IF(A75&gt;=$B$4,"",MAX(D75-E75,0))</x:f>
@@ -2681,7 +2681,7 @@
         <x:f>IF(A75&gt;$B$4,"",SUM($E$15:E75))</x:f>
       </x:c>
       <x:c r="J75" s="1" t="str">
-        <x:f>IF(A75&gt;$B$4,"Future",IF(A75=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A75,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E75=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A75&gt;$B$4,"Future",IF(A75=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A75,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E75=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2701,7 +2701,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E76" s="6" t="str">
-        <x:f>IF(A76&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A76,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A76&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A76,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F76" s="6" t="str">
         <x:f>IF(A76&gt;=$B$4,"",MAX(D76-E76,0))</x:f>
@@ -2716,7 +2716,7 @@
         <x:f>IF(A76&gt;$B$4,"",SUM($E$15:E76))</x:f>
       </x:c>
       <x:c r="J76" s="1" t="str">
-        <x:f>IF(A76&gt;$B$4,"Future",IF(A76=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A76,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E76=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A76&gt;$B$4,"Future",IF(A76=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A76,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E76=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2736,7 +2736,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E77" s="6" t="str">
-        <x:f>IF(A77&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A77,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A77&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A77,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F77" s="6" t="str">
         <x:f>IF(A77&gt;=$B$4,"",MAX(D77-E77,0))</x:f>
@@ -2751,7 +2751,7 @@
         <x:f>IF(A77&gt;$B$4,"",SUM($E$15:E77))</x:f>
       </x:c>
       <x:c r="J77" s="1" t="str">
-        <x:f>IF(A77&gt;$B$4,"Future",IF(A77=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A77,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E77=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A77&gt;$B$4,"Future",IF(A77=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A77,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E77=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2771,7 +2771,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E78" s="6" t="str">
-        <x:f>IF(A78&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A78,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A78&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A78,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F78" s="6" t="str">
         <x:f>IF(A78&gt;=$B$4,"",MAX(D78-E78,0))</x:f>
@@ -2786,7 +2786,7 @@
         <x:f>IF(A78&gt;$B$4,"",SUM($E$15:E78))</x:f>
       </x:c>
       <x:c r="J78" s="1" t="str">
-        <x:f>IF(A78&gt;$B$4,"Future",IF(A78=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A78,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E78=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A78&gt;$B$4,"Future",IF(A78=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A78,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E78=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2806,7 +2806,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E79" s="6" t="str">
-        <x:f>IF(A79&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A79,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A79&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A79,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F79" s="6" t="str">
         <x:f>IF(A79&gt;=$B$4,"",MAX(D79-E79,0))</x:f>
@@ -2821,7 +2821,7 @@
         <x:f>IF(A79&gt;$B$4,"",SUM($E$15:E79))</x:f>
       </x:c>
       <x:c r="J79" s="1" t="str">
-        <x:f>IF(A79&gt;$B$4,"Future",IF(A79=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A79,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E79=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A79&gt;$B$4,"Future",IF(A79=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A79,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E79=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2841,7 +2841,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E80" s="6" t="str">
-        <x:f>IF(A80&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A80,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A80&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A80,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F80" s="6" t="str">
         <x:f>IF(A80&gt;=$B$4,"",MAX(D80-E80,0))</x:f>
@@ -2856,7 +2856,7 @@
         <x:f>IF(A80&gt;$B$4,"",SUM($E$15:E80))</x:f>
       </x:c>
       <x:c r="J80" s="1" t="str">
-        <x:f>IF(A80&gt;$B$4,"Future",IF(A80=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A80,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E80=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A80&gt;$B$4,"Future",IF(A80=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A80,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E80=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2876,7 +2876,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E81" s="6" t="str">
-        <x:f>IF(A81&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A81,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A81&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A81,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F81" s="6" t="str">
         <x:f>IF(A81&gt;=$B$4,"",MAX(D81-E81,0))</x:f>
@@ -2891,7 +2891,7 @@
         <x:f>IF(A81&gt;$B$4,"",SUM($E$15:E81))</x:f>
       </x:c>
       <x:c r="J81" s="1" t="str">
-        <x:f>IF(A81&gt;$B$4,"Future",IF(A81=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A81,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E81=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A81&gt;$B$4,"Future",IF(A81=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A81,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E81=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2911,7 +2911,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E82" s="6" t="str">
-        <x:f>IF(A82&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A82,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A82&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A82,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F82" s="6" t="str">
         <x:f>IF(A82&gt;=$B$4,"",MAX(D82-E82,0))</x:f>
@@ -2926,7 +2926,7 @@
         <x:f>IF(A82&gt;$B$4,"",SUM($E$15:E82))</x:f>
       </x:c>
       <x:c r="J82" s="1" t="str">
-        <x:f>IF(A82&gt;$B$4,"Future",IF(A82=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A82,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E82=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A82&gt;$B$4,"Future",IF(A82=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A82,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E82=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2946,7 +2946,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E83" s="6" t="str">
-        <x:f>IF(A83&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A83,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A83&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A83,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F83" s="6" t="str">
         <x:f>IF(A83&gt;=$B$4,"",MAX(D83-E83,0))</x:f>
@@ -2961,7 +2961,7 @@
         <x:f>IF(A83&gt;$B$4,"",SUM($E$15:E83))</x:f>
       </x:c>
       <x:c r="J83" s="1" t="str">
-        <x:f>IF(A83&gt;$B$4,"Future",IF(A83=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A83,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E83=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A83&gt;$B$4,"Future",IF(A83=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A83,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E83=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2981,7 +2981,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E84" s="6" t="str">
-        <x:f>IF(A84&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A84,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A84&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A84,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F84" s="6" t="str">
         <x:f>IF(A84&gt;=$B$4,"",MAX(D84-E84,0))</x:f>
@@ -2996,7 +2996,7 @@
         <x:f>IF(A84&gt;$B$4,"",SUM($E$15:E84))</x:f>
       </x:c>
       <x:c r="J84" s="1" t="str">
-        <x:f>IF(A84&gt;$B$4,"Future",IF(A84=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A84,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E84=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A84&gt;$B$4,"Future",IF(A84=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A84,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E84=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3016,7 +3016,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E85" s="6" t="str">
-        <x:f>IF(A85&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A85,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A85&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A85,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F85" s="6" t="str">
         <x:f>IF(A85&gt;=$B$4,"",MAX(D85-E85,0))</x:f>
@@ -3031,7 +3031,7 @@
         <x:f>IF(A85&gt;$B$4,"",SUM($E$15:E85))</x:f>
       </x:c>
       <x:c r="J85" s="1" t="str">
-        <x:f>IF(A85&gt;$B$4,"Future",IF(A85=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A85,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E85=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A85&gt;$B$4,"Future",IF(A85=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A85,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E85=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3051,7 +3051,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E86" s="6" t="str">
-        <x:f>IF(A86&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A86,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A86&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A86,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F86" s="6" t="str">
         <x:f>IF(A86&gt;=$B$4,"",MAX(D86-E86,0))</x:f>
@@ -3066,7 +3066,7 @@
         <x:f>IF(A86&gt;$B$4,"",SUM($E$15:E86))</x:f>
       </x:c>
       <x:c r="J86" s="1" t="str">
-        <x:f>IF(A86&gt;$B$4,"Future",IF(A86=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A86,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E86=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A86&gt;$B$4,"Future",IF(A86=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A86,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E86=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3086,7 +3086,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E87" s="6" t="str">
-        <x:f>IF(A87&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A87,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A87&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A87,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F87" s="6" t="str">
         <x:f>IF(A87&gt;=$B$4,"",MAX(D87-E87,0))</x:f>
@@ -3101,7 +3101,7 @@
         <x:f>IF(A87&gt;$B$4,"",SUM($E$15:E87))</x:f>
       </x:c>
       <x:c r="J87" s="1" t="str">
-        <x:f>IF(A87&gt;$B$4,"Future",IF(A87=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A87,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E87=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A87&gt;$B$4,"Future",IF(A87=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A87,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E87=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3121,7 +3121,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E88" s="6" t="str">
-        <x:f>IF(A88&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A88,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A88&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A88,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F88" s="6" t="str">
         <x:f>IF(A88&gt;=$B$4,"",MAX(D88-E88,0))</x:f>
@@ -3136,7 +3136,7 @@
         <x:f>IF(A88&gt;$B$4,"",SUM($E$15:E88))</x:f>
       </x:c>
       <x:c r="J88" s="1" t="str">
-        <x:f>IF(A88&gt;$B$4,"Future",IF(A88=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A88,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E88=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A88&gt;$B$4,"Future",IF(A88=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A88,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E88=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3156,7 +3156,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E89" s="6" t="str">
-        <x:f>IF(A89&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A89,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A89&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A89,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F89" s="6" t="str">
         <x:f>IF(A89&gt;=$B$4,"",MAX(D89-E89,0))</x:f>
@@ -3171,7 +3171,7 @@
         <x:f>IF(A89&gt;$B$4,"",SUM($E$15:E89))</x:f>
       </x:c>
       <x:c r="J89" s="1" t="str">
-        <x:f>IF(A89&gt;$B$4,"Future",IF(A89=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A89,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E89=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A89&gt;$B$4,"Future",IF(A89=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A89,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E89=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3191,7 +3191,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E90" s="6" t="str">
-        <x:f>IF(A90&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A90,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A90&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A90,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F90" s="6" t="str">
         <x:f>IF(A90&gt;=$B$4,"",MAX(D90-E90,0))</x:f>
@@ -3206,7 +3206,7 @@
         <x:f>IF(A90&gt;$B$4,"",SUM($E$15:E90))</x:f>
       </x:c>
       <x:c r="J90" s="1" t="str">
-        <x:f>IF(A90&gt;$B$4,"Future",IF(A90=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A90,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E90=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A90&gt;$B$4,"Future",IF(A90=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A90,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E90=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3226,7 +3226,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E91" s="6" t="str">
-        <x:f>IF(A91&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A91,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A91&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A91,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F91" s="6" t="str">
         <x:f>IF(A91&gt;=$B$4,"",MAX(D91-E91,0))</x:f>
@@ -3241,7 +3241,7 @@
         <x:f>IF(A91&gt;$B$4,"",SUM($E$15:E91))</x:f>
       </x:c>
       <x:c r="J91" s="1" t="str">
-        <x:f>IF(A91&gt;$B$4,"Future",IF(A91=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A91,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E91=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A91&gt;$B$4,"Future",IF(A91=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A91,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E91=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3261,7 +3261,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E92" s="6" t="str">
-        <x:f>IF(A92&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A92,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A92&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A92,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F92" s="6" t="str">
         <x:f>IF(A92&gt;=$B$4,"",MAX(D92-E92,0))</x:f>
@@ -3276,7 +3276,7 @@
         <x:f>IF(A92&gt;$B$4,"",SUM($E$15:E92))</x:f>
       </x:c>
       <x:c r="J92" s="1" t="str">
-        <x:f>IF(A92&gt;$B$4,"Future",IF(A92=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A92,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E92=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A92&gt;$B$4,"Future",IF(A92=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A92,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E92=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3296,7 +3296,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E93" s="6" t="str">
-        <x:f>IF(A93&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A93,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A93&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A93,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F93" s="6" t="str">
         <x:f>IF(A93&gt;=$B$4,"",MAX(D93-E93,0))</x:f>
@@ -3311,7 +3311,7 @@
         <x:f>IF(A93&gt;$B$4,"",SUM($E$15:E93))</x:f>
       </x:c>
       <x:c r="J93" s="1" t="str">
-        <x:f>IF(A93&gt;$B$4,"Future",IF(A93=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A93,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E93=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A93&gt;$B$4,"Future",IF(A93=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A93,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E93=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3331,7 +3331,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E94" s="6" t="str">
-        <x:f>IF(A94&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A94,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A94&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A94,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F94" s="6" t="str">
         <x:f>IF(A94&gt;=$B$4,"",MAX(D94-E94,0))</x:f>
@@ -3346,7 +3346,7 @@
         <x:f>IF(A94&gt;$B$4,"",SUM($E$15:E94))</x:f>
       </x:c>
       <x:c r="J94" s="1" t="str">
-        <x:f>IF(A94&gt;$B$4,"Future",IF(A94=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A94,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E94=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A94&gt;$B$4,"Future",IF(A94=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A94,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E94=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3366,7 +3366,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E95" s="6" t="str">
-        <x:f>IF(A95&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A95,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A95&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A95,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F95" s="6" t="str">
         <x:f>IF(A95&gt;=$B$4,"",MAX(D95-E95,0))</x:f>
@@ -3381,7 +3381,7 @@
         <x:f>IF(A95&gt;$B$4,"",SUM($E$15:E95))</x:f>
       </x:c>
       <x:c r="J95" s="1" t="str">
-        <x:f>IF(A95&gt;$B$4,"Future",IF(A95=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A95,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E95=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A95&gt;$B$4,"Future",IF(A95=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A95,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E95=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3401,7 +3401,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E96" s="6" t="str">
-        <x:f>IF(A96&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A96,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A96&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A96,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F96" s="6" t="str">
         <x:f>IF(A96&gt;=$B$4,"",MAX(D96-E96,0))</x:f>
@@ -3416,7 +3416,7 @@
         <x:f>IF(A96&gt;$B$4,"",SUM($E$15:E96))</x:f>
       </x:c>
       <x:c r="J96" s="1" t="str">
-        <x:f>IF(A96&gt;$B$4,"Future",IF(A96=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A96,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E96=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A96&gt;$B$4,"Future",IF(A96=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A96,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E96=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3436,7 +3436,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E97" s="6" t="str">
-        <x:f>IF(A97&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A97,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A97&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A97,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F97" s="6" t="str">
         <x:f>IF(A97&gt;=$B$4,"",MAX(D97-E97,0))</x:f>
@@ -3451,7 +3451,7 @@
         <x:f>IF(A97&gt;$B$4,"",SUM($E$15:E97))</x:f>
       </x:c>
       <x:c r="J97" s="1" t="str">
-        <x:f>IF(A97&gt;$B$4,"Future",IF(A97=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A97,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E97=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A97&gt;$B$4,"Future",IF(A97=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A97,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E97=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3471,7 +3471,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E98" s="6" t="str">
-        <x:f>IF(A98&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A98,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A98&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A98,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F98" s="6" t="str">
         <x:f>IF(A98&gt;=$B$4,"",MAX(D98-E98,0))</x:f>
@@ -3486,7 +3486,7 @@
         <x:f>IF(A98&gt;$B$4,"",SUM($E$15:E98))</x:f>
       </x:c>
       <x:c r="J98" s="1" t="str">
-        <x:f>IF(A98&gt;$B$4,"Future",IF(A98=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A98,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E98=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A98&gt;$B$4,"Future",IF(A98=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A98,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E98=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3506,7 +3506,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E99" s="6" t="str">
-        <x:f>IF(A99&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A99,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A99&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A99,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F99" s="6" t="str">
         <x:f>IF(A99&gt;=$B$4,"",MAX(D99-E99,0))</x:f>
@@ -3521,7 +3521,7 @@
         <x:f>IF(A99&gt;$B$4,"",SUM($E$15:E99))</x:f>
       </x:c>
       <x:c r="J99" s="1" t="str">
-        <x:f>IF(A99&gt;$B$4,"Future",IF(A99=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A99,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E99=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A99&gt;$B$4,"Future",IF(A99=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A99,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E99=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3541,7 +3541,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E100" s="6" t="str">
-        <x:f>IF(A100&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A100,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A100&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A100,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F100" s="6" t="str">
         <x:f>IF(A100&gt;=$B$4,"",MAX(D100-E100,0))</x:f>
@@ -3556,7 +3556,7 @@
         <x:f>IF(A100&gt;$B$4,"",SUM($E$15:E100))</x:f>
       </x:c>
       <x:c r="J100" s="1" t="str">
-        <x:f>IF(A100&gt;$B$4,"Future",IF(A100=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A100,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E100=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A100&gt;$B$4,"Future",IF(A100=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A100,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E100=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3576,7 +3576,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E101" s="6" t="str">
-        <x:f>IF(A101&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A101,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A101&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A101,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F101" s="6" t="str">
         <x:f>IF(A101&gt;=$B$4,"",MAX(D101-E101,0))</x:f>
@@ -3591,7 +3591,7 @@
         <x:f>IF(A101&gt;$B$4,"",SUM($E$15:E101))</x:f>
       </x:c>
       <x:c r="J101" s="1" t="str">
-        <x:f>IF(A101&gt;$B$4,"Future",IF(A101=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A101,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E101=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A101&gt;$B$4,"Future",IF(A101=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A101,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E101=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3611,7 +3611,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E102" s="6" t="str">
-        <x:f>IF(A102&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A102,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A102&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A102,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F102" s="6" t="str">
         <x:f>IF(A102&gt;=$B$4,"",MAX(D102-E102,0))</x:f>
@@ -3626,7 +3626,7 @@
         <x:f>IF(A102&gt;$B$4,"",SUM($E$15:E102))</x:f>
       </x:c>
       <x:c r="J102" s="1" t="str">
-        <x:f>IF(A102&gt;$B$4,"Future",IF(A102=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A102,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E102=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A102&gt;$B$4,"Future",IF(A102=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A102,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E102=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3646,7 +3646,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E103" s="6" t="str">
-        <x:f>IF(A103&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A103,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A103&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A103,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F103" s="6" t="str">
         <x:f>IF(A103&gt;=$B$4,"",MAX(D103-E103,0))</x:f>
@@ -3661,7 +3661,7 @@
         <x:f>IF(A103&gt;$B$4,"",SUM($E$15:E103))</x:f>
       </x:c>
       <x:c r="J103" s="1" t="str">
-        <x:f>IF(A103&gt;$B$4,"Future",IF(A103=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A103,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E103=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A103&gt;$B$4,"Future",IF(A103=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A103,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E103=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3681,7 +3681,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E104" s="6" t="str">
-        <x:f>IF(A104&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A104,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A104&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A104,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F104" s="6" t="str">
         <x:f>IF(A104&gt;=$B$4,"",MAX(D104-E104,0))</x:f>
@@ -3696,7 +3696,7 @@
         <x:f>IF(A104&gt;$B$4,"",SUM($E$15:E104))</x:f>
       </x:c>
       <x:c r="J104" s="1" t="str">
-        <x:f>IF(A104&gt;$B$4,"Future",IF(A104=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A104,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E104=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A104&gt;$B$4,"Future",IF(A104=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A104,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E104=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3716,7 +3716,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E105" s="6" t="str">
-        <x:f>IF(A105&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A105,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A105&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A105,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F105" s="6" t="str">
         <x:f>IF(A105&gt;=$B$4,"",MAX(D105-E105,0))</x:f>
@@ -3731,7 +3731,7 @@
         <x:f>IF(A105&gt;$B$4,"",SUM($E$15:E105))</x:f>
       </x:c>
       <x:c r="J105" s="1" t="str">
-        <x:f>IF(A105&gt;$B$4,"Future",IF(A105=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A105,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E105=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A105&gt;$B$4,"Future",IF(A105=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A105,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E105=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3751,7 +3751,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E106" s="6" t="str">
-        <x:f>IF(A106&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A106,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A106&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A106,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F106" s="6" t="str">
         <x:f>IF(A106&gt;=$B$4,"",MAX(D106-E106,0))</x:f>
@@ -3766,7 +3766,7 @@
         <x:f>IF(A106&gt;$B$4,"",SUM($E$15:E106))</x:f>
       </x:c>
       <x:c r="J106" s="1" t="str">
-        <x:f>IF(A106&gt;$B$4,"Future",IF(A106=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A106,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E106=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A106&gt;$B$4,"Future",IF(A106=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A106,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E106=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3786,7 +3786,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E107" s="6" t="str">
-        <x:f>IF(A107&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A107,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A107&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A107,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F107" s="6" t="str">
         <x:f>IF(A107&gt;=$B$4,"",MAX(D107-E107,0))</x:f>
@@ -3801,7 +3801,7 @@
         <x:f>IF(A107&gt;$B$4,"",SUM($E$15:E107))</x:f>
       </x:c>
       <x:c r="J107" s="1" t="str">
-        <x:f>IF(A107&gt;$B$4,"Future",IF(A107=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A107,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E107=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A107&gt;$B$4,"Future",IF(A107=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A107,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E107=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3821,7 +3821,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E108" s="6" t="str">
-        <x:f>IF(A108&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A108,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A108&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A108,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F108" s="6" t="str">
         <x:f>IF(A108&gt;=$B$4,"",MAX(D108-E108,0))</x:f>
@@ -3836,7 +3836,7 @@
         <x:f>IF(A108&gt;$B$4,"",SUM($E$15:E108))</x:f>
       </x:c>
       <x:c r="J108" s="1" t="str">
-        <x:f>IF(A108&gt;$B$4,"Future",IF(A108=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A108,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E108=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A108&gt;$B$4,"Future",IF(A108=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A108,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E108=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3856,7 +3856,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E109" s="6" t="str">
-        <x:f>IF(A109&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A109,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A109&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A109,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F109" s="6" t="str">
         <x:f>IF(A109&gt;=$B$4,"",MAX(D109-E109,0))</x:f>
@@ -3871,7 +3871,7 @@
         <x:f>IF(A109&gt;$B$4,"",SUM($E$15:E109))</x:f>
       </x:c>
       <x:c r="J109" s="1" t="str">
-        <x:f>IF(A109&gt;$B$4,"Future",IF(A109=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A109,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E109=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A109&gt;$B$4,"Future",IF(A109=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A109,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E109=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3891,7 +3891,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E110" s="6" t="str">
-        <x:f>IF(A110&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A110,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A110&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A110,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F110" s="6" t="str">
         <x:f>IF(A110&gt;=$B$4,"",MAX(D110-E110,0))</x:f>
@@ -3906,7 +3906,7 @@
         <x:f>IF(A110&gt;$B$4,"",SUM($E$15:E110))</x:f>
       </x:c>
       <x:c r="J110" s="1" t="str">
-        <x:f>IF(A110&gt;$B$4,"Future",IF(A110=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A110,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E110=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A110&gt;$B$4,"Future",IF(A110=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A110,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E110=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3926,7 +3926,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E111" s="6" t="str">
-        <x:f>IF(A111&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A111,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A111&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A111,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F111" s="6" t="str">
         <x:f>IF(A111&gt;=$B$4,"",MAX(D111-E111,0))</x:f>
@@ -3941,7 +3941,7 @@
         <x:f>IF(A111&gt;$B$4,"",SUM($E$15:E111))</x:f>
       </x:c>
       <x:c r="J111" s="1" t="str">
-        <x:f>IF(A111&gt;$B$4,"Future",IF(A111=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A111,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E111=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A111&gt;$B$4,"Future",IF(A111=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A111,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E111=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3961,7 +3961,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E112" s="6" t="str">
-        <x:f>IF(A112&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A112,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A112&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A112,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F112" s="6" t="str">
         <x:f>IF(A112&gt;=$B$4,"",MAX(D112-E112,0))</x:f>
@@ -3976,7 +3976,7 @@
         <x:f>IF(A112&gt;$B$4,"",SUM($E$15:E112))</x:f>
       </x:c>
       <x:c r="J112" s="1" t="str">
-        <x:f>IF(A112&gt;$B$4,"Future",IF(A112=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A112,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E112=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A112&gt;$B$4,"Future",IF(A112=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A112,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E112=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3996,7 +3996,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E113" s="6" t="str">
-        <x:f>IF(A113&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A113,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A113&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A113,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F113" s="6" t="str">
         <x:f>IF(A113&gt;=$B$4,"",MAX(D113-E113,0))</x:f>
@@ -4011,7 +4011,7 @@
         <x:f>IF(A113&gt;$B$4,"",SUM($E$15:E113))</x:f>
       </x:c>
       <x:c r="J113" s="1" t="str">
-        <x:f>IF(A113&gt;$B$4,"Future",IF(A113=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A113,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E113=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A113&gt;$B$4,"Future",IF(A113=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A113,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E113=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4031,7 +4031,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E114" s="6" t="str">
-        <x:f>IF(A114&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A114,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A114&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A114,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F114" s="6" t="str">
         <x:f>IF(A114&gt;=$B$4,"",MAX(D114-E114,0))</x:f>
@@ -4046,7 +4046,7 @@
         <x:f>IF(A114&gt;$B$4,"",SUM($E$15:E114))</x:f>
       </x:c>
       <x:c r="J114" s="1" t="str">
-        <x:f>IF(A114&gt;$B$4,"Future",IF(A114=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A114,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E114=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A114&gt;$B$4,"Future",IF(A114=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A114,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E114=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4066,7 +4066,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E115" s="6" t="str">
-        <x:f>IF(A115&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A115,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A115&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A115,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F115" s="6" t="str">
         <x:f>IF(A115&gt;=$B$4,"",MAX(D115-E115,0))</x:f>
@@ -4081,7 +4081,7 @@
         <x:f>IF(A115&gt;$B$4,"",SUM($E$15:E115))</x:f>
       </x:c>
       <x:c r="J115" s="1" t="str">
-        <x:f>IF(A115&gt;$B$4,"Future",IF(A115=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A115,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E115=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A115&gt;$B$4,"Future",IF(A115=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A115,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E115=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4101,7 +4101,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E116" s="6" t="str">
-        <x:f>IF(A116&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A116,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A116&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A116,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F116" s="6" t="str">
         <x:f>IF(A116&gt;=$B$4,"",MAX(D116-E116,0))</x:f>
@@ -4116,7 +4116,7 @@
         <x:f>IF(A116&gt;$B$4,"",SUM($E$15:E116))</x:f>
       </x:c>
       <x:c r="J116" s="1" t="str">
-        <x:f>IF(A116&gt;$B$4,"Future",IF(A116=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A116,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E116=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A116&gt;$B$4,"Future",IF(A116=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A116,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E116=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4136,7 +4136,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E117" s="6" t="str">
-        <x:f>IF(A117&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A117,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A117&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A117,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F117" s="6" t="str">
         <x:f>IF(A117&gt;=$B$4,"",MAX(D117-E117,0))</x:f>
@@ -4151,7 +4151,7 @@
         <x:f>IF(A117&gt;$B$4,"",SUM($E$15:E117))</x:f>
       </x:c>
       <x:c r="J117" s="1" t="str">
-        <x:f>IF(A117&gt;$B$4,"Future",IF(A117=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A117,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E117=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A117&gt;$B$4,"Future",IF(A117=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A117,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E117=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4171,7 +4171,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E118" s="6" t="str">
-        <x:f>IF(A118&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A118,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A118&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A118,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F118" s="6" t="str">
         <x:f>IF(A118&gt;=$B$4,"",MAX(D118-E118,0))</x:f>
@@ -4186,7 +4186,7 @@
         <x:f>IF(A118&gt;$B$4,"",SUM($E$15:E118))</x:f>
       </x:c>
       <x:c r="J118" s="1" t="str">
-        <x:f>IF(A118&gt;$B$4,"Future",IF(A118=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A118,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E118=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A118&gt;$B$4,"Future",IF(A118=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A118,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E118=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4206,7 +4206,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E119" s="6" t="str">
-        <x:f>IF(A119&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A119,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A119&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A119,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F119" s="6" t="str">
         <x:f>IF(A119&gt;=$B$4,"",MAX(D119-E119,0))</x:f>
@@ -4221,7 +4221,7 @@
         <x:f>IF(A119&gt;$B$4,"",SUM($E$15:E119))</x:f>
       </x:c>
       <x:c r="J119" s="1" t="str">
-        <x:f>IF(A119&gt;$B$4,"Future",IF(A119=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A119,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E119=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A119&gt;$B$4,"Future",IF(A119=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A119,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E119=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4241,7 +4241,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E120" s="6" t="str">
-        <x:f>IF(A120&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A120,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A120&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A120,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F120" s="6" t="str">
         <x:f>IF(A120&gt;=$B$4,"",MAX(D120-E120,0))</x:f>
@@ -4256,7 +4256,7 @@
         <x:f>IF(A120&gt;$B$4,"",SUM($E$15:E120))</x:f>
       </x:c>
       <x:c r="J120" s="1" t="str">
-        <x:f>IF(A120&gt;$B$4,"Future",IF(A120=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A120,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E120=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A120&gt;$B$4,"Future",IF(A120=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A120,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E120=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4276,7 +4276,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E121" s="6" t="str">
-        <x:f>IF(A121&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A121,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A121&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A121,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F121" s="6" t="str">
         <x:f>IF(A121&gt;=$B$4,"",MAX(D121-E121,0))</x:f>
@@ -4291,7 +4291,7 @@
         <x:f>IF(A121&gt;$B$4,"",SUM($E$15:E121))</x:f>
       </x:c>
       <x:c r="J121" s="1" t="str">
-        <x:f>IF(A121&gt;$B$4,"Future",IF(A121=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A121,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E121=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A121&gt;$B$4,"Future",IF(A121=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A121,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E121=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4311,7 +4311,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E122" s="6" t="str">
-        <x:f>IF(A122&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A122,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A122&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A122,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F122" s="6" t="str">
         <x:f>IF(A122&gt;=$B$4,"",MAX(D122-E122,0))</x:f>
@@ -4326,7 +4326,7 @@
         <x:f>IF(A122&gt;$B$4,"",SUM($E$15:E122))</x:f>
       </x:c>
       <x:c r="J122" s="1" t="str">
-        <x:f>IF(A122&gt;$B$4,"Future",IF(A122=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A122,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E122=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A122&gt;$B$4,"Future",IF(A122=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A122,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E122=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4346,7 +4346,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E123" s="6" t="str">
-        <x:f>IF(A123&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A123,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A123&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A123,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F123" s="6" t="str">
         <x:f>IF(A123&gt;=$B$4,"",MAX(D123-E123,0))</x:f>
@@ -4361,7 +4361,7 @@
         <x:f>IF(A123&gt;$B$4,"",SUM($E$15:E123))</x:f>
       </x:c>
       <x:c r="J123" s="1" t="str">
-        <x:f>IF(A123&gt;$B$4,"Future",IF(A123=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A123,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E123=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A123&gt;$B$4,"Future",IF(A123=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A123,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E123=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4381,7 +4381,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E124" s="6" t="str">
-        <x:f>IF(A124&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A124,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A124&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A124,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F124" s="6" t="str">
         <x:f>IF(A124&gt;=$B$4,"",MAX(D124-E124,0))</x:f>
@@ -4396,7 +4396,7 @@
         <x:f>IF(A124&gt;$B$4,"",SUM($E$15:E124))</x:f>
       </x:c>
       <x:c r="J124" s="1" t="str">
-        <x:f>IF(A124&gt;$B$4,"Future",IF(A124=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A124,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E124=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A124&gt;$B$4,"Future",IF(A124=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A124,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E124=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4416,7 +4416,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E125" s="6" t="str">
-        <x:f>IF(A125&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A125,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A125&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A125,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F125" s="6" t="str">
         <x:f>IF(A125&gt;=$B$4,"",MAX(D125-E125,0))</x:f>
@@ -4431,7 +4431,7 @@
         <x:f>IF(A125&gt;$B$4,"",SUM($E$15:E125))</x:f>
       </x:c>
       <x:c r="J125" s="1" t="str">
-        <x:f>IF(A125&gt;$B$4,"Future",IF(A125=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A125,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E125=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A125&gt;$B$4,"Future",IF(A125=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A125,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E125=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4451,7 +4451,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E126" s="6" t="str">
-        <x:f>IF(A126&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A126,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A126&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A126,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F126" s="6" t="str">
         <x:f>IF(A126&gt;=$B$4,"",MAX(D126-E126,0))</x:f>
@@ -4466,7 +4466,7 @@
         <x:f>IF(A126&gt;$B$4,"",SUM($E$15:E126))</x:f>
       </x:c>
       <x:c r="J126" s="1" t="str">
-        <x:f>IF(A126&gt;$B$4,"Future",IF(A126=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A126,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E126=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A126&gt;$B$4,"Future",IF(A126=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A126,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E126=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4486,7 +4486,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E127" s="6" t="str">
-        <x:f>IF(A127&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A127,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A127&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A127,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F127" s="6" t="str">
         <x:f>IF(A127&gt;=$B$4,"",MAX(D127-E127,0))</x:f>
@@ -4501,7 +4501,7 @@
         <x:f>IF(A127&gt;$B$4,"",SUM($E$15:E127))</x:f>
       </x:c>
       <x:c r="J127" s="1" t="str">
-        <x:f>IF(A127&gt;$B$4,"Future",IF(A127=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A127,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E127=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A127&gt;$B$4,"Future",IF(A127=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A127,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E127=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4521,7 +4521,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E128" s="6" t="str">
-        <x:f>IF(A128&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A128,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A128&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A128,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F128" s="6" t="str">
         <x:f>IF(A128&gt;=$B$4,"",MAX(D128-E128,0))</x:f>
@@ -4536,7 +4536,7 @@
         <x:f>IF(A128&gt;$B$4,"",SUM($E$15:E128))</x:f>
       </x:c>
       <x:c r="J128" s="1" t="str">
-        <x:f>IF(A128&gt;$B$4,"Future",IF(A128=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A128,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E128=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A128&gt;$B$4,"Future",IF(A128=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A128,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E128=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4556,7 +4556,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E129" s="6" t="str">
-        <x:f>IF(A129&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A129,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A129&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A129,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F129" s="6" t="str">
         <x:f>IF(A129&gt;=$B$4,"",MAX(D129-E129,0))</x:f>
@@ -4571,7 +4571,7 @@
         <x:f>IF(A129&gt;$B$4,"",SUM($E$15:E129))</x:f>
       </x:c>
       <x:c r="J129" s="1" t="str">
-        <x:f>IF(A129&gt;$B$4,"Future",IF(A129=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A129,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E129=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A129&gt;$B$4,"Future",IF(A129=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A129,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E129=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4591,7 +4591,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E130" s="6" t="str">
-        <x:f>IF(A130&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$8,'Sessions'!$B$2:$B$8,A130,'Sessions'!$G$2:$G$8,"completed")/60)</x:f>
+        <x:f>IF(A130&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A130,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
       </x:c>
       <x:c r="F130" s="6" t="str">
         <x:f>IF(A130&gt;=$B$4,"",MAX(D130-E130,0))</x:f>
@@ -4606,7 +4606,7 @@
         <x:f>IF(A130&gt;$B$4,"",SUM($E$15:E130))</x:f>
       </x:c>
       <x:c r="J130" s="1" t="str">
-        <x:f>IF(A130&gt;$B$4,"Future",IF(A130=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$8,A130,'Sessions'!$G$2:$G$8,"needs_confirmation")&gt;0,"Uncertain time",IF(E130=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A130&gt;$B$4,"Future",IF(A130=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A130,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E130=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4730,7 +4730,7 @@
       </x:c>
       <x:c r="D8" s="6" t="n">
         <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A8)</x:f>
-        <x:v>1.9563888888899998</x:v>
+        <x:v>2.8094444444449995</x:v>
       </x:c>
       <x:c r="E8" s="6" t="n">
         <x:f>MAX(C8-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A8,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
@@ -4742,11 +4742,11 @@
       </x:c>
       <x:c r="G8" s="6" t="n">
         <x:f>MAX(B8-D8,0)</x:f>
-        <x:v>30.04361111111</x:v>
+        <x:v>29.190555555555</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
         <x:f>IF(B8=0,0,D8/B8)</x:f>
-        <x:v>0.061137152777812495</x:v>
+        <x:v>0.08779513888890624</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
@@ -5505,6 +5505,58 @@
         <x:v>Explicit pause at first request; clock timestamp; 7 minutes 11 seconds; learner requested dictionary foundations; repeated pause does not extend interval</x:v>
       </x:c>
     </x:row>
+    <x:row r="9" ht="22" customHeight="1">
+      <x:c r="A9" s="1" t="str">
+        <x:v>PY-20261015T134259</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="C9" s="1" t="str">
+        <x:v>Python: dictionary foundations in Jupyter</x:v>
+      </x:c>
+      <x:c r="D9" s="1" t="str">
+        <x:v>IST 2026-10-15 13:42:59</x:v>
+      </x:c>
+      <x:c r="E9" s="1" t="str">
+        <x:v>IST 2026-10-15 13:48:32</x:v>
+      </x:c>
+      <x:c r="F9" s="1" t="n">
+        <x:v>5.55</x:v>
+      </x:c>
+      <x:c r="G9" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H9" s="1" t="str">
+        <x:v>Explicit resume and pause; clock timestamps; 5 minutes 33 seconds; no notebook attempt or output submitted</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="22" customHeight="1">
+      <x:c r="A10" s="1" t="str">
+        <x:v>PY-20261015T141407</x:v>
+      </x:c>
+      <x:c r="B10" s="7" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="C10" s="1" t="str">
+        <x:v>Python: dictionary foundations in Jupyter</x:v>
+      </x:c>
+      <x:c r="D10" s="1" t="str">
+        <x:v>IST 2026-10-15 14:14:07</x:v>
+      </x:c>
+      <x:c r="E10" s="1" t="str">
+        <x:v>IST 2026-10-15 14:59:45</x:v>
+      </x:c>
+      <x:c r="F10" s="1" t="n">
+        <x:v>45.6333333333</x:v>
+      </x:c>
+      <x:c r="G10" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H10" s="1" t="str">
+        <x:v>Explicit resume and pause; clock timestamps; 45 minutes 38 seconds; no notebook code or output submitted for review</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Drive revision from learning notes and save daily handoff
</commit_message>
<xml_diff>
--- a/outputs/study-tracker/study-hours.xlsx
+++ b/outputs/study-tracker/study-hours.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="R5b131d87a3eb4221"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="R6125572898c64ece"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="Rc300a46b03f14ebd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="Rbc6d7cc6059248a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="R801fa213fbf44f98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="R6913d5206433495b"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Save Python learning progress and command-based checkpoints
</commit_message>
<xml_diff>
--- a/outputs/study-tracker/study-hours.xlsx
+++ b/outputs/study-tracker/study-hours.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="Rbc6d7cc6059248a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="R801fa213fbf44f98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="R6913d5206433495b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="Rb1591a1a45824674"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="Rc75e3e2caf614c15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="Raa35522b94e94052"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -354,7 +354,7 @@
         <x:v>Reporting date (IST)</x:v>
       </x:c>
       <x:c r="B4" s="8" t="n">
-        <x:v>46310</x:v>
+        <x:v>46311</x:v>
       </x:c>
       <x:c r="C4" s="1"/>
       <x:c r="D4" s="1" t="str">
@@ -362,7 +362,7 @@
       </x:c>
       <x:c r="E4" s="6" t="n">
         <x:f>SUM(E15:E130)</x:f>
-        <x:v>2.8094444444449995</x:v>
+        <x:v>4.371944444444999</x:v>
       </x:c>
       <x:c r="F4" s="1"/>
       <x:c r="G4" s="1"/>
@@ -383,7 +383,7 @@
       </x:c>
       <x:c r="E5" s="6" t="n">
         <x:f>SUMIFS(D15:D130,A15:A130,"&lt;"&amp;B4)</x:f>
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F5" s="1"/>
       <x:c r="G5" s="1"/>
@@ -404,7 +404,7 @@
       </x:c>
       <x:c r="E6" s="6" t="n">
         <x:f>MAX(E5-SUMIFS(E15:E130,A15:A130,"&lt;"&amp;B4),0)</x:f>
-        <x:v>0</x:v>
+        <x:v>3.1905555555550005</x:v>
       </x:c>
       <x:c r="F6" s="1"/>
       <x:c r="G6" s="1"/>
@@ -442,7 +442,7 @@
       </x:c>
       <x:c r="E8" s="6" t="n">
         <x:f>MAX(SUMIFS(D15:D130,A15:A130,B4)-SUMIFS(E15:E130,A15:A130,B4),0)</x:f>
-        <x:v>3.1905555555550005</x:v>
+        <x:v>4.4375</x:v>
       </x:c>
       <x:c r="F8" s="1"/>
       <x:c r="G8" s="1"/>
@@ -564,25 +564,28 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E15" s="6" t="n">
-        <x:f>IF(A15&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A15,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A15&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A15,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
         <x:v>2.8094444444449995</x:v>
       </x:c>
-      <x:c r="F15" s="6" t="str">
+      <x:c r="F15" s="6" t="n">
         <x:f>IF(A15&gt;=$B$4,"",MAX(D15-E15,0))</x:f>
-      </x:c>
-      <x:c r="G15" s="6" t="str">
+        <x:v>3.1905555555550005</x:v>
+      </x:c>
+      <x:c r="G15" s="6" t="n">
         <x:f>IF(A15&gt;=$B$4,"",MAX(E15-D15,0))</x:f>
-      </x:c>
-      <x:c r="H15" s="6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H15" s="6" t="n">
         <x:f>IF(A15&gt;=$B$4,"",SUM($D$15:D15))</x:f>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="I15" s="6" t="n">
         <x:f>IF(A15&gt;$B$4,"",SUM($E$15:E15))</x:f>
         <x:v>2.8094444444449995</x:v>
       </x:c>
       <x:c r="J15" s="1" t="str">
-        <x:f>IF(A15&gt;$B$4,"Future",IF(A15=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A15,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E15=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>In progress</x:v>
+        <x:f>IF(A15&gt;$B$4,"Future",IF(A15=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A15,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E15=0,"No confirmed time","Logged"))))</x:f>
+        <x:v>Uncertain time</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
@@ -600,8 +603,9 @@
         <x:f>IF(WEEKDAY(A16,2)&gt;5,$B$7,$B$6)</x:f>
         <x:v>6</x:v>
       </x:c>
-      <x:c r="E16" s="6" t="str">
-        <x:f>IF(A16&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A16,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+      <x:c r="E16" s="6" t="n">
+        <x:f>IF(A16&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A16,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:v>1.5625</x:v>
       </x:c>
       <x:c r="F16" s="6" t="str">
         <x:f>IF(A16&gt;=$B$4,"",MAX(D16-E16,0))</x:f>
@@ -612,12 +616,13 @@
       <x:c r="H16" s="6" t="str">
         <x:f>IF(A16&gt;=$B$4,"",SUM($D$15:D16))</x:f>
       </x:c>
-      <x:c r="I16" s="6" t="str">
+      <x:c r="I16" s="6" t="n">
         <x:f>IF(A16&gt;$B$4,"",SUM($E$15:E16))</x:f>
+        <x:v>4.371944444444999</x:v>
       </x:c>
       <x:c r="J16" s="1" t="str">
-        <x:f>IF(A16&gt;$B$4,"Future",IF(A16=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A16,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E16=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
+        <x:f>IF(A16&gt;$B$4,"Future",IF(A16=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A16,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E16=0,"No confirmed time","Logged"))))</x:f>
+        <x:v>In progress</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
@@ -636,7 +641,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E17" s="6" t="str">
-        <x:f>IF(A17&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A17,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A17&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A17,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F17" s="6" t="str">
         <x:f>IF(A17&gt;=$B$4,"",MAX(D17-E17,0))</x:f>
@@ -651,7 +656,7 @@
         <x:f>IF(A17&gt;$B$4,"",SUM($E$15:E17))</x:f>
       </x:c>
       <x:c r="J17" s="1" t="str">
-        <x:f>IF(A17&gt;$B$4,"Future",IF(A17=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A17,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E17=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A17&gt;$B$4,"Future",IF(A17=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A17,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E17=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -671,7 +676,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E18" s="6" t="str">
-        <x:f>IF(A18&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A18,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A18&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A18,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F18" s="6" t="str">
         <x:f>IF(A18&gt;=$B$4,"",MAX(D18-E18,0))</x:f>
@@ -686,7 +691,7 @@
         <x:f>IF(A18&gt;$B$4,"",SUM($E$15:E18))</x:f>
       </x:c>
       <x:c r="J18" s="1" t="str">
-        <x:f>IF(A18&gt;$B$4,"Future",IF(A18=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A18,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E18=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A18&gt;$B$4,"Future",IF(A18=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A18,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E18=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -706,7 +711,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E19" s="6" t="str">
-        <x:f>IF(A19&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A19,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A19&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A19,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F19" s="6" t="str">
         <x:f>IF(A19&gt;=$B$4,"",MAX(D19-E19,0))</x:f>
@@ -721,7 +726,7 @@
         <x:f>IF(A19&gt;$B$4,"",SUM($E$15:E19))</x:f>
       </x:c>
       <x:c r="J19" s="1" t="str">
-        <x:f>IF(A19&gt;$B$4,"Future",IF(A19=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A19,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E19=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A19&gt;$B$4,"Future",IF(A19=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A19,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E19=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -741,7 +746,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E20" s="6" t="str">
-        <x:f>IF(A20&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A20,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A20&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A20,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F20" s="6" t="str">
         <x:f>IF(A20&gt;=$B$4,"",MAX(D20-E20,0))</x:f>
@@ -756,7 +761,7 @@
         <x:f>IF(A20&gt;$B$4,"",SUM($E$15:E20))</x:f>
       </x:c>
       <x:c r="J20" s="1" t="str">
-        <x:f>IF(A20&gt;$B$4,"Future",IF(A20=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A20,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E20=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A20&gt;$B$4,"Future",IF(A20=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A20,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E20=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -776,7 +781,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E21" s="6" t="str">
-        <x:f>IF(A21&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A21,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A21&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A21,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F21" s="6" t="str">
         <x:f>IF(A21&gt;=$B$4,"",MAX(D21-E21,0))</x:f>
@@ -791,7 +796,7 @@
         <x:f>IF(A21&gt;$B$4,"",SUM($E$15:E21))</x:f>
       </x:c>
       <x:c r="J21" s="1" t="str">
-        <x:f>IF(A21&gt;$B$4,"Future",IF(A21=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A21,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E21=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A21&gt;$B$4,"Future",IF(A21=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A21,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E21=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -811,7 +816,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E22" s="6" t="str">
-        <x:f>IF(A22&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A22,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A22&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A22,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F22" s="6" t="str">
         <x:f>IF(A22&gt;=$B$4,"",MAX(D22-E22,0))</x:f>
@@ -826,7 +831,7 @@
         <x:f>IF(A22&gt;$B$4,"",SUM($E$15:E22))</x:f>
       </x:c>
       <x:c r="J22" s="1" t="str">
-        <x:f>IF(A22&gt;$B$4,"Future",IF(A22=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A22,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E22=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A22&gt;$B$4,"Future",IF(A22=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A22,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E22=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -846,7 +851,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E23" s="6" t="str">
-        <x:f>IF(A23&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A23,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A23&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A23,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F23" s="6" t="str">
         <x:f>IF(A23&gt;=$B$4,"",MAX(D23-E23,0))</x:f>
@@ -861,7 +866,7 @@
         <x:f>IF(A23&gt;$B$4,"",SUM($E$15:E23))</x:f>
       </x:c>
       <x:c r="J23" s="1" t="str">
-        <x:f>IF(A23&gt;$B$4,"Future",IF(A23=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A23,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E23=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A23&gt;$B$4,"Future",IF(A23=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A23,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E23=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -881,7 +886,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E24" s="6" t="str">
-        <x:f>IF(A24&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A24,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A24&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A24,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F24" s="6" t="str">
         <x:f>IF(A24&gt;=$B$4,"",MAX(D24-E24,0))</x:f>
@@ -896,7 +901,7 @@
         <x:f>IF(A24&gt;$B$4,"",SUM($E$15:E24))</x:f>
       </x:c>
       <x:c r="J24" s="1" t="str">
-        <x:f>IF(A24&gt;$B$4,"Future",IF(A24=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A24,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E24=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A24&gt;$B$4,"Future",IF(A24=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A24,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E24=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -916,7 +921,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E25" s="6" t="str">
-        <x:f>IF(A25&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A25,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A25&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A25,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F25" s="6" t="str">
         <x:f>IF(A25&gt;=$B$4,"",MAX(D25-E25,0))</x:f>
@@ -931,7 +936,7 @@
         <x:f>IF(A25&gt;$B$4,"",SUM($E$15:E25))</x:f>
       </x:c>
       <x:c r="J25" s="1" t="str">
-        <x:f>IF(A25&gt;$B$4,"Future",IF(A25=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A25,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E25=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A25&gt;$B$4,"Future",IF(A25=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A25,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E25=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -951,7 +956,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E26" s="6" t="str">
-        <x:f>IF(A26&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A26,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A26&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A26,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F26" s="6" t="str">
         <x:f>IF(A26&gt;=$B$4,"",MAX(D26-E26,0))</x:f>
@@ -966,7 +971,7 @@
         <x:f>IF(A26&gt;$B$4,"",SUM($E$15:E26))</x:f>
       </x:c>
       <x:c r="J26" s="1" t="str">
-        <x:f>IF(A26&gt;$B$4,"Future",IF(A26=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A26,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E26=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A26&gt;$B$4,"Future",IF(A26=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A26,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E26=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -986,7 +991,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E27" s="6" t="str">
-        <x:f>IF(A27&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A27,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A27&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A27,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F27" s="6" t="str">
         <x:f>IF(A27&gt;=$B$4,"",MAX(D27-E27,0))</x:f>
@@ -1001,7 +1006,7 @@
         <x:f>IF(A27&gt;$B$4,"",SUM($E$15:E27))</x:f>
       </x:c>
       <x:c r="J27" s="1" t="str">
-        <x:f>IF(A27&gt;$B$4,"Future",IF(A27=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A27,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E27=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A27&gt;$B$4,"Future",IF(A27=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A27,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E27=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1021,7 +1026,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E28" s="6" t="str">
-        <x:f>IF(A28&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A28,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A28&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A28,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F28" s="6" t="str">
         <x:f>IF(A28&gt;=$B$4,"",MAX(D28-E28,0))</x:f>
@@ -1036,7 +1041,7 @@
         <x:f>IF(A28&gt;$B$4,"",SUM($E$15:E28))</x:f>
       </x:c>
       <x:c r="J28" s="1" t="str">
-        <x:f>IF(A28&gt;$B$4,"Future",IF(A28=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A28,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E28=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A28&gt;$B$4,"Future",IF(A28=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A28,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E28=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1056,7 +1061,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E29" s="6" t="str">
-        <x:f>IF(A29&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A29,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A29&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A29,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F29" s="6" t="str">
         <x:f>IF(A29&gt;=$B$4,"",MAX(D29-E29,0))</x:f>
@@ -1071,7 +1076,7 @@
         <x:f>IF(A29&gt;$B$4,"",SUM($E$15:E29))</x:f>
       </x:c>
       <x:c r="J29" s="1" t="str">
-        <x:f>IF(A29&gt;$B$4,"Future",IF(A29=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A29,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E29=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A29&gt;$B$4,"Future",IF(A29=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A29,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E29=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1091,7 +1096,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E30" s="6" t="str">
-        <x:f>IF(A30&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A30,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A30&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A30,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F30" s="6" t="str">
         <x:f>IF(A30&gt;=$B$4,"",MAX(D30-E30,0))</x:f>
@@ -1106,7 +1111,7 @@
         <x:f>IF(A30&gt;$B$4,"",SUM($E$15:E30))</x:f>
       </x:c>
       <x:c r="J30" s="1" t="str">
-        <x:f>IF(A30&gt;$B$4,"Future",IF(A30=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A30,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E30=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A30&gt;$B$4,"Future",IF(A30=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A30,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E30=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1126,7 +1131,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E31" s="6" t="str">
-        <x:f>IF(A31&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A31,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A31&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A31,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F31" s="6" t="str">
         <x:f>IF(A31&gt;=$B$4,"",MAX(D31-E31,0))</x:f>
@@ -1141,7 +1146,7 @@
         <x:f>IF(A31&gt;$B$4,"",SUM($E$15:E31))</x:f>
       </x:c>
       <x:c r="J31" s="1" t="str">
-        <x:f>IF(A31&gt;$B$4,"Future",IF(A31=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A31,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E31=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A31&gt;$B$4,"Future",IF(A31=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A31,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E31=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1161,7 +1166,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E32" s="6" t="str">
-        <x:f>IF(A32&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A32,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A32&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A32,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F32" s="6" t="str">
         <x:f>IF(A32&gt;=$B$4,"",MAX(D32-E32,0))</x:f>
@@ -1176,7 +1181,7 @@
         <x:f>IF(A32&gt;$B$4,"",SUM($E$15:E32))</x:f>
       </x:c>
       <x:c r="J32" s="1" t="str">
-        <x:f>IF(A32&gt;$B$4,"Future",IF(A32=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A32,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E32=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A32&gt;$B$4,"Future",IF(A32=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A32,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E32=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1196,7 +1201,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E33" s="6" t="str">
-        <x:f>IF(A33&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A33,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A33&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A33,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F33" s="6" t="str">
         <x:f>IF(A33&gt;=$B$4,"",MAX(D33-E33,0))</x:f>
@@ -1211,7 +1216,7 @@
         <x:f>IF(A33&gt;$B$4,"",SUM($E$15:E33))</x:f>
       </x:c>
       <x:c r="J33" s="1" t="str">
-        <x:f>IF(A33&gt;$B$4,"Future",IF(A33=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A33,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E33=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A33&gt;$B$4,"Future",IF(A33=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A33,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E33=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1231,7 +1236,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E34" s="6" t="str">
-        <x:f>IF(A34&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A34,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A34&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A34,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F34" s="6" t="str">
         <x:f>IF(A34&gt;=$B$4,"",MAX(D34-E34,0))</x:f>
@@ -1246,7 +1251,7 @@
         <x:f>IF(A34&gt;$B$4,"",SUM($E$15:E34))</x:f>
       </x:c>
       <x:c r="J34" s="1" t="str">
-        <x:f>IF(A34&gt;$B$4,"Future",IF(A34=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A34,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E34=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A34&gt;$B$4,"Future",IF(A34=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A34,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E34=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1266,7 +1271,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E35" s="6" t="str">
-        <x:f>IF(A35&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A35,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A35&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A35,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F35" s="6" t="str">
         <x:f>IF(A35&gt;=$B$4,"",MAX(D35-E35,0))</x:f>
@@ -1281,7 +1286,7 @@
         <x:f>IF(A35&gt;$B$4,"",SUM($E$15:E35))</x:f>
       </x:c>
       <x:c r="J35" s="1" t="str">
-        <x:f>IF(A35&gt;$B$4,"Future",IF(A35=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A35,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E35=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A35&gt;$B$4,"Future",IF(A35=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A35,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E35=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1301,7 +1306,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E36" s="6" t="str">
-        <x:f>IF(A36&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A36,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A36&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A36,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F36" s="6" t="str">
         <x:f>IF(A36&gt;=$B$4,"",MAX(D36-E36,0))</x:f>
@@ -1316,7 +1321,7 @@
         <x:f>IF(A36&gt;$B$4,"",SUM($E$15:E36))</x:f>
       </x:c>
       <x:c r="J36" s="1" t="str">
-        <x:f>IF(A36&gt;$B$4,"Future",IF(A36=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A36,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E36=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A36&gt;$B$4,"Future",IF(A36=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A36,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E36=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1336,7 +1341,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E37" s="6" t="str">
-        <x:f>IF(A37&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A37,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A37&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A37,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F37" s="6" t="str">
         <x:f>IF(A37&gt;=$B$4,"",MAX(D37-E37,0))</x:f>
@@ -1351,7 +1356,7 @@
         <x:f>IF(A37&gt;$B$4,"",SUM($E$15:E37))</x:f>
       </x:c>
       <x:c r="J37" s="1" t="str">
-        <x:f>IF(A37&gt;$B$4,"Future",IF(A37=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A37,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E37=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A37&gt;$B$4,"Future",IF(A37=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A37,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E37=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1371,7 +1376,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E38" s="6" t="str">
-        <x:f>IF(A38&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A38,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A38&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A38,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F38" s="6" t="str">
         <x:f>IF(A38&gt;=$B$4,"",MAX(D38-E38,0))</x:f>
@@ -1386,7 +1391,7 @@
         <x:f>IF(A38&gt;$B$4,"",SUM($E$15:E38))</x:f>
       </x:c>
       <x:c r="J38" s="1" t="str">
-        <x:f>IF(A38&gt;$B$4,"Future",IF(A38=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A38,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E38=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A38&gt;$B$4,"Future",IF(A38=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A38,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E38=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1406,7 +1411,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E39" s="6" t="str">
-        <x:f>IF(A39&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A39,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A39&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A39,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F39" s="6" t="str">
         <x:f>IF(A39&gt;=$B$4,"",MAX(D39-E39,0))</x:f>
@@ -1421,7 +1426,7 @@
         <x:f>IF(A39&gt;$B$4,"",SUM($E$15:E39))</x:f>
       </x:c>
       <x:c r="J39" s="1" t="str">
-        <x:f>IF(A39&gt;$B$4,"Future",IF(A39=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A39,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E39=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A39&gt;$B$4,"Future",IF(A39=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A39,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E39=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1441,7 +1446,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E40" s="6" t="str">
-        <x:f>IF(A40&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A40,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A40&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A40,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F40" s="6" t="str">
         <x:f>IF(A40&gt;=$B$4,"",MAX(D40-E40,0))</x:f>
@@ -1456,7 +1461,7 @@
         <x:f>IF(A40&gt;$B$4,"",SUM($E$15:E40))</x:f>
       </x:c>
       <x:c r="J40" s="1" t="str">
-        <x:f>IF(A40&gt;$B$4,"Future",IF(A40=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A40,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E40=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A40&gt;$B$4,"Future",IF(A40=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A40,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E40=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1476,7 +1481,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E41" s="6" t="str">
-        <x:f>IF(A41&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A41,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A41&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A41,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F41" s="6" t="str">
         <x:f>IF(A41&gt;=$B$4,"",MAX(D41-E41,0))</x:f>
@@ -1491,7 +1496,7 @@
         <x:f>IF(A41&gt;$B$4,"",SUM($E$15:E41))</x:f>
       </x:c>
       <x:c r="J41" s="1" t="str">
-        <x:f>IF(A41&gt;$B$4,"Future",IF(A41=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A41,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E41=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A41&gt;$B$4,"Future",IF(A41=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A41,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E41=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1511,7 +1516,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E42" s="6" t="str">
-        <x:f>IF(A42&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A42,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A42&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A42,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F42" s="6" t="str">
         <x:f>IF(A42&gt;=$B$4,"",MAX(D42-E42,0))</x:f>
@@ -1526,7 +1531,7 @@
         <x:f>IF(A42&gt;$B$4,"",SUM($E$15:E42))</x:f>
       </x:c>
       <x:c r="J42" s="1" t="str">
-        <x:f>IF(A42&gt;$B$4,"Future",IF(A42=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A42,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E42=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A42&gt;$B$4,"Future",IF(A42=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A42,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E42=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1546,7 +1551,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E43" s="6" t="str">
-        <x:f>IF(A43&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A43,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A43&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A43,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F43" s="6" t="str">
         <x:f>IF(A43&gt;=$B$4,"",MAX(D43-E43,0))</x:f>
@@ -1561,7 +1566,7 @@
         <x:f>IF(A43&gt;$B$4,"",SUM($E$15:E43))</x:f>
       </x:c>
       <x:c r="J43" s="1" t="str">
-        <x:f>IF(A43&gt;$B$4,"Future",IF(A43=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A43,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E43=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A43&gt;$B$4,"Future",IF(A43=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A43,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E43=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1581,7 +1586,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E44" s="6" t="str">
-        <x:f>IF(A44&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A44,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A44&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A44,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F44" s="6" t="str">
         <x:f>IF(A44&gt;=$B$4,"",MAX(D44-E44,0))</x:f>
@@ -1596,7 +1601,7 @@
         <x:f>IF(A44&gt;$B$4,"",SUM($E$15:E44))</x:f>
       </x:c>
       <x:c r="J44" s="1" t="str">
-        <x:f>IF(A44&gt;$B$4,"Future",IF(A44=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A44,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E44=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A44&gt;$B$4,"Future",IF(A44=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A44,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E44=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1616,7 +1621,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E45" s="6" t="str">
-        <x:f>IF(A45&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A45,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A45&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A45,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F45" s="6" t="str">
         <x:f>IF(A45&gt;=$B$4,"",MAX(D45-E45,0))</x:f>
@@ -1631,7 +1636,7 @@
         <x:f>IF(A45&gt;$B$4,"",SUM($E$15:E45))</x:f>
       </x:c>
       <x:c r="J45" s="1" t="str">
-        <x:f>IF(A45&gt;$B$4,"Future",IF(A45=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A45,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E45=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A45&gt;$B$4,"Future",IF(A45=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A45,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E45=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1651,7 +1656,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E46" s="6" t="str">
-        <x:f>IF(A46&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A46,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A46&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A46,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F46" s="6" t="str">
         <x:f>IF(A46&gt;=$B$4,"",MAX(D46-E46,0))</x:f>
@@ -1666,7 +1671,7 @@
         <x:f>IF(A46&gt;$B$4,"",SUM($E$15:E46))</x:f>
       </x:c>
       <x:c r="J46" s="1" t="str">
-        <x:f>IF(A46&gt;$B$4,"Future",IF(A46=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A46,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E46=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A46&gt;$B$4,"Future",IF(A46=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A46,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E46=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1686,7 +1691,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E47" s="6" t="str">
-        <x:f>IF(A47&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A47,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A47&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A47,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F47" s="6" t="str">
         <x:f>IF(A47&gt;=$B$4,"",MAX(D47-E47,0))</x:f>
@@ -1701,7 +1706,7 @@
         <x:f>IF(A47&gt;$B$4,"",SUM($E$15:E47))</x:f>
       </x:c>
       <x:c r="J47" s="1" t="str">
-        <x:f>IF(A47&gt;$B$4,"Future",IF(A47=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A47,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E47=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A47&gt;$B$4,"Future",IF(A47=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A47,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E47=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1721,7 +1726,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E48" s="6" t="str">
-        <x:f>IF(A48&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A48,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A48&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A48,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F48" s="6" t="str">
         <x:f>IF(A48&gt;=$B$4,"",MAX(D48-E48,0))</x:f>
@@ -1736,7 +1741,7 @@
         <x:f>IF(A48&gt;$B$4,"",SUM($E$15:E48))</x:f>
       </x:c>
       <x:c r="J48" s="1" t="str">
-        <x:f>IF(A48&gt;$B$4,"Future",IF(A48=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A48,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E48=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A48&gt;$B$4,"Future",IF(A48=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A48,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E48=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1756,7 +1761,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E49" s="6" t="str">
-        <x:f>IF(A49&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A49,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A49&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A49,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F49" s="6" t="str">
         <x:f>IF(A49&gt;=$B$4,"",MAX(D49-E49,0))</x:f>
@@ -1771,7 +1776,7 @@
         <x:f>IF(A49&gt;$B$4,"",SUM($E$15:E49))</x:f>
       </x:c>
       <x:c r="J49" s="1" t="str">
-        <x:f>IF(A49&gt;$B$4,"Future",IF(A49=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A49,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E49=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A49&gt;$B$4,"Future",IF(A49=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A49,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E49=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1791,7 +1796,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E50" s="6" t="str">
-        <x:f>IF(A50&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A50,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A50&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A50,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F50" s="6" t="str">
         <x:f>IF(A50&gt;=$B$4,"",MAX(D50-E50,0))</x:f>
@@ -1806,7 +1811,7 @@
         <x:f>IF(A50&gt;$B$4,"",SUM($E$15:E50))</x:f>
       </x:c>
       <x:c r="J50" s="1" t="str">
-        <x:f>IF(A50&gt;$B$4,"Future",IF(A50=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A50,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E50=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A50&gt;$B$4,"Future",IF(A50=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A50,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E50=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1826,7 +1831,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E51" s="6" t="str">
-        <x:f>IF(A51&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A51,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A51&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A51,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F51" s="6" t="str">
         <x:f>IF(A51&gt;=$B$4,"",MAX(D51-E51,0))</x:f>
@@ -1841,7 +1846,7 @@
         <x:f>IF(A51&gt;$B$4,"",SUM($E$15:E51))</x:f>
       </x:c>
       <x:c r="J51" s="1" t="str">
-        <x:f>IF(A51&gt;$B$4,"Future",IF(A51=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A51,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E51=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A51&gt;$B$4,"Future",IF(A51=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A51,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E51=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1861,7 +1866,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E52" s="6" t="str">
-        <x:f>IF(A52&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A52,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A52&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A52,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F52" s="6" t="str">
         <x:f>IF(A52&gt;=$B$4,"",MAX(D52-E52,0))</x:f>
@@ -1876,7 +1881,7 @@
         <x:f>IF(A52&gt;$B$4,"",SUM($E$15:E52))</x:f>
       </x:c>
       <x:c r="J52" s="1" t="str">
-        <x:f>IF(A52&gt;$B$4,"Future",IF(A52=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A52,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E52=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A52&gt;$B$4,"Future",IF(A52=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A52,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E52=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1896,7 +1901,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E53" s="6" t="str">
-        <x:f>IF(A53&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A53,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A53&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A53,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F53" s="6" t="str">
         <x:f>IF(A53&gt;=$B$4,"",MAX(D53-E53,0))</x:f>
@@ -1911,7 +1916,7 @@
         <x:f>IF(A53&gt;$B$4,"",SUM($E$15:E53))</x:f>
       </x:c>
       <x:c r="J53" s="1" t="str">
-        <x:f>IF(A53&gt;$B$4,"Future",IF(A53=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A53,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E53=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A53&gt;$B$4,"Future",IF(A53=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A53,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E53=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1931,7 +1936,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E54" s="6" t="str">
-        <x:f>IF(A54&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A54,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A54&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A54,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F54" s="6" t="str">
         <x:f>IF(A54&gt;=$B$4,"",MAX(D54-E54,0))</x:f>
@@ -1946,7 +1951,7 @@
         <x:f>IF(A54&gt;$B$4,"",SUM($E$15:E54))</x:f>
       </x:c>
       <x:c r="J54" s="1" t="str">
-        <x:f>IF(A54&gt;$B$4,"Future",IF(A54=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A54,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E54=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A54&gt;$B$4,"Future",IF(A54=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A54,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E54=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1966,7 +1971,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E55" s="6" t="str">
-        <x:f>IF(A55&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A55,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A55&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A55,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F55" s="6" t="str">
         <x:f>IF(A55&gt;=$B$4,"",MAX(D55-E55,0))</x:f>
@@ -1981,7 +1986,7 @@
         <x:f>IF(A55&gt;$B$4,"",SUM($E$15:E55))</x:f>
       </x:c>
       <x:c r="J55" s="1" t="str">
-        <x:f>IF(A55&gt;$B$4,"Future",IF(A55=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A55,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E55=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A55&gt;$B$4,"Future",IF(A55=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A55,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E55=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2001,7 +2006,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E56" s="6" t="str">
-        <x:f>IF(A56&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A56,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A56&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A56,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F56" s="6" t="str">
         <x:f>IF(A56&gt;=$B$4,"",MAX(D56-E56,0))</x:f>
@@ -2016,7 +2021,7 @@
         <x:f>IF(A56&gt;$B$4,"",SUM($E$15:E56))</x:f>
       </x:c>
       <x:c r="J56" s="1" t="str">
-        <x:f>IF(A56&gt;$B$4,"Future",IF(A56=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A56,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E56=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A56&gt;$B$4,"Future",IF(A56=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A56,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E56=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2036,7 +2041,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E57" s="6" t="str">
-        <x:f>IF(A57&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A57,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A57&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A57,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F57" s="6" t="str">
         <x:f>IF(A57&gt;=$B$4,"",MAX(D57-E57,0))</x:f>
@@ -2051,7 +2056,7 @@
         <x:f>IF(A57&gt;$B$4,"",SUM($E$15:E57))</x:f>
       </x:c>
       <x:c r="J57" s="1" t="str">
-        <x:f>IF(A57&gt;$B$4,"Future",IF(A57=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A57,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E57=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A57&gt;$B$4,"Future",IF(A57=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A57,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E57=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2071,7 +2076,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E58" s="6" t="str">
-        <x:f>IF(A58&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A58,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A58&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A58,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F58" s="6" t="str">
         <x:f>IF(A58&gt;=$B$4,"",MAX(D58-E58,0))</x:f>
@@ -2086,7 +2091,7 @@
         <x:f>IF(A58&gt;$B$4,"",SUM($E$15:E58))</x:f>
       </x:c>
       <x:c r="J58" s="1" t="str">
-        <x:f>IF(A58&gt;$B$4,"Future",IF(A58=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A58,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E58=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A58&gt;$B$4,"Future",IF(A58=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A58,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E58=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2106,7 +2111,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E59" s="6" t="str">
-        <x:f>IF(A59&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A59,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A59&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A59,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F59" s="6" t="str">
         <x:f>IF(A59&gt;=$B$4,"",MAX(D59-E59,0))</x:f>
@@ -2121,7 +2126,7 @@
         <x:f>IF(A59&gt;$B$4,"",SUM($E$15:E59))</x:f>
       </x:c>
       <x:c r="J59" s="1" t="str">
-        <x:f>IF(A59&gt;$B$4,"Future",IF(A59=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A59,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E59=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A59&gt;$B$4,"Future",IF(A59=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A59,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E59=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2141,7 +2146,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E60" s="6" t="str">
-        <x:f>IF(A60&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A60,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A60&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A60,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F60" s="6" t="str">
         <x:f>IF(A60&gt;=$B$4,"",MAX(D60-E60,0))</x:f>
@@ -2156,7 +2161,7 @@
         <x:f>IF(A60&gt;$B$4,"",SUM($E$15:E60))</x:f>
       </x:c>
       <x:c r="J60" s="1" t="str">
-        <x:f>IF(A60&gt;$B$4,"Future",IF(A60=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A60,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E60=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A60&gt;$B$4,"Future",IF(A60=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A60,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E60=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2176,7 +2181,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E61" s="6" t="str">
-        <x:f>IF(A61&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A61,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A61&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A61,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F61" s="6" t="str">
         <x:f>IF(A61&gt;=$B$4,"",MAX(D61-E61,0))</x:f>
@@ -2191,7 +2196,7 @@
         <x:f>IF(A61&gt;$B$4,"",SUM($E$15:E61))</x:f>
       </x:c>
       <x:c r="J61" s="1" t="str">
-        <x:f>IF(A61&gt;$B$4,"Future",IF(A61=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A61,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E61=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A61&gt;$B$4,"Future",IF(A61=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A61,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E61=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2211,7 +2216,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E62" s="6" t="str">
-        <x:f>IF(A62&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A62,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A62&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A62,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F62" s="6" t="str">
         <x:f>IF(A62&gt;=$B$4,"",MAX(D62-E62,0))</x:f>
@@ -2226,7 +2231,7 @@
         <x:f>IF(A62&gt;$B$4,"",SUM($E$15:E62))</x:f>
       </x:c>
       <x:c r="J62" s="1" t="str">
-        <x:f>IF(A62&gt;$B$4,"Future",IF(A62=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A62,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E62=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A62&gt;$B$4,"Future",IF(A62=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A62,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E62=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2246,7 +2251,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E63" s="6" t="str">
-        <x:f>IF(A63&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A63,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A63&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A63,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F63" s="6" t="str">
         <x:f>IF(A63&gt;=$B$4,"",MAX(D63-E63,0))</x:f>
@@ -2261,7 +2266,7 @@
         <x:f>IF(A63&gt;$B$4,"",SUM($E$15:E63))</x:f>
       </x:c>
       <x:c r="J63" s="1" t="str">
-        <x:f>IF(A63&gt;$B$4,"Future",IF(A63=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A63,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E63=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A63&gt;$B$4,"Future",IF(A63=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A63,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E63=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2281,7 +2286,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E64" s="6" t="str">
-        <x:f>IF(A64&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A64,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A64&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A64,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F64" s="6" t="str">
         <x:f>IF(A64&gt;=$B$4,"",MAX(D64-E64,0))</x:f>
@@ -2296,7 +2301,7 @@
         <x:f>IF(A64&gt;$B$4,"",SUM($E$15:E64))</x:f>
       </x:c>
       <x:c r="J64" s="1" t="str">
-        <x:f>IF(A64&gt;$B$4,"Future",IF(A64=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A64,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E64=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A64&gt;$B$4,"Future",IF(A64=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A64,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E64=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2316,7 +2321,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E65" s="6" t="str">
-        <x:f>IF(A65&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A65,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A65&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A65,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F65" s="6" t="str">
         <x:f>IF(A65&gt;=$B$4,"",MAX(D65-E65,0))</x:f>
@@ -2331,7 +2336,7 @@
         <x:f>IF(A65&gt;$B$4,"",SUM($E$15:E65))</x:f>
       </x:c>
       <x:c r="J65" s="1" t="str">
-        <x:f>IF(A65&gt;$B$4,"Future",IF(A65=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A65,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E65=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A65&gt;$B$4,"Future",IF(A65=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A65,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E65=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2351,7 +2356,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E66" s="6" t="str">
-        <x:f>IF(A66&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A66,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A66&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A66,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F66" s="6" t="str">
         <x:f>IF(A66&gt;=$B$4,"",MAX(D66-E66,0))</x:f>
@@ -2366,7 +2371,7 @@
         <x:f>IF(A66&gt;$B$4,"",SUM($E$15:E66))</x:f>
       </x:c>
       <x:c r="J66" s="1" t="str">
-        <x:f>IF(A66&gt;$B$4,"Future",IF(A66=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A66,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E66=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A66&gt;$B$4,"Future",IF(A66=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A66,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E66=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2386,7 +2391,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E67" s="6" t="str">
-        <x:f>IF(A67&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A67,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A67&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A67,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F67" s="6" t="str">
         <x:f>IF(A67&gt;=$B$4,"",MAX(D67-E67,0))</x:f>
@@ -2401,7 +2406,7 @@
         <x:f>IF(A67&gt;$B$4,"",SUM($E$15:E67))</x:f>
       </x:c>
       <x:c r="J67" s="1" t="str">
-        <x:f>IF(A67&gt;$B$4,"Future",IF(A67=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A67,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E67=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A67&gt;$B$4,"Future",IF(A67=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A67,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E67=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2421,7 +2426,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E68" s="6" t="str">
-        <x:f>IF(A68&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A68,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A68&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A68,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F68" s="6" t="str">
         <x:f>IF(A68&gt;=$B$4,"",MAX(D68-E68,0))</x:f>
@@ -2436,7 +2441,7 @@
         <x:f>IF(A68&gt;$B$4,"",SUM($E$15:E68))</x:f>
       </x:c>
       <x:c r="J68" s="1" t="str">
-        <x:f>IF(A68&gt;$B$4,"Future",IF(A68=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A68,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E68=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A68&gt;$B$4,"Future",IF(A68=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A68,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E68=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2456,7 +2461,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E69" s="6" t="str">
-        <x:f>IF(A69&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A69,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A69&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A69,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F69" s="6" t="str">
         <x:f>IF(A69&gt;=$B$4,"",MAX(D69-E69,0))</x:f>
@@ -2471,7 +2476,7 @@
         <x:f>IF(A69&gt;$B$4,"",SUM($E$15:E69))</x:f>
       </x:c>
       <x:c r="J69" s="1" t="str">
-        <x:f>IF(A69&gt;$B$4,"Future",IF(A69=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A69,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E69=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A69&gt;$B$4,"Future",IF(A69=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A69,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E69=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2491,7 +2496,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E70" s="6" t="str">
-        <x:f>IF(A70&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A70,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A70&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A70,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F70" s="6" t="str">
         <x:f>IF(A70&gt;=$B$4,"",MAX(D70-E70,0))</x:f>
@@ -2506,7 +2511,7 @@
         <x:f>IF(A70&gt;$B$4,"",SUM($E$15:E70))</x:f>
       </x:c>
       <x:c r="J70" s="1" t="str">
-        <x:f>IF(A70&gt;$B$4,"Future",IF(A70=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A70,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E70=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A70&gt;$B$4,"Future",IF(A70=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A70,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E70=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2526,7 +2531,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E71" s="6" t="str">
-        <x:f>IF(A71&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A71,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A71&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A71,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F71" s="6" t="str">
         <x:f>IF(A71&gt;=$B$4,"",MAX(D71-E71,0))</x:f>
@@ -2541,7 +2546,7 @@
         <x:f>IF(A71&gt;$B$4,"",SUM($E$15:E71))</x:f>
       </x:c>
       <x:c r="J71" s="1" t="str">
-        <x:f>IF(A71&gt;$B$4,"Future",IF(A71=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A71,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E71=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A71&gt;$B$4,"Future",IF(A71=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A71,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E71=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2561,7 +2566,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E72" s="6" t="str">
-        <x:f>IF(A72&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A72,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A72&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A72,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F72" s="6" t="str">
         <x:f>IF(A72&gt;=$B$4,"",MAX(D72-E72,0))</x:f>
@@ -2576,7 +2581,7 @@
         <x:f>IF(A72&gt;$B$4,"",SUM($E$15:E72))</x:f>
       </x:c>
       <x:c r="J72" s="1" t="str">
-        <x:f>IF(A72&gt;$B$4,"Future",IF(A72=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A72,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E72=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A72&gt;$B$4,"Future",IF(A72=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A72,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E72=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2596,7 +2601,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E73" s="6" t="str">
-        <x:f>IF(A73&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A73,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A73&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A73,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F73" s="6" t="str">
         <x:f>IF(A73&gt;=$B$4,"",MAX(D73-E73,0))</x:f>
@@ -2611,7 +2616,7 @@
         <x:f>IF(A73&gt;$B$4,"",SUM($E$15:E73))</x:f>
       </x:c>
       <x:c r="J73" s="1" t="str">
-        <x:f>IF(A73&gt;$B$4,"Future",IF(A73=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A73,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E73=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A73&gt;$B$4,"Future",IF(A73=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A73,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E73=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2631,7 +2636,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E74" s="6" t="str">
-        <x:f>IF(A74&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A74,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A74&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A74,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F74" s="6" t="str">
         <x:f>IF(A74&gt;=$B$4,"",MAX(D74-E74,0))</x:f>
@@ -2646,7 +2651,7 @@
         <x:f>IF(A74&gt;$B$4,"",SUM($E$15:E74))</x:f>
       </x:c>
       <x:c r="J74" s="1" t="str">
-        <x:f>IF(A74&gt;$B$4,"Future",IF(A74=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A74,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E74=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A74&gt;$B$4,"Future",IF(A74=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A74,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E74=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2666,7 +2671,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E75" s="6" t="str">
-        <x:f>IF(A75&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A75,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A75&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A75,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F75" s="6" t="str">
         <x:f>IF(A75&gt;=$B$4,"",MAX(D75-E75,0))</x:f>
@@ -2681,7 +2686,7 @@
         <x:f>IF(A75&gt;$B$4,"",SUM($E$15:E75))</x:f>
       </x:c>
       <x:c r="J75" s="1" t="str">
-        <x:f>IF(A75&gt;$B$4,"Future",IF(A75=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A75,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E75=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A75&gt;$B$4,"Future",IF(A75=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A75,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E75=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2701,7 +2706,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E76" s="6" t="str">
-        <x:f>IF(A76&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A76,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A76&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A76,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F76" s="6" t="str">
         <x:f>IF(A76&gt;=$B$4,"",MAX(D76-E76,0))</x:f>
@@ -2716,7 +2721,7 @@
         <x:f>IF(A76&gt;$B$4,"",SUM($E$15:E76))</x:f>
       </x:c>
       <x:c r="J76" s="1" t="str">
-        <x:f>IF(A76&gt;$B$4,"Future",IF(A76=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A76,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E76=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A76&gt;$B$4,"Future",IF(A76=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A76,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E76=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2736,7 +2741,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E77" s="6" t="str">
-        <x:f>IF(A77&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A77,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A77&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A77,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F77" s="6" t="str">
         <x:f>IF(A77&gt;=$B$4,"",MAX(D77-E77,0))</x:f>
@@ -2751,7 +2756,7 @@
         <x:f>IF(A77&gt;$B$4,"",SUM($E$15:E77))</x:f>
       </x:c>
       <x:c r="J77" s="1" t="str">
-        <x:f>IF(A77&gt;$B$4,"Future",IF(A77=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A77,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E77=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A77&gt;$B$4,"Future",IF(A77=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A77,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E77=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2771,7 +2776,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E78" s="6" t="str">
-        <x:f>IF(A78&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A78,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A78&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A78,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F78" s="6" t="str">
         <x:f>IF(A78&gt;=$B$4,"",MAX(D78-E78,0))</x:f>
@@ -2786,7 +2791,7 @@
         <x:f>IF(A78&gt;$B$4,"",SUM($E$15:E78))</x:f>
       </x:c>
       <x:c r="J78" s="1" t="str">
-        <x:f>IF(A78&gt;$B$4,"Future",IF(A78=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A78,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E78=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A78&gt;$B$4,"Future",IF(A78=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A78,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E78=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2806,7 +2811,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E79" s="6" t="str">
-        <x:f>IF(A79&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A79,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A79&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A79,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F79" s="6" t="str">
         <x:f>IF(A79&gt;=$B$4,"",MAX(D79-E79,0))</x:f>
@@ -2821,7 +2826,7 @@
         <x:f>IF(A79&gt;$B$4,"",SUM($E$15:E79))</x:f>
       </x:c>
       <x:c r="J79" s="1" t="str">
-        <x:f>IF(A79&gt;$B$4,"Future",IF(A79=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A79,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E79=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A79&gt;$B$4,"Future",IF(A79=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A79,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E79=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2841,7 +2846,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E80" s="6" t="str">
-        <x:f>IF(A80&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A80,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A80&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A80,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F80" s="6" t="str">
         <x:f>IF(A80&gt;=$B$4,"",MAX(D80-E80,0))</x:f>
@@ -2856,7 +2861,7 @@
         <x:f>IF(A80&gt;$B$4,"",SUM($E$15:E80))</x:f>
       </x:c>
       <x:c r="J80" s="1" t="str">
-        <x:f>IF(A80&gt;$B$4,"Future",IF(A80=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A80,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E80=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A80&gt;$B$4,"Future",IF(A80=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A80,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E80=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2876,7 +2881,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E81" s="6" t="str">
-        <x:f>IF(A81&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A81,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A81&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A81,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F81" s="6" t="str">
         <x:f>IF(A81&gt;=$B$4,"",MAX(D81-E81,0))</x:f>
@@ -2891,7 +2896,7 @@
         <x:f>IF(A81&gt;$B$4,"",SUM($E$15:E81))</x:f>
       </x:c>
       <x:c r="J81" s="1" t="str">
-        <x:f>IF(A81&gt;$B$4,"Future",IF(A81=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A81,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E81=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A81&gt;$B$4,"Future",IF(A81=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A81,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E81=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2911,7 +2916,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E82" s="6" t="str">
-        <x:f>IF(A82&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A82,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A82&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A82,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F82" s="6" t="str">
         <x:f>IF(A82&gt;=$B$4,"",MAX(D82-E82,0))</x:f>
@@ -2926,7 +2931,7 @@
         <x:f>IF(A82&gt;$B$4,"",SUM($E$15:E82))</x:f>
       </x:c>
       <x:c r="J82" s="1" t="str">
-        <x:f>IF(A82&gt;$B$4,"Future",IF(A82=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A82,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E82=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A82&gt;$B$4,"Future",IF(A82=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A82,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E82=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2946,7 +2951,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E83" s="6" t="str">
-        <x:f>IF(A83&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A83,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A83&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A83,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F83" s="6" t="str">
         <x:f>IF(A83&gt;=$B$4,"",MAX(D83-E83,0))</x:f>
@@ -2961,7 +2966,7 @@
         <x:f>IF(A83&gt;$B$4,"",SUM($E$15:E83))</x:f>
       </x:c>
       <x:c r="J83" s="1" t="str">
-        <x:f>IF(A83&gt;$B$4,"Future",IF(A83=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A83,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E83=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A83&gt;$B$4,"Future",IF(A83=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A83,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E83=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2981,7 +2986,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E84" s="6" t="str">
-        <x:f>IF(A84&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A84,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A84&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A84,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F84" s="6" t="str">
         <x:f>IF(A84&gt;=$B$4,"",MAX(D84-E84,0))</x:f>
@@ -2996,7 +3001,7 @@
         <x:f>IF(A84&gt;$B$4,"",SUM($E$15:E84))</x:f>
       </x:c>
       <x:c r="J84" s="1" t="str">
-        <x:f>IF(A84&gt;$B$4,"Future",IF(A84=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A84,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E84=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A84&gt;$B$4,"Future",IF(A84=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A84,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E84=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3016,7 +3021,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E85" s="6" t="str">
-        <x:f>IF(A85&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A85,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A85&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A85,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F85" s="6" t="str">
         <x:f>IF(A85&gt;=$B$4,"",MAX(D85-E85,0))</x:f>
@@ -3031,7 +3036,7 @@
         <x:f>IF(A85&gt;$B$4,"",SUM($E$15:E85))</x:f>
       </x:c>
       <x:c r="J85" s="1" t="str">
-        <x:f>IF(A85&gt;$B$4,"Future",IF(A85=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A85,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E85=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A85&gt;$B$4,"Future",IF(A85=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A85,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E85=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3051,7 +3056,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E86" s="6" t="str">
-        <x:f>IF(A86&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A86,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A86&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A86,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F86" s="6" t="str">
         <x:f>IF(A86&gt;=$B$4,"",MAX(D86-E86,0))</x:f>
@@ -3066,7 +3071,7 @@
         <x:f>IF(A86&gt;$B$4,"",SUM($E$15:E86))</x:f>
       </x:c>
       <x:c r="J86" s="1" t="str">
-        <x:f>IF(A86&gt;$B$4,"Future",IF(A86=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A86,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E86=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A86&gt;$B$4,"Future",IF(A86=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A86,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E86=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3086,7 +3091,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E87" s="6" t="str">
-        <x:f>IF(A87&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A87,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A87&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A87,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F87" s="6" t="str">
         <x:f>IF(A87&gt;=$B$4,"",MAX(D87-E87,0))</x:f>
@@ -3101,7 +3106,7 @@
         <x:f>IF(A87&gt;$B$4,"",SUM($E$15:E87))</x:f>
       </x:c>
       <x:c r="J87" s="1" t="str">
-        <x:f>IF(A87&gt;$B$4,"Future",IF(A87=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A87,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E87=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A87&gt;$B$4,"Future",IF(A87=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A87,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E87=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3121,7 +3126,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E88" s="6" t="str">
-        <x:f>IF(A88&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A88,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A88&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A88,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F88" s="6" t="str">
         <x:f>IF(A88&gt;=$B$4,"",MAX(D88-E88,0))</x:f>
@@ -3136,7 +3141,7 @@
         <x:f>IF(A88&gt;$B$4,"",SUM($E$15:E88))</x:f>
       </x:c>
       <x:c r="J88" s="1" t="str">
-        <x:f>IF(A88&gt;$B$4,"Future",IF(A88=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A88,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E88=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A88&gt;$B$4,"Future",IF(A88=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A88,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E88=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3156,7 +3161,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E89" s="6" t="str">
-        <x:f>IF(A89&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A89,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A89&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A89,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F89" s="6" t="str">
         <x:f>IF(A89&gt;=$B$4,"",MAX(D89-E89,0))</x:f>
@@ -3171,7 +3176,7 @@
         <x:f>IF(A89&gt;$B$4,"",SUM($E$15:E89))</x:f>
       </x:c>
       <x:c r="J89" s="1" t="str">
-        <x:f>IF(A89&gt;$B$4,"Future",IF(A89=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A89,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E89=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A89&gt;$B$4,"Future",IF(A89=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A89,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E89=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3191,7 +3196,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E90" s="6" t="str">
-        <x:f>IF(A90&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A90,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A90&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A90,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F90" s="6" t="str">
         <x:f>IF(A90&gt;=$B$4,"",MAX(D90-E90,0))</x:f>
@@ -3206,7 +3211,7 @@
         <x:f>IF(A90&gt;$B$4,"",SUM($E$15:E90))</x:f>
       </x:c>
       <x:c r="J90" s="1" t="str">
-        <x:f>IF(A90&gt;$B$4,"Future",IF(A90=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A90,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E90=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A90&gt;$B$4,"Future",IF(A90=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A90,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E90=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3226,7 +3231,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E91" s="6" t="str">
-        <x:f>IF(A91&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A91,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A91&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A91,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F91" s="6" t="str">
         <x:f>IF(A91&gt;=$B$4,"",MAX(D91-E91,0))</x:f>
@@ -3241,7 +3246,7 @@
         <x:f>IF(A91&gt;$B$4,"",SUM($E$15:E91))</x:f>
       </x:c>
       <x:c r="J91" s="1" t="str">
-        <x:f>IF(A91&gt;$B$4,"Future",IF(A91=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A91,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E91=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A91&gt;$B$4,"Future",IF(A91=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A91,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E91=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3261,7 +3266,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E92" s="6" t="str">
-        <x:f>IF(A92&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A92,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A92&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A92,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F92" s="6" t="str">
         <x:f>IF(A92&gt;=$B$4,"",MAX(D92-E92,0))</x:f>
@@ -3276,7 +3281,7 @@
         <x:f>IF(A92&gt;$B$4,"",SUM($E$15:E92))</x:f>
       </x:c>
       <x:c r="J92" s="1" t="str">
-        <x:f>IF(A92&gt;$B$4,"Future",IF(A92=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A92,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E92=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A92&gt;$B$4,"Future",IF(A92=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A92,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E92=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3296,7 +3301,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E93" s="6" t="str">
-        <x:f>IF(A93&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A93,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A93&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A93,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F93" s="6" t="str">
         <x:f>IF(A93&gt;=$B$4,"",MAX(D93-E93,0))</x:f>
@@ -3311,7 +3316,7 @@
         <x:f>IF(A93&gt;$B$4,"",SUM($E$15:E93))</x:f>
       </x:c>
       <x:c r="J93" s="1" t="str">
-        <x:f>IF(A93&gt;$B$4,"Future",IF(A93=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A93,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E93=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A93&gt;$B$4,"Future",IF(A93=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A93,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E93=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3331,7 +3336,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E94" s="6" t="str">
-        <x:f>IF(A94&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A94,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A94&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A94,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F94" s="6" t="str">
         <x:f>IF(A94&gt;=$B$4,"",MAX(D94-E94,0))</x:f>
@@ -3346,7 +3351,7 @@
         <x:f>IF(A94&gt;$B$4,"",SUM($E$15:E94))</x:f>
       </x:c>
       <x:c r="J94" s="1" t="str">
-        <x:f>IF(A94&gt;$B$4,"Future",IF(A94=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A94,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E94=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A94&gt;$B$4,"Future",IF(A94=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A94,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E94=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3366,7 +3371,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E95" s="6" t="str">
-        <x:f>IF(A95&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A95,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A95&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A95,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F95" s="6" t="str">
         <x:f>IF(A95&gt;=$B$4,"",MAX(D95-E95,0))</x:f>
@@ -3381,7 +3386,7 @@
         <x:f>IF(A95&gt;$B$4,"",SUM($E$15:E95))</x:f>
       </x:c>
       <x:c r="J95" s="1" t="str">
-        <x:f>IF(A95&gt;$B$4,"Future",IF(A95=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A95,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E95=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A95&gt;$B$4,"Future",IF(A95=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A95,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E95=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3401,7 +3406,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E96" s="6" t="str">
-        <x:f>IF(A96&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A96,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A96&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A96,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F96" s="6" t="str">
         <x:f>IF(A96&gt;=$B$4,"",MAX(D96-E96,0))</x:f>
@@ -3416,7 +3421,7 @@
         <x:f>IF(A96&gt;$B$4,"",SUM($E$15:E96))</x:f>
       </x:c>
       <x:c r="J96" s="1" t="str">
-        <x:f>IF(A96&gt;$B$4,"Future",IF(A96=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A96,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E96=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A96&gt;$B$4,"Future",IF(A96=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A96,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E96=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3436,7 +3441,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E97" s="6" t="str">
-        <x:f>IF(A97&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A97,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A97&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A97,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F97" s="6" t="str">
         <x:f>IF(A97&gt;=$B$4,"",MAX(D97-E97,0))</x:f>
@@ -3451,7 +3456,7 @@
         <x:f>IF(A97&gt;$B$4,"",SUM($E$15:E97))</x:f>
       </x:c>
       <x:c r="J97" s="1" t="str">
-        <x:f>IF(A97&gt;$B$4,"Future",IF(A97=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A97,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E97=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A97&gt;$B$4,"Future",IF(A97=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A97,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E97=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3471,7 +3476,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E98" s="6" t="str">
-        <x:f>IF(A98&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A98,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A98&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A98,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F98" s="6" t="str">
         <x:f>IF(A98&gt;=$B$4,"",MAX(D98-E98,0))</x:f>
@@ -3486,7 +3491,7 @@
         <x:f>IF(A98&gt;$B$4,"",SUM($E$15:E98))</x:f>
       </x:c>
       <x:c r="J98" s="1" t="str">
-        <x:f>IF(A98&gt;$B$4,"Future",IF(A98=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A98,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E98=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A98&gt;$B$4,"Future",IF(A98=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A98,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E98=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3506,7 +3511,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E99" s="6" t="str">
-        <x:f>IF(A99&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A99,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A99&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A99,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F99" s="6" t="str">
         <x:f>IF(A99&gt;=$B$4,"",MAX(D99-E99,0))</x:f>
@@ -3521,7 +3526,7 @@
         <x:f>IF(A99&gt;$B$4,"",SUM($E$15:E99))</x:f>
       </x:c>
       <x:c r="J99" s="1" t="str">
-        <x:f>IF(A99&gt;$B$4,"Future",IF(A99=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A99,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E99=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A99&gt;$B$4,"Future",IF(A99=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A99,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E99=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3541,7 +3546,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E100" s="6" t="str">
-        <x:f>IF(A100&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A100,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A100&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A100,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F100" s="6" t="str">
         <x:f>IF(A100&gt;=$B$4,"",MAX(D100-E100,0))</x:f>
@@ -3556,7 +3561,7 @@
         <x:f>IF(A100&gt;$B$4,"",SUM($E$15:E100))</x:f>
       </x:c>
       <x:c r="J100" s="1" t="str">
-        <x:f>IF(A100&gt;$B$4,"Future",IF(A100=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A100,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E100=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A100&gt;$B$4,"Future",IF(A100=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A100,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E100=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3576,7 +3581,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E101" s="6" t="str">
-        <x:f>IF(A101&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A101,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A101&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A101,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F101" s="6" t="str">
         <x:f>IF(A101&gt;=$B$4,"",MAX(D101-E101,0))</x:f>
@@ -3591,7 +3596,7 @@
         <x:f>IF(A101&gt;$B$4,"",SUM($E$15:E101))</x:f>
       </x:c>
       <x:c r="J101" s="1" t="str">
-        <x:f>IF(A101&gt;$B$4,"Future",IF(A101=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A101,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E101=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A101&gt;$B$4,"Future",IF(A101=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A101,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E101=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3611,7 +3616,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E102" s="6" t="str">
-        <x:f>IF(A102&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A102,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A102&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A102,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F102" s="6" t="str">
         <x:f>IF(A102&gt;=$B$4,"",MAX(D102-E102,0))</x:f>
@@ -3626,7 +3631,7 @@
         <x:f>IF(A102&gt;$B$4,"",SUM($E$15:E102))</x:f>
       </x:c>
       <x:c r="J102" s="1" t="str">
-        <x:f>IF(A102&gt;$B$4,"Future",IF(A102=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A102,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E102=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A102&gt;$B$4,"Future",IF(A102=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A102,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E102=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3646,7 +3651,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E103" s="6" t="str">
-        <x:f>IF(A103&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A103,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A103&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A103,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F103" s="6" t="str">
         <x:f>IF(A103&gt;=$B$4,"",MAX(D103-E103,0))</x:f>
@@ -3661,7 +3666,7 @@
         <x:f>IF(A103&gt;$B$4,"",SUM($E$15:E103))</x:f>
       </x:c>
       <x:c r="J103" s="1" t="str">
-        <x:f>IF(A103&gt;$B$4,"Future",IF(A103=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A103,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E103=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A103&gt;$B$4,"Future",IF(A103=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A103,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E103=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3681,7 +3686,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E104" s="6" t="str">
-        <x:f>IF(A104&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A104,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A104&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A104,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F104" s="6" t="str">
         <x:f>IF(A104&gt;=$B$4,"",MAX(D104-E104,0))</x:f>
@@ -3696,7 +3701,7 @@
         <x:f>IF(A104&gt;$B$4,"",SUM($E$15:E104))</x:f>
       </x:c>
       <x:c r="J104" s="1" t="str">
-        <x:f>IF(A104&gt;$B$4,"Future",IF(A104=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A104,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E104=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A104&gt;$B$4,"Future",IF(A104=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A104,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E104=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3716,7 +3721,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E105" s="6" t="str">
-        <x:f>IF(A105&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A105,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A105&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A105,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F105" s="6" t="str">
         <x:f>IF(A105&gt;=$B$4,"",MAX(D105-E105,0))</x:f>
@@ -3731,7 +3736,7 @@
         <x:f>IF(A105&gt;$B$4,"",SUM($E$15:E105))</x:f>
       </x:c>
       <x:c r="J105" s="1" t="str">
-        <x:f>IF(A105&gt;$B$4,"Future",IF(A105=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A105,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E105=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A105&gt;$B$4,"Future",IF(A105=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A105,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E105=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3751,7 +3756,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E106" s="6" t="str">
-        <x:f>IF(A106&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A106,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A106&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A106,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F106" s="6" t="str">
         <x:f>IF(A106&gt;=$B$4,"",MAX(D106-E106,0))</x:f>
@@ -3766,7 +3771,7 @@
         <x:f>IF(A106&gt;$B$4,"",SUM($E$15:E106))</x:f>
       </x:c>
       <x:c r="J106" s="1" t="str">
-        <x:f>IF(A106&gt;$B$4,"Future",IF(A106=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A106,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E106=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A106&gt;$B$4,"Future",IF(A106=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A106,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E106=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3786,7 +3791,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E107" s="6" t="str">
-        <x:f>IF(A107&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A107,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A107&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A107,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F107" s="6" t="str">
         <x:f>IF(A107&gt;=$B$4,"",MAX(D107-E107,0))</x:f>
@@ -3801,7 +3806,7 @@
         <x:f>IF(A107&gt;$B$4,"",SUM($E$15:E107))</x:f>
       </x:c>
       <x:c r="J107" s="1" t="str">
-        <x:f>IF(A107&gt;$B$4,"Future",IF(A107=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A107,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E107=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A107&gt;$B$4,"Future",IF(A107=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A107,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E107=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3821,7 +3826,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E108" s="6" t="str">
-        <x:f>IF(A108&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A108,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A108&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A108,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F108" s="6" t="str">
         <x:f>IF(A108&gt;=$B$4,"",MAX(D108-E108,0))</x:f>
@@ -3836,7 +3841,7 @@
         <x:f>IF(A108&gt;$B$4,"",SUM($E$15:E108))</x:f>
       </x:c>
       <x:c r="J108" s="1" t="str">
-        <x:f>IF(A108&gt;$B$4,"Future",IF(A108=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A108,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E108=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A108&gt;$B$4,"Future",IF(A108=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A108,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E108=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3856,7 +3861,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E109" s="6" t="str">
-        <x:f>IF(A109&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A109,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A109&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A109,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F109" s="6" t="str">
         <x:f>IF(A109&gt;=$B$4,"",MAX(D109-E109,0))</x:f>
@@ -3871,7 +3876,7 @@
         <x:f>IF(A109&gt;$B$4,"",SUM($E$15:E109))</x:f>
       </x:c>
       <x:c r="J109" s="1" t="str">
-        <x:f>IF(A109&gt;$B$4,"Future",IF(A109=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A109,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E109=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A109&gt;$B$4,"Future",IF(A109=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A109,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E109=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3891,7 +3896,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E110" s="6" t="str">
-        <x:f>IF(A110&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A110,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A110&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A110,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F110" s="6" t="str">
         <x:f>IF(A110&gt;=$B$4,"",MAX(D110-E110,0))</x:f>
@@ -3906,7 +3911,7 @@
         <x:f>IF(A110&gt;$B$4,"",SUM($E$15:E110))</x:f>
       </x:c>
       <x:c r="J110" s="1" t="str">
-        <x:f>IF(A110&gt;$B$4,"Future",IF(A110=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A110,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E110=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A110&gt;$B$4,"Future",IF(A110=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A110,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E110=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3926,7 +3931,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E111" s="6" t="str">
-        <x:f>IF(A111&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A111,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A111&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A111,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F111" s="6" t="str">
         <x:f>IF(A111&gt;=$B$4,"",MAX(D111-E111,0))</x:f>
@@ -3941,7 +3946,7 @@
         <x:f>IF(A111&gt;$B$4,"",SUM($E$15:E111))</x:f>
       </x:c>
       <x:c r="J111" s="1" t="str">
-        <x:f>IF(A111&gt;$B$4,"Future",IF(A111=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A111,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E111=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A111&gt;$B$4,"Future",IF(A111=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A111,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E111=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3961,7 +3966,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E112" s="6" t="str">
-        <x:f>IF(A112&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A112,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A112&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A112,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F112" s="6" t="str">
         <x:f>IF(A112&gt;=$B$4,"",MAX(D112-E112,0))</x:f>
@@ -3976,7 +3981,7 @@
         <x:f>IF(A112&gt;$B$4,"",SUM($E$15:E112))</x:f>
       </x:c>
       <x:c r="J112" s="1" t="str">
-        <x:f>IF(A112&gt;$B$4,"Future",IF(A112=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A112,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E112=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A112&gt;$B$4,"Future",IF(A112=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A112,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E112=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3996,7 +4001,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E113" s="6" t="str">
-        <x:f>IF(A113&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A113,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A113&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A113,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F113" s="6" t="str">
         <x:f>IF(A113&gt;=$B$4,"",MAX(D113-E113,0))</x:f>
@@ -4011,7 +4016,7 @@
         <x:f>IF(A113&gt;$B$4,"",SUM($E$15:E113))</x:f>
       </x:c>
       <x:c r="J113" s="1" t="str">
-        <x:f>IF(A113&gt;$B$4,"Future",IF(A113=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A113,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E113=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A113&gt;$B$4,"Future",IF(A113=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A113,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E113=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4031,7 +4036,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E114" s="6" t="str">
-        <x:f>IF(A114&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A114,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A114&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A114,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F114" s="6" t="str">
         <x:f>IF(A114&gt;=$B$4,"",MAX(D114-E114,0))</x:f>
@@ -4046,7 +4051,7 @@
         <x:f>IF(A114&gt;$B$4,"",SUM($E$15:E114))</x:f>
       </x:c>
       <x:c r="J114" s="1" t="str">
-        <x:f>IF(A114&gt;$B$4,"Future",IF(A114=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A114,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E114=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A114&gt;$B$4,"Future",IF(A114=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A114,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E114=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4066,7 +4071,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E115" s="6" t="str">
-        <x:f>IF(A115&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A115,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A115&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A115,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F115" s="6" t="str">
         <x:f>IF(A115&gt;=$B$4,"",MAX(D115-E115,0))</x:f>
@@ -4081,7 +4086,7 @@
         <x:f>IF(A115&gt;$B$4,"",SUM($E$15:E115))</x:f>
       </x:c>
       <x:c r="J115" s="1" t="str">
-        <x:f>IF(A115&gt;$B$4,"Future",IF(A115=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A115,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E115=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A115&gt;$B$4,"Future",IF(A115=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A115,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E115=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4101,7 +4106,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E116" s="6" t="str">
-        <x:f>IF(A116&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A116,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A116&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A116,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F116" s="6" t="str">
         <x:f>IF(A116&gt;=$B$4,"",MAX(D116-E116,0))</x:f>
@@ -4116,7 +4121,7 @@
         <x:f>IF(A116&gt;$B$4,"",SUM($E$15:E116))</x:f>
       </x:c>
       <x:c r="J116" s="1" t="str">
-        <x:f>IF(A116&gt;$B$4,"Future",IF(A116=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A116,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E116=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A116&gt;$B$4,"Future",IF(A116=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A116,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E116=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4136,7 +4141,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E117" s="6" t="str">
-        <x:f>IF(A117&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A117,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A117&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A117,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F117" s="6" t="str">
         <x:f>IF(A117&gt;=$B$4,"",MAX(D117-E117,0))</x:f>
@@ -4151,7 +4156,7 @@
         <x:f>IF(A117&gt;$B$4,"",SUM($E$15:E117))</x:f>
       </x:c>
       <x:c r="J117" s="1" t="str">
-        <x:f>IF(A117&gt;$B$4,"Future",IF(A117=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A117,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E117=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A117&gt;$B$4,"Future",IF(A117=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A117,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E117=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4171,7 +4176,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E118" s="6" t="str">
-        <x:f>IF(A118&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A118,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A118&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A118,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F118" s="6" t="str">
         <x:f>IF(A118&gt;=$B$4,"",MAX(D118-E118,0))</x:f>
@@ -4186,7 +4191,7 @@
         <x:f>IF(A118&gt;$B$4,"",SUM($E$15:E118))</x:f>
       </x:c>
       <x:c r="J118" s="1" t="str">
-        <x:f>IF(A118&gt;$B$4,"Future",IF(A118=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A118,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E118=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A118&gt;$B$4,"Future",IF(A118=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A118,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E118=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4206,7 +4211,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E119" s="6" t="str">
-        <x:f>IF(A119&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A119,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A119&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A119,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F119" s="6" t="str">
         <x:f>IF(A119&gt;=$B$4,"",MAX(D119-E119,0))</x:f>
@@ -4221,7 +4226,7 @@
         <x:f>IF(A119&gt;$B$4,"",SUM($E$15:E119))</x:f>
       </x:c>
       <x:c r="J119" s="1" t="str">
-        <x:f>IF(A119&gt;$B$4,"Future",IF(A119=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A119,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E119=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A119&gt;$B$4,"Future",IF(A119=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A119,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E119=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4241,7 +4246,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E120" s="6" t="str">
-        <x:f>IF(A120&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A120,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A120&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A120,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F120" s="6" t="str">
         <x:f>IF(A120&gt;=$B$4,"",MAX(D120-E120,0))</x:f>
@@ -4256,7 +4261,7 @@
         <x:f>IF(A120&gt;$B$4,"",SUM($E$15:E120))</x:f>
       </x:c>
       <x:c r="J120" s="1" t="str">
-        <x:f>IF(A120&gt;$B$4,"Future",IF(A120=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A120,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E120=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A120&gt;$B$4,"Future",IF(A120=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A120,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E120=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4276,7 +4281,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E121" s="6" t="str">
-        <x:f>IF(A121&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A121,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A121&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A121,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F121" s="6" t="str">
         <x:f>IF(A121&gt;=$B$4,"",MAX(D121-E121,0))</x:f>
@@ -4291,7 +4296,7 @@
         <x:f>IF(A121&gt;$B$4,"",SUM($E$15:E121))</x:f>
       </x:c>
       <x:c r="J121" s="1" t="str">
-        <x:f>IF(A121&gt;$B$4,"Future",IF(A121=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A121,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E121=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A121&gt;$B$4,"Future",IF(A121=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A121,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E121=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4311,7 +4316,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E122" s="6" t="str">
-        <x:f>IF(A122&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A122,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A122&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A122,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F122" s="6" t="str">
         <x:f>IF(A122&gt;=$B$4,"",MAX(D122-E122,0))</x:f>
@@ -4326,7 +4331,7 @@
         <x:f>IF(A122&gt;$B$4,"",SUM($E$15:E122))</x:f>
       </x:c>
       <x:c r="J122" s="1" t="str">
-        <x:f>IF(A122&gt;$B$4,"Future",IF(A122=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A122,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E122=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A122&gt;$B$4,"Future",IF(A122=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A122,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E122=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4346,7 +4351,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E123" s="6" t="str">
-        <x:f>IF(A123&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A123,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A123&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A123,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F123" s="6" t="str">
         <x:f>IF(A123&gt;=$B$4,"",MAX(D123-E123,0))</x:f>
@@ -4361,7 +4366,7 @@
         <x:f>IF(A123&gt;$B$4,"",SUM($E$15:E123))</x:f>
       </x:c>
       <x:c r="J123" s="1" t="str">
-        <x:f>IF(A123&gt;$B$4,"Future",IF(A123=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A123,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E123=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A123&gt;$B$4,"Future",IF(A123=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A123,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E123=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4381,7 +4386,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E124" s="6" t="str">
-        <x:f>IF(A124&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A124,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A124&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A124,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F124" s="6" t="str">
         <x:f>IF(A124&gt;=$B$4,"",MAX(D124-E124,0))</x:f>
@@ -4396,7 +4401,7 @@
         <x:f>IF(A124&gt;$B$4,"",SUM($E$15:E124))</x:f>
       </x:c>
       <x:c r="J124" s="1" t="str">
-        <x:f>IF(A124&gt;$B$4,"Future",IF(A124=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A124,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E124=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A124&gt;$B$4,"Future",IF(A124=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A124,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E124=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4416,7 +4421,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E125" s="6" t="str">
-        <x:f>IF(A125&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A125,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A125&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A125,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F125" s="6" t="str">
         <x:f>IF(A125&gt;=$B$4,"",MAX(D125-E125,0))</x:f>
@@ -4431,7 +4436,7 @@
         <x:f>IF(A125&gt;$B$4,"",SUM($E$15:E125))</x:f>
       </x:c>
       <x:c r="J125" s="1" t="str">
-        <x:f>IF(A125&gt;$B$4,"Future",IF(A125=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A125,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E125=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A125&gt;$B$4,"Future",IF(A125=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A125,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E125=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4451,7 +4456,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E126" s="6" t="str">
-        <x:f>IF(A126&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A126,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A126&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A126,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F126" s="6" t="str">
         <x:f>IF(A126&gt;=$B$4,"",MAX(D126-E126,0))</x:f>
@@ -4466,7 +4471,7 @@
         <x:f>IF(A126&gt;$B$4,"",SUM($E$15:E126))</x:f>
       </x:c>
       <x:c r="J126" s="1" t="str">
-        <x:f>IF(A126&gt;$B$4,"Future",IF(A126=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A126,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E126=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A126&gt;$B$4,"Future",IF(A126=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A126,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E126=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4486,7 +4491,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E127" s="6" t="str">
-        <x:f>IF(A127&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A127,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A127&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A127,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F127" s="6" t="str">
         <x:f>IF(A127&gt;=$B$4,"",MAX(D127-E127,0))</x:f>
@@ -4501,7 +4506,7 @@
         <x:f>IF(A127&gt;$B$4,"",SUM($E$15:E127))</x:f>
       </x:c>
       <x:c r="J127" s="1" t="str">
-        <x:f>IF(A127&gt;$B$4,"Future",IF(A127=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A127,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E127=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A127&gt;$B$4,"Future",IF(A127=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A127,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E127=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4521,7 +4526,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E128" s="6" t="str">
-        <x:f>IF(A128&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A128,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A128&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A128,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F128" s="6" t="str">
         <x:f>IF(A128&gt;=$B$4,"",MAX(D128-E128,0))</x:f>
@@ -4536,7 +4541,7 @@
         <x:f>IF(A128&gt;$B$4,"",SUM($E$15:E128))</x:f>
       </x:c>
       <x:c r="J128" s="1" t="str">
-        <x:f>IF(A128&gt;$B$4,"Future",IF(A128=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A128,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E128=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A128&gt;$B$4,"Future",IF(A128=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A128,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E128=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4556,7 +4561,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E129" s="6" t="str">
-        <x:f>IF(A129&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A129,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A129&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A129,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F129" s="6" t="str">
         <x:f>IF(A129&gt;=$B$4,"",MAX(D129-E129,0))</x:f>
@@ -4571,7 +4576,7 @@
         <x:f>IF(A129&gt;$B$4,"",SUM($E$15:E129))</x:f>
       </x:c>
       <x:c r="J129" s="1" t="str">
-        <x:f>IF(A129&gt;$B$4,"Future",IF(A129=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A129,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E129=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A129&gt;$B$4,"Future",IF(A129=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A129,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E129=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4591,7 +4596,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E130" s="6" t="str">
-        <x:f>IF(A130&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$10,'Sessions'!$B$2:$B$10,A130,'Sessions'!$G$2:$G$10,"completed")/60)</x:f>
+        <x:f>IF(A130&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A130,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
       </x:c>
       <x:c r="F130" s="6" t="str">
         <x:f>IF(A130&gt;=$B$4,"",MAX(D130-E130,0))</x:f>
@@ -4606,7 +4611,7 @@
         <x:f>IF(A130&gt;$B$4,"",SUM($E$15:E130))</x:f>
       </x:c>
       <x:c r="J130" s="1" t="str">
-        <x:f>IF(A130&gt;$B$4,"Future",IF(A130=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$10,A130,'Sessions'!$G$2:$G$10,"needs_confirmation")&gt;0,"Uncertain time",IF(E130=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A130&gt;$B$4,"Future",IF(A130=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A130,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E130=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4726,15 +4731,15 @@
       </x:c>
       <x:c r="C8" s="6" t="n">
         <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A8,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D8" s="6" t="n">
         <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A8)</x:f>
-        <x:v>2.8094444444449995</x:v>
+        <x:v>4.371944444444999</x:v>
       </x:c>
       <x:c r="E8" s="6" t="n">
         <x:f>MAX(C8-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A8,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
-        <x:v>0</x:v>
+        <x:v>3.1905555555550005</x:v>
       </x:c>
       <x:c r="F8" s="6" t="n">
         <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A8,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C8,0)</x:f>
@@ -4742,11 +4747,11 @@
       </x:c>
       <x:c r="G8" s="6" t="n">
         <x:f>MAX(B8-D8,0)</x:f>
-        <x:v>29.190555555555</x:v>
+        <x:v>27.628055555555</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
         <x:f>IF(B8=0,0,D8/B8)</x:f>
-        <x:v>0.08779513888890624</x:v>
+        <x:v>0.13662326388890622</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
@@ -5557,6 +5562,84 @@
         <x:v>Explicit resume and pause; clock timestamps; 45 minutes 38 seconds; no notebook code or output submitted for review</x:v>
       </x:c>
     </x:row>
+    <x:row r="11" ht="22" customHeight="1">
+      <x:c r="A11" s="1" t="str">
+        <x:v>PY-20261016T094020</x:v>
+      </x:c>
+      <x:c r="B11" s="7" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="C11" s="1" t="str">
+        <x:v>Python: dictionary foundations in Jupyter</x:v>
+      </x:c>
+      <x:c r="D11" s="1" t="str">
+        <x:v>IST 2026-10-16 09:40:20</x:v>
+      </x:c>
+      <x:c r="E11" s="1" t="str">
+        <x:v>IST 2026-10-16 10:27:42</x:v>
+      </x:c>
+      <x:c r="F11" s="1" t="n">
+        <x:v>47.36666666666667</x:v>
+      </x:c>
+      <x:c r="G11" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H11" s="1" t="str">
+        <x:v>Explicit Start Python; dictionary read/update code submitted; actual output and assistance confirmation pending; Explicit pause at 10:27:42 IST; 47m22s; dictionary/list/conversion/error-handling practice; cleaner list construction corrections pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="22" customHeight="1">
+      <x:c r="A12" s="1" t="str">
+        <x:v>PY-20261016T103447</x:v>
+      </x:c>
+      <x:c r="B12" s="7" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="C12" s="1" t="str">
+        <x:v>Python: valid and rejected record lists</x:v>
+      </x:c>
+      <x:c r="D12" s="1" t="str">
+        <x:v>IST 2026-10-16 10:34:47</x:v>
+      </x:c>
+      <x:c r="E12" s="1" t="str">
+        <x:v>IST 2026-10-16 10:51:42</x:v>
+      </x:c>
+      <x:c r="F12" s="1" t="n">
+        <x:v>16.916666666666668</x:v>
+      </x:c>
+      <x:c r="G12" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H12" s="1" t="str">
+        <x:v>Explicit Resume Python; break excluded; pending integer output dictionaries rejection reasons and removal of positivity filter; Explicit pause at 10:51:42 IST; 16m55s; copy/input-preservation correction with guidance; changed blank spaces zero dataset pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="22" customHeight="1">
+      <x:c r="A13" s="1" t="str">
+        <x:v>PY-20261016T113047</x:v>
+      </x:c>
+      <x:c r="B13" s="7" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="C13" s="1" t="str">
+        <x:v>Python: cleaner changed-input check</x:v>
+      </x:c>
+      <x:c r="D13" s="1" t="str">
+        <x:v>IST 2026-10-16 11:30:47</x:v>
+      </x:c>
+      <x:c r="E13" s="1" t="str">
+        <x:v>IST 2026-10-16 12:00:15</x:v>
+      </x:c>
+      <x:c r="F13" s="1" t="n">
+        <x:v>29.466666666666665</x:v>
+      </x:c>
+      <x:c r="G13" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H13" s="1" t="str">
+        <x:v>Explicit resume-timer; prior topic Python; break excluded; blank spaces zero check pending; no new learning evidence to duplicate; Explicit pause 12:00:15 IST; 29m28s; cleaner function and CSV reading completed with guidance; CSV output task pending</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Save CSV study checkpoint and practice setup
</commit_message>
<xml_diff>
--- a/outputs/study-tracker/study-hours.xlsx
+++ b/outputs/study-tracker/study-hours.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="Rb1591a1a45824674"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="Rc75e3e2caf614c15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="Raa35522b94e94052"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="R8c3ed5d77fed4b78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="R08394828940a4f03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="R9a38385d7c2843d0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -362,7 +362,7 @@
       </x:c>
       <x:c r="E4" s="6" t="n">
         <x:f>SUM(E15:E130)</x:f>
-        <x:v>4.371944444444999</x:v>
+        <x:v>4.499166666667222</x:v>
       </x:c>
       <x:c r="F4" s="1"/>
       <x:c r="G4" s="1"/>
@@ -442,7 +442,7 @@
       </x:c>
       <x:c r="E8" s="6" t="n">
         <x:f>MAX(SUMIFS(D15:D130,A15:A130,B4)-SUMIFS(E15:E130,A15:A130,B4),0)</x:f>
-        <x:v>4.4375</x:v>
+        <x:v>4.310277777777777</x:v>
       </x:c>
       <x:c r="F8" s="1"/>
       <x:c r="G8" s="1"/>
@@ -564,7 +564,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E15" s="6" t="n">
-        <x:f>IF(A15&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A15,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A15&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A15,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
         <x:v>2.8094444444449995</x:v>
       </x:c>
       <x:c r="F15" s="6" t="n">
@@ -584,7 +584,7 @@
         <x:v>2.8094444444449995</x:v>
       </x:c>
       <x:c r="J15" s="1" t="str">
-        <x:f>IF(A15&gt;$B$4,"Future",IF(A15=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A15,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E15=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A15&gt;$B$4,"Future",IF(A15=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A15,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E15=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Uncertain time</x:v>
       </x:c>
     </x:row>
@@ -604,8 +604,8 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E16" s="6" t="n">
-        <x:f>IF(A16&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A16,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
-        <x:v>1.5625</x:v>
+        <x:f>IF(A16&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A16,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:v>1.6897222222222223</x:v>
       </x:c>
       <x:c r="F16" s="6" t="str">
         <x:f>IF(A16&gt;=$B$4,"",MAX(D16-E16,0))</x:f>
@@ -618,10 +618,10 @@
       </x:c>
       <x:c r="I16" s="6" t="n">
         <x:f>IF(A16&gt;$B$4,"",SUM($E$15:E16))</x:f>
-        <x:v>4.371944444444999</x:v>
+        <x:v>4.499166666667222</x:v>
       </x:c>
       <x:c r="J16" s="1" t="str">
-        <x:f>IF(A16&gt;$B$4,"Future",IF(A16=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A16,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E16=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A16&gt;$B$4,"Future",IF(A16=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A16,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E16=0,"No confirmed time","Logged"))))</x:f>
         <x:v>In progress</x:v>
       </x:c>
     </x:row>
@@ -641,7 +641,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E17" s="6" t="str">
-        <x:f>IF(A17&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A17,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A17&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A17,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F17" s="6" t="str">
         <x:f>IF(A17&gt;=$B$4,"",MAX(D17-E17,0))</x:f>
@@ -656,7 +656,7 @@
         <x:f>IF(A17&gt;$B$4,"",SUM($E$15:E17))</x:f>
       </x:c>
       <x:c r="J17" s="1" t="str">
-        <x:f>IF(A17&gt;$B$4,"Future",IF(A17=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A17,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E17=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A17&gt;$B$4,"Future",IF(A17=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A17,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E17=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -676,7 +676,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E18" s="6" t="str">
-        <x:f>IF(A18&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A18,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A18&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A18,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F18" s="6" t="str">
         <x:f>IF(A18&gt;=$B$4,"",MAX(D18-E18,0))</x:f>
@@ -691,7 +691,7 @@
         <x:f>IF(A18&gt;$B$4,"",SUM($E$15:E18))</x:f>
       </x:c>
       <x:c r="J18" s="1" t="str">
-        <x:f>IF(A18&gt;$B$4,"Future",IF(A18=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A18,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E18=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A18&gt;$B$4,"Future",IF(A18=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A18,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E18=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -711,7 +711,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E19" s="6" t="str">
-        <x:f>IF(A19&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A19,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A19&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A19,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F19" s="6" t="str">
         <x:f>IF(A19&gt;=$B$4,"",MAX(D19-E19,0))</x:f>
@@ -726,7 +726,7 @@
         <x:f>IF(A19&gt;$B$4,"",SUM($E$15:E19))</x:f>
       </x:c>
       <x:c r="J19" s="1" t="str">
-        <x:f>IF(A19&gt;$B$4,"Future",IF(A19=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A19,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E19=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A19&gt;$B$4,"Future",IF(A19=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A19,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E19=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -746,7 +746,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E20" s="6" t="str">
-        <x:f>IF(A20&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A20,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A20&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A20,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F20" s="6" t="str">
         <x:f>IF(A20&gt;=$B$4,"",MAX(D20-E20,0))</x:f>
@@ -761,7 +761,7 @@
         <x:f>IF(A20&gt;$B$4,"",SUM($E$15:E20))</x:f>
       </x:c>
       <x:c r="J20" s="1" t="str">
-        <x:f>IF(A20&gt;$B$4,"Future",IF(A20=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A20,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E20=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A20&gt;$B$4,"Future",IF(A20=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A20,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E20=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -781,7 +781,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E21" s="6" t="str">
-        <x:f>IF(A21&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A21,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A21&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A21,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F21" s="6" t="str">
         <x:f>IF(A21&gt;=$B$4,"",MAX(D21-E21,0))</x:f>
@@ -796,7 +796,7 @@
         <x:f>IF(A21&gt;$B$4,"",SUM($E$15:E21))</x:f>
       </x:c>
       <x:c r="J21" s="1" t="str">
-        <x:f>IF(A21&gt;$B$4,"Future",IF(A21=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A21,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E21=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A21&gt;$B$4,"Future",IF(A21=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A21,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E21=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -816,7 +816,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E22" s="6" t="str">
-        <x:f>IF(A22&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A22,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A22&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A22,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F22" s="6" t="str">
         <x:f>IF(A22&gt;=$B$4,"",MAX(D22-E22,0))</x:f>
@@ -831,7 +831,7 @@
         <x:f>IF(A22&gt;$B$4,"",SUM($E$15:E22))</x:f>
       </x:c>
       <x:c r="J22" s="1" t="str">
-        <x:f>IF(A22&gt;$B$4,"Future",IF(A22=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A22,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E22=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A22&gt;$B$4,"Future",IF(A22=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A22,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E22=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -851,7 +851,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E23" s="6" t="str">
-        <x:f>IF(A23&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A23,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A23&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A23,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F23" s="6" t="str">
         <x:f>IF(A23&gt;=$B$4,"",MAX(D23-E23,0))</x:f>
@@ -866,7 +866,7 @@
         <x:f>IF(A23&gt;$B$4,"",SUM($E$15:E23))</x:f>
       </x:c>
       <x:c r="J23" s="1" t="str">
-        <x:f>IF(A23&gt;$B$4,"Future",IF(A23=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A23,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E23=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A23&gt;$B$4,"Future",IF(A23=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A23,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E23=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -886,7 +886,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E24" s="6" t="str">
-        <x:f>IF(A24&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A24,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A24&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A24,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F24" s="6" t="str">
         <x:f>IF(A24&gt;=$B$4,"",MAX(D24-E24,0))</x:f>
@@ -901,7 +901,7 @@
         <x:f>IF(A24&gt;$B$4,"",SUM($E$15:E24))</x:f>
       </x:c>
       <x:c r="J24" s="1" t="str">
-        <x:f>IF(A24&gt;$B$4,"Future",IF(A24=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A24,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E24=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A24&gt;$B$4,"Future",IF(A24=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A24,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E24=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -921,7 +921,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E25" s="6" t="str">
-        <x:f>IF(A25&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A25,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A25&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A25,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F25" s="6" t="str">
         <x:f>IF(A25&gt;=$B$4,"",MAX(D25-E25,0))</x:f>
@@ -936,7 +936,7 @@
         <x:f>IF(A25&gt;$B$4,"",SUM($E$15:E25))</x:f>
       </x:c>
       <x:c r="J25" s="1" t="str">
-        <x:f>IF(A25&gt;$B$4,"Future",IF(A25=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A25,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E25=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A25&gt;$B$4,"Future",IF(A25=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A25,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E25=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -956,7 +956,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E26" s="6" t="str">
-        <x:f>IF(A26&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A26,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A26&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A26,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F26" s="6" t="str">
         <x:f>IF(A26&gt;=$B$4,"",MAX(D26-E26,0))</x:f>
@@ -971,7 +971,7 @@
         <x:f>IF(A26&gt;$B$4,"",SUM($E$15:E26))</x:f>
       </x:c>
       <x:c r="J26" s="1" t="str">
-        <x:f>IF(A26&gt;$B$4,"Future",IF(A26=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A26,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E26=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A26&gt;$B$4,"Future",IF(A26=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A26,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E26=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -991,7 +991,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E27" s="6" t="str">
-        <x:f>IF(A27&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A27,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A27&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A27,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F27" s="6" t="str">
         <x:f>IF(A27&gt;=$B$4,"",MAX(D27-E27,0))</x:f>
@@ -1006,7 +1006,7 @@
         <x:f>IF(A27&gt;$B$4,"",SUM($E$15:E27))</x:f>
       </x:c>
       <x:c r="J27" s="1" t="str">
-        <x:f>IF(A27&gt;$B$4,"Future",IF(A27=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A27,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E27=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A27&gt;$B$4,"Future",IF(A27=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A27,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E27=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1026,7 +1026,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E28" s="6" t="str">
-        <x:f>IF(A28&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A28,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A28&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A28,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F28" s="6" t="str">
         <x:f>IF(A28&gt;=$B$4,"",MAX(D28-E28,0))</x:f>
@@ -1041,7 +1041,7 @@
         <x:f>IF(A28&gt;$B$4,"",SUM($E$15:E28))</x:f>
       </x:c>
       <x:c r="J28" s="1" t="str">
-        <x:f>IF(A28&gt;$B$4,"Future",IF(A28=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A28,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E28=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A28&gt;$B$4,"Future",IF(A28=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A28,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E28=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1061,7 +1061,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E29" s="6" t="str">
-        <x:f>IF(A29&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A29,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A29&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A29,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F29" s="6" t="str">
         <x:f>IF(A29&gt;=$B$4,"",MAX(D29-E29,0))</x:f>
@@ -1076,7 +1076,7 @@
         <x:f>IF(A29&gt;$B$4,"",SUM($E$15:E29))</x:f>
       </x:c>
       <x:c r="J29" s="1" t="str">
-        <x:f>IF(A29&gt;$B$4,"Future",IF(A29=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A29,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E29=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A29&gt;$B$4,"Future",IF(A29=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A29,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E29=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1096,7 +1096,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E30" s="6" t="str">
-        <x:f>IF(A30&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A30,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A30&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A30,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F30" s="6" t="str">
         <x:f>IF(A30&gt;=$B$4,"",MAX(D30-E30,0))</x:f>
@@ -1111,7 +1111,7 @@
         <x:f>IF(A30&gt;$B$4,"",SUM($E$15:E30))</x:f>
       </x:c>
       <x:c r="J30" s="1" t="str">
-        <x:f>IF(A30&gt;$B$4,"Future",IF(A30=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A30,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E30=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A30&gt;$B$4,"Future",IF(A30=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A30,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E30=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1131,7 +1131,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E31" s="6" t="str">
-        <x:f>IF(A31&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A31,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A31&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A31,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F31" s="6" t="str">
         <x:f>IF(A31&gt;=$B$4,"",MAX(D31-E31,0))</x:f>
@@ -1146,7 +1146,7 @@
         <x:f>IF(A31&gt;$B$4,"",SUM($E$15:E31))</x:f>
       </x:c>
       <x:c r="J31" s="1" t="str">
-        <x:f>IF(A31&gt;$B$4,"Future",IF(A31=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A31,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E31=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A31&gt;$B$4,"Future",IF(A31=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A31,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E31=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1166,7 +1166,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E32" s="6" t="str">
-        <x:f>IF(A32&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A32,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A32&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A32,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F32" s="6" t="str">
         <x:f>IF(A32&gt;=$B$4,"",MAX(D32-E32,0))</x:f>
@@ -1181,7 +1181,7 @@
         <x:f>IF(A32&gt;$B$4,"",SUM($E$15:E32))</x:f>
       </x:c>
       <x:c r="J32" s="1" t="str">
-        <x:f>IF(A32&gt;$B$4,"Future",IF(A32=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A32,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E32=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A32&gt;$B$4,"Future",IF(A32=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A32,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E32=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1201,7 +1201,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E33" s="6" t="str">
-        <x:f>IF(A33&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A33,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A33&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A33,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F33" s="6" t="str">
         <x:f>IF(A33&gt;=$B$4,"",MAX(D33-E33,0))</x:f>
@@ -1216,7 +1216,7 @@
         <x:f>IF(A33&gt;$B$4,"",SUM($E$15:E33))</x:f>
       </x:c>
       <x:c r="J33" s="1" t="str">
-        <x:f>IF(A33&gt;$B$4,"Future",IF(A33=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A33,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E33=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A33&gt;$B$4,"Future",IF(A33=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A33,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E33=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1236,7 +1236,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E34" s="6" t="str">
-        <x:f>IF(A34&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A34,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A34&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A34,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F34" s="6" t="str">
         <x:f>IF(A34&gt;=$B$4,"",MAX(D34-E34,0))</x:f>
@@ -1251,7 +1251,7 @@
         <x:f>IF(A34&gt;$B$4,"",SUM($E$15:E34))</x:f>
       </x:c>
       <x:c r="J34" s="1" t="str">
-        <x:f>IF(A34&gt;$B$4,"Future",IF(A34=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A34,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E34=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A34&gt;$B$4,"Future",IF(A34=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A34,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E34=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1271,7 +1271,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E35" s="6" t="str">
-        <x:f>IF(A35&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A35,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A35&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A35,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F35" s="6" t="str">
         <x:f>IF(A35&gt;=$B$4,"",MAX(D35-E35,0))</x:f>
@@ -1286,7 +1286,7 @@
         <x:f>IF(A35&gt;$B$4,"",SUM($E$15:E35))</x:f>
       </x:c>
       <x:c r="J35" s="1" t="str">
-        <x:f>IF(A35&gt;$B$4,"Future",IF(A35=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A35,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E35=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A35&gt;$B$4,"Future",IF(A35=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A35,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E35=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1306,7 +1306,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E36" s="6" t="str">
-        <x:f>IF(A36&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A36,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A36&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A36,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F36" s="6" t="str">
         <x:f>IF(A36&gt;=$B$4,"",MAX(D36-E36,0))</x:f>
@@ -1321,7 +1321,7 @@
         <x:f>IF(A36&gt;$B$4,"",SUM($E$15:E36))</x:f>
       </x:c>
       <x:c r="J36" s="1" t="str">
-        <x:f>IF(A36&gt;$B$4,"Future",IF(A36=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A36,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E36=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A36&gt;$B$4,"Future",IF(A36=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A36,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E36=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1341,7 +1341,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E37" s="6" t="str">
-        <x:f>IF(A37&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A37,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A37&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A37,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F37" s="6" t="str">
         <x:f>IF(A37&gt;=$B$4,"",MAX(D37-E37,0))</x:f>
@@ -1356,7 +1356,7 @@
         <x:f>IF(A37&gt;$B$4,"",SUM($E$15:E37))</x:f>
       </x:c>
       <x:c r="J37" s="1" t="str">
-        <x:f>IF(A37&gt;$B$4,"Future",IF(A37=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A37,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E37=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A37&gt;$B$4,"Future",IF(A37=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A37,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E37=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1376,7 +1376,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E38" s="6" t="str">
-        <x:f>IF(A38&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A38,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A38&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A38,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F38" s="6" t="str">
         <x:f>IF(A38&gt;=$B$4,"",MAX(D38-E38,0))</x:f>
@@ -1391,7 +1391,7 @@
         <x:f>IF(A38&gt;$B$4,"",SUM($E$15:E38))</x:f>
       </x:c>
       <x:c r="J38" s="1" t="str">
-        <x:f>IF(A38&gt;$B$4,"Future",IF(A38=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A38,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E38=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A38&gt;$B$4,"Future",IF(A38=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A38,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E38=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1411,7 +1411,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E39" s="6" t="str">
-        <x:f>IF(A39&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A39,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A39&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A39,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F39" s="6" t="str">
         <x:f>IF(A39&gt;=$B$4,"",MAX(D39-E39,0))</x:f>
@@ -1426,7 +1426,7 @@
         <x:f>IF(A39&gt;$B$4,"",SUM($E$15:E39))</x:f>
       </x:c>
       <x:c r="J39" s="1" t="str">
-        <x:f>IF(A39&gt;$B$4,"Future",IF(A39=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A39,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E39=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A39&gt;$B$4,"Future",IF(A39=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A39,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E39=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1446,7 +1446,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E40" s="6" t="str">
-        <x:f>IF(A40&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A40,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A40&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A40,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F40" s="6" t="str">
         <x:f>IF(A40&gt;=$B$4,"",MAX(D40-E40,0))</x:f>
@@ -1461,7 +1461,7 @@
         <x:f>IF(A40&gt;$B$4,"",SUM($E$15:E40))</x:f>
       </x:c>
       <x:c r="J40" s="1" t="str">
-        <x:f>IF(A40&gt;$B$4,"Future",IF(A40=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A40,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E40=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A40&gt;$B$4,"Future",IF(A40=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A40,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E40=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1481,7 +1481,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E41" s="6" t="str">
-        <x:f>IF(A41&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A41,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A41&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A41,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F41" s="6" t="str">
         <x:f>IF(A41&gt;=$B$4,"",MAX(D41-E41,0))</x:f>
@@ -1496,7 +1496,7 @@
         <x:f>IF(A41&gt;$B$4,"",SUM($E$15:E41))</x:f>
       </x:c>
       <x:c r="J41" s="1" t="str">
-        <x:f>IF(A41&gt;$B$4,"Future",IF(A41=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A41,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E41=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A41&gt;$B$4,"Future",IF(A41=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A41,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E41=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1516,7 +1516,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E42" s="6" t="str">
-        <x:f>IF(A42&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A42,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A42&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A42,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F42" s="6" t="str">
         <x:f>IF(A42&gt;=$B$4,"",MAX(D42-E42,0))</x:f>
@@ -1531,7 +1531,7 @@
         <x:f>IF(A42&gt;$B$4,"",SUM($E$15:E42))</x:f>
       </x:c>
       <x:c r="J42" s="1" t="str">
-        <x:f>IF(A42&gt;$B$4,"Future",IF(A42=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A42,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E42=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A42&gt;$B$4,"Future",IF(A42=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A42,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E42=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1551,7 +1551,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E43" s="6" t="str">
-        <x:f>IF(A43&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A43,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A43&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A43,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F43" s="6" t="str">
         <x:f>IF(A43&gt;=$B$4,"",MAX(D43-E43,0))</x:f>
@@ -1566,7 +1566,7 @@
         <x:f>IF(A43&gt;$B$4,"",SUM($E$15:E43))</x:f>
       </x:c>
       <x:c r="J43" s="1" t="str">
-        <x:f>IF(A43&gt;$B$4,"Future",IF(A43=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A43,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E43=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A43&gt;$B$4,"Future",IF(A43=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A43,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E43=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1586,7 +1586,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E44" s="6" t="str">
-        <x:f>IF(A44&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A44,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A44&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A44,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F44" s="6" t="str">
         <x:f>IF(A44&gt;=$B$4,"",MAX(D44-E44,0))</x:f>
@@ -1601,7 +1601,7 @@
         <x:f>IF(A44&gt;$B$4,"",SUM($E$15:E44))</x:f>
       </x:c>
       <x:c r="J44" s="1" t="str">
-        <x:f>IF(A44&gt;$B$4,"Future",IF(A44=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A44,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E44=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A44&gt;$B$4,"Future",IF(A44=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A44,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E44=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1621,7 +1621,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E45" s="6" t="str">
-        <x:f>IF(A45&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A45,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A45&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A45,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F45" s="6" t="str">
         <x:f>IF(A45&gt;=$B$4,"",MAX(D45-E45,0))</x:f>
@@ -1636,7 +1636,7 @@
         <x:f>IF(A45&gt;$B$4,"",SUM($E$15:E45))</x:f>
       </x:c>
       <x:c r="J45" s="1" t="str">
-        <x:f>IF(A45&gt;$B$4,"Future",IF(A45=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A45,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E45=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A45&gt;$B$4,"Future",IF(A45=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A45,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E45=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1656,7 +1656,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E46" s="6" t="str">
-        <x:f>IF(A46&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A46,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A46&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A46,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F46" s="6" t="str">
         <x:f>IF(A46&gt;=$B$4,"",MAX(D46-E46,0))</x:f>
@@ -1671,7 +1671,7 @@
         <x:f>IF(A46&gt;$B$4,"",SUM($E$15:E46))</x:f>
       </x:c>
       <x:c r="J46" s="1" t="str">
-        <x:f>IF(A46&gt;$B$4,"Future",IF(A46=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A46,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E46=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A46&gt;$B$4,"Future",IF(A46=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A46,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E46=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1691,7 +1691,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E47" s="6" t="str">
-        <x:f>IF(A47&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A47,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A47&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A47,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F47" s="6" t="str">
         <x:f>IF(A47&gt;=$B$4,"",MAX(D47-E47,0))</x:f>
@@ -1706,7 +1706,7 @@
         <x:f>IF(A47&gt;$B$4,"",SUM($E$15:E47))</x:f>
       </x:c>
       <x:c r="J47" s="1" t="str">
-        <x:f>IF(A47&gt;$B$4,"Future",IF(A47=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A47,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E47=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A47&gt;$B$4,"Future",IF(A47=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A47,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E47=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1726,7 +1726,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E48" s="6" t="str">
-        <x:f>IF(A48&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A48,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A48&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A48,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F48" s="6" t="str">
         <x:f>IF(A48&gt;=$B$4,"",MAX(D48-E48,0))</x:f>
@@ -1741,7 +1741,7 @@
         <x:f>IF(A48&gt;$B$4,"",SUM($E$15:E48))</x:f>
       </x:c>
       <x:c r="J48" s="1" t="str">
-        <x:f>IF(A48&gt;$B$4,"Future",IF(A48=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A48,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E48=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A48&gt;$B$4,"Future",IF(A48=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A48,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E48=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1761,7 +1761,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E49" s="6" t="str">
-        <x:f>IF(A49&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A49,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A49&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A49,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F49" s="6" t="str">
         <x:f>IF(A49&gt;=$B$4,"",MAX(D49-E49,0))</x:f>
@@ -1776,7 +1776,7 @@
         <x:f>IF(A49&gt;$B$4,"",SUM($E$15:E49))</x:f>
       </x:c>
       <x:c r="J49" s="1" t="str">
-        <x:f>IF(A49&gt;$B$4,"Future",IF(A49=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A49,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E49=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A49&gt;$B$4,"Future",IF(A49=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A49,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E49=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1796,7 +1796,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E50" s="6" t="str">
-        <x:f>IF(A50&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A50,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A50&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A50,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F50" s="6" t="str">
         <x:f>IF(A50&gt;=$B$4,"",MAX(D50-E50,0))</x:f>
@@ -1811,7 +1811,7 @@
         <x:f>IF(A50&gt;$B$4,"",SUM($E$15:E50))</x:f>
       </x:c>
       <x:c r="J50" s="1" t="str">
-        <x:f>IF(A50&gt;$B$4,"Future",IF(A50=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A50,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E50=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A50&gt;$B$4,"Future",IF(A50=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A50,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E50=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1831,7 +1831,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E51" s="6" t="str">
-        <x:f>IF(A51&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A51,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A51&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A51,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F51" s="6" t="str">
         <x:f>IF(A51&gt;=$B$4,"",MAX(D51-E51,0))</x:f>
@@ -1846,7 +1846,7 @@
         <x:f>IF(A51&gt;$B$4,"",SUM($E$15:E51))</x:f>
       </x:c>
       <x:c r="J51" s="1" t="str">
-        <x:f>IF(A51&gt;$B$4,"Future",IF(A51=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A51,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E51=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A51&gt;$B$4,"Future",IF(A51=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A51,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E51=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1866,7 +1866,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E52" s="6" t="str">
-        <x:f>IF(A52&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A52,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A52&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A52,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F52" s="6" t="str">
         <x:f>IF(A52&gt;=$B$4,"",MAX(D52-E52,0))</x:f>
@@ -1881,7 +1881,7 @@
         <x:f>IF(A52&gt;$B$4,"",SUM($E$15:E52))</x:f>
       </x:c>
       <x:c r="J52" s="1" t="str">
-        <x:f>IF(A52&gt;$B$4,"Future",IF(A52=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A52,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E52=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A52&gt;$B$4,"Future",IF(A52=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A52,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E52=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1901,7 +1901,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E53" s="6" t="str">
-        <x:f>IF(A53&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A53,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A53&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A53,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F53" s="6" t="str">
         <x:f>IF(A53&gt;=$B$4,"",MAX(D53-E53,0))</x:f>
@@ -1916,7 +1916,7 @@
         <x:f>IF(A53&gt;$B$4,"",SUM($E$15:E53))</x:f>
       </x:c>
       <x:c r="J53" s="1" t="str">
-        <x:f>IF(A53&gt;$B$4,"Future",IF(A53=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A53,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E53=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A53&gt;$B$4,"Future",IF(A53=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A53,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E53=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1936,7 +1936,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E54" s="6" t="str">
-        <x:f>IF(A54&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A54,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A54&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A54,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F54" s="6" t="str">
         <x:f>IF(A54&gt;=$B$4,"",MAX(D54-E54,0))</x:f>
@@ -1951,7 +1951,7 @@
         <x:f>IF(A54&gt;$B$4,"",SUM($E$15:E54))</x:f>
       </x:c>
       <x:c r="J54" s="1" t="str">
-        <x:f>IF(A54&gt;$B$4,"Future",IF(A54=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A54,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E54=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A54&gt;$B$4,"Future",IF(A54=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A54,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E54=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1971,7 +1971,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E55" s="6" t="str">
-        <x:f>IF(A55&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A55,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A55&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A55,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F55" s="6" t="str">
         <x:f>IF(A55&gt;=$B$4,"",MAX(D55-E55,0))</x:f>
@@ -1986,7 +1986,7 @@
         <x:f>IF(A55&gt;$B$4,"",SUM($E$15:E55))</x:f>
       </x:c>
       <x:c r="J55" s="1" t="str">
-        <x:f>IF(A55&gt;$B$4,"Future",IF(A55=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A55,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E55=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A55&gt;$B$4,"Future",IF(A55=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A55,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E55=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2006,7 +2006,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E56" s="6" t="str">
-        <x:f>IF(A56&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A56,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A56&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A56,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F56" s="6" t="str">
         <x:f>IF(A56&gt;=$B$4,"",MAX(D56-E56,0))</x:f>
@@ -2021,7 +2021,7 @@
         <x:f>IF(A56&gt;$B$4,"",SUM($E$15:E56))</x:f>
       </x:c>
       <x:c r="J56" s="1" t="str">
-        <x:f>IF(A56&gt;$B$4,"Future",IF(A56=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A56,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E56=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A56&gt;$B$4,"Future",IF(A56=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A56,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E56=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2041,7 +2041,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E57" s="6" t="str">
-        <x:f>IF(A57&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A57,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A57&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A57,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F57" s="6" t="str">
         <x:f>IF(A57&gt;=$B$4,"",MAX(D57-E57,0))</x:f>
@@ -2056,7 +2056,7 @@
         <x:f>IF(A57&gt;$B$4,"",SUM($E$15:E57))</x:f>
       </x:c>
       <x:c r="J57" s="1" t="str">
-        <x:f>IF(A57&gt;$B$4,"Future",IF(A57=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A57,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E57=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A57&gt;$B$4,"Future",IF(A57=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A57,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E57=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2076,7 +2076,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E58" s="6" t="str">
-        <x:f>IF(A58&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A58,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A58&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A58,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F58" s="6" t="str">
         <x:f>IF(A58&gt;=$B$4,"",MAX(D58-E58,0))</x:f>
@@ -2091,7 +2091,7 @@
         <x:f>IF(A58&gt;$B$4,"",SUM($E$15:E58))</x:f>
       </x:c>
       <x:c r="J58" s="1" t="str">
-        <x:f>IF(A58&gt;$B$4,"Future",IF(A58=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A58,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E58=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A58&gt;$B$4,"Future",IF(A58=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A58,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E58=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2111,7 +2111,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E59" s="6" t="str">
-        <x:f>IF(A59&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A59,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A59&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A59,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F59" s="6" t="str">
         <x:f>IF(A59&gt;=$B$4,"",MAX(D59-E59,0))</x:f>
@@ -2126,7 +2126,7 @@
         <x:f>IF(A59&gt;$B$4,"",SUM($E$15:E59))</x:f>
       </x:c>
       <x:c r="J59" s="1" t="str">
-        <x:f>IF(A59&gt;$B$4,"Future",IF(A59=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A59,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E59=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A59&gt;$B$4,"Future",IF(A59=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A59,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E59=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2146,7 +2146,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E60" s="6" t="str">
-        <x:f>IF(A60&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A60,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A60&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A60,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F60" s="6" t="str">
         <x:f>IF(A60&gt;=$B$4,"",MAX(D60-E60,0))</x:f>
@@ -2161,7 +2161,7 @@
         <x:f>IF(A60&gt;$B$4,"",SUM($E$15:E60))</x:f>
       </x:c>
       <x:c r="J60" s="1" t="str">
-        <x:f>IF(A60&gt;$B$4,"Future",IF(A60=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A60,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E60=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A60&gt;$B$4,"Future",IF(A60=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A60,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E60=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2181,7 +2181,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E61" s="6" t="str">
-        <x:f>IF(A61&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A61,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A61&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A61,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F61" s="6" t="str">
         <x:f>IF(A61&gt;=$B$4,"",MAX(D61-E61,0))</x:f>
@@ -2196,7 +2196,7 @@
         <x:f>IF(A61&gt;$B$4,"",SUM($E$15:E61))</x:f>
       </x:c>
       <x:c r="J61" s="1" t="str">
-        <x:f>IF(A61&gt;$B$4,"Future",IF(A61=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A61,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E61=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A61&gt;$B$4,"Future",IF(A61=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A61,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E61=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2216,7 +2216,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E62" s="6" t="str">
-        <x:f>IF(A62&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A62,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A62&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A62,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F62" s="6" t="str">
         <x:f>IF(A62&gt;=$B$4,"",MAX(D62-E62,0))</x:f>
@@ -2231,7 +2231,7 @@
         <x:f>IF(A62&gt;$B$4,"",SUM($E$15:E62))</x:f>
       </x:c>
       <x:c r="J62" s="1" t="str">
-        <x:f>IF(A62&gt;$B$4,"Future",IF(A62=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A62,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E62=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A62&gt;$B$4,"Future",IF(A62=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A62,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E62=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2251,7 +2251,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E63" s="6" t="str">
-        <x:f>IF(A63&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A63,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A63&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A63,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F63" s="6" t="str">
         <x:f>IF(A63&gt;=$B$4,"",MAX(D63-E63,0))</x:f>
@@ -2266,7 +2266,7 @@
         <x:f>IF(A63&gt;$B$4,"",SUM($E$15:E63))</x:f>
       </x:c>
       <x:c r="J63" s="1" t="str">
-        <x:f>IF(A63&gt;$B$4,"Future",IF(A63=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A63,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E63=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A63&gt;$B$4,"Future",IF(A63=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A63,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E63=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2286,7 +2286,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E64" s="6" t="str">
-        <x:f>IF(A64&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A64,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A64&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A64,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F64" s="6" t="str">
         <x:f>IF(A64&gt;=$B$4,"",MAX(D64-E64,0))</x:f>
@@ -2301,7 +2301,7 @@
         <x:f>IF(A64&gt;$B$4,"",SUM($E$15:E64))</x:f>
       </x:c>
       <x:c r="J64" s="1" t="str">
-        <x:f>IF(A64&gt;$B$4,"Future",IF(A64=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A64,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E64=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A64&gt;$B$4,"Future",IF(A64=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A64,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E64=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2321,7 +2321,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E65" s="6" t="str">
-        <x:f>IF(A65&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A65,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A65&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A65,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F65" s="6" t="str">
         <x:f>IF(A65&gt;=$B$4,"",MAX(D65-E65,0))</x:f>
@@ -2336,7 +2336,7 @@
         <x:f>IF(A65&gt;$B$4,"",SUM($E$15:E65))</x:f>
       </x:c>
       <x:c r="J65" s="1" t="str">
-        <x:f>IF(A65&gt;$B$4,"Future",IF(A65=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A65,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E65=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A65&gt;$B$4,"Future",IF(A65=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A65,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E65=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2356,7 +2356,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E66" s="6" t="str">
-        <x:f>IF(A66&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A66,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A66&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A66,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F66" s="6" t="str">
         <x:f>IF(A66&gt;=$B$4,"",MAX(D66-E66,0))</x:f>
@@ -2371,7 +2371,7 @@
         <x:f>IF(A66&gt;$B$4,"",SUM($E$15:E66))</x:f>
       </x:c>
       <x:c r="J66" s="1" t="str">
-        <x:f>IF(A66&gt;$B$4,"Future",IF(A66=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A66,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E66=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A66&gt;$B$4,"Future",IF(A66=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A66,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E66=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2391,7 +2391,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E67" s="6" t="str">
-        <x:f>IF(A67&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A67,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A67&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A67,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F67" s="6" t="str">
         <x:f>IF(A67&gt;=$B$4,"",MAX(D67-E67,0))</x:f>
@@ -2406,7 +2406,7 @@
         <x:f>IF(A67&gt;$B$4,"",SUM($E$15:E67))</x:f>
       </x:c>
       <x:c r="J67" s="1" t="str">
-        <x:f>IF(A67&gt;$B$4,"Future",IF(A67=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A67,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E67=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A67&gt;$B$4,"Future",IF(A67=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A67,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E67=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2426,7 +2426,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E68" s="6" t="str">
-        <x:f>IF(A68&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A68,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A68&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A68,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F68" s="6" t="str">
         <x:f>IF(A68&gt;=$B$4,"",MAX(D68-E68,0))</x:f>
@@ -2441,7 +2441,7 @@
         <x:f>IF(A68&gt;$B$4,"",SUM($E$15:E68))</x:f>
       </x:c>
       <x:c r="J68" s="1" t="str">
-        <x:f>IF(A68&gt;$B$4,"Future",IF(A68=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A68,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E68=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A68&gt;$B$4,"Future",IF(A68=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A68,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E68=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2461,7 +2461,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E69" s="6" t="str">
-        <x:f>IF(A69&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A69,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A69&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A69,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F69" s="6" t="str">
         <x:f>IF(A69&gt;=$B$4,"",MAX(D69-E69,0))</x:f>
@@ -2476,7 +2476,7 @@
         <x:f>IF(A69&gt;$B$4,"",SUM($E$15:E69))</x:f>
       </x:c>
       <x:c r="J69" s="1" t="str">
-        <x:f>IF(A69&gt;$B$4,"Future",IF(A69=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A69,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E69=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A69&gt;$B$4,"Future",IF(A69=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A69,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E69=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2496,7 +2496,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E70" s="6" t="str">
-        <x:f>IF(A70&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A70,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A70&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A70,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F70" s="6" t="str">
         <x:f>IF(A70&gt;=$B$4,"",MAX(D70-E70,0))</x:f>
@@ -2511,7 +2511,7 @@
         <x:f>IF(A70&gt;$B$4,"",SUM($E$15:E70))</x:f>
       </x:c>
       <x:c r="J70" s="1" t="str">
-        <x:f>IF(A70&gt;$B$4,"Future",IF(A70=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A70,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E70=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A70&gt;$B$4,"Future",IF(A70=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A70,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E70=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2531,7 +2531,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E71" s="6" t="str">
-        <x:f>IF(A71&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A71,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A71&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A71,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F71" s="6" t="str">
         <x:f>IF(A71&gt;=$B$4,"",MAX(D71-E71,0))</x:f>
@@ -2546,7 +2546,7 @@
         <x:f>IF(A71&gt;$B$4,"",SUM($E$15:E71))</x:f>
       </x:c>
       <x:c r="J71" s="1" t="str">
-        <x:f>IF(A71&gt;$B$4,"Future",IF(A71=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A71,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E71=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A71&gt;$B$4,"Future",IF(A71=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A71,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E71=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2566,7 +2566,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E72" s="6" t="str">
-        <x:f>IF(A72&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A72,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A72&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A72,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F72" s="6" t="str">
         <x:f>IF(A72&gt;=$B$4,"",MAX(D72-E72,0))</x:f>
@@ -2581,7 +2581,7 @@
         <x:f>IF(A72&gt;$B$4,"",SUM($E$15:E72))</x:f>
       </x:c>
       <x:c r="J72" s="1" t="str">
-        <x:f>IF(A72&gt;$B$4,"Future",IF(A72=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A72,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E72=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A72&gt;$B$4,"Future",IF(A72=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A72,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E72=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2601,7 +2601,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E73" s="6" t="str">
-        <x:f>IF(A73&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A73,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A73&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A73,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F73" s="6" t="str">
         <x:f>IF(A73&gt;=$B$4,"",MAX(D73-E73,0))</x:f>
@@ -2616,7 +2616,7 @@
         <x:f>IF(A73&gt;$B$4,"",SUM($E$15:E73))</x:f>
       </x:c>
       <x:c r="J73" s="1" t="str">
-        <x:f>IF(A73&gt;$B$4,"Future",IF(A73=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A73,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E73=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A73&gt;$B$4,"Future",IF(A73=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A73,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E73=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2636,7 +2636,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E74" s="6" t="str">
-        <x:f>IF(A74&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A74,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A74&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A74,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F74" s="6" t="str">
         <x:f>IF(A74&gt;=$B$4,"",MAX(D74-E74,0))</x:f>
@@ -2651,7 +2651,7 @@
         <x:f>IF(A74&gt;$B$4,"",SUM($E$15:E74))</x:f>
       </x:c>
       <x:c r="J74" s="1" t="str">
-        <x:f>IF(A74&gt;$B$4,"Future",IF(A74=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A74,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E74=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A74&gt;$B$4,"Future",IF(A74=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A74,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E74=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2671,7 +2671,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E75" s="6" t="str">
-        <x:f>IF(A75&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A75,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A75&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A75,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F75" s="6" t="str">
         <x:f>IF(A75&gt;=$B$4,"",MAX(D75-E75,0))</x:f>
@@ -2686,7 +2686,7 @@
         <x:f>IF(A75&gt;$B$4,"",SUM($E$15:E75))</x:f>
       </x:c>
       <x:c r="J75" s="1" t="str">
-        <x:f>IF(A75&gt;$B$4,"Future",IF(A75=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A75,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E75=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A75&gt;$B$4,"Future",IF(A75=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A75,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E75=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2706,7 +2706,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E76" s="6" t="str">
-        <x:f>IF(A76&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A76,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A76&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A76,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F76" s="6" t="str">
         <x:f>IF(A76&gt;=$B$4,"",MAX(D76-E76,0))</x:f>
@@ -2721,7 +2721,7 @@
         <x:f>IF(A76&gt;$B$4,"",SUM($E$15:E76))</x:f>
       </x:c>
       <x:c r="J76" s="1" t="str">
-        <x:f>IF(A76&gt;$B$4,"Future",IF(A76=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A76,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E76=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A76&gt;$B$4,"Future",IF(A76=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A76,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E76=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2741,7 +2741,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E77" s="6" t="str">
-        <x:f>IF(A77&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A77,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A77&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A77,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F77" s="6" t="str">
         <x:f>IF(A77&gt;=$B$4,"",MAX(D77-E77,0))</x:f>
@@ -2756,7 +2756,7 @@
         <x:f>IF(A77&gt;$B$4,"",SUM($E$15:E77))</x:f>
       </x:c>
       <x:c r="J77" s="1" t="str">
-        <x:f>IF(A77&gt;$B$4,"Future",IF(A77=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A77,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E77=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A77&gt;$B$4,"Future",IF(A77=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A77,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E77=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2776,7 +2776,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E78" s="6" t="str">
-        <x:f>IF(A78&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A78,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A78&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A78,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F78" s="6" t="str">
         <x:f>IF(A78&gt;=$B$4,"",MAX(D78-E78,0))</x:f>
@@ -2791,7 +2791,7 @@
         <x:f>IF(A78&gt;$B$4,"",SUM($E$15:E78))</x:f>
       </x:c>
       <x:c r="J78" s="1" t="str">
-        <x:f>IF(A78&gt;$B$4,"Future",IF(A78=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A78,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E78=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A78&gt;$B$4,"Future",IF(A78=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A78,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E78=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2811,7 +2811,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E79" s="6" t="str">
-        <x:f>IF(A79&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A79,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A79&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A79,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F79" s="6" t="str">
         <x:f>IF(A79&gt;=$B$4,"",MAX(D79-E79,0))</x:f>
@@ -2826,7 +2826,7 @@
         <x:f>IF(A79&gt;$B$4,"",SUM($E$15:E79))</x:f>
       </x:c>
       <x:c r="J79" s="1" t="str">
-        <x:f>IF(A79&gt;$B$4,"Future",IF(A79=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A79,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E79=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A79&gt;$B$4,"Future",IF(A79=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A79,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E79=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2846,7 +2846,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E80" s="6" t="str">
-        <x:f>IF(A80&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A80,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A80&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A80,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F80" s="6" t="str">
         <x:f>IF(A80&gt;=$B$4,"",MAX(D80-E80,0))</x:f>
@@ -2861,7 +2861,7 @@
         <x:f>IF(A80&gt;$B$4,"",SUM($E$15:E80))</x:f>
       </x:c>
       <x:c r="J80" s="1" t="str">
-        <x:f>IF(A80&gt;$B$4,"Future",IF(A80=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A80,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E80=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A80&gt;$B$4,"Future",IF(A80=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A80,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E80=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2881,7 +2881,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E81" s="6" t="str">
-        <x:f>IF(A81&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A81,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A81&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A81,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F81" s="6" t="str">
         <x:f>IF(A81&gt;=$B$4,"",MAX(D81-E81,0))</x:f>
@@ -2896,7 +2896,7 @@
         <x:f>IF(A81&gt;$B$4,"",SUM($E$15:E81))</x:f>
       </x:c>
       <x:c r="J81" s="1" t="str">
-        <x:f>IF(A81&gt;$B$4,"Future",IF(A81=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A81,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E81=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A81&gt;$B$4,"Future",IF(A81=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A81,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E81=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2916,7 +2916,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E82" s="6" t="str">
-        <x:f>IF(A82&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A82,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A82&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A82,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F82" s="6" t="str">
         <x:f>IF(A82&gt;=$B$4,"",MAX(D82-E82,0))</x:f>
@@ -2931,7 +2931,7 @@
         <x:f>IF(A82&gt;$B$4,"",SUM($E$15:E82))</x:f>
       </x:c>
       <x:c r="J82" s="1" t="str">
-        <x:f>IF(A82&gt;$B$4,"Future",IF(A82=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A82,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E82=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A82&gt;$B$4,"Future",IF(A82=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A82,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E82=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2951,7 +2951,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E83" s="6" t="str">
-        <x:f>IF(A83&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A83,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A83&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A83,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F83" s="6" t="str">
         <x:f>IF(A83&gt;=$B$4,"",MAX(D83-E83,0))</x:f>
@@ -2966,7 +2966,7 @@
         <x:f>IF(A83&gt;$B$4,"",SUM($E$15:E83))</x:f>
       </x:c>
       <x:c r="J83" s="1" t="str">
-        <x:f>IF(A83&gt;$B$4,"Future",IF(A83=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A83,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E83=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A83&gt;$B$4,"Future",IF(A83=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A83,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E83=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2986,7 +2986,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E84" s="6" t="str">
-        <x:f>IF(A84&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A84,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A84&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A84,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F84" s="6" t="str">
         <x:f>IF(A84&gt;=$B$4,"",MAX(D84-E84,0))</x:f>
@@ -3001,7 +3001,7 @@
         <x:f>IF(A84&gt;$B$4,"",SUM($E$15:E84))</x:f>
       </x:c>
       <x:c r="J84" s="1" t="str">
-        <x:f>IF(A84&gt;$B$4,"Future",IF(A84=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A84,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E84=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A84&gt;$B$4,"Future",IF(A84=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A84,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E84=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3021,7 +3021,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E85" s="6" t="str">
-        <x:f>IF(A85&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A85,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A85&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A85,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F85" s="6" t="str">
         <x:f>IF(A85&gt;=$B$4,"",MAX(D85-E85,0))</x:f>
@@ -3036,7 +3036,7 @@
         <x:f>IF(A85&gt;$B$4,"",SUM($E$15:E85))</x:f>
       </x:c>
       <x:c r="J85" s="1" t="str">
-        <x:f>IF(A85&gt;$B$4,"Future",IF(A85=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A85,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E85=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A85&gt;$B$4,"Future",IF(A85=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A85,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E85=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3056,7 +3056,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E86" s="6" t="str">
-        <x:f>IF(A86&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A86,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A86&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A86,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F86" s="6" t="str">
         <x:f>IF(A86&gt;=$B$4,"",MAX(D86-E86,0))</x:f>
@@ -3071,7 +3071,7 @@
         <x:f>IF(A86&gt;$B$4,"",SUM($E$15:E86))</x:f>
       </x:c>
       <x:c r="J86" s="1" t="str">
-        <x:f>IF(A86&gt;$B$4,"Future",IF(A86=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A86,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E86=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A86&gt;$B$4,"Future",IF(A86=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A86,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E86=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3091,7 +3091,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E87" s="6" t="str">
-        <x:f>IF(A87&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A87,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A87&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A87,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F87" s="6" t="str">
         <x:f>IF(A87&gt;=$B$4,"",MAX(D87-E87,0))</x:f>
@@ -3106,7 +3106,7 @@
         <x:f>IF(A87&gt;$B$4,"",SUM($E$15:E87))</x:f>
       </x:c>
       <x:c r="J87" s="1" t="str">
-        <x:f>IF(A87&gt;$B$4,"Future",IF(A87=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A87,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E87=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A87&gt;$B$4,"Future",IF(A87=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A87,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E87=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3126,7 +3126,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E88" s="6" t="str">
-        <x:f>IF(A88&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A88,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A88&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A88,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F88" s="6" t="str">
         <x:f>IF(A88&gt;=$B$4,"",MAX(D88-E88,0))</x:f>
@@ -3141,7 +3141,7 @@
         <x:f>IF(A88&gt;$B$4,"",SUM($E$15:E88))</x:f>
       </x:c>
       <x:c r="J88" s="1" t="str">
-        <x:f>IF(A88&gt;$B$4,"Future",IF(A88=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A88,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E88=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A88&gt;$B$4,"Future",IF(A88=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A88,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E88=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3161,7 +3161,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E89" s="6" t="str">
-        <x:f>IF(A89&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A89,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A89&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A89,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F89" s="6" t="str">
         <x:f>IF(A89&gt;=$B$4,"",MAX(D89-E89,0))</x:f>
@@ -3176,7 +3176,7 @@
         <x:f>IF(A89&gt;$B$4,"",SUM($E$15:E89))</x:f>
       </x:c>
       <x:c r="J89" s="1" t="str">
-        <x:f>IF(A89&gt;$B$4,"Future",IF(A89=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A89,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E89=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A89&gt;$B$4,"Future",IF(A89=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A89,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E89=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3196,7 +3196,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E90" s="6" t="str">
-        <x:f>IF(A90&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A90,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A90&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A90,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F90" s="6" t="str">
         <x:f>IF(A90&gt;=$B$4,"",MAX(D90-E90,0))</x:f>
@@ -3211,7 +3211,7 @@
         <x:f>IF(A90&gt;$B$4,"",SUM($E$15:E90))</x:f>
       </x:c>
       <x:c r="J90" s="1" t="str">
-        <x:f>IF(A90&gt;$B$4,"Future",IF(A90=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A90,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E90=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A90&gt;$B$4,"Future",IF(A90=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A90,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E90=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3231,7 +3231,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E91" s="6" t="str">
-        <x:f>IF(A91&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A91,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A91&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A91,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F91" s="6" t="str">
         <x:f>IF(A91&gt;=$B$4,"",MAX(D91-E91,0))</x:f>
@@ -3246,7 +3246,7 @@
         <x:f>IF(A91&gt;$B$4,"",SUM($E$15:E91))</x:f>
       </x:c>
       <x:c r="J91" s="1" t="str">
-        <x:f>IF(A91&gt;$B$4,"Future",IF(A91=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A91,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E91=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A91&gt;$B$4,"Future",IF(A91=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A91,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E91=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3266,7 +3266,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E92" s="6" t="str">
-        <x:f>IF(A92&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A92,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A92&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A92,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F92" s="6" t="str">
         <x:f>IF(A92&gt;=$B$4,"",MAX(D92-E92,0))</x:f>
@@ -3281,7 +3281,7 @@
         <x:f>IF(A92&gt;$B$4,"",SUM($E$15:E92))</x:f>
       </x:c>
       <x:c r="J92" s="1" t="str">
-        <x:f>IF(A92&gt;$B$4,"Future",IF(A92=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A92,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E92=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A92&gt;$B$4,"Future",IF(A92=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A92,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E92=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3301,7 +3301,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E93" s="6" t="str">
-        <x:f>IF(A93&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A93,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A93&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A93,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F93" s="6" t="str">
         <x:f>IF(A93&gt;=$B$4,"",MAX(D93-E93,0))</x:f>
@@ -3316,7 +3316,7 @@
         <x:f>IF(A93&gt;$B$4,"",SUM($E$15:E93))</x:f>
       </x:c>
       <x:c r="J93" s="1" t="str">
-        <x:f>IF(A93&gt;$B$4,"Future",IF(A93=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A93,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E93=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A93&gt;$B$4,"Future",IF(A93=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A93,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E93=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3336,7 +3336,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E94" s="6" t="str">
-        <x:f>IF(A94&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A94,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A94&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A94,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F94" s="6" t="str">
         <x:f>IF(A94&gt;=$B$4,"",MAX(D94-E94,0))</x:f>
@@ -3351,7 +3351,7 @@
         <x:f>IF(A94&gt;$B$4,"",SUM($E$15:E94))</x:f>
       </x:c>
       <x:c r="J94" s="1" t="str">
-        <x:f>IF(A94&gt;$B$4,"Future",IF(A94=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A94,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E94=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A94&gt;$B$4,"Future",IF(A94=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A94,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E94=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3371,7 +3371,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E95" s="6" t="str">
-        <x:f>IF(A95&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A95,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A95&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A95,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F95" s="6" t="str">
         <x:f>IF(A95&gt;=$B$4,"",MAX(D95-E95,0))</x:f>
@@ -3386,7 +3386,7 @@
         <x:f>IF(A95&gt;$B$4,"",SUM($E$15:E95))</x:f>
       </x:c>
       <x:c r="J95" s="1" t="str">
-        <x:f>IF(A95&gt;$B$4,"Future",IF(A95=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A95,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E95=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A95&gt;$B$4,"Future",IF(A95=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A95,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E95=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3406,7 +3406,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E96" s="6" t="str">
-        <x:f>IF(A96&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A96,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A96&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A96,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F96" s="6" t="str">
         <x:f>IF(A96&gt;=$B$4,"",MAX(D96-E96,0))</x:f>
@@ -3421,7 +3421,7 @@
         <x:f>IF(A96&gt;$B$4,"",SUM($E$15:E96))</x:f>
       </x:c>
       <x:c r="J96" s="1" t="str">
-        <x:f>IF(A96&gt;$B$4,"Future",IF(A96=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A96,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E96=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A96&gt;$B$4,"Future",IF(A96=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A96,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E96=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3441,7 +3441,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E97" s="6" t="str">
-        <x:f>IF(A97&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A97,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A97&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A97,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F97" s="6" t="str">
         <x:f>IF(A97&gt;=$B$4,"",MAX(D97-E97,0))</x:f>
@@ -3456,7 +3456,7 @@
         <x:f>IF(A97&gt;$B$4,"",SUM($E$15:E97))</x:f>
       </x:c>
       <x:c r="J97" s="1" t="str">
-        <x:f>IF(A97&gt;$B$4,"Future",IF(A97=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A97,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E97=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A97&gt;$B$4,"Future",IF(A97=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A97,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E97=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3476,7 +3476,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E98" s="6" t="str">
-        <x:f>IF(A98&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A98,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A98&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A98,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F98" s="6" t="str">
         <x:f>IF(A98&gt;=$B$4,"",MAX(D98-E98,0))</x:f>
@@ -3491,7 +3491,7 @@
         <x:f>IF(A98&gt;$B$4,"",SUM($E$15:E98))</x:f>
       </x:c>
       <x:c r="J98" s="1" t="str">
-        <x:f>IF(A98&gt;$B$4,"Future",IF(A98=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A98,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E98=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A98&gt;$B$4,"Future",IF(A98=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A98,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E98=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3511,7 +3511,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E99" s="6" t="str">
-        <x:f>IF(A99&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A99,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A99&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A99,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F99" s="6" t="str">
         <x:f>IF(A99&gt;=$B$4,"",MAX(D99-E99,0))</x:f>
@@ -3526,7 +3526,7 @@
         <x:f>IF(A99&gt;$B$4,"",SUM($E$15:E99))</x:f>
       </x:c>
       <x:c r="J99" s="1" t="str">
-        <x:f>IF(A99&gt;$B$4,"Future",IF(A99=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A99,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E99=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A99&gt;$B$4,"Future",IF(A99=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A99,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E99=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3546,7 +3546,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E100" s="6" t="str">
-        <x:f>IF(A100&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A100,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A100&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A100,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F100" s="6" t="str">
         <x:f>IF(A100&gt;=$B$4,"",MAX(D100-E100,0))</x:f>
@@ -3561,7 +3561,7 @@
         <x:f>IF(A100&gt;$B$4,"",SUM($E$15:E100))</x:f>
       </x:c>
       <x:c r="J100" s="1" t="str">
-        <x:f>IF(A100&gt;$B$4,"Future",IF(A100=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A100,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E100=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A100&gt;$B$4,"Future",IF(A100=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A100,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E100=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3581,7 +3581,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E101" s="6" t="str">
-        <x:f>IF(A101&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A101,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A101&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A101,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F101" s="6" t="str">
         <x:f>IF(A101&gt;=$B$4,"",MAX(D101-E101,0))</x:f>
@@ -3596,7 +3596,7 @@
         <x:f>IF(A101&gt;$B$4,"",SUM($E$15:E101))</x:f>
       </x:c>
       <x:c r="J101" s="1" t="str">
-        <x:f>IF(A101&gt;$B$4,"Future",IF(A101=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A101,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E101=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A101&gt;$B$4,"Future",IF(A101=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A101,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E101=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3616,7 +3616,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E102" s="6" t="str">
-        <x:f>IF(A102&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A102,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A102&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A102,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F102" s="6" t="str">
         <x:f>IF(A102&gt;=$B$4,"",MAX(D102-E102,0))</x:f>
@@ -3631,7 +3631,7 @@
         <x:f>IF(A102&gt;$B$4,"",SUM($E$15:E102))</x:f>
       </x:c>
       <x:c r="J102" s="1" t="str">
-        <x:f>IF(A102&gt;$B$4,"Future",IF(A102=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A102,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E102=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A102&gt;$B$4,"Future",IF(A102=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A102,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E102=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3651,7 +3651,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E103" s="6" t="str">
-        <x:f>IF(A103&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A103,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A103&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A103,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F103" s="6" t="str">
         <x:f>IF(A103&gt;=$B$4,"",MAX(D103-E103,0))</x:f>
@@ -3666,7 +3666,7 @@
         <x:f>IF(A103&gt;$B$4,"",SUM($E$15:E103))</x:f>
       </x:c>
       <x:c r="J103" s="1" t="str">
-        <x:f>IF(A103&gt;$B$4,"Future",IF(A103=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A103,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E103=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A103&gt;$B$4,"Future",IF(A103=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A103,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E103=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3686,7 +3686,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E104" s="6" t="str">
-        <x:f>IF(A104&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A104,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A104&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A104,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F104" s="6" t="str">
         <x:f>IF(A104&gt;=$B$4,"",MAX(D104-E104,0))</x:f>
@@ -3701,7 +3701,7 @@
         <x:f>IF(A104&gt;$B$4,"",SUM($E$15:E104))</x:f>
       </x:c>
       <x:c r="J104" s="1" t="str">
-        <x:f>IF(A104&gt;$B$4,"Future",IF(A104=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A104,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E104=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A104&gt;$B$4,"Future",IF(A104=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A104,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E104=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3721,7 +3721,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E105" s="6" t="str">
-        <x:f>IF(A105&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A105,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A105&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A105,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F105" s="6" t="str">
         <x:f>IF(A105&gt;=$B$4,"",MAX(D105-E105,0))</x:f>
@@ -3736,7 +3736,7 @@
         <x:f>IF(A105&gt;$B$4,"",SUM($E$15:E105))</x:f>
       </x:c>
       <x:c r="J105" s="1" t="str">
-        <x:f>IF(A105&gt;$B$4,"Future",IF(A105=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A105,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E105=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A105&gt;$B$4,"Future",IF(A105=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A105,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E105=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3756,7 +3756,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E106" s="6" t="str">
-        <x:f>IF(A106&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A106,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A106&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A106,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F106" s="6" t="str">
         <x:f>IF(A106&gt;=$B$4,"",MAX(D106-E106,0))</x:f>
@@ -3771,7 +3771,7 @@
         <x:f>IF(A106&gt;$B$4,"",SUM($E$15:E106))</x:f>
       </x:c>
       <x:c r="J106" s="1" t="str">
-        <x:f>IF(A106&gt;$B$4,"Future",IF(A106=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A106,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E106=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A106&gt;$B$4,"Future",IF(A106=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A106,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E106=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3791,7 +3791,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E107" s="6" t="str">
-        <x:f>IF(A107&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A107,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A107&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A107,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F107" s="6" t="str">
         <x:f>IF(A107&gt;=$B$4,"",MAX(D107-E107,0))</x:f>
@@ -3806,7 +3806,7 @@
         <x:f>IF(A107&gt;$B$4,"",SUM($E$15:E107))</x:f>
       </x:c>
       <x:c r="J107" s="1" t="str">
-        <x:f>IF(A107&gt;$B$4,"Future",IF(A107=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A107,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E107=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A107&gt;$B$4,"Future",IF(A107=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A107,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E107=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3826,7 +3826,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E108" s="6" t="str">
-        <x:f>IF(A108&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A108,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A108&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A108,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F108" s="6" t="str">
         <x:f>IF(A108&gt;=$B$4,"",MAX(D108-E108,0))</x:f>
@@ -3841,7 +3841,7 @@
         <x:f>IF(A108&gt;$B$4,"",SUM($E$15:E108))</x:f>
       </x:c>
       <x:c r="J108" s="1" t="str">
-        <x:f>IF(A108&gt;$B$4,"Future",IF(A108=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A108,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E108=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A108&gt;$B$4,"Future",IF(A108=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A108,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E108=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3861,7 +3861,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E109" s="6" t="str">
-        <x:f>IF(A109&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A109,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A109&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A109,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F109" s="6" t="str">
         <x:f>IF(A109&gt;=$B$4,"",MAX(D109-E109,0))</x:f>
@@ -3876,7 +3876,7 @@
         <x:f>IF(A109&gt;$B$4,"",SUM($E$15:E109))</x:f>
       </x:c>
       <x:c r="J109" s="1" t="str">
-        <x:f>IF(A109&gt;$B$4,"Future",IF(A109=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A109,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E109=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A109&gt;$B$4,"Future",IF(A109=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A109,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E109=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3896,7 +3896,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E110" s="6" t="str">
-        <x:f>IF(A110&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A110,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A110&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A110,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F110" s="6" t="str">
         <x:f>IF(A110&gt;=$B$4,"",MAX(D110-E110,0))</x:f>
@@ -3911,7 +3911,7 @@
         <x:f>IF(A110&gt;$B$4,"",SUM($E$15:E110))</x:f>
       </x:c>
       <x:c r="J110" s="1" t="str">
-        <x:f>IF(A110&gt;$B$4,"Future",IF(A110=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A110,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E110=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A110&gt;$B$4,"Future",IF(A110=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A110,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E110=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3931,7 +3931,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E111" s="6" t="str">
-        <x:f>IF(A111&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A111,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A111&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A111,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F111" s="6" t="str">
         <x:f>IF(A111&gt;=$B$4,"",MAX(D111-E111,0))</x:f>
@@ -3946,7 +3946,7 @@
         <x:f>IF(A111&gt;$B$4,"",SUM($E$15:E111))</x:f>
       </x:c>
       <x:c r="J111" s="1" t="str">
-        <x:f>IF(A111&gt;$B$4,"Future",IF(A111=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A111,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E111=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A111&gt;$B$4,"Future",IF(A111=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A111,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E111=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3966,7 +3966,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E112" s="6" t="str">
-        <x:f>IF(A112&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A112,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A112&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A112,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F112" s="6" t="str">
         <x:f>IF(A112&gt;=$B$4,"",MAX(D112-E112,0))</x:f>
@@ -3981,7 +3981,7 @@
         <x:f>IF(A112&gt;$B$4,"",SUM($E$15:E112))</x:f>
       </x:c>
       <x:c r="J112" s="1" t="str">
-        <x:f>IF(A112&gt;$B$4,"Future",IF(A112=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A112,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E112=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A112&gt;$B$4,"Future",IF(A112=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A112,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E112=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4001,7 +4001,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E113" s="6" t="str">
-        <x:f>IF(A113&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A113,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A113&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A113,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F113" s="6" t="str">
         <x:f>IF(A113&gt;=$B$4,"",MAX(D113-E113,0))</x:f>
@@ -4016,7 +4016,7 @@
         <x:f>IF(A113&gt;$B$4,"",SUM($E$15:E113))</x:f>
       </x:c>
       <x:c r="J113" s="1" t="str">
-        <x:f>IF(A113&gt;$B$4,"Future",IF(A113=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A113,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E113=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A113&gt;$B$4,"Future",IF(A113=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A113,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E113=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4036,7 +4036,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E114" s="6" t="str">
-        <x:f>IF(A114&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A114,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A114&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A114,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F114" s="6" t="str">
         <x:f>IF(A114&gt;=$B$4,"",MAX(D114-E114,0))</x:f>
@@ -4051,7 +4051,7 @@
         <x:f>IF(A114&gt;$B$4,"",SUM($E$15:E114))</x:f>
       </x:c>
       <x:c r="J114" s="1" t="str">
-        <x:f>IF(A114&gt;$B$4,"Future",IF(A114=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A114,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E114=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A114&gt;$B$4,"Future",IF(A114=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A114,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E114=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4071,7 +4071,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E115" s="6" t="str">
-        <x:f>IF(A115&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A115,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A115&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A115,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F115" s="6" t="str">
         <x:f>IF(A115&gt;=$B$4,"",MAX(D115-E115,0))</x:f>
@@ -4086,7 +4086,7 @@
         <x:f>IF(A115&gt;$B$4,"",SUM($E$15:E115))</x:f>
       </x:c>
       <x:c r="J115" s="1" t="str">
-        <x:f>IF(A115&gt;$B$4,"Future",IF(A115=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A115,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E115=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A115&gt;$B$4,"Future",IF(A115=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A115,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E115=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4106,7 +4106,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E116" s="6" t="str">
-        <x:f>IF(A116&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A116,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A116&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A116,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F116" s="6" t="str">
         <x:f>IF(A116&gt;=$B$4,"",MAX(D116-E116,0))</x:f>
@@ -4121,7 +4121,7 @@
         <x:f>IF(A116&gt;$B$4,"",SUM($E$15:E116))</x:f>
       </x:c>
       <x:c r="J116" s="1" t="str">
-        <x:f>IF(A116&gt;$B$4,"Future",IF(A116=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A116,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E116=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A116&gt;$B$4,"Future",IF(A116=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A116,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E116=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4141,7 +4141,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E117" s="6" t="str">
-        <x:f>IF(A117&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A117,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A117&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A117,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F117" s="6" t="str">
         <x:f>IF(A117&gt;=$B$4,"",MAX(D117-E117,0))</x:f>
@@ -4156,7 +4156,7 @@
         <x:f>IF(A117&gt;$B$4,"",SUM($E$15:E117))</x:f>
       </x:c>
       <x:c r="J117" s="1" t="str">
-        <x:f>IF(A117&gt;$B$4,"Future",IF(A117=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A117,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E117=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A117&gt;$B$4,"Future",IF(A117=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A117,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E117=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4176,7 +4176,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E118" s="6" t="str">
-        <x:f>IF(A118&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A118,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A118&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A118,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F118" s="6" t="str">
         <x:f>IF(A118&gt;=$B$4,"",MAX(D118-E118,0))</x:f>
@@ -4191,7 +4191,7 @@
         <x:f>IF(A118&gt;$B$4,"",SUM($E$15:E118))</x:f>
       </x:c>
       <x:c r="J118" s="1" t="str">
-        <x:f>IF(A118&gt;$B$4,"Future",IF(A118=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A118,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E118=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A118&gt;$B$4,"Future",IF(A118=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A118,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E118=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4211,7 +4211,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E119" s="6" t="str">
-        <x:f>IF(A119&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A119,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A119&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A119,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F119" s="6" t="str">
         <x:f>IF(A119&gt;=$B$4,"",MAX(D119-E119,0))</x:f>
@@ -4226,7 +4226,7 @@
         <x:f>IF(A119&gt;$B$4,"",SUM($E$15:E119))</x:f>
       </x:c>
       <x:c r="J119" s="1" t="str">
-        <x:f>IF(A119&gt;$B$4,"Future",IF(A119=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A119,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E119=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A119&gt;$B$4,"Future",IF(A119=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A119,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E119=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4246,7 +4246,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E120" s="6" t="str">
-        <x:f>IF(A120&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A120,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A120&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A120,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F120" s="6" t="str">
         <x:f>IF(A120&gt;=$B$4,"",MAX(D120-E120,0))</x:f>
@@ -4261,7 +4261,7 @@
         <x:f>IF(A120&gt;$B$4,"",SUM($E$15:E120))</x:f>
       </x:c>
       <x:c r="J120" s="1" t="str">
-        <x:f>IF(A120&gt;$B$4,"Future",IF(A120=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A120,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E120=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A120&gt;$B$4,"Future",IF(A120=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A120,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E120=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4281,7 +4281,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E121" s="6" t="str">
-        <x:f>IF(A121&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A121,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A121&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A121,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F121" s="6" t="str">
         <x:f>IF(A121&gt;=$B$4,"",MAX(D121-E121,0))</x:f>
@@ -4296,7 +4296,7 @@
         <x:f>IF(A121&gt;$B$4,"",SUM($E$15:E121))</x:f>
       </x:c>
       <x:c r="J121" s="1" t="str">
-        <x:f>IF(A121&gt;$B$4,"Future",IF(A121=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A121,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E121=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A121&gt;$B$4,"Future",IF(A121=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A121,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E121=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4316,7 +4316,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E122" s="6" t="str">
-        <x:f>IF(A122&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A122,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A122&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A122,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F122" s="6" t="str">
         <x:f>IF(A122&gt;=$B$4,"",MAX(D122-E122,0))</x:f>
@@ -4331,7 +4331,7 @@
         <x:f>IF(A122&gt;$B$4,"",SUM($E$15:E122))</x:f>
       </x:c>
       <x:c r="J122" s="1" t="str">
-        <x:f>IF(A122&gt;$B$4,"Future",IF(A122=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A122,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E122=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A122&gt;$B$4,"Future",IF(A122=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A122,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E122=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4351,7 +4351,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E123" s="6" t="str">
-        <x:f>IF(A123&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A123,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A123&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A123,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F123" s="6" t="str">
         <x:f>IF(A123&gt;=$B$4,"",MAX(D123-E123,0))</x:f>
@@ -4366,7 +4366,7 @@
         <x:f>IF(A123&gt;$B$4,"",SUM($E$15:E123))</x:f>
       </x:c>
       <x:c r="J123" s="1" t="str">
-        <x:f>IF(A123&gt;$B$4,"Future",IF(A123=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A123,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E123=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A123&gt;$B$4,"Future",IF(A123=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A123,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E123=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4386,7 +4386,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E124" s="6" t="str">
-        <x:f>IF(A124&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A124,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A124&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A124,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F124" s="6" t="str">
         <x:f>IF(A124&gt;=$B$4,"",MAX(D124-E124,0))</x:f>
@@ -4401,7 +4401,7 @@
         <x:f>IF(A124&gt;$B$4,"",SUM($E$15:E124))</x:f>
       </x:c>
       <x:c r="J124" s="1" t="str">
-        <x:f>IF(A124&gt;$B$4,"Future",IF(A124=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A124,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E124=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A124&gt;$B$4,"Future",IF(A124=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A124,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E124=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4421,7 +4421,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E125" s="6" t="str">
-        <x:f>IF(A125&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A125,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A125&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A125,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F125" s="6" t="str">
         <x:f>IF(A125&gt;=$B$4,"",MAX(D125-E125,0))</x:f>
@@ -4436,7 +4436,7 @@
         <x:f>IF(A125&gt;$B$4,"",SUM($E$15:E125))</x:f>
       </x:c>
       <x:c r="J125" s="1" t="str">
-        <x:f>IF(A125&gt;$B$4,"Future",IF(A125=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A125,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E125=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A125&gt;$B$4,"Future",IF(A125=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A125,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E125=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4456,7 +4456,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E126" s="6" t="str">
-        <x:f>IF(A126&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A126,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A126&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A126,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F126" s="6" t="str">
         <x:f>IF(A126&gt;=$B$4,"",MAX(D126-E126,0))</x:f>
@@ -4471,7 +4471,7 @@
         <x:f>IF(A126&gt;$B$4,"",SUM($E$15:E126))</x:f>
       </x:c>
       <x:c r="J126" s="1" t="str">
-        <x:f>IF(A126&gt;$B$4,"Future",IF(A126=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A126,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E126=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A126&gt;$B$4,"Future",IF(A126=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A126,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E126=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4491,7 +4491,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E127" s="6" t="str">
-        <x:f>IF(A127&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A127,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A127&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A127,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F127" s="6" t="str">
         <x:f>IF(A127&gt;=$B$4,"",MAX(D127-E127,0))</x:f>
@@ -4506,7 +4506,7 @@
         <x:f>IF(A127&gt;$B$4,"",SUM($E$15:E127))</x:f>
       </x:c>
       <x:c r="J127" s="1" t="str">
-        <x:f>IF(A127&gt;$B$4,"Future",IF(A127=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A127,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E127=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A127&gt;$B$4,"Future",IF(A127=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A127,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E127=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4526,7 +4526,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E128" s="6" t="str">
-        <x:f>IF(A128&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A128,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A128&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A128,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F128" s="6" t="str">
         <x:f>IF(A128&gt;=$B$4,"",MAX(D128-E128,0))</x:f>
@@ -4541,7 +4541,7 @@
         <x:f>IF(A128&gt;$B$4,"",SUM($E$15:E128))</x:f>
       </x:c>
       <x:c r="J128" s="1" t="str">
-        <x:f>IF(A128&gt;$B$4,"Future",IF(A128=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A128,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E128=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A128&gt;$B$4,"Future",IF(A128=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A128,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E128=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4561,7 +4561,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E129" s="6" t="str">
-        <x:f>IF(A129&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A129,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A129&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A129,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F129" s="6" t="str">
         <x:f>IF(A129&gt;=$B$4,"",MAX(D129-E129,0))</x:f>
@@ -4576,7 +4576,7 @@
         <x:f>IF(A129&gt;$B$4,"",SUM($E$15:E129))</x:f>
       </x:c>
       <x:c r="J129" s="1" t="str">
-        <x:f>IF(A129&gt;$B$4,"Future",IF(A129=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A129,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E129=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A129&gt;$B$4,"Future",IF(A129=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A129,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E129=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4596,7 +4596,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E130" s="6" t="str">
-        <x:f>IF(A130&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$13,'Sessions'!$B$2:$B$13,A130,'Sessions'!$G$2:$G$13,"completed")/60)</x:f>
+        <x:f>IF(A130&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A130,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
       </x:c>
       <x:c r="F130" s="6" t="str">
         <x:f>IF(A130&gt;=$B$4,"",MAX(D130-E130,0))</x:f>
@@ -4611,7 +4611,7 @@
         <x:f>IF(A130&gt;$B$4,"",SUM($E$15:E130))</x:f>
       </x:c>
       <x:c r="J130" s="1" t="str">
-        <x:f>IF(A130&gt;$B$4,"Future",IF(A130=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$13,A130,'Sessions'!$G$2:$G$13,"needs_confirmation")&gt;0,"Uncertain time",IF(E130=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A130&gt;$B$4,"Future",IF(A130=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A130,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E130=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4735,7 +4735,7 @@
       </x:c>
       <x:c r="D8" s="6" t="n">
         <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A8)</x:f>
-        <x:v>4.371944444444999</x:v>
+        <x:v>4.499166666667222</x:v>
       </x:c>
       <x:c r="E8" s="6" t="n">
         <x:f>MAX(C8-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A8,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
@@ -4747,11 +4747,11 @@
       </x:c>
       <x:c r="G8" s="6" t="n">
         <x:f>MAX(B8-D8,0)</x:f>
-        <x:v>27.628055555555</x:v>
+        <x:v>27.50083333333278</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
         <x:f>IF(B8=0,0,D8/B8)</x:f>
-        <x:v>0.13662326388890622</x:v>
+        <x:v>0.14059895833335068</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
@@ -5640,6 +5640,32 @@
         <x:v>Explicit resume-timer; prior topic Python; break excluded; blank spaces zero check pending; no new learning evidence to duplicate; Explicit pause 12:00:15 IST; 29m28s; cleaner function and CSV reading completed with guidance; CSV output task pending</x:v>
       </x:c>
     </x:row>
+    <x:row r="14" ht="22" customHeight="1">
+      <x:c r="A14" s="1" t="str">
+        <x:v>PY-20261016T133137</x:v>
+      </x:c>
+      <x:c r="B14" s="7" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="C14" s="1" t="str">
+        <x:v>Python: CSV reading and writing</x:v>
+      </x:c>
+      <x:c r="D14" s="1" t="str">
+        <x:v>IST 2026-10-16 13:31:37</x:v>
+      </x:c>
+      <x:c r="E14" s="1" t="str">
+        <x:v>IST 2026-10-16 13:39:15</x:v>
+      </x:c>
+      <x:c r="F14" s="1" t="n">
+        <x:v>7.633333333333334</x:v>
+      </x:c>
+      <x:c r="G14" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H14" s="1" t="str">
+        <x:v>Explicit start-timer for CSV; break excluded; pending output-file task; earlier 15 October uncertain interval remains excluded; Explicit pause 13:39:15 IST; 7m38s; no new submitted code or output; CSV writing task pending</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Save RRDAP setup, Python practice notes and study checkpoints
</commit_message>
<xml_diff>
--- a/outputs/study-tracker/study-hours.xlsx
+++ b/outputs/study-tracker/study-hours.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="R8c3ed5d77fed4b78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="R08394828940a4f03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="R9a38385d7c2843d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="R0756837246834773"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="R621daf9bb6f74648"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="R6e15d754381d424b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -354,7 +354,7 @@
         <x:v>Reporting date (IST)</x:v>
       </x:c>
       <x:c r="B4" s="8" t="n">
-        <x:v>46311</x:v>
+        <x:v>46312</x:v>
       </x:c>
       <x:c r="C4" s="1"/>
       <x:c r="D4" s="1" t="str">
@@ -362,7 +362,7 @@
       </x:c>
       <x:c r="E4" s="6" t="n">
         <x:f>SUM(E15:E130)</x:f>
-        <x:v>4.499166666667222</x:v>
+        <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="F4" s="1"/>
       <x:c r="G4" s="1"/>
@@ -383,7 +383,7 @@
       </x:c>
       <x:c r="E5" s="6" t="n">
         <x:f>SUMIFS(D15:D130,A15:A130,"&lt;"&amp;B4)</x:f>
-        <x:v>6</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F5" s="1"/>
       <x:c r="G5" s="1"/>
@@ -404,7 +404,7 @@
       </x:c>
       <x:c r="E6" s="6" t="n">
         <x:f>MAX(E5-SUMIFS(E15:E130,A15:A130,"&lt;"&amp;B4),0)</x:f>
-        <x:v>3.1905555555550005</x:v>
+        <x:v>7.500833333332778</x:v>
       </x:c>
       <x:c r="F6" s="1"/>
       <x:c r="G6" s="1"/>
@@ -442,7 +442,7 @@
       </x:c>
       <x:c r="E8" s="6" t="n">
         <x:f>MAX(SUMIFS(D15:D130,A15:A130,B4)-SUMIFS(E15:E130,A15:A130,B4),0)</x:f>
-        <x:v>4.310277777777777</x:v>
+        <x:v>3.347777777777777</x:v>
       </x:c>
       <x:c r="F8" s="1"/>
       <x:c r="G8" s="1"/>
@@ -564,7 +564,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E15" s="6" t="n">
-        <x:f>IF(A15&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A15,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A15&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A15,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
         <x:v>2.8094444444449995</x:v>
       </x:c>
       <x:c r="F15" s="6" t="n">
@@ -584,7 +584,7 @@
         <x:v>2.8094444444449995</x:v>
       </x:c>
       <x:c r="J15" s="1" t="str">
-        <x:f>IF(A15&gt;$B$4,"Future",IF(A15=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A15,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E15=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A15&gt;$B$4,"Future",IF(A15=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A15,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E15=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Uncertain time</x:v>
       </x:c>
     </x:row>
@@ -604,25 +604,28 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E16" s="6" t="n">
-        <x:f>IF(A16&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A16,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A16&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A16,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
         <x:v>1.6897222222222223</x:v>
       </x:c>
-      <x:c r="F16" s="6" t="str">
+      <x:c r="F16" s="6" t="n">
         <x:f>IF(A16&gt;=$B$4,"",MAX(D16-E16,0))</x:f>
-      </x:c>
-      <x:c r="G16" s="6" t="str">
+        <x:v>4.310277777777777</x:v>
+      </x:c>
+      <x:c r="G16" s="6" t="n">
         <x:f>IF(A16&gt;=$B$4,"",MAX(E16-D16,0))</x:f>
-      </x:c>
-      <x:c r="H16" s="6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H16" s="6" t="n">
         <x:f>IF(A16&gt;=$B$4,"",SUM($D$15:D16))</x:f>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="I16" s="6" t="n">
         <x:f>IF(A16&gt;$B$4,"",SUM($E$15:E16))</x:f>
         <x:v>4.499166666667222</x:v>
       </x:c>
       <x:c r="J16" s="1" t="str">
-        <x:f>IF(A16&gt;$B$4,"Future",IF(A16=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A16,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E16=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>In progress</x:v>
+        <x:f>IF(A16&gt;$B$4,"Future",IF(A16=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A16,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E16=0,"No confirmed time","Logged"))))</x:f>
+        <x:v>Logged</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
@@ -640,8 +643,9 @@
         <x:f>IF(WEEKDAY(A17,2)&gt;5,$B$7,$B$6)</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="E17" s="6" t="str">
-        <x:f>IF(A17&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A17,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+      <x:c r="E17" s="6" t="n">
+        <x:f>IF(A17&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A17,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:v>6.652222222222223</x:v>
       </x:c>
       <x:c r="F17" s="6" t="str">
         <x:f>IF(A17&gt;=$B$4,"",MAX(D17-E17,0))</x:f>
@@ -652,12 +656,13 @@
       <x:c r="H17" s="6" t="str">
         <x:f>IF(A17&gt;=$B$4,"",SUM($D$15:D17))</x:f>
       </x:c>
-      <x:c r="I17" s="6" t="str">
+      <x:c r="I17" s="6" t="n">
         <x:f>IF(A17&gt;$B$4,"",SUM($E$15:E17))</x:f>
+        <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J17" s="1" t="str">
-        <x:f>IF(A17&gt;$B$4,"Future",IF(A17=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A17,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E17=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
+        <x:f>IF(A17&gt;$B$4,"Future",IF(A17=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A17,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E17=0,"No confirmed time","Logged"))))</x:f>
+        <x:v>In progress</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
@@ -676,7 +681,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E18" s="6" t="str">
-        <x:f>IF(A18&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A18,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A18&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A18,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F18" s="6" t="str">
         <x:f>IF(A18&gt;=$B$4,"",MAX(D18-E18,0))</x:f>
@@ -691,7 +696,7 @@
         <x:f>IF(A18&gt;$B$4,"",SUM($E$15:E18))</x:f>
       </x:c>
       <x:c r="J18" s="1" t="str">
-        <x:f>IF(A18&gt;$B$4,"Future",IF(A18=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A18,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E18=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A18&gt;$B$4,"Future",IF(A18=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A18,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E18=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -711,7 +716,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E19" s="6" t="str">
-        <x:f>IF(A19&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A19,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A19&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A19,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F19" s="6" t="str">
         <x:f>IF(A19&gt;=$B$4,"",MAX(D19-E19,0))</x:f>
@@ -726,7 +731,7 @@
         <x:f>IF(A19&gt;$B$4,"",SUM($E$15:E19))</x:f>
       </x:c>
       <x:c r="J19" s="1" t="str">
-        <x:f>IF(A19&gt;$B$4,"Future",IF(A19=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A19,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E19=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A19&gt;$B$4,"Future",IF(A19=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A19,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E19=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -746,7 +751,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E20" s="6" t="str">
-        <x:f>IF(A20&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A20,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A20&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A20,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F20" s="6" t="str">
         <x:f>IF(A20&gt;=$B$4,"",MAX(D20-E20,0))</x:f>
@@ -761,7 +766,7 @@
         <x:f>IF(A20&gt;$B$4,"",SUM($E$15:E20))</x:f>
       </x:c>
       <x:c r="J20" s="1" t="str">
-        <x:f>IF(A20&gt;$B$4,"Future",IF(A20=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A20,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E20=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A20&gt;$B$4,"Future",IF(A20=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A20,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E20=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -781,7 +786,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E21" s="6" t="str">
-        <x:f>IF(A21&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A21,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A21&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A21,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F21" s="6" t="str">
         <x:f>IF(A21&gt;=$B$4,"",MAX(D21-E21,0))</x:f>
@@ -796,7 +801,7 @@
         <x:f>IF(A21&gt;$B$4,"",SUM($E$15:E21))</x:f>
       </x:c>
       <x:c r="J21" s="1" t="str">
-        <x:f>IF(A21&gt;$B$4,"Future",IF(A21=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A21,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E21=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A21&gt;$B$4,"Future",IF(A21=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A21,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E21=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -816,7 +821,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E22" s="6" t="str">
-        <x:f>IF(A22&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A22,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A22&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A22,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F22" s="6" t="str">
         <x:f>IF(A22&gt;=$B$4,"",MAX(D22-E22,0))</x:f>
@@ -831,7 +836,7 @@
         <x:f>IF(A22&gt;$B$4,"",SUM($E$15:E22))</x:f>
       </x:c>
       <x:c r="J22" s="1" t="str">
-        <x:f>IF(A22&gt;$B$4,"Future",IF(A22=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A22,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E22=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A22&gt;$B$4,"Future",IF(A22=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A22,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E22=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -851,7 +856,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E23" s="6" t="str">
-        <x:f>IF(A23&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A23,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A23&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A23,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F23" s="6" t="str">
         <x:f>IF(A23&gt;=$B$4,"",MAX(D23-E23,0))</x:f>
@@ -866,7 +871,7 @@
         <x:f>IF(A23&gt;$B$4,"",SUM($E$15:E23))</x:f>
       </x:c>
       <x:c r="J23" s="1" t="str">
-        <x:f>IF(A23&gt;$B$4,"Future",IF(A23=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A23,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E23=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A23&gt;$B$4,"Future",IF(A23=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A23,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E23=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -886,7 +891,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E24" s="6" t="str">
-        <x:f>IF(A24&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A24,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A24&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A24,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F24" s="6" t="str">
         <x:f>IF(A24&gt;=$B$4,"",MAX(D24-E24,0))</x:f>
@@ -901,7 +906,7 @@
         <x:f>IF(A24&gt;$B$4,"",SUM($E$15:E24))</x:f>
       </x:c>
       <x:c r="J24" s="1" t="str">
-        <x:f>IF(A24&gt;$B$4,"Future",IF(A24=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A24,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E24=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A24&gt;$B$4,"Future",IF(A24=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A24,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E24=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -921,7 +926,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E25" s="6" t="str">
-        <x:f>IF(A25&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A25,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A25&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A25,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F25" s="6" t="str">
         <x:f>IF(A25&gt;=$B$4,"",MAX(D25-E25,0))</x:f>
@@ -936,7 +941,7 @@
         <x:f>IF(A25&gt;$B$4,"",SUM($E$15:E25))</x:f>
       </x:c>
       <x:c r="J25" s="1" t="str">
-        <x:f>IF(A25&gt;$B$4,"Future",IF(A25=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A25,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E25=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A25&gt;$B$4,"Future",IF(A25=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A25,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E25=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -956,7 +961,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E26" s="6" t="str">
-        <x:f>IF(A26&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A26,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A26&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A26,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F26" s="6" t="str">
         <x:f>IF(A26&gt;=$B$4,"",MAX(D26-E26,0))</x:f>
@@ -971,7 +976,7 @@
         <x:f>IF(A26&gt;$B$4,"",SUM($E$15:E26))</x:f>
       </x:c>
       <x:c r="J26" s="1" t="str">
-        <x:f>IF(A26&gt;$B$4,"Future",IF(A26=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A26,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E26=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A26&gt;$B$4,"Future",IF(A26=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A26,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E26=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -991,7 +996,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E27" s="6" t="str">
-        <x:f>IF(A27&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A27,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A27&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A27,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F27" s="6" t="str">
         <x:f>IF(A27&gt;=$B$4,"",MAX(D27-E27,0))</x:f>
@@ -1006,7 +1011,7 @@
         <x:f>IF(A27&gt;$B$4,"",SUM($E$15:E27))</x:f>
       </x:c>
       <x:c r="J27" s="1" t="str">
-        <x:f>IF(A27&gt;$B$4,"Future",IF(A27=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A27,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E27=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A27&gt;$B$4,"Future",IF(A27=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A27,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E27=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1026,7 +1031,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E28" s="6" t="str">
-        <x:f>IF(A28&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A28,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A28&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A28,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F28" s="6" t="str">
         <x:f>IF(A28&gt;=$B$4,"",MAX(D28-E28,0))</x:f>
@@ -1041,7 +1046,7 @@
         <x:f>IF(A28&gt;$B$4,"",SUM($E$15:E28))</x:f>
       </x:c>
       <x:c r="J28" s="1" t="str">
-        <x:f>IF(A28&gt;$B$4,"Future",IF(A28=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A28,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E28=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A28&gt;$B$4,"Future",IF(A28=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A28,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E28=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1061,7 +1066,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E29" s="6" t="str">
-        <x:f>IF(A29&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A29,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A29&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A29,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F29" s="6" t="str">
         <x:f>IF(A29&gt;=$B$4,"",MAX(D29-E29,0))</x:f>
@@ -1076,7 +1081,7 @@
         <x:f>IF(A29&gt;$B$4,"",SUM($E$15:E29))</x:f>
       </x:c>
       <x:c r="J29" s="1" t="str">
-        <x:f>IF(A29&gt;$B$4,"Future",IF(A29=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A29,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E29=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A29&gt;$B$4,"Future",IF(A29=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A29,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E29=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1096,7 +1101,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E30" s="6" t="str">
-        <x:f>IF(A30&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A30,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A30&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A30,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F30" s="6" t="str">
         <x:f>IF(A30&gt;=$B$4,"",MAX(D30-E30,0))</x:f>
@@ -1111,7 +1116,7 @@
         <x:f>IF(A30&gt;$B$4,"",SUM($E$15:E30))</x:f>
       </x:c>
       <x:c r="J30" s="1" t="str">
-        <x:f>IF(A30&gt;$B$4,"Future",IF(A30=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A30,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E30=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A30&gt;$B$4,"Future",IF(A30=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A30,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E30=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1131,7 +1136,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E31" s="6" t="str">
-        <x:f>IF(A31&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A31,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A31&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A31,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F31" s="6" t="str">
         <x:f>IF(A31&gt;=$B$4,"",MAX(D31-E31,0))</x:f>
@@ -1146,7 +1151,7 @@
         <x:f>IF(A31&gt;$B$4,"",SUM($E$15:E31))</x:f>
       </x:c>
       <x:c r="J31" s="1" t="str">
-        <x:f>IF(A31&gt;$B$4,"Future",IF(A31=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A31,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E31=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A31&gt;$B$4,"Future",IF(A31=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A31,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E31=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1166,7 +1171,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E32" s="6" t="str">
-        <x:f>IF(A32&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A32,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A32&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A32,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F32" s="6" t="str">
         <x:f>IF(A32&gt;=$B$4,"",MAX(D32-E32,0))</x:f>
@@ -1181,7 +1186,7 @@
         <x:f>IF(A32&gt;$B$4,"",SUM($E$15:E32))</x:f>
       </x:c>
       <x:c r="J32" s="1" t="str">
-        <x:f>IF(A32&gt;$B$4,"Future",IF(A32=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A32,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E32=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A32&gt;$B$4,"Future",IF(A32=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A32,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E32=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1201,7 +1206,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E33" s="6" t="str">
-        <x:f>IF(A33&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A33,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A33&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A33,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F33" s="6" t="str">
         <x:f>IF(A33&gt;=$B$4,"",MAX(D33-E33,0))</x:f>
@@ -1216,7 +1221,7 @@
         <x:f>IF(A33&gt;$B$4,"",SUM($E$15:E33))</x:f>
       </x:c>
       <x:c r="J33" s="1" t="str">
-        <x:f>IF(A33&gt;$B$4,"Future",IF(A33=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A33,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E33=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A33&gt;$B$4,"Future",IF(A33=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A33,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E33=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1236,7 +1241,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E34" s="6" t="str">
-        <x:f>IF(A34&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A34,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A34&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A34,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F34" s="6" t="str">
         <x:f>IF(A34&gt;=$B$4,"",MAX(D34-E34,0))</x:f>
@@ -1251,7 +1256,7 @@
         <x:f>IF(A34&gt;$B$4,"",SUM($E$15:E34))</x:f>
       </x:c>
       <x:c r="J34" s="1" t="str">
-        <x:f>IF(A34&gt;$B$4,"Future",IF(A34=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A34,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E34=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A34&gt;$B$4,"Future",IF(A34=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A34,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E34=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1271,7 +1276,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E35" s="6" t="str">
-        <x:f>IF(A35&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A35,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A35&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A35,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F35" s="6" t="str">
         <x:f>IF(A35&gt;=$B$4,"",MAX(D35-E35,0))</x:f>
@@ -1286,7 +1291,7 @@
         <x:f>IF(A35&gt;$B$4,"",SUM($E$15:E35))</x:f>
       </x:c>
       <x:c r="J35" s="1" t="str">
-        <x:f>IF(A35&gt;$B$4,"Future",IF(A35=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A35,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E35=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A35&gt;$B$4,"Future",IF(A35=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A35,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E35=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1306,7 +1311,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E36" s="6" t="str">
-        <x:f>IF(A36&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A36,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A36&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A36,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F36" s="6" t="str">
         <x:f>IF(A36&gt;=$B$4,"",MAX(D36-E36,0))</x:f>
@@ -1321,7 +1326,7 @@
         <x:f>IF(A36&gt;$B$4,"",SUM($E$15:E36))</x:f>
       </x:c>
       <x:c r="J36" s="1" t="str">
-        <x:f>IF(A36&gt;$B$4,"Future",IF(A36=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A36,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E36=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A36&gt;$B$4,"Future",IF(A36=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A36,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E36=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1341,7 +1346,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E37" s="6" t="str">
-        <x:f>IF(A37&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A37,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A37&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A37,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F37" s="6" t="str">
         <x:f>IF(A37&gt;=$B$4,"",MAX(D37-E37,0))</x:f>
@@ -1356,7 +1361,7 @@
         <x:f>IF(A37&gt;$B$4,"",SUM($E$15:E37))</x:f>
       </x:c>
       <x:c r="J37" s="1" t="str">
-        <x:f>IF(A37&gt;$B$4,"Future",IF(A37=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A37,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E37=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A37&gt;$B$4,"Future",IF(A37=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A37,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E37=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1376,7 +1381,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E38" s="6" t="str">
-        <x:f>IF(A38&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A38,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A38&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A38,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F38" s="6" t="str">
         <x:f>IF(A38&gt;=$B$4,"",MAX(D38-E38,0))</x:f>
@@ -1391,7 +1396,7 @@
         <x:f>IF(A38&gt;$B$4,"",SUM($E$15:E38))</x:f>
       </x:c>
       <x:c r="J38" s="1" t="str">
-        <x:f>IF(A38&gt;$B$4,"Future",IF(A38=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A38,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E38=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A38&gt;$B$4,"Future",IF(A38=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A38,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E38=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1411,7 +1416,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E39" s="6" t="str">
-        <x:f>IF(A39&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A39,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A39&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A39,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F39" s="6" t="str">
         <x:f>IF(A39&gt;=$B$4,"",MAX(D39-E39,0))</x:f>
@@ -1426,7 +1431,7 @@
         <x:f>IF(A39&gt;$B$4,"",SUM($E$15:E39))</x:f>
       </x:c>
       <x:c r="J39" s="1" t="str">
-        <x:f>IF(A39&gt;$B$4,"Future",IF(A39=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A39,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E39=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A39&gt;$B$4,"Future",IF(A39=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A39,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E39=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1446,7 +1451,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E40" s="6" t="str">
-        <x:f>IF(A40&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A40,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A40&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A40,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F40" s="6" t="str">
         <x:f>IF(A40&gt;=$B$4,"",MAX(D40-E40,0))</x:f>
@@ -1461,7 +1466,7 @@
         <x:f>IF(A40&gt;$B$4,"",SUM($E$15:E40))</x:f>
       </x:c>
       <x:c r="J40" s="1" t="str">
-        <x:f>IF(A40&gt;$B$4,"Future",IF(A40=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A40,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E40=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A40&gt;$B$4,"Future",IF(A40=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A40,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E40=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1481,7 +1486,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E41" s="6" t="str">
-        <x:f>IF(A41&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A41,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A41&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A41,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F41" s="6" t="str">
         <x:f>IF(A41&gt;=$B$4,"",MAX(D41-E41,0))</x:f>
@@ -1496,7 +1501,7 @@
         <x:f>IF(A41&gt;$B$4,"",SUM($E$15:E41))</x:f>
       </x:c>
       <x:c r="J41" s="1" t="str">
-        <x:f>IF(A41&gt;$B$4,"Future",IF(A41=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A41,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E41=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A41&gt;$B$4,"Future",IF(A41=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A41,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E41=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1516,7 +1521,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E42" s="6" t="str">
-        <x:f>IF(A42&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A42,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A42&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A42,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F42" s="6" t="str">
         <x:f>IF(A42&gt;=$B$4,"",MAX(D42-E42,0))</x:f>
@@ -1531,7 +1536,7 @@
         <x:f>IF(A42&gt;$B$4,"",SUM($E$15:E42))</x:f>
       </x:c>
       <x:c r="J42" s="1" t="str">
-        <x:f>IF(A42&gt;$B$4,"Future",IF(A42=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A42,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E42=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A42&gt;$B$4,"Future",IF(A42=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A42,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E42=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1551,7 +1556,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E43" s="6" t="str">
-        <x:f>IF(A43&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A43,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A43&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A43,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F43" s="6" t="str">
         <x:f>IF(A43&gt;=$B$4,"",MAX(D43-E43,0))</x:f>
@@ -1566,7 +1571,7 @@
         <x:f>IF(A43&gt;$B$4,"",SUM($E$15:E43))</x:f>
       </x:c>
       <x:c r="J43" s="1" t="str">
-        <x:f>IF(A43&gt;$B$4,"Future",IF(A43=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A43,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E43=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A43&gt;$B$4,"Future",IF(A43=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A43,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E43=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1586,7 +1591,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E44" s="6" t="str">
-        <x:f>IF(A44&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A44,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A44&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A44,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F44" s="6" t="str">
         <x:f>IF(A44&gt;=$B$4,"",MAX(D44-E44,0))</x:f>
@@ -1601,7 +1606,7 @@
         <x:f>IF(A44&gt;$B$4,"",SUM($E$15:E44))</x:f>
       </x:c>
       <x:c r="J44" s="1" t="str">
-        <x:f>IF(A44&gt;$B$4,"Future",IF(A44=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A44,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E44=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A44&gt;$B$4,"Future",IF(A44=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A44,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E44=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1621,7 +1626,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E45" s="6" t="str">
-        <x:f>IF(A45&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A45,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A45&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A45,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F45" s="6" t="str">
         <x:f>IF(A45&gt;=$B$4,"",MAX(D45-E45,0))</x:f>
@@ -1636,7 +1641,7 @@
         <x:f>IF(A45&gt;$B$4,"",SUM($E$15:E45))</x:f>
       </x:c>
       <x:c r="J45" s="1" t="str">
-        <x:f>IF(A45&gt;$B$4,"Future",IF(A45=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A45,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E45=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A45&gt;$B$4,"Future",IF(A45=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A45,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E45=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1656,7 +1661,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E46" s="6" t="str">
-        <x:f>IF(A46&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A46,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A46&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A46,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F46" s="6" t="str">
         <x:f>IF(A46&gt;=$B$4,"",MAX(D46-E46,0))</x:f>
@@ -1671,7 +1676,7 @@
         <x:f>IF(A46&gt;$B$4,"",SUM($E$15:E46))</x:f>
       </x:c>
       <x:c r="J46" s="1" t="str">
-        <x:f>IF(A46&gt;$B$4,"Future",IF(A46=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A46,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E46=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A46&gt;$B$4,"Future",IF(A46=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A46,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E46=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1691,7 +1696,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E47" s="6" t="str">
-        <x:f>IF(A47&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A47,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A47&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A47,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F47" s="6" t="str">
         <x:f>IF(A47&gt;=$B$4,"",MAX(D47-E47,0))</x:f>
@@ -1706,7 +1711,7 @@
         <x:f>IF(A47&gt;$B$4,"",SUM($E$15:E47))</x:f>
       </x:c>
       <x:c r="J47" s="1" t="str">
-        <x:f>IF(A47&gt;$B$4,"Future",IF(A47=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A47,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E47=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A47&gt;$B$4,"Future",IF(A47=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A47,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E47=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1726,7 +1731,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E48" s="6" t="str">
-        <x:f>IF(A48&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A48,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A48&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A48,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F48" s="6" t="str">
         <x:f>IF(A48&gt;=$B$4,"",MAX(D48-E48,0))</x:f>
@@ -1741,7 +1746,7 @@
         <x:f>IF(A48&gt;$B$4,"",SUM($E$15:E48))</x:f>
       </x:c>
       <x:c r="J48" s="1" t="str">
-        <x:f>IF(A48&gt;$B$4,"Future",IF(A48=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A48,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E48=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A48&gt;$B$4,"Future",IF(A48=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A48,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E48=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1761,7 +1766,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E49" s="6" t="str">
-        <x:f>IF(A49&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A49,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A49&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A49,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F49" s="6" t="str">
         <x:f>IF(A49&gt;=$B$4,"",MAX(D49-E49,0))</x:f>
@@ -1776,7 +1781,7 @@
         <x:f>IF(A49&gt;$B$4,"",SUM($E$15:E49))</x:f>
       </x:c>
       <x:c r="J49" s="1" t="str">
-        <x:f>IF(A49&gt;$B$4,"Future",IF(A49=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A49,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E49=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A49&gt;$B$4,"Future",IF(A49=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A49,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E49=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1796,7 +1801,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E50" s="6" t="str">
-        <x:f>IF(A50&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A50,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A50&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A50,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F50" s="6" t="str">
         <x:f>IF(A50&gt;=$B$4,"",MAX(D50-E50,0))</x:f>
@@ -1811,7 +1816,7 @@
         <x:f>IF(A50&gt;$B$4,"",SUM($E$15:E50))</x:f>
       </x:c>
       <x:c r="J50" s="1" t="str">
-        <x:f>IF(A50&gt;$B$4,"Future",IF(A50=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A50,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E50=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A50&gt;$B$4,"Future",IF(A50=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A50,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E50=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1831,7 +1836,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E51" s="6" t="str">
-        <x:f>IF(A51&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A51,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A51&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A51,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F51" s="6" t="str">
         <x:f>IF(A51&gt;=$B$4,"",MAX(D51-E51,0))</x:f>
@@ -1846,7 +1851,7 @@
         <x:f>IF(A51&gt;$B$4,"",SUM($E$15:E51))</x:f>
       </x:c>
       <x:c r="J51" s="1" t="str">
-        <x:f>IF(A51&gt;$B$4,"Future",IF(A51=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A51,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E51=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A51&gt;$B$4,"Future",IF(A51=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A51,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E51=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1866,7 +1871,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E52" s="6" t="str">
-        <x:f>IF(A52&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A52,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A52&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A52,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F52" s="6" t="str">
         <x:f>IF(A52&gt;=$B$4,"",MAX(D52-E52,0))</x:f>
@@ -1881,7 +1886,7 @@
         <x:f>IF(A52&gt;$B$4,"",SUM($E$15:E52))</x:f>
       </x:c>
       <x:c r="J52" s="1" t="str">
-        <x:f>IF(A52&gt;$B$4,"Future",IF(A52=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A52,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E52=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A52&gt;$B$4,"Future",IF(A52=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A52,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E52=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1901,7 +1906,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E53" s="6" t="str">
-        <x:f>IF(A53&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A53,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A53&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A53,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F53" s="6" t="str">
         <x:f>IF(A53&gt;=$B$4,"",MAX(D53-E53,0))</x:f>
@@ -1916,7 +1921,7 @@
         <x:f>IF(A53&gt;$B$4,"",SUM($E$15:E53))</x:f>
       </x:c>
       <x:c r="J53" s="1" t="str">
-        <x:f>IF(A53&gt;$B$4,"Future",IF(A53=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A53,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E53=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A53&gt;$B$4,"Future",IF(A53=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A53,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E53=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1936,7 +1941,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E54" s="6" t="str">
-        <x:f>IF(A54&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A54,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A54&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A54,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F54" s="6" t="str">
         <x:f>IF(A54&gt;=$B$4,"",MAX(D54-E54,0))</x:f>
@@ -1951,7 +1956,7 @@
         <x:f>IF(A54&gt;$B$4,"",SUM($E$15:E54))</x:f>
       </x:c>
       <x:c r="J54" s="1" t="str">
-        <x:f>IF(A54&gt;$B$4,"Future",IF(A54=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A54,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E54=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A54&gt;$B$4,"Future",IF(A54=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A54,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E54=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1971,7 +1976,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E55" s="6" t="str">
-        <x:f>IF(A55&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A55,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A55&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A55,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F55" s="6" t="str">
         <x:f>IF(A55&gt;=$B$4,"",MAX(D55-E55,0))</x:f>
@@ -1986,7 +1991,7 @@
         <x:f>IF(A55&gt;$B$4,"",SUM($E$15:E55))</x:f>
       </x:c>
       <x:c r="J55" s="1" t="str">
-        <x:f>IF(A55&gt;$B$4,"Future",IF(A55=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A55,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E55=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A55&gt;$B$4,"Future",IF(A55=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A55,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E55=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2006,7 +2011,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E56" s="6" t="str">
-        <x:f>IF(A56&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A56,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A56&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A56,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F56" s="6" t="str">
         <x:f>IF(A56&gt;=$B$4,"",MAX(D56-E56,0))</x:f>
@@ -2021,7 +2026,7 @@
         <x:f>IF(A56&gt;$B$4,"",SUM($E$15:E56))</x:f>
       </x:c>
       <x:c r="J56" s="1" t="str">
-        <x:f>IF(A56&gt;$B$4,"Future",IF(A56=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A56,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E56=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A56&gt;$B$4,"Future",IF(A56=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A56,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E56=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2041,7 +2046,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E57" s="6" t="str">
-        <x:f>IF(A57&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A57,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A57&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A57,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F57" s="6" t="str">
         <x:f>IF(A57&gt;=$B$4,"",MAX(D57-E57,0))</x:f>
@@ -2056,7 +2061,7 @@
         <x:f>IF(A57&gt;$B$4,"",SUM($E$15:E57))</x:f>
       </x:c>
       <x:c r="J57" s="1" t="str">
-        <x:f>IF(A57&gt;$B$4,"Future",IF(A57=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A57,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E57=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A57&gt;$B$4,"Future",IF(A57=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A57,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E57=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2076,7 +2081,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E58" s="6" t="str">
-        <x:f>IF(A58&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A58,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A58&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A58,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F58" s="6" t="str">
         <x:f>IF(A58&gt;=$B$4,"",MAX(D58-E58,0))</x:f>
@@ -2091,7 +2096,7 @@
         <x:f>IF(A58&gt;$B$4,"",SUM($E$15:E58))</x:f>
       </x:c>
       <x:c r="J58" s="1" t="str">
-        <x:f>IF(A58&gt;$B$4,"Future",IF(A58=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A58,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E58=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A58&gt;$B$4,"Future",IF(A58=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A58,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E58=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2111,7 +2116,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E59" s="6" t="str">
-        <x:f>IF(A59&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A59,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A59&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A59,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F59" s="6" t="str">
         <x:f>IF(A59&gt;=$B$4,"",MAX(D59-E59,0))</x:f>
@@ -2126,7 +2131,7 @@
         <x:f>IF(A59&gt;$B$4,"",SUM($E$15:E59))</x:f>
       </x:c>
       <x:c r="J59" s="1" t="str">
-        <x:f>IF(A59&gt;$B$4,"Future",IF(A59=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A59,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E59=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A59&gt;$B$4,"Future",IF(A59=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A59,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E59=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2146,7 +2151,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E60" s="6" t="str">
-        <x:f>IF(A60&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A60,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A60&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A60,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F60" s="6" t="str">
         <x:f>IF(A60&gt;=$B$4,"",MAX(D60-E60,0))</x:f>
@@ -2161,7 +2166,7 @@
         <x:f>IF(A60&gt;$B$4,"",SUM($E$15:E60))</x:f>
       </x:c>
       <x:c r="J60" s="1" t="str">
-        <x:f>IF(A60&gt;$B$4,"Future",IF(A60=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A60,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E60=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A60&gt;$B$4,"Future",IF(A60=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A60,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E60=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2181,7 +2186,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E61" s="6" t="str">
-        <x:f>IF(A61&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A61,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A61&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A61,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F61" s="6" t="str">
         <x:f>IF(A61&gt;=$B$4,"",MAX(D61-E61,0))</x:f>
@@ -2196,7 +2201,7 @@
         <x:f>IF(A61&gt;$B$4,"",SUM($E$15:E61))</x:f>
       </x:c>
       <x:c r="J61" s="1" t="str">
-        <x:f>IF(A61&gt;$B$4,"Future",IF(A61=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A61,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E61=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A61&gt;$B$4,"Future",IF(A61=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A61,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E61=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2216,7 +2221,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E62" s="6" t="str">
-        <x:f>IF(A62&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A62,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A62&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A62,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F62" s="6" t="str">
         <x:f>IF(A62&gt;=$B$4,"",MAX(D62-E62,0))</x:f>
@@ -2231,7 +2236,7 @@
         <x:f>IF(A62&gt;$B$4,"",SUM($E$15:E62))</x:f>
       </x:c>
       <x:c r="J62" s="1" t="str">
-        <x:f>IF(A62&gt;$B$4,"Future",IF(A62=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A62,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E62=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A62&gt;$B$4,"Future",IF(A62=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A62,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E62=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2251,7 +2256,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E63" s="6" t="str">
-        <x:f>IF(A63&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A63,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A63&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A63,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F63" s="6" t="str">
         <x:f>IF(A63&gt;=$B$4,"",MAX(D63-E63,0))</x:f>
@@ -2266,7 +2271,7 @@
         <x:f>IF(A63&gt;$B$4,"",SUM($E$15:E63))</x:f>
       </x:c>
       <x:c r="J63" s="1" t="str">
-        <x:f>IF(A63&gt;$B$4,"Future",IF(A63=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A63,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E63=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A63&gt;$B$4,"Future",IF(A63=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A63,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E63=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2286,7 +2291,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E64" s="6" t="str">
-        <x:f>IF(A64&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A64,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A64&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A64,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F64" s="6" t="str">
         <x:f>IF(A64&gt;=$B$4,"",MAX(D64-E64,0))</x:f>
@@ -2301,7 +2306,7 @@
         <x:f>IF(A64&gt;$B$4,"",SUM($E$15:E64))</x:f>
       </x:c>
       <x:c r="J64" s="1" t="str">
-        <x:f>IF(A64&gt;$B$4,"Future",IF(A64=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A64,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E64=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A64&gt;$B$4,"Future",IF(A64=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A64,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E64=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2321,7 +2326,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E65" s="6" t="str">
-        <x:f>IF(A65&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A65,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A65&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A65,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F65" s="6" t="str">
         <x:f>IF(A65&gt;=$B$4,"",MAX(D65-E65,0))</x:f>
@@ -2336,7 +2341,7 @@
         <x:f>IF(A65&gt;$B$4,"",SUM($E$15:E65))</x:f>
       </x:c>
       <x:c r="J65" s="1" t="str">
-        <x:f>IF(A65&gt;$B$4,"Future",IF(A65=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A65,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E65=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A65&gt;$B$4,"Future",IF(A65=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A65,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E65=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2356,7 +2361,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E66" s="6" t="str">
-        <x:f>IF(A66&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A66,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A66&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A66,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F66" s="6" t="str">
         <x:f>IF(A66&gt;=$B$4,"",MAX(D66-E66,0))</x:f>
@@ -2371,7 +2376,7 @@
         <x:f>IF(A66&gt;$B$4,"",SUM($E$15:E66))</x:f>
       </x:c>
       <x:c r="J66" s="1" t="str">
-        <x:f>IF(A66&gt;$B$4,"Future",IF(A66=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A66,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E66=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A66&gt;$B$4,"Future",IF(A66=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A66,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E66=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2391,7 +2396,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E67" s="6" t="str">
-        <x:f>IF(A67&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A67,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A67&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A67,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F67" s="6" t="str">
         <x:f>IF(A67&gt;=$B$4,"",MAX(D67-E67,0))</x:f>
@@ -2406,7 +2411,7 @@
         <x:f>IF(A67&gt;$B$4,"",SUM($E$15:E67))</x:f>
       </x:c>
       <x:c r="J67" s="1" t="str">
-        <x:f>IF(A67&gt;$B$4,"Future",IF(A67=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A67,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E67=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A67&gt;$B$4,"Future",IF(A67=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A67,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E67=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2426,7 +2431,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E68" s="6" t="str">
-        <x:f>IF(A68&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A68,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A68&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A68,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F68" s="6" t="str">
         <x:f>IF(A68&gt;=$B$4,"",MAX(D68-E68,0))</x:f>
@@ -2441,7 +2446,7 @@
         <x:f>IF(A68&gt;$B$4,"",SUM($E$15:E68))</x:f>
       </x:c>
       <x:c r="J68" s="1" t="str">
-        <x:f>IF(A68&gt;$B$4,"Future",IF(A68=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A68,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E68=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A68&gt;$B$4,"Future",IF(A68=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A68,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E68=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2461,7 +2466,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E69" s="6" t="str">
-        <x:f>IF(A69&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A69,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A69&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A69,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F69" s="6" t="str">
         <x:f>IF(A69&gt;=$B$4,"",MAX(D69-E69,0))</x:f>
@@ -2476,7 +2481,7 @@
         <x:f>IF(A69&gt;$B$4,"",SUM($E$15:E69))</x:f>
       </x:c>
       <x:c r="J69" s="1" t="str">
-        <x:f>IF(A69&gt;$B$4,"Future",IF(A69=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A69,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E69=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A69&gt;$B$4,"Future",IF(A69=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A69,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E69=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2496,7 +2501,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E70" s="6" t="str">
-        <x:f>IF(A70&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A70,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A70&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A70,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F70" s="6" t="str">
         <x:f>IF(A70&gt;=$B$4,"",MAX(D70-E70,0))</x:f>
@@ -2511,7 +2516,7 @@
         <x:f>IF(A70&gt;$B$4,"",SUM($E$15:E70))</x:f>
       </x:c>
       <x:c r="J70" s="1" t="str">
-        <x:f>IF(A70&gt;$B$4,"Future",IF(A70=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A70,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E70=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A70&gt;$B$4,"Future",IF(A70=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A70,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E70=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2531,7 +2536,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E71" s="6" t="str">
-        <x:f>IF(A71&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A71,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A71&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A71,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F71" s="6" t="str">
         <x:f>IF(A71&gt;=$B$4,"",MAX(D71-E71,0))</x:f>
@@ -2546,7 +2551,7 @@
         <x:f>IF(A71&gt;$B$4,"",SUM($E$15:E71))</x:f>
       </x:c>
       <x:c r="J71" s="1" t="str">
-        <x:f>IF(A71&gt;$B$4,"Future",IF(A71=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A71,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E71=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A71&gt;$B$4,"Future",IF(A71=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A71,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E71=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2566,7 +2571,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E72" s="6" t="str">
-        <x:f>IF(A72&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A72,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A72&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A72,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F72" s="6" t="str">
         <x:f>IF(A72&gt;=$B$4,"",MAX(D72-E72,0))</x:f>
@@ -2581,7 +2586,7 @@
         <x:f>IF(A72&gt;$B$4,"",SUM($E$15:E72))</x:f>
       </x:c>
       <x:c r="J72" s="1" t="str">
-        <x:f>IF(A72&gt;$B$4,"Future",IF(A72=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A72,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E72=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A72&gt;$B$4,"Future",IF(A72=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A72,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E72=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2601,7 +2606,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E73" s="6" t="str">
-        <x:f>IF(A73&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A73,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A73&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A73,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F73" s="6" t="str">
         <x:f>IF(A73&gt;=$B$4,"",MAX(D73-E73,0))</x:f>
@@ -2616,7 +2621,7 @@
         <x:f>IF(A73&gt;$B$4,"",SUM($E$15:E73))</x:f>
       </x:c>
       <x:c r="J73" s="1" t="str">
-        <x:f>IF(A73&gt;$B$4,"Future",IF(A73=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A73,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E73=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A73&gt;$B$4,"Future",IF(A73=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A73,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E73=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2636,7 +2641,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E74" s="6" t="str">
-        <x:f>IF(A74&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A74,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A74&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A74,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F74" s="6" t="str">
         <x:f>IF(A74&gt;=$B$4,"",MAX(D74-E74,0))</x:f>
@@ -2651,7 +2656,7 @@
         <x:f>IF(A74&gt;$B$4,"",SUM($E$15:E74))</x:f>
       </x:c>
       <x:c r="J74" s="1" t="str">
-        <x:f>IF(A74&gt;$B$4,"Future",IF(A74=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A74,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E74=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A74&gt;$B$4,"Future",IF(A74=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A74,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E74=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2671,7 +2676,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E75" s="6" t="str">
-        <x:f>IF(A75&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A75,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A75&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A75,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F75" s="6" t="str">
         <x:f>IF(A75&gt;=$B$4,"",MAX(D75-E75,0))</x:f>
@@ -2686,7 +2691,7 @@
         <x:f>IF(A75&gt;$B$4,"",SUM($E$15:E75))</x:f>
       </x:c>
       <x:c r="J75" s="1" t="str">
-        <x:f>IF(A75&gt;$B$4,"Future",IF(A75=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A75,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E75=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A75&gt;$B$4,"Future",IF(A75=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A75,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E75=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2706,7 +2711,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E76" s="6" t="str">
-        <x:f>IF(A76&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A76,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A76&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A76,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F76" s="6" t="str">
         <x:f>IF(A76&gt;=$B$4,"",MAX(D76-E76,0))</x:f>
@@ -2721,7 +2726,7 @@
         <x:f>IF(A76&gt;$B$4,"",SUM($E$15:E76))</x:f>
       </x:c>
       <x:c r="J76" s="1" t="str">
-        <x:f>IF(A76&gt;$B$4,"Future",IF(A76=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A76,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E76=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A76&gt;$B$4,"Future",IF(A76=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A76,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E76=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2741,7 +2746,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E77" s="6" t="str">
-        <x:f>IF(A77&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A77,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A77&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A77,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F77" s="6" t="str">
         <x:f>IF(A77&gt;=$B$4,"",MAX(D77-E77,0))</x:f>
@@ -2756,7 +2761,7 @@
         <x:f>IF(A77&gt;$B$4,"",SUM($E$15:E77))</x:f>
       </x:c>
       <x:c r="J77" s="1" t="str">
-        <x:f>IF(A77&gt;$B$4,"Future",IF(A77=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A77,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E77=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A77&gt;$B$4,"Future",IF(A77=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A77,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E77=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2776,7 +2781,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E78" s="6" t="str">
-        <x:f>IF(A78&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A78,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A78&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A78,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F78" s="6" t="str">
         <x:f>IF(A78&gt;=$B$4,"",MAX(D78-E78,0))</x:f>
@@ -2791,7 +2796,7 @@
         <x:f>IF(A78&gt;$B$4,"",SUM($E$15:E78))</x:f>
       </x:c>
       <x:c r="J78" s="1" t="str">
-        <x:f>IF(A78&gt;$B$4,"Future",IF(A78=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A78,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E78=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A78&gt;$B$4,"Future",IF(A78=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A78,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E78=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2811,7 +2816,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E79" s="6" t="str">
-        <x:f>IF(A79&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A79,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A79&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A79,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F79" s="6" t="str">
         <x:f>IF(A79&gt;=$B$4,"",MAX(D79-E79,0))</x:f>
@@ -2826,7 +2831,7 @@
         <x:f>IF(A79&gt;$B$4,"",SUM($E$15:E79))</x:f>
       </x:c>
       <x:c r="J79" s="1" t="str">
-        <x:f>IF(A79&gt;$B$4,"Future",IF(A79=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A79,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E79=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A79&gt;$B$4,"Future",IF(A79=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A79,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E79=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2846,7 +2851,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E80" s="6" t="str">
-        <x:f>IF(A80&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A80,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A80&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A80,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F80" s="6" t="str">
         <x:f>IF(A80&gt;=$B$4,"",MAX(D80-E80,0))</x:f>
@@ -2861,7 +2866,7 @@
         <x:f>IF(A80&gt;$B$4,"",SUM($E$15:E80))</x:f>
       </x:c>
       <x:c r="J80" s="1" t="str">
-        <x:f>IF(A80&gt;$B$4,"Future",IF(A80=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A80,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E80=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A80&gt;$B$4,"Future",IF(A80=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A80,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E80=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2881,7 +2886,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E81" s="6" t="str">
-        <x:f>IF(A81&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A81,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A81&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A81,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F81" s="6" t="str">
         <x:f>IF(A81&gt;=$B$4,"",MAX(D81-E81,0))</x:f>
@@ -2896,7 +2901,7 @@
         <x:f>IF(A81&gt;$B$4,"",SUM($E$15:E81))</x:f>
       </x:c>
       <x:c r="J81" s="1" t="str">
-        <x:f>IF(A81&gt;$B$4,"Future",IF(A81=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A81,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E81=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A81&gt;$B$4,"Future",IF(A81=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A81,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E81=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2916,7 +2921,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E82" s="6" t="str">
-        <x:f>IF(A82&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A82,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A82&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A82,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F82" s="6" t="str">
         <x:f>IF(A82&gt;=$B$4,"",MAX(D82-E82,0))</x:f>
@@ -2931,7 +2936,7 @@
         <x:f>IF(A82&gt;$B$4,"",SUM($E$15:E82))</x:f>
       </x:c>
       <x:c r="J82" s="1" t="str">
-        <x:f>IF(A82&gt;$B$4,"Future",IF(A82=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A82,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E82=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A82&gt;$B$4,"Future",IF(A82=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A82,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E82=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2951,7 +2956,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E83" s="6" t="str">
-        <x:f>IF(A83&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A83,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A83&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A83,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F83" s="6" t="str">
         <x:f>IF(A83&gt;=$B$4,"",MAX(D83-E83,0))</x:f>
@@ -2966,7 +2971,7 @@
         <x:f>IF(A83&gt;$B$4,"",SUM($E$15:E83))</x:f>
       </x:c>
       <x:c r="J83" s="1" t="str">
-        <x:f>IF(A83&gt;$B$4,"Future",IF(A83=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A83,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E83=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A83&gt;$B$4,"Future",IF(A83=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A83,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E83=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2986,7 +2991,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E84" s="6" t="str">
-        <x:f>IF(A84&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A84,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A84&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A84,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F84" s="6" t="str">
         <x:f>IF(A84&gt;=$B$4,"",MAX(D84-E84,0))</x:f>
@@ -3001,7 +3006,7 @@
         <x:f>IF(A84&gt;$B$4,"",SUM($E$15:E84))</x:f>
       </x:c>
       <x:c r="J84" s="1" t="str">
-        <x:f>IF(A84&gt;$B$4,"Future",IF(A84=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A84,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E84=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A84&gt;$B$4,"Future",IF(A84=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A84,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E84=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3021,7 +3026,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E85" s="6" t="str">
-        <x:f>IF(A85&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A85,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A85&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A85,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F85" s="6" t="str">
         <x:f>IF(A85&gt;=$B$4,"",MAX(D85-E85,0))</x:f>
@@ -3036,7 +3041,7 @@
         <x:f>IF(A85&gt;$B$4,"",SUM($E$15:E85))</x:f>
       </x:c>
       <x:c r="J85" s="1" t="str">
-        <x:f>IF(A85&gt;$B$4,"Future",IF(A85=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A85,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E85=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A85&gt;$B$4,"Future",IF(A85=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A85,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E85=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3056,7 +3061,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E86" s="6" t="str">
-        <x:f>IF(A86&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A86,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A86&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A86,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F86" s="6" t="str">
         <x:f>IF(A86&gt;=$B$4,"",MAX(D86-E86,0))</x:f>
@@ -3071,7 +3076,7 @@
         <x:f>IF(A86&gt;$B$4,"",SUM($E$15:E86))</x:f>
       </x:c>
       <x:c r="J86" s="1" t="str">
-        <x:f>IF(A86&gt;$B$4,"Future",IF(A86=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A86,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E86=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A86&gt;$B$4,"Future",IF(A86=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A86,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E86=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3091,7 +3096,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E87" s="6" t="str">
-        <x:f>IF(A87&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A87,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A87&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A87,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F87" s="6" t="str">
         <x:f>IF(A87&gt;=$B$4,"",MAX(D87-E87,0))</x:f>
@@ -3106,7 +3111,7 @@
         <x:f>IF(A87&gt;$B$4,"",SUM($E$15:E87))</x:f>
       </x:c>
       <x:c r="J87" s="1" t="str">
-        <x:f>IF(A87&gt;$B$4,"Future",IF(A87=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A87,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E87=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A87&gt;$B$4,"Future",IF(A87=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A87,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E87=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3126,7 +3131,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E88" s="6" t="str">
-        <x:f>IF(A88&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A88,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A88&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A88,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F88" s="6" t="str">
         <x:f>IF(A88&gt;=$B$4,"",MAX(D88-E88,0))</x:f>
@@ -3141,7 +3146,7 @@
         <x:f>IF(A88&gt;$B$4,"",SUM($E$15:E88))</x:f>
       </x:c>
       <x:c r="J88" s="1" t="str">
-        <x:f>IF(A88&gt;$B$4,"Future",IF(A88=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A88,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E88=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A88&gt;$B$4,"Future",IF(A88=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A88,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E88=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3161,7 +3166,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E89" s="6" t="str">
-        <x:f>IF(A89&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A89,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A89&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A89,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F89" s="6" t="str">
         <x:f>IF(A89&gt;=$B$4,"",MAX(D89-E89,0))</x:f>
@@ -3176,7 +3181,7 @@
         <x:f>IF(A89&gt;$B$4,"",SUM($E$15:E89))</x:f>
       </x:c>
       <x:c r="J89" s="1" t="str">
-        <x:f>IF(A89&gt;$B$4,"Future",IF(A89=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A89,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E89=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A89&gt;$B$4,"Future",IF(A89=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A89,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E89=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3196,7 +3201,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E90" s="6" t="str">
-        <x:f>IF(A90&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A90,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A90&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A90,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F90" s="6" t="str">
         <x:f>IF(A90&gt;=$B$4,"",MAX(D90-E90,0))</x:f>
@@ -3211,7 +3216,7 @@
         <x:f>IF(A90&gt;$B$4,"",SUM($E$15:E90))</x:f>
       </x:c>
       <x:c r="J90" s="1" t="str">
-        <x:f>IF(A90&gt;$B$4,"Future",IF(A90=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A90,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E90=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A90&gt;$B$4,"Future",IF(A90=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A90,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E90=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3231,7 +3236,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E91" s="6" t="str">
-        <x:f>IF(A91&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A91,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A91&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A91,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F91" s="6" t="str">
         <x:f>IF(A91&gt;=$B$4,"",MAX(D91-E91,0))</x:f>
@@ -3246,7 +3251,7 @@
         <x:f>IF(A91&gt;$B$4,"",SUM($E$15:E91))</x:f>
       </x:c>
       <x:c r="J91" s="1" t="str">
-        <x:f>IF(A91&gt;$B$4,"Future",IF(A91=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A91,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E91=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A91&gt;$B$4,"Future",IF(A91=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A91,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E91=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3266,7 +3271,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E92" s="6" t="str">
-        <x:f>IF(A92&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A92,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A92&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A92,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F92" s="6" t="str">
         <x:f>IF(A92&gt;=$B$4,"",MAX(D92-E92,0))</x:f>
@@ -3281,7 +3286,7 @@
         <x:f>IF(A92&gt;$B$4,"",SUM($E$15:E92))</x:f>
       </x:c>
       <x:c r="J92" s="1" t="str">
-        <x:f>IF(A92&gt;$B$4,"Future",IF(A92=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A92,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E92=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A92&gt;$B$4,"Future",IF(A92=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A92,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E92=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3301,7 +3306,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E93" s="6" t="str">
-        <x:f>IF(A93&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A93,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A93&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A93,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F93" s="6" t="str">
         <x:f>IF(A93&gt;=$B$4,"",MAX(D93-E93,0))</x:f>
@@ -3316,7 +3321,7 @@
         <x:f>IF(A93&gt;$B$4,"",SUM($E$15:E93))</x:f>
       </x:c>
       <x:c r="J93" s="1" t="str">
-        <x:f>IF(A93&gt;$B$4,"Future",IF(A93=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A93,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E93=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A93&gt;$B$4,"Future",IF(A93=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A93,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E93=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3336,7 +3341,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E94" s="6" t="str">
-        <x:f>IF(A94&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A94,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A94&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A94,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F94" s="6" t="str">
         <x:f>IF(A94&gt;=$B$4,"",MAX(D94-E94,0))</x:f>
@@ -3351,7 +3356,7 @@
         <x:f>IF(A94&gt;$B$4,"",SUM($E$15:E94))</x:f>
       </x:c>
       <x:c r="J94" s="1" t="str">
-        <x:f>IF(A94&gt;$B$4,"Future",IF(A94=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A94,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E94=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A94&gt;$B$4,"Future",IF(A94=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A94,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E94=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3371,7 +3376,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E95" s="6" t="str">
-        <x:f>IF(A95&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A95,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A95&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A95,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F95" s="6" t="str">
         <x:f>IF(A95&gt;=$B$4,"",MAX(D95-E95,0))</x:f>
@@ -3386,7 +3391,7 @@
         <x:f>IF(A95&gt;$B$4,"",SUM($E$15:E95))</x:f>
       </x:c>
       <x:c r="J95" s="1" t="str">
-        <x:f>IF(A95&gt;$B$4,"Future",IF(A95=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A95,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E95=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A95&gt;$B$4,"Future",IF(A95=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A95,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E95=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3406,7 +3411,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E96" s="6" t="str">
-        <x:f>IF(A96&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A96,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A96&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A96,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F96" s="6" t="str">
         <x:f>IF(A96&gt;=$B$4,"",MAX(D96-E96,0))</x:f>
@@ -3421,7 +3426,7 @@
         <x:f>IF(A96&gt;$B$4,"",SUM($E$15:E96))</x:f>
       </x:c>
       <x:c r="J96" s="1" t="str">
-        <x:f>IF(A96&gt;$B$4,"Future",IF(A96=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A96,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E96=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A96&gt;$B$4,"Future",IF(A96=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A96,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E96=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3441,7 +3446,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E97" s="6" t="str">
-        <x:f>IF(A97&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A97,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A97&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A97,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F97" s="6" t="str">
         <x:f>IF(A97&gt;=$B$4,"",MAX(D97-E97,0))</x:f>
@@ -3456,7 +3461,7 @@
         <x:f>IF(A97&gt;$B$4,"",SUM($E$15:E97))</x:f>
       </x:c>
       <x:c r="J97" s="1" t="str">
-        <x:f>IF(A97&gt;$B$4,"Future",IF(A97=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A97,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E97=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A97&gt;$B$4,"Future",IF(A97=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A97,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E97=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3476,7 +3481,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E98" s="6" t="str">
-        <x:f>IF(A98&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A98,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A98&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A98,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F98" s="6" t="str">
         <x:f>IF(A98&gt;=$B$4,"",MAX(D98-E98,0))</x:f>
@@ -3491,7 +3496,7 @@
         <x:f>IF(A98&gt;$B$4,"",SUM($E$15:E98))</x:f>
       </x:c>
       <x:c r="J98" s="1" t="str">
-        <x:f>IF(A98&gt;$B$4,"Future",IF(A98=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A98,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E98=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A98&gt;$B$4,"Future",IF(A98=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A98,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E98=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3511,7 +3516,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E99" s="6" t="str">
-        <x:f>IF(A99&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A99,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A99&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A99,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F99" s="6" t="str">
         <x:f>IF(A99&gt;=$B$4,"",MAX(D99-E99,0))</x:f>
@@ -3526,7 +3531,7 @@
         <x:f>IF(A99&gt;$B$4,"",SUM($E$15:E99))</x:f>
       </x:c>
       <x:c r="J99" s="1" t="str">
-        <x:f>IF(A99&gt;$B$4,"Future",IF(A99=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A99,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E99=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A99&gt;$B$4,"Future",IF(A99=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A99,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E99=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3546,7 +3551,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E100" s="6" t="str">
-        <x:f>IF(A100&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A100,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A100&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A100,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F100" s="6" t="str">
         <x:f>IF(A100&gt;=$B$4,"",MAX(D100-E100,0))</x:f>
@@ -3561,7 +3566,7 @@
         <x:f>IF(A100&gt;$B$4,"",SUM($E$15:E100))</x:f>
       </x:c>
       <x:c r="J100" s="1" t="str">
-        <x:f>IF(A100&gt;$B$4,"Future",IF(A100=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A100,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E100=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A100&gt;$B$4,"Future",IF(A100=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A100,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E100=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3581,7 +3586,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E101" s="6" t="str">
-        <x:f>IF(A101&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A101,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A101&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A101,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F101" s="6" t="str">
         <x:f>IF(A101&gt;=$B$4,"",MAX(D101-E101,0))</x:f>
@@ -3596,7 +3601,7 @@
         <x:f>IF(A101&gt;$B$4,"",SUM($E$15:E101))</x:f>
       </x:c>
       <x:c r="J101" s="1" t="str">
-        <x:f>IF(A101&gt;$B$4,"Future",IF(A101=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A101,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E101=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A101&gt;$B$4,"Future",IF(A101=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A101,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E101=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3616,7 +3621,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E102" s="6" t="str">
-        <x:f>IF(A102&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A102,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A102&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A102,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F102" s="6" t="str">
         <x:f>IF(A102&gt;=$B$4,"",MAX(D102-E102,0))</x:f>
@@ -3631,7 +3636,7 @@
         <x:f>IF(A102&gt;$B$4,"",SUM($E$15:E102))</x:f>
       </x:c>
       <x:c r="J102" s="1" t="str">
-        <x:f>IF(A102&gt;$B$4,"Future",IF(A102=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A102,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E102=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A102&gt;$B$4,"Future",IF(A102=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A102,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E102=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3651,7 +3656,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E103" s="6" t="str">
-        <x:f>IF(A103&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A103,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A103&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A103,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F103" s="6" t="str">
         <x:f>IF(A103&gt;=$B$4,"",MAX(D103-E103,0))</x:f>
@@ -3666,7 +3671,7 @@
         <x:f>IF(A103&gt;$B$4,"",SUM($E$15:E103))</x:f>
       </x:c>
       <x:c r="J103" s="1" t="str">
-        <x:f>IF(A103&gt;$B$4,"Future",IF(A103=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A103,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E103=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A103&gt;$B$4,"Future",IF(A103=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A103,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E103=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3686,7 +3691,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E104" s="6" t="str">
-        <x:f>IF(A104&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A104,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A104&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A104,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F104" s="6" t="str">
         <x:f>IF(A104&gt;=$B$4,"",MAX(D104-E104,0))</x:f>
@@ -3701,7 +3706,7 @@
         <x:f>IF(A104&gt;$B$4,"",SUM($E$15:E104))</x:f>
       </x:c>
       <x:c r="J104" s="1" t="str">
-        <x:f>IF(A104&gt;$B$4,"Future",IF(A104=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A104,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E104=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A104&gt;$B$4,"Future",IF(A104=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A104,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E104=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3721,7 +3726,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E105" s="6" t="str">
-        <x:f>IF(A105&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A105,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A105&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A105,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F105" s="6" t="str">
         <x:f>IF(A105&gt;=$B$4,"",MAX(D105-E105,0))</x:f>
@@ -3736,7 +3741,7 @@
         <x:f>IF(A105&gt;$B$4,"",SUM($E$15:E105))</x:f>
       </x:c>
       <x:c r="J105" s="1" t="str">
-        <x:f>IF(A105&gt;$B$4,"Future",IF(A105=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A105,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E105=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A105&gt;$B$4,"Future",IF(A105=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A105,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E105=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3756,7 +3761,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E106" s="6" t="str">
-        <x:f>IF(A106&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A106,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A106&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A106,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F106" s="6" t="str">
         <x:f>IF(A106&gt;=$B$4,"",MAX(D106-E106,0))</x:f>
@@ -3771,7 +3776,7 @@
         <x:f>IF(A106&gt;$B$4,"",SUM($E$15:E106))</x:f>
       </x:c>
       <x:c r="J106" s="1" t="str">
-        <x:f>IF(A106&gt;$B$4,"Future",IF(A106=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A106,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E106=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A106&gt;$B$4,"Future",IF(A106=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A106,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E106=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3791,7 +3796,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E107" s="6" t="str">
-        <x:f>IF(A107&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A107,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A107&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A107,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F107" s="6" t="str">
         <x:f>IF(A107&gt;=$B$4,"",MAX(D107-E107,0))</x:f>
@@ -3806,7 +3811,7 @@
         <x:f>IF(A107&gt;$B$4,"",SUM($E$15:E107))</x:f>
       </x:c>
       <x:c r="J107" s="1" t="str">
-        <x:f>IF(A107&gt;$B$4,"Future",IF(A107=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A107,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E107=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A107&gt;$B$4,"Future",IF(A107=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A107,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E107=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3826,7 +3831,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E108" s="6" t="str">
-        <x:f>IF(A108&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A108,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A108&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A108,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F108" s="6" t="str">
         <x:f>IF(A108&gt;=$B$4,"",MAX(D108-E108,0))</x:f>
@@ -3841,7 +3846,7 @@
         <x:f>IF(A108&gt;$B$4,"",SUM($E$15:E108))</x:f>
       </x:c>
       <x:c r="J108" s="1" t="str">
-        <x:f>IF(A108&gt;$B$4,"Future",IF(A108=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A108,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E108=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A108&gt;$B$4,"Future",IF(A108=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A108,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E108=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3861,7 +3866,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E109" s="6" t="str">
-        <x:f>IF(A109&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A109,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A109&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A109,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F109" s="6" t="str">
         <x:f>IF(A109&gt;=$B$4,"",MAX(D109-E109,0))</x:f>
@@ -3876,7 +3881,7 @@
         <x:f>IF(A109&gt;$B$4,"",SUM($E$15:E109))</x:f>
       </x:c>
       <x:c r="J109" s="1" t="str">
-        <x:f>IF(A109&gt;$B$4,"Future",IF(A109=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A109,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E109=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A109&gt;$B$4,"Future",IF(A109=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A109,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E109=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3896,7 +3901,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E110" s="6" t="str">
-        <x:f>IF(A110&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A110,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A110&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A110,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F110" s="6" t="str">
         <x:f>IF(A110&gt;=$B$4,"",MAX(D110-E110,0))</x:f>
@@ -3911,7 +3916,7 @@
         <x:f>IF(A110&gt;$B$4,"",SUM($E$15:E110))</x:f>
       </x:c>
       <x:c r="J110" s="1" t="str">
-        <x:f>IF(A110&gt;$B$4,"Future",IF(A110=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A110,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E110=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A110&gt;$B$4,"Future",IF(A110=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A110,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E110=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3931,7 +3936,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E111" s="6" t="str">
-        <x:f>IF(A111&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A111,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A111&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A111,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F111" s="6" t="str">
         <x:f>IF(A111&gt;=$B$4,"",MAX(D111-E111,0))</x:f>
@@ -3946,7 +3951,7 @@
         <x:f>IF(A111&gt;$B$4,"",SUM($E$15:E111))</x:f>
       </x:c>
       <x:c r="J111" s="1" t="str">
-        <x:f>IF(A111&gt;$B$4,"Future",IF(A111=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A111,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E111=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A111&gt;$B$4,"Future",IF(A111=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A111,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E111=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3966,7 +3971,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E112" s="6" t="str">
-        <x:f>IF(A112&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A112,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A112&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A112,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F112" s="6" t="str">
         <x:f>IF(A112&gt;=$B$4,"",MAX(D112-E112,0))</x:f>
@@ -3981,7 +3986,7 @@
         <x:f>IF(A112&gt;$B$4,"",SUM($E$15:E112))</x:f>
       </x:c>
       <x:c r="J112" s="1" t="str">
-        <x:f>IF(A112&gt;$B$4,"Future",IF(A112=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A112,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E112=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A112&gt;$B$4,"Future",IF(A112=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A112,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E112=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4001,7 +4006,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E113" s="6" t="str">
-        <x:f>IF(A113&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A113,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A113&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A113,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F113" s="6" t="str">
         <x:f>IF(A113&gt;=$B$4,"",MAX(D113-E113,0))</x:f>
@@ -4016,7 +4021,7 @@
         <x:f>IF(A113&gt;$B$4,"",SUM($E$15:E113))</x:f>
       </x:c>
       <x:c r="J113" s="1" t="str">
-        <x:f>IF(A113&gt;$B$4,"Future",IF(A113=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A113,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E113=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A113&gt;$B$4,"Future",IF(A113=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A113,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E113=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4036,7 +4041,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E114" s="6" t="str">
-        <x:f>IF(A114&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A114,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A114&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A114,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F114" s="6" t="str">
         <x:f>IF(A114&gt;=$B$4,"",MAX(D114-E114,0))</x:f>
@@ -4051,7 +4056,7 @@
         <x:f>IF(A114&gt;$B$4,"",SUM($E$15:E114))</x:f>
       </x:c>
       <x:c r="J114" s="1" t="str">
-        <x:f>IF(A114&gt;$B$4,"Future",IF(A114=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A114,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E114=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A114&gt;$B$4,"Future",IF(A114=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A114,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E114=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4071,7 +4076,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E115" s="6" t="str">
-        <x:f>IF(A115&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A115,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A115&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A115,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F115" s="6" t="str">
         <x:f>IF(A115&gt;=$B$4,"",MAX(D115-E115,0))</x:f>
@@ -4086,7 +4091,7 @@
         <x:f>IF(A115&gt;$B$4,"",SUM($E$15:E115))</x:f>
       </x:c>
       <x:c r="J115" s="1" t="str">
-        <x:f>IF(A115&gt;$B$4,"Future",IF(A115=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A115,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E115=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A115&gt;$B$4,"Future",IF(A115=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A115,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E115=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4106,7 +4111,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E116" s="6" t="str">
-        <x:f>IF(A116&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A116,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A116&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A116,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F116" s="6" t="str">
         <x:f>IF(A116&gt;=$B$4,"",MAX(D116-E116,0))</x:f>
@@ -4121,7 +4126,7 @@
         <x:f>IF(A116&gt;$B$4,"",SUM($E$15:E116))</x:f>
       </x:c>
       <x:c r="J116" s="1" t="str">
-        <x:f>IF(A116&gt;$B$4,"Future",IF(A116=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A116,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E116=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A116&gt;$B$4,"Future",IF(A116=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A116,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E116=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4141,7 +4146,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E117" s="6" t="str">
-        <x:f>IF(A117&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A117,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A117&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A117,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F117" s="6" t="str">
         <x:f>IF(A117&gt;=$B$4,"",MAX(D117-E117,0))</x:f>
@@ -4156,7 +4161,7 @@
         <x:f>IF(A117&gt;$B$4,"",SUM($E$15:E117))</x:f>
       </x:c>
       <x:c r="J117" s="1" t="str">
-        <x:f>IF(A117&gt;$B$4,"Future",IF(A117=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A117,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E117=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A117&gt;$B$4,"Future",IF(A117=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A117,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E117=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4176,7 +4181,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E118" s="6" t="str">
-        <x:f>IF(A118&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A118,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A118&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A118,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F118" s="6" t="str">
         <x:f>IF(A118&gt;=$B$4,"",MAX(D118-E118,0))</x:f>
@@ -4191,7 +4196,7 @@
         <x:f>IF(A118&gt;$B$4,"",SUM($E$15:E118))</x:f>
       </x:c>
       <x:c r="J118" s="1" t="str">
-        <x:f>IF(A118&gt;$B$4,"Future",IF(A118=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A118,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E118=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A118&gt;$B$4,"Future",IF(A118=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A118,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E118=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4211,7 +4216,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E119" s="6" t="str">
-        <x:f>IF(A119&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A119,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A119&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A119,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F119" s="6" t="str">
         <x:f>IF(A119&gt;=$B$4,"",MAX(D119-E119,0))</x:f>
@@ -4226,7 +4231,7 @@
         <x:f>IF(A119&gt;$B$4,"",SUM($E$15:E119))</x:f>
       </x:c>
       <x:c r="J119" s="1" t="str">
-        <x:f>IF(A119&gt;$B$4,"Future",IF(A119=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A119,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E119=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A119&gt;$B$4,"Future",IF(A119=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A119,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E119=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4246,7 +4251,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E120" s="6" t="str">
-        <x:f>IF(A120&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A120,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A120&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A120,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F120" s="6" t="str">
         <x:f>IF(A120&gt;=$B$4,"",MAX(D120-E120,0))</x:f>
@@ -4261,7 +4266,7 @@
         <x:f>IF(A120&gt;$B$4,"",SUM($E$15:E120))</x:f>
       </x:c>
       <x:c r="J120" s="1" t="str">
-        <x:f>IF(A120&gt;$B$4,"Future",IF(A120=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A120,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E120=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A120&gt;$B$4,"Future",IF(A120=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A120,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E120=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4281,7 +4286,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E121" s="6" t="str">
-        <x:f>IF(A121&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A121,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A121&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A121,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F121" s="6" t="str">
         <x:f>IF(A121&gt;=$B$4,"",MAX(D121-E121,0))</x:f>
@@ -4296,7 +4301,7 @@
         <x:f>IF(A121&gt;$B$4,"",SUM($E$15:E121))</x:f>
       </x:c>
       <x:c r="J121" s="1" t="str">
-        <x:f>IF(A121&gt;$B$4,"Future",IF(A121=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A121,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E121=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A121&gt;$B$4,"Future",IF(A121=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A121,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E121=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4316,7 +4321,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E122" s="6" t="str">
-        <x:f>IF(A122&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A122,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A122&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A122,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F122" s="6" t="str">
         <x:f>IF(A122&gt;=$B$4,"",MAX(D122-E122,0))</x:f>
@@ -4331,7 +4336,7 @@
         <x:f>IF(A122&gt;$B$4,"",SUM($E$15:E122))</x:f>
       </x:c>
       <x:c r="J122" s="1" t="str">
-        <x:f>IF(A122&gt;$B$4,"Future",IF(A122=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A122,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E122=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A122&gt;$B$4,"Future",IF(A122=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A122,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E122=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4351,7 +4356,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E123" s="6" t="str">
-        <x:f>IF(A123&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A123,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A123&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A123,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F123" s="6" t="str">
         <x:f>IF(A123&gt;=$B$4,"",MAX(D123-E123,0))</x:f>
@@ -4366,7 +4371,7 @@
         <x:f>IF(A123&gt;$B$4,"",SUM($E$15:E123))</x:f>
       </x:c>
       <x:c r="J123" s="1" t="str">
-        <x:f>IF(A123&gt;$B$4,"Future",IF(A123=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A123,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E123=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A123&gt;$B$4,"Future",IF(A123=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A123,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E123=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4386,7 +4391,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E124" s="6" t="str">
-        <x:f>IF(A124&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A124,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A124&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A124,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F124" s="6" t="str">
         <x:f>IF(A124&gt;=$B$4,"",MAX(D124-E124,0))</x:f>
@@ -4401,7 +4406,7 @@
         <x:f>IF(A124&gt;$B$4,"",SUM($E$15:E124))</x:f>
       </x:c>
       <x:c r="J124" s="1" t="str">
-        <x:f>IF(A124&gt;$B$4,"Future",IF(A124=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A124,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E124=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A124&gt;$B$4,"Future",IF(A124=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A124,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E124=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4421,7 +4426,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E125" s="6" t="str">
-        <x:f>IF(A125&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A125,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A125&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A125,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F125" s="6" t="str">
         <x:f>IF(A125&gt;=$B$4,"",MAX(D125-E125,0))</x:f>
@@ -4436,7 +4441,7 @@
         <x:f>IF(A125&gt;$B$4,"",SUM($E$15:E125))</x:f>
       </x:c>
       <x:c r="J125" s="1" t="str">
-        <x:f>IF(A125&gt;$B$4,"Future",IF(A125=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A125,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E125=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A125&gt;$B$4,"Future",IF(A125=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A125,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E125=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4456,7 +4461,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E126" s="6" t="str">
-        <x:f>IF(A126&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A126,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A126&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A126,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F126" s="6" t="str">
         <x:f>IF(A126&gt;=$B$4,"",MAX(D126-E126,0))</x:f>
@@ -4471,7 +4476,7 @@
         <x:f>IF(A126&gt;$B$4,"",SUM($E$15:E126))</x:f>
       </x:c>
       <x:c r="J126" s="1" t="str">
-        <x:f>IF(A126&gt;$B$4,"Future",IF(A126=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A126,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E126=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A126&gt;$B$4,"Future",IF(A126=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A126,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E126=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4491,7 +4496,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E127" s="6" t="str">
-        <x:f>IF(A127&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A127,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A127&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A127,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F127" s="6" t="str">
         <x:f>IF(A127&gt;=$B$4,"",MAX(D127-E127,0))</x:f>
@@ -4506,7 +4511,7 @@
         <x:f>IF(A127&gt;$B$4,"",SUM($E$15:E127))</x:f>
       </x:c>
       <x:c r="J127" s="1" t="str">
-        <x:f>IF(A127&gt;$B$4,"Future",IF(A127=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A127,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E127=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A127&gt;$B$4,"Future",IF(A127=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A127,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E127=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4526,7 +4531,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E128" s="6" t="str">
-        <x:f>IF(A128&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A128,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A128&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A128,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F128" s="6" t="str">
         <x:f>IF(A128&gt;=$B$4,"",MAX(D128-E128,0))</x:f>
@@ -4541,7 +4546,7 @@
         <x:f>IF(A128&gt;$B$4,"",SUM($E$15:E128))</x:f>
       </x:c>
       <x:c r="J128" s="1" t="str">
-        <x:f>IF(A128&gt;$B$4,"Future",IF(A128=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A128,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E128=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A128&gt;$B$4,"Future",IF(A128=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A128,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E128=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4561,7 +4566,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E129" s="6" t="str">
-        <x:f>IF(A129&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A129,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A129&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A129,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F129" s="6" t="str">
         <x:f>IF(A129&gt;=$B$4,"",MAX(D129-E129,0))</x:f>
@@ -4576,7 +4581,7 @@
         <x:f>IF(A129&gt;$B$4,"",SUM($E$15:E129))</x:f>
       </x:c>
       <x:c r="J129" s="1" t="str">
-        <x:f>IF(A129&gt;$B$4,"Future",IF(A129=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A129,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E129=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A129&gt;$B$4,"Future",IF(A129=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A129,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E129=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4596,7 +4601,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E130" s="6" t="str">
-        <x:f>IF(A130&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$14,'Sessions'!$B$2:$B$14,A130,'Sessions'!$G$2:$G$14,"completed")/60)</x:f>
+        <x:f>IF(A130&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A130,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
       </x:c>
       <x:c r="F130" s="6" t="str">
         <x:f>IF(A130&gt;=$B$4,"",MAX(D130-E130,0))</x:f>
@@ -4611,7 +4616,7 @@
         <x:f>IF(A130&gt;$B$4,"",SUM($E$15:E130))</x:f>
       </x:c>
       <x:c r="J130" s="1" t="str">
-        <x:f>IF(A130&gt;$B$4,"Future",IF(A130=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$14,A130,'Sessions'!$G$2:$G$14,"needs_confirmation")&gt;0,"Uncertain time",IF(E130=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A130&gt;$B$4,"Future",IF(A130=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A130,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E130=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4731,15 +4736,15 @@
       </x:c>
       <x:c r="C8" s="6" t="n">
         <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A8,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
-        <x:v>6</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D8" s="6" t="n">
         <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A8)</x:f>
-        <x:v>4.499166666667222</x:v>
+        <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="E8" s="6" t="n">
         <x:f>MAX(C8-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A8,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
-        <x:v>3.1905555555550005</x:v>
+        <x:v>7.500833333332778</x:v>
       </x:c>
       <x:c r="F8" s="6" t="n">
         <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A8,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C8,0)</x:f>
@@ -4747,11 +4752,11 @@
       </x:c>
       <x:c r="G8" s="6" t="n">
         <x:f>MAX(B8-D8,0)</x:f>
-        <x:v>27.50083333333278</x:v>
+        <x:v>20.848611111110557</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
         <x:f>IF(B8=0,0,D8/B8)</x:f>
-        <x:v>0.14059895833335068</x:v>
+        <x:v>0.34848090277779514</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
@@ -5666,6 +5671,188 @@
         <x:v>Explicit start-timer for CSV; break excluded; pending output-file task; earlier 15 October uncertain interval remains excluded; Explicit pause 13:39:15 IST; 7m38s; no new submitted code or output; CSV writing task pending</x:v>
       </x:c>
     </x:row>
+    <x:row r="15" ht="22" customHeight="1">
+      <x:c r="A15" s="1" t="str">
+        <x:v>PY-20261017T103739</x:v>
+      </x:c>
+      <x:c r="B15" s="7" t="n">
+        <x:v>46312</x:v>
+      </x:c>
+      <x:c r="C15" s="1" t="str">
+        <x:v>Python: CSV writing and read-back</x:v>
+      </x:c>
+      <x:c r="D15" s="1" t="str">
+        <x:v>IST 2026-10-17 10:37:39</x:v>
+      </x:c>
+      <x:c r="E15" s="1" t="str">
+        <x:v>IST 2026-10-17 11:25:08</x:v>
+      </x:c>
+      <x:c r="F15" s="1" t="n">
+        <x:v>47.483333333333334</x:v>
+      </x:c>
+      <x:c r="G15" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H15" s="1" t="str">
+        <x:v>Explicit Start Python; clock timestamp; resume pending valid/rejected CSV writing and read-back; breaks and old 15 October uncertain interval excluded; no new assessed learning. Explicit pause 11:25:08 IST; 47m29s. Requested split() reference saved earlier; no learner code/output or assessment submitted; CSV writing/read-back remains pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="22" customHeight="1">
+      <x:c r="A16" s="1" t="str">
+        <x:v>PY-20261017T113412</x:v>
+      </x:c>
+      <x:c r="B16" s="7" t="n">
+        <x:v>46312</x:v>
+      </x:c>
+      <x:c r="C16" s="1" t="str">
+        <x:v>Python: CSV writing and read-back</x:v>
+      </x:c>
+      <x:c r="D16" s="1" t="str">
+        <x:v>IST 2026-10-17 11:34:12</x:v>
+      </x:c>
+      <x:c r="E16" s="1" t="str">
+        <x:v>IST 2026-10-17 11:45:31</x:v>
+      </x:c>
+      <x:c r="F16" s="1" t="n">
+        <x:v>11.316666666666666</x:v>
+      </x:c>
+      <x:c r="G16" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H16" s="1" t="str">
+        <x:v>Explicit resume-timer; prior Python topic retained; 11:25:08-11:34:12 break excluded; CSV writing/read-back pending; no new learning evidence. Explicit pause 11:45:31 IST; 11m19s; no new submitted code/output; CSV writing/read-back pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="22" customHeight="1">
+      <x:c r="A17" s="1" t="str">
+        <x:v>PY-20261017T120153</x:v>
+      </x:c>
+      <x:c r="B17" s="7" t="n">
+        <x:v>46312</x:v>
+      </x:c>
+      <x:c r="C17" s="1" t="str">
+        <x:v>Python: CSV writing and read-back</x:v>
+      </x:c>
+      <x:c r="D17" s="1" t="str">
+        <x:v>IST 2026-10-17 12:01:53</x:v>
+      </x:c>
+      <x:c r="E17" s="1" t="str">
+        <x:v>IST 2026-10-17 12:32:30</x:v>
+      </x:c>
+      <x:c r="F17" s="1" t="n">
+        <x:v>30.616666666666667</x:v>
+      </x:c>
+      <x:c r="G17" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H17" s="1" t="str">
+        <x:v>Explicit resume-timer; prior Python topic retained; 11:45:31-12:01:53 break excluded; CSV writing/read-back pending; no new learning evidence. Explicit pause 12:32:30 IST; 30m37s; no new submitted code/output; CSV writing/read-back pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="22" customHeight="1">
+      <x:c r="A18" s="1" t="str">
+        <x:v>PY-20261017T152016</x:v>
+      </x:c>
+      <x:c r="B18" s="7" t="n">
+        <x:v>46312</x:v>
+      </x:c>
+      <x:c r="C18" s="1" t="str">
+        <x:v>Python: CSV writing and read-back</x:v>
+      </x:c>
+      <x:c r="D18" s="1" t="str">
+        <x:v>IST 2026-10-17 15:20:16</x:v>
+      </x:c>
+      <x:c r="E18" s="1" t="str">
+        <x:v>IST 2026-10-17 16:39:54</x:v>
+      </x:c>
+      <x:c r="F18" s="1" t="n">
+        <x:v>79.63333333333334</x:v>
+      </x:c>
+      <x:c r="G18" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H18" s="1" t="str">
+        <x:v>Explicit start-timer; established Python topic retained; break since 12:32:30 excluded; CSV writing/read-back pending; no new learning evidence. Topic switched to RetailFlow at 16:39:54 IST on explicit integration request; no new code reviewed; outgoing interval not attributed to RetailFlow.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="22" customHeight="1">
+      <x:c r="A19" s="1" t="str">
+        <x:v>RF-20261017T163954</x:v>
+      </x:c>
+      <x:c r="B19" s="7" t="n">
+        <x:v>46312</x:v>
+      </x:c>
+      <x:c r="C19" s="1" t="str">
+        <x:v>Python / RetailFlow: setup and RF-001</x:v>
+      </x:c>
+      <x:c r="D19" s="1" t="str">
+        <x:v>IST 2026-10-17 16:39:54</x:v>
+      </x:c>
+      <x:c r="E19" s="1" t="str">
+        <x:v>IST 2026-10-17 17:45:25</x:v>
+      </x:c>
+      <x:c r="F19" s="1" t="n">
+        <x:v>65.51666666666667</x:v>
+      </x:c>
+      <x:c r="G19" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H19" s="1" t="str">
+        <x:v>Existing authorised Python timer continues across explicit project switch; no break/overlap; RetailFlow setup is not learning success; only completed RF-prefixed intervals count toward confirmed project hours. Switched to RRDAP at 17:45:25 IST on explicit replacement request; setup/planning interval, no verified implementation; preserve separately from RRDAP time.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="22" customHeight="1">
+      <x:c r="A20" s="1" t="str">
+        <x:v>RDS-20261017T174525</x:v>
+      </x:c>
+      <x:c r="B20" s="7" t="n">
+        <x:v>46312</x:v>
+      </x:c>
+      <x:c r="C20" s="1" t="str">
+        <x:v>Python / RRDAP: setup and RDS-001</x:v>
+      </x:c>
+      <x:c r="D20" s="1" t="str">
+        <x:v>IST 2026-10-17 17:45:25</x:v>
+      </x:c>
+      <x:c r="E20" s="1" t="str">
+        <x:v>IST 2026-10-17 19:58:56</x:v>
+      </x:c>
+      <x:c r="F20" s="1" t="n">
+        <x:v>133.51666666666668</x:v>
+      </x:c>
+      <x:c r="G20" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H20" s="1" t="str">
+        <x:v>Existing authorised study timer continues across explicit project replacement without overlap; RRDAP setup is not learning success; completed RDS-prefixed intervals own project time. Explicit pause at 19:58:56 IST; 2h13m31s. No new learner code/output or assessment available in this chat; RDS-001 remains pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="22" customHeight="1">
+      <x:c r="A21" s="1" t="str">
+        <x:v>RDS-20261017T205651</x:v>
+      </x:c>
+      <x:c r="B21" s="7" t="n">
+        <x:v>46312</x:v>
+      </x:c>
+      <x:c r="C21" s="1" t="str">
+        <x:v>Python / RRDAP: RDS-001 Product Catalogue</x:v>
+      </x:c>
+      <x:c r="D21" s="1" t="str">
+        <x:v>IST 2026-10-17 20:56:51</x:v>
+      </x:c>
+      <x:c r="E21" s="1" t="str">
+        <x:v>IST 2026-10-17 21:27:54</x:v>
+      </x:c>
+      <x:c r="F21" s="1" t="n">
+        <x:v>31.05</x:v>
+      </x:c>
+      <x:c r="G21" s="1" t="str">
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="H21" s="1" t="str">
+        <x:v>Explicit resume-timer; established RRDAP topic retained. Break 19:58:56-20:56:51 (57m55s) excluded. RDS-001 approach/implementation pending; no new assessed learning. Explicit pause at 21:27:54 IST; 31m03s. No new learner submission or assessed learning in this chat; RDS-001 pending.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Upgrade Azure interview roadmap and date-effective study tracking
</commit_message>
<xml_diff>
--- a/outputs/study-tracker/study-hours.xlsx
+++ b/outputs/study-tracker/study-hours.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="R0756837246834773"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="R621daf9bb6f74648"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="R6e15d754381d424b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="R645b99787c3941f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="R3a925f8c45464b2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="Reb46c3304c5a464d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topics" sheetId="4" r:id="Rfdc3a107eac445e4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -354,19 +355,23 @@
         <x:v>Reporting date (IST)</x:v>
       </x:c>
       <x:c r="B4" s="8" t="n">
-        <x:v>46312</x:v>
+        <x:v>46317</x:v>
       </x:c>
       <x:c r="C4" s="1"/>
       <x:c r="D4" s="1" t="str">
         <x:v>Confirmed hours</x:v>
       </x:c>
       <x:c r="E4" s="6" t="n">
-        <x:f>SUM(E15:E130)</x:f>
+        <x:f>SUM(E15:E114)</x:f>
         <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="F4" s="1"/>
-      <x:c r="G4" s="1"/>
-      <x:c r="H4" s="1"/>
+      <x:c r="G4" s="1" t="str">
+        <x:v>Earlier weekday target</x:v>
+      </x:c>
+      <x:c r="H4" s="1" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="I4" s="1"/>
       <x:c r="J4" s="1"/>
     </x:row>
@@ -382,29 +387,33 @@
         <x:v>Target: closed days</x:v>
       </x:c>
       <x:c r="E5" s="6" t="n">
-        <x:f>SUMIFS(D15:D130,A15:A130,"&lt;"&amp;B4)</x:f>
-        <x:v>12</x:v>
+        <x:f>SUMIFS(D15:D114,A15:A114,"&lt;"&amp;B4)</x:f>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="F5" s="1"/>
-      <x:c r="G5" s="1"/>
-      <x:c r="H5" s="1"/>
+      <x:c r="G5" s="1" t="str">
+        <x:v>Target source</x:v>
+      </x:c>
+      <x:c r="H5" s="1" t="str">
+        <x:v>tracking/study-targets.json</x:v>
+      </x:c>
       <x:c r="I5" s="1"/>
       <x:c r="J5" s="1"/>
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
       <x:c r="A6" s="1" t="str">
-        <x:v>Weekday target (hours)</x:v>
+        <x:v>Weekday target (from 22 Oct)</x:v>
       </x:c>
       <x:c r="B6" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C6" s="1"/>
       <x:c r="D6" s="1" t="str">
         <x:v>Behind: closed days</x:v>
       </x:c>
       <x:c r="E6" s="6" t="n">
-        <x:f>MAX(E5-SUMIFS(E15:E130,A15:A130,"&lt;"&amp;B4),0)</x:f>
-        <x:v>7.500833333332778</x:v>
+        <x:f>MAX(E5-SUMIFS(E15:E114,A15:A114,"&lt;"&amp;B4),0)</x:f>
+        <x:v>38.84861111111056</x:v>
       </x:c>
       <x:c r="F6" s="1"/>
       <x:c r="G6" s="1"/>
@@ -424,7 +433,7 @@
         <x:v>Ahead: closed days</x:v>
       </x:c>
       <x:c r="E7" s="6" t="n">
-        <x:f>MAX(SUMIFS(E15:E130,A15:A130,"&lt;"&amp;B4)-E5,0)</x:f>
+        <x:f>MAX(SUMIFS(E15:E114,A15:A114,"&lt;"&amp;B4)-E5,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="1"/>
@@ -434,15 +443,19 @@
       <x:c r="J7" s="1"/>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">
-      <x:c r="A8" s="1"/>
-      <x:c r="B8" s="1"/>
+      <x:c r="A8" s="1" t="str">
+        <x:v>New target effective</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="n">
+        <x:v>46317</x:v>
+      </x:c>
       <x:c r="C8" s="1"/>
       <x:c r="D8" s="1" t="str">
         <x:v>Remaining today</x:v>
       </x:c>
       <x:c r="E8" s="6" t="n">
-        <x:f>MAX(SUMIFS(D15:D130,A15:A130,B4)-SUMIFS(E15:E130,A15:A130,B4),0)</x:f>
-        <x:v>3.347777777777777</x:v>
+        <x:f>MAX(SUMIFS(D15:D114,A15:A114,B4)-SUMIFS(E15:E114,A15:A114,B4),0)</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F8" s="1"/>
       <x:c r="G8" s="1"/>
@@ -451,8 +464,12 @@
       <x:c r="J8" s="1"/>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
-      <x:c r="A9" s="1"/>
-      <x:c r="B9" s="1"/>
+      <x:c r="A9" s="1" t="str">
+        <x:v>Preparation deadline</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="n">
+        <x:v>46409</x:v>
+      </x:c>
       <x:c r="C9" s="1"/>
       <x:c r="D9" s="1"/>
       <x:c r="E9" s="1"/>
@@ -560,7 +577,7 @@
         <x:v>46307</x:v>
       </x:c>
       <x:c r="D15" s="6" t="n">
-        <x:f>IF(WEEKDAY(A15,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A15,2)&gt;5,$B$7,IF(A15&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="E15" s="6" t="n">
@@ -600,7 +617,7 @@
         <x:v>46307</x:v>
       </x:c>
       <x:c r="D16" s="6" t="n">
-        <x:f>IF(WEEKDAY(A16,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A16,2)&gt;5,$B$7,IF(A16&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="E16" s="6" t="n">
@@ -640,21 +657,24 @@
         <x:v>46307</x:v>
       </x:c>
       <x:c r="D17" s="6" t="n">
-        <x:f>IF(WEEKDAY(A17,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A17,2)&gt;5,$B$7,IF(A17&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E17" s="6" t="n">
         <x:f>IF(A17&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A17,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
         <x:v>6.652222222222223</x:v>
       </x:c>
-      <x:c r="F17" s="6" t="str">
+      <x:c r="F17" s="6" t="n">
         <x:f>IF(A17&gt;=$B$4,"",MAX(D17-E17,0))</x:f>
-      </x:c>
-      <x:c r="G17" s="6" t="str">
+        <x:v>3.347777777777777</x:v>
+      </x:c>
+      <x:c r="G17" s="6" t="n">
         <x:f>IF(A17&gt;=$B$4,"",MAX(E17-D17,0))</x:f>
-      </x:c>
-      <x:c r="H17" s="6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H17" s="6" t="n">
         <x:f>IF(A17&gt;=$B$4,"",SUM($D$15:D17))</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="I17" s="6" t="n">
         <x:f>IF(A17&gt;$B$4,"",SUM($E$15:E17))</x:f>
@@ -662,7 +682,7 @@
       </x:c>
       <x:c r="J17" s="1" t="str">
         <x:f>IF(A17&gt;$B$4,"Future",IF(A17=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A17,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E17=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>In progress</x:v>
+        <x:v>Logged</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
@@ -677,27 +697,32 @@
         <x:v>46307</x:v>
       </x:c>
       <x:c r="D18" s="6" t="n">
-        <x:f>IF(WEEKDAY(A18,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A18,2)&gt;5,$B$7,IF(A18&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="E18" s="6" t="str">
+      <x:c r="E18" s="6" t="n">
         <x:f>IF(A18&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A18,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F18" s="6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F18" s="6" t="n">
         <x:f>IF(A18&gt;=$B$4,"",MAX(D18-E18,0))</x:f>
-      </x:c>
-      <x:c r="G18" s="6" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G18" s="6" t="n">
         <x:f>IF(A18&gt;=$B$4,"",MAX(E18-D18,0))</x:f>
-      </x:c>
-      <x:c r="H18" s="6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H18" s="6" t="n">
         <x:f>IF(A18&gt;=$B$4,"",SUM($D$15:D18))</x:f>
-      </x:c>
-      <x:c r="I18" s="6" t="str">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="I18" s="6" t="n">
         <x:f>IF(A18&gt;$B$4,"",SUM($E$15:E18))</x:f>
+        <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J18" s="1" t="str">
         <x:f>IF(A18&gt;$B$4,"Future",IF(A18=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A18,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E18=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
+        <x:v>No confirmed time</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
@@ -712,27 +737,32 @@
         <x:v>46314</x:v>
       </x:c>
       <x:c r="D19" s="6" t="n">
-        <x:f>IF(WEEKDAY(A19,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A19,2)&gt;5,$B$7,IF(A19&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>6</x:v>
       </x:c>
-      <x:c r="E19" s="6" t="str">
+      <x:c r="E19" s="6" t="n">
         <x:f>IF(A19&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A19,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F19" s="6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F19" s="6" t="n">
         <x:f>IF(A19&gt;=$B$4,"",MAX(D19-E19,0))</x:f>
-      </x:c>
-      <x:c r="G19" s="6" t="str">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G19" s="6" t="n">
         <x:f>IF(A19&gt;=$B$4,"",MAX(E19-D19,0))</x:f>
-      </x:c>
-      <x:c r="H19" s="6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H19" s="6" t="n">
         <x:f>IF(A19&gt;=$B$4,"",SUM($D$15:D19))</x:f>
-      </x:c>
-      <x:c r="I19" s="6" t="str">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="I19" s="6" t="n">
         <x:f>IF(A19&gt;$B$4,"",SUM($E$15:E19))</x:f>
+        <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J19" s="1" t="str">
         <x:f>IF(A19&gt;$B$4,"Future",IF(A19=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A19,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E19=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
+        <x:v>No confirmed time</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
@@ -747,27 +777,32 @@
         <x:v>46314</x:v>
       </x:c>
       <x:c r="D20" s="6" t="n">
-        <x:f>IF(WEEKDAY(A20,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A20,2)&gt;5,$B$7,IF(A20&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>6</x:v>
       </x:c>
-      <x:c r="E20" s="6" t="str">
+      <x:c r="E20" s="6" t="n">
         <x:f>IF(A20&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A20,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F20" s="6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F20" s="6" t="n">
         <x:f>IF(A20&gt;=$B$4,"",MAX(D20-E20,0))</x:f>
-      </x:c>
-      <x:c r="G20" s="6" t="str">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G20" s="6" t="n">
         <x:f>IF(A20&gt;=$B$4,"",MAX(E20-D20,0))</x:f>
-      </x:c>
-      <x:c r="H20" s="6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H20" s="6" t="n">
         <x:f>IF(A20&gt;=$B$4,"",SUM($D$15:D20))</x:f>
-      </x:c>
-      <x:c r="I20" s="6" t="str">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="I20" s="6" t="n">
         <x:f>IF(A20&gt;$B$4,"",SUM($E$15:E20))</x:f>
+        <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J20" s="1" t="str">
         <x:f>IF(A20&gt;$B$4,"Future",IF(A20=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A20,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E20=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
+        <x:v>No confirmed time</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="22" customHeight="1">
@@ -782,27 +817,32 @@
         <x:v>46314</x:v>
       </x:c>
       <x:c r="D21" s="6" t="n">
-        <x:f>IF(WEEKDAY(A21,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A21,2)&gt;5,$B$7,IF(A21&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>6</x:v>
       </x:c>
-      <x:c r="E21" s="6" t="str">
+      <x:c r="E21" s="6" t="n">
         <x:f>IF(A21&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A21,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F21" s="6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F21" s="6" t="n">
         <x:f>IF(A21&gt;=$B$4,"",MAX(D21-E21,0))</x:f>
-      </x:c>
-      <x:c r="G21" s="6" t="str">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G21" s="6" t="n">
         <x:f>IF(A21&gt;=$B$4,"",MAX(E21-D21,0))</x:f>
-      </x:c>
-      <x:c r="H21" s="6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H21" s="6" t="n">
         <x:f>IF(A21&gt;=$B$4,"",SUM($D$15:D21))</x:f>
-      </x:c>
-      <x:c r="I21" s="6" t="str">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="I21" s="6" t="n">
         <x:f>IF(A21&gt;$B$4,"",SUM($E$15:E21))</x:f>
+        <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J21" s="1" t="str">
         <x:f>IF(A21&gt;$B$4,"Future",IF(A21=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A21,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E21=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
+        <x:v>No confirmed time</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="22" customHeight="1">
@@ -817,11 +857,12 @@
         <x:v>46314</x:v>
       </x:c>
       <x:c r="D22" s="6" t="n">
-        <x:f>IF(WEEKDAY(A22,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="E22" s="6" t="str">
+        <x:f>IF(WEEKDAY(A22,2)&gt;5,$B$7,IF(A22&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E22" s="6" t="n">
         <x:f>IF(A22&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A22,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F22" s="6" t="str">
         <x:f>IF(A22&gt;=$B$4,"",MAX(D22-E22,0))</x:f>
@@ -832,12 +873,13 @@
       <x:c r="H22" s="6" t="str">
         <x:f>IF(A22&gt;=$B$4,"",SUM($D$15:D22))</x:f>
       </x:c>
-      <x:c r="I22" s="6" t="str">
+      <x:c r="I22" s="6" t="n">
         <x:f>IF(A22&gt;$B$4,"",SUM($E$15:E22))</x:f>
+        <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J22" s="1" t="str">
         <x:f>IF(A22&gt;$B$4,"Future",IF(A22=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A22,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E22=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
+        <x:v>In progress</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="22" customHeight="1">
@@ -852,8 +894,8 @@
         <x:v>46314</x:v>
       </x:c>
       <x:c r="D23" s="6" t="n">
-        <x:f>IF(WEEKDAY(A23,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A23,2)&gt;5,$B$7,IF(A23&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E23" s="6" t="str">
         <x:f>IF(A23&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A23,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -887,7 +929,7 @@
         <x:v>46314</x:v>
       </x:c>
       <x:c r="D24" s="6" t="n">
-        <x:f>IF(WEEKDAY(A24,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A24,2)&gt;5,$B$7,IF(A24&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E24" s="6" t="str">
@@ -922,7 +964,7 @@
         <x:v>46314</x:v>
       </x:c>
       <x:c r="D25" s="6" t="n">
-        <x:f>IF(WEEKDAY(A25,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A25,2)&gt;5,$B$7,IF(A25&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E25" s="6" t="str">
@@ -957,8 +999,8 @@
         <x:v>46321</x:v>
       </x:c>
       <x:c r="D26" s="6" t="n">
-        <x:f>IF(WEEKDAY(A26,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A26,2)&gt;5,$B$7,IF(A26&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E26" s="6" t="str">
         <x:f>IF(A26&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A26,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -992,8 +1034,8 @@
         <x:v>46321</x:v>
       </x:c>
       <x:c r="D27" s="6" t="n">
-        <x:f>IF(WEEKDAY(A27,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A27,2)&gt;5,$B$7,IF(A27&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E27" s="6" t="str">
         <x:f>IF(A27&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A27,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1027,8 +1069,8 @@
         <x:v>46321</x:v>
       </x:c>
       <x:c r="D28" s="6" t="n">
-        <x:f>IF(WEEKDAY(A28,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A28,2)&gt;5,$B$7,IF(A28&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E28" s="6" t="str">
         <x:f>IF(A28&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A28,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1062,8 +1104,8 @@
         <x:v>46321</x:v>
       </x:c>
       <x:c r="D29" s="6" t="n">
-        <x:f>IF(WEEKDAY(A29,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A29,2)&gt;5,$B$7,IF(A29&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E29" s="6" t="str">
         <x:f>IF(A29&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A29,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1097,8 +1139,8 @@
         <x:v>46321</x:v>
       </x:c>
       <x:c r="D30" s="6" t="n">
-        <x:f>IF(WEEKDAY(A30,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A30,2)&gt;5,$B$7,IF(A30&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E30" s="6" t="str">
         <x:f>IF(A30&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A30,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1132,7 +1174,7 @@
         <x:v>46321</x:v>
       </x:c>
       <x:c r="D31" s="6" t="n">
-        <x:f>IF(WEEKDAY(A31,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A31,2)&gt;5,$B$7,IF(A31&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E31" s="6" t="str">
@@ -1167,7 +1209,7 @@
         <x:v>46321</x:v>
       </x:c>
       <x:c r="D32" s="6" t="n">
-        <x:f>IF(WEEKDAY(A32,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A32,2)&gt;5,$B$7,IF(A32&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E32" s="6" t="str">
@@ -1202,8 +1244,8 @@
         <x:v>46328</x:v>
       </x:c>
       <x:c r="D33" s="6" t="n">
-        <x:f>IF(WEEKDAY(A33,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A33,2)&gt;5,$B$7,IF(A33&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E33" s="6" t="str">
         <x:f>IF(A33&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A33,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1237,8 +1279,8 @@
         <x:v>46328</x:v>
       </x:c>
       <x:c r="D34" s="6" t="n">
-        <x:f>IF(WEEKDAY(A34,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A34,2)&gt;5,$B$7,IF(A34&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E34" s="6" t="str">
         <x:f>IF(A34&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A34,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1272,8 +1314,8 @@
         <x:v>46328</x:v>
       </x:c>
       <x:c r="D35" s="6" t="n">
-        <x:f>IF(WEEKDAY(A35,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A35,2)&gt;5,$B$7,IF(A35&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E35" s="6" t="str">
         <x:f>IF(A35&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A35,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1307,8 +1349,8 @@
         <x:v>46328</x:v>
       </x:c>
       <x:c r="D36" s="6" t="n">
-        <x:f>IF(WEEKDAY(A36,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A36,2)&gt;5,$B$7,IF(A36&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E36" s="6" t="str">
         <x:f>IF(A36&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A36,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1342,8 +1384,8 @@
         <x:v>46328</x:v>
       </x:c>
       <x:c r="D37" s="6" t="n">
-        <x:f>IF(WEEKDAY(A37,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A37,2)&gt;5,$B$7,IF(A37&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E37" s="6" t="str">
         <x:f>IF(A37&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A37,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1377,7 +1419,7 @@
         <x:v>46328</x:v>
       </x:c>
       <x:c r="D38" s="6" t="n">
-        <x:f>IF(WEEKDAY(A38,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A38,2)&gt;5,$B$7,IF(A38&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E38" s="6" t="str">
@@ -1412,7 +1454,7 @@
         <x:v>46328</x:v>
       </x:c>
       <x:c r="D39" s="6" t="n">
-        <x:f>IF(WEEKDAY(A39,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A39,2)&gt;5,$B$7,IF(A39&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E39" s="6" t="str">
@@ -1447,8 +1489,8 @@
         <x:v>46335</x:v>
       </x:c>
       <x:c r="D40" s="6" t="n">
-        <x:f>IF(WEEKDAY(A40,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A40,2)&gt;5,$B$7,IF(A40&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E40" s="6" t="str">
         <x:f>IF(A40&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A40,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1482,8 +1524,8 @@
         <x:v>46335</x:v>
       </x:c>
       <x:c r="D41" s="6" t="n">
-        <x:f>IF(WEEKDAY(A41,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A41,2)&gt;5,$B$7,IF(A41&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E41" s="6" t="str">
         <x:f>IF(A41&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A41,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1517,8 +1559,8 @@
         <x:v>46335</x:v>
       </x:c>
       <x:c r="D42" s="6" t="n">
-        <x:f>IF(WEEKDAY(A42,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A42,2)&gt;5,$B$7,IF(A42&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E42" s="6" t="str">
         <x:f>IF(A42&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A42,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1552,8 +1594,8 @@
         <x:v>46335</x:v>
       </x:c>
       <x:c r="D43" s="6" t="n">
-        <x:f>IF(WEEKDAY(A43,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A43,2)&gt;5,$B$7,IF(A43&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E43" s="6" t="str">
         <x:f>IF(A43&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A43,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1587,8 +1629,8 @@
         <x:v>46335</x:v>
       </x:c>
       <x:c r="D44" s="6" t="n">
-        <x:f>IF(WEEKDAY(A44,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A44,2)&gt;5,$B$7,IF(A44&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E44" s="6" t="str">
         <x:f>IF(A44&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A44,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1622,7 +1664,7 @@
         <x:v>46335</x:v>
       </x:c>
       <x:c r="D45" s="6" t="n">
-        <x:f>IF(WEEKDAY(A45,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A45,2)&gt;5,$B$7,IF(A45&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E45" s="6" t="str">
@@ -1657,7 +1699,7 @@
         <x:v>46335</x:v>
       </x:c>
       <x:c r="D46" s="6" t="n">
-        <x:f>IF(WEEKDAY(A46,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A46,2)&gt;5,$B$7,IF(A46&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E46" s="6" t="str">
@@ -1692,8 +1734,8 @@
         <x:v>46342</x:v>
       </x:c>
       <x:c r="D47" s="6" t="n">
-        <x:f>IF(WEEKDAY(A47,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A47,2)&gt;5,$B$7,IF(A47&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E47" s="6" t="str">
         <x:f>IF(A47&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A47,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1727,8 +1769,8 @@
         <x:v>46342</x:v>
       </x:c>
       <x:c r="D48" s="6" t="n">
-        <x:f>IF(WEEKDAY(A48,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A48,2)&gt;5,$B$7,IF(A48&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E48" s="6" t="str">
         <x:f>IF(A48&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A48,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1762,8 +1804,8 @@
         <x:v>46342</x:v>
       </x:c>
       <x:c r="D49" s="6" t="n">
-        <x:f>IF(WEEKDAY(A49,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A49,2)&gt;5,$B$7,IF(A49&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E49" s="6" t="str">
         <x:f>IF(A49&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A49,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1797,8 +1839,8 @@
         <x:v>46342</x:v>
       </x:c>
       <x:c r="D50" s="6" t="n">
-        <x:f>IF(WEEKDAY(A50,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A50,2)&gt;5,$B$7,IF(A50&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E50" s="6" t="str">
         <x:f>IF(A50&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A50,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1832,8 +1874,8 @@
         <x:v>46342</x:v>
       </x:c>
       <x:c r="D51" s="6" t="n">
-        <x:f>IF(WEEKDAY(A51,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A51,2)&gt;5,$B$7,IF(A51&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E51" s="6" t="str">
         <x:f>IF(A51&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A51,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1867,7 +1909,7 @@
         <x:v>46342</x:v>
       </x:c>
       <x:c r="D52" s="6" t="n">
-        <x:f>IF(WEEKDAY(A52,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A52,2)&gt;5,$B$7,IF(A52&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E52" s="6" t="str">
@@ -1902,7 +1944,7 @@
         <x:v>46342</x:v>
       </x:c>
       <x:c r="D53" s="6" t="n">
-        <x:f>IF(WEEKDAY(A53,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A53,2)&gt;5,$B$7,IF(A53&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E53" s="6" t="str">
@@ -1937,8 +1979,8 @@
         <x:v>46349</x:v>
       </x:c>
       <x:c r="D54" s="6" t="n">
-        <x:f>IF(WEEKDAY(A54,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A54,2)&gt;5,$B$7,IF(A54&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E54" s="6" t="str">
         <x:f>IF(A54&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A54,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -1972,8 +2014,8 @@
         <x:v>46349</x:v>
       </x:c>
       <x:c r="D55" s="6" t="n">
-        <x:f>IF(WEEKDAY(A55,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A55,2)&gt;5,$B$7,IF(A55&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E55" s="6" t="str">
         <x:f>IF(A55&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A55,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2007,8 +2049,8 @@
         <x:v>46349</x:v>
       </x:c>
       <x:c r="D56" s="6" t="n">
-        <x:f>IF(WEEKDAY(A56,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A56,2)&gt;5,$B$7,IF(A56&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E56" s="6" t="str">
         <x:f>IF(A56&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A56,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2042,8 +2084,8 @@
         <x:v>46349</x:v>
       </x:c>
       <x:c r="D57" s="6" t="n">
-        <x:f>IF(WEEKDAY(A57,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A57,2)&gt;5,$B$7,IF(A57&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E57" s="6" t="str">
         <x:f>IF(A57&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A57,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2077,8 +2119,8 @@
         <x:v>46349</x:v>
       </x:c>
       <x:c r="D58" s="6" t="n">
-        <x:f>IF(WEEKDAY(A58,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A58,2)&gt;5,$B$7,IF(A58&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E58" s="6" t="str">
         <x:f>IF(A58&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A58,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2112,7 +2154,7 @@
         <x:v>46349</x:v>
       </x:c>
       <x:c r="D59" s="6" t="n">
-        <x:f>IF(WEEKDAY(A59,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A59,2)&gt;5,$B$7,IF(A59&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E59" s="6" t="str">
@@ -2147,7 +2189,7 @@
         <x:v>46349</x:v>
       </x:c>
       <x:c r="D60" s="6" t="n">
-        <x:f>IF(WEEKDAY(A60,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A60,2)&gt;5,$B$7,IF(A60&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E60" s="6" t="str">
@@ -2182,8 +2224,8 @@
         <x:v>46356</x:v>
       </x:c>
       <x:c r="D61" s="6" t="n">
-        <x:f>IF(WEEKDAY(A61,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A61,2)&gt;5,$B$7,IF(A61&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E61" s="6" t="str">
         <x:f>IF(A61&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A61,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2217,8 +2259,8 @@
         <x:v>46356</x:v>
       </x:c>
       <x:c r="D62" s="6" t="n">
-        <x:f>IF(WEEKDAY(A62,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A62,2)&gt;5,$B$7,IF(A62&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E62" s="6" t="str">
         <x:f>IF(A62&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A62,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2252,8 +2294,8 @@
         <x:v>46356</x:v>
       </x:c>
       <x:c r="D63" s="6" t="n">
-        <x:f>IF(WEEKDAY(A63,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A63,2)&gt;5,$B$7,IF(A63&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E63" s="6" t="str">
         <x:f>IF(A63&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A63,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2287,8 +2329,8 @@
         <x:v>46356</x:v>
       </x:c>
       <x:c r="D64" s="6" t="n">
-        <x:f>IF(WEEKDAY(A64,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A64,2)&gt;5,$B$7,IF(A64&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E64" s="6" t="str">
         <x:f>IF(A64&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A64,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2322,8 +2364,8 @@
         <x:v>46356</x:v>
       </x:c>
       <x:c r="D65" s="6" t="n">
-        <x:f>IF(WEEKDAY(A65,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A65,2)&gt;5,$B$7,IF(A65&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E65" s="6" t="str">
         <x:f>IF(A65&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A65,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2357,7 +2399,7 @@
         <x:v>46356</x:v>
       </x:c>
       <x:c r="D66" s="6" t="n">
-        <x:f>IF(WEEKDAY(A66,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A66,2)&gt;5,$B$7,IF(A66&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E66" s="6" t="str">
@@ -2392,7 +2434,7 @@
         <x:v>46356</x:v>
       </x:c>
       <x:c r="D67" s="6" t="n">
-        <x:f>IF(WEEKDAY(A67,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A67,2)&gt;5,$B$7,IF(A67&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E67" s="6" t="str">
@@ -2427,8 +2469,8 @@
         <x:v>46363</x:v>
       </x:c>
       <x:c r="D68" s="6" t="n">
-        <x:f>IF(WEEKDAY(A68,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A68,2)&gt;5,$B$7,IF(A68&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E68" s="6" t="str">
         <x:f>IF(A68&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A68,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2462,8 +2504,8 @@
         <x:v>46363</x:v>
       </x:c>
       <x:c r="D69" s="6" t="n">
-        <x:f>IF(WEEKDAY(A69,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A69,2)&gt;5,$B$7,IF(A69&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E69" s="6" t="str">
         <x:f>IF(A69&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A69,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2497,8 +2539,8 @@
         <x:v>46363</x:v>
       </x:c>
       <x:c r="D70" s="6" t="n">
-        <x:f>IF(WEEKDAY(A70,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A70,2)&gt;5,$B$7,IF(A70&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E70" s="6" t="str">
         <x:f>IF(A70&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A70,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2532,8 +2574,8 @@
         <x:v>46363</x:v>
       </x:c>
       <x:c r="D71" s="6" t="n">
-        <x:f>IF(WEEKDAY(A71,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A71,2)&gt;5,$B$7,IF(A71&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E71" s="6" t="str">
         <x:f>IF(A71&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A71,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2567,8 +2609,8 @@
         <x:v>46363</x:v>
       </x:c>
       <x:c r="D72" s="6" t="n">
-        <x:f>IF(WEEKDAY(A72,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A72,2)&gt;5,$B$7,IF(A72&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E72" s="6" t="str">
         <x:f>IF(A72&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A72,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2602,7 +2644,7 @@
         <x:v>46363</x:v>
       </x:c>
       <x:c r="D73" s="6" t="n">
-        <x:f>IF(WEEKDAY(A73,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A73,2)&gt;5,$B$7,IF(A73&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E73" s="6" t="str">
@@ -2637,7 +2679,7 @@
         <x:v>46363</x:v>
       </x:c>
       <x:c r="D74" s="6" t="n">
-        <x:f>IF(WEEKDAY(A74,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A74,2)&gt;5,$B$7,IF(A74&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E74" s="6" t="str">
@@ -2672,8 +2714,8 @@
         <x:v>46370</x:v>
       </x:c>
       <x:c r="D75" s="6" t="n">
-        <x:f>IF(WEEKDAY(A75,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A75,2)&gt;5,$B$7,IF(A75&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E75" s="6" t="str">
         <x:f>IF(A75&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A75,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2707,8 +2749,8 @@
         <x:v>46370</x:v>
       </x:c>
       <x:c r="D76" s="6" t="n">
-        <x:f>IF(WEEKDAY(A76,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A76,2)&gt;5,$B$7,IF(A76&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E76" s="6" t="str">
         <x:f>IF(A76&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A76,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2742,8 +2784,8 @@
         <x:v>46370</x:v>
       </x:c>
       <x:c r="D77" s="6" t="n">
-        <x:f>IF(WEEKDAY(A77,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A77,2)&gt;5,$B$7,IF(A77&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E77" s="6" t="str">
         <x:f>IF(A77&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A77,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2777,8 +2819,8 @@
         <x:v>46370</x:v>
       </x:c>
       <x:c r="D78" s="6" t="n">
-        <x:f>IF(WEEKDAY(A78,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A78,2)&gt;5,$B$7,IF(A78&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E78" s="6" t="str">
         <x:f>IF(A78&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A78,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2812,8 +2854,8 @@
         <x:v>46370</x:v>
       </x:c>
       <x:c r="D79" s="6" t="n">
-        <x:f>IF(WEEKDAY(A79,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A79,2)&gt;5,$B$7,IF(A79&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E79" s="6" t="str">
         <x:f>IF(A79&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A79,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2847,7 +2889,7 @@
         <x:v>46370</x:v>
       </x:c>
       <x:c r="D80" s="6" t="n">
-        <x:f>IF(WEEKDAY(A80,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A80,2)&gt;5,$B$7,IF(A80&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E80" s="6" t="str">
@@ -2882,7 +2924,7 @@
         <x:v>46370</x:v>
       </x:c>
       <x:c r="D81" s="6" t="n">
-        <x:f>IF(WEEKDAY(A81,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A81,2)&gt;5,$B$7,IF(A81&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E81" s="6" t="str">
@@ -2917,8 +2959,8 @@
         <x:v>46377</x:v>
       </x:c>
       <x:c r="D82" s="6" t="n">
-        <x:f>IF(WEEKDAY(A82,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A82,2)&gt;5,$B$7,IF(A82&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E82" s="6" t="str">
         <x:f>IF(A82&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A82,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2952,8 +2994,8 @@
         <x:v>46377</x:v>
       </x:c>
       <x:c r="D83" s="6" t="n">
-        <x:f>IF(WEEKDAY(A83,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A83,2)&gt;5,$B$7,IF(A83&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E83" s="6" t="str">
         <x:f>IF(A83&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A83,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -2987,8 +3029,8 @@
         <x:v>46377</x:v>
       </x:c>
       <x:c r="D84" s="6" t="n">
-        <x:f>IF(WEEKDAY(A84,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A84,2)&gt;5,$B$7,IF(A84&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E84" s="6" t="str">
         <x:f>IF(A84&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A84,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3022,8 +3064,8 @@
         <x:v>46377</x:v>
       </x:c>
       <x:c r="D85" s="6" t="n">
-        <x:f>IF(WEEKDAY(A85,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A85,2)&gt;5,$B$7,IF(A85&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E85" s="6" t="str">
         <x:f>IF(A85&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A85,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3057,8 +3099,8 @@
         <x:v>46377</x:v>
       </x:c>
       <x:c r="D86" s="6" t="n">
-        <x:f>IF(WEEKDAY(A86,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A86,2)&gt;5,$B$7,IF(A86&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E86" s="6" t="str">
         <x:f>IF(A86&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A86,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3092,7 +3134,7 @@
         <x:v>46377</x:v>
       </x:c>
       <x:c r="D87" s="6" t="n">
-        <x:f>IF(WEEKDAY(A87,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A87,2)&gt;5,$B$7,IF(A87&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E87" s="6" t="str">
@@ -3127,7 +3169,7 @@
         <x:v>46377</x:v>
       </x:c>
       <x:c r="D88" s="6" t="n">
-        <x:f>IF(WEEKDAY(A88,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A88,2)&gt;5,$B$7,IF(A88&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E88" s="6" t="str">
@@ -3162,8 +3204,8 @@
         <x:v>46384</x:v>
       </x:c>
       <x:c r="D89" s="6" t="n">
-        <x:f>IF(WEEKDAY(A89,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A89,2)&gt;5,$B$7,IF(A89&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E89" s="6" t="str">
         <x:f>IF(A89&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A89,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3197,8 +3239,8 @@
         <x:v>46384</x:v>
       </x:c>
       <x:c r="D90" s="6" t="n">
-        <x:f>IF(WEEKDAY(A90,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A90,2)&gt;5,$B$7,IF(A90&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E90" s="6" t="str">
         <x:f>IF(A90&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A90,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3232,8 +3274,8 @@
         <x:v>46384</x:v>
       </x:c>
       <x:c r="D91" s="6" t="n">
-        <x:f>IF(WEEKDAY(A91,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A91,2)&gt;5,$B$7,IF(A91&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E91" s="6" t="str">
         <x:f>IF(A91&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A91,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3267,8 +3309,8 @@
         <x:v>46384</x:v>
       </x:c>
       <x:c r="D92" s="6" t="n">
-        <x:f>IF(WEEKDAY(A92,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A92,2)&gt;5,$B$7,IF(A92&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E92" s="6" t="str">
         <x:f>IF(A92&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A92,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3302,8 +3344,8 @@
         <x:v>46384</x:v>
       </x:c>
       <x:c r="D93" s="6" t="n">
-        <x:f>IF(WEEKDAY(A93,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A93,2)&gt;5,$B$7,IF(A93&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E93" s="6" t="str">
         <x:f>IF(A93&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A93,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3337,7 +3379,7 @@
         <x:v>46384</x:v>
       </x:c>
       <x:c r="D94" s="6" t="n">
-        <x:f>IF(WEEKDAY(A94,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A94,2)&gt;5,$B$7,IF(A94&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E94" s="6" t="str">
@@ -3372,7 +3414,7 @@
         <x:v>46384</x:v>
       </x:c>
       <x:c r="D95" s="6" t="n">
-        <x:f>IF(WEEKDAY(A95,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A95,2)&gt;5,$B$7,IF(A95&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E95" s="6" t="str">
@@ -3407,8 +3449,8 @@
         <x:v>46391</x:v>
       </x:c>
       <x:c r="D96" s="6" t="n">
-        <x:f>IF(WEEKDAY(A96,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A96,2)&gt;5,$B$7,IF(A96&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E96" s="6" t="str">
         <x:f>IF(A96&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A96,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3442,8 +3484,8 @@
         <x:v>46391</x:v>
       </x:c>
       <x:c r="D97" s="6" t="n">
-        <x:f>IF(WEEKDAY(A97,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A97,2)&gt;5,$B$7,IF(A97&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E97" s="6" t="str">
         <x:f>IF(A97&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A97,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3477,8 +3519,8 @@
         <x:v>46391</x:v>
       </x:c>
       <x:c r="D98" s="6" t="n">
-        <x:f>IF(WEEKDAY(A98,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A98,2)&gt;5,$B$7,IF(A98&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E98" s="6" t="str">
         <x:f>IF(A98&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A98,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3512,8 +3554,8 @@
         <x:v>46391</x:v>
       </x:c>
       <x:c r="D99" s="6" t="n">
-        <x:f>IF(WEEKDAY(A99,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A99,2)&gt;5,$B$7,IF(A99&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E99" s="6" t="str">
         <x:f>IF(A99&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A99,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3547,8 +3589,8 @@
         <x:v>46391</x:v>
       </x:c>
       <x:c r="D100" s="6" t="n">
-        <x:f>IF(WEEKDAY(A100,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A100,2)&gt;5,$B$7,IF(A100&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E100" s="6" t="str">
         <x:f>IF(A100&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A100,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3582,7 +3624,7 @@
         <x:v>46391</x:v>
       </x:c>
       <x:c r="D101" s="6" t="n">
-        <x:f>IF(WEEKDAY(A101,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A101,2)&gt;5,$B$7,IF(A101&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E101" s="6" t="str">
@@ -3617,7 +3659,7 @@
         <x:v>46391</x:v>
       </x:c>
       <x:c r="D102" s="6" t="n">
-        <x:f>IF(WEEKDAY(A102,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A102,2)&gt;5,$B$7,IF(A102&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E102" s="6" t="str">
@@ -3652,8 +3694,8 @@
         <x:v>46398</x:v>
       </x:c>
       <x:c r="D103" s="6" t="n">
-        <x:f>IF(WEEKDAY(A103,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A103,2)&gt;5,$B$7,IF(A103&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E103" s="6" t="str">
         <x:f>IF(A103&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A103,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3687,8 +3729,8 @@
         <x:v>46398</x:v>
       </x:c>
       <x:c r="D104" s="6" t="n">
-        <x:f>IF(WEEKDAY(A104,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A104,2)&gt;5,$B$7,IF(A104&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E104" s="6" t="str">
         <x:f>IF(A104&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A104,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3722,8 +3764,8 @@
         <x:v>46398</x:v>
       </x:c>
       <x:c r="D105" s="6" t="n">
-        <x:f>IF(WEEKDAY(A105,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A105,2)&gt;5,$B$7,IF(A105&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E105" s="6" t="str">
         <x:f>IF(A105&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A105,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3757,8 +3799,8 @@
         <x:v>46398</x:v>
       </x:c>
       <x:c r="D106" s="6" t="n">
-        <x:f>IF(WEEKDAY(A106,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A106,2)&gt;5,$B$7,IF(A106&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E106" s="6" t="str">
         <x:f>IF(A106&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A106,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3792,8 +3834,8 @@
         <x:v>46398</x:v>
       </x:c>
       <x:c r="D107" s="6" t="n">
-        <x:f>IF(WEEKDAY(A107,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A107,2)&gt;5,$B$7,IF(A107&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E107" s="6" t="str">
         <x:f>IF(A107&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A107,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3827,7 +3869,7 @@
         <x:v>46398</x:v>
       </x:c>
       <x:c r="D108" s="6" t="n">
-        <x:f>IF(WEEKDAY(A108,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A108,2)&gt;5,$B$7,IF(A108&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E108" s="6" t="str">
@@ -3862,7 +3904,7 @@
         <x:v>46398</x:v>
       </x:c>
       <x:c r="D109" s="6" t="n">
-        <x:f>IF(WEEKDAY(A109,2)&gt;5,$B$7,$B$6)</x:f>
+        <x:f>IF(WEEKDAY(A109,2)&gt;5,$B$7,IF(A109&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E109" s="6" t="str">
@@ -3897,8 +3939,8 @@
         <x:v>46405</x:v>
       </x:c>
       <x:c r="D110" s="6" t="n">
-        <x:f>IF(WEEKDAY(A110,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A110,2)&gt;5,$B$7,IF(A110&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E110" s="6" t="str">
         <x:f>IF(A110&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A110,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3932,8 +3974,8 @@
         <x:v>46405</x:v>
       </x:c>
       <x:c r="D111" s="6" t="n">
-        <x:f>IF(WEEKDAY(A111,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A111,2)&gt;5,$B$7,IF(A111&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E111" s="6" t="str">
         <x:f>IF(A111&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A111,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -3967,8 +4009,8 @@
         <x:v>46405</x:v>
       </x:c>
       <x:c r="D112" s="6" t="n">
-        <x:f>IF(WEEKDAY(A112,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A112,2)&gt;5,$B$7,IF(A112&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E112" s="6" t="str">
         <x:f>IF(A112&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A112,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -4002,8 +4044,8 @@
         <x:v>46405</x:v>
       </x:c>
       <x:c r="D113" s="6" t="n">
-        <x:f>IF(WEEKDAY(A113,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A113,2)&gt;5,$B$7,IF(A113&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E113" s="6" t="str">
         <x:f>IF(A113&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A113,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -4037,8 +4079,8 @@
         <x:v>46405</x:v>
       </x:c>
       <x:c r="D114" s="6" t="n">
-        <x:f>IF(WEEKDAY(A114,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
+        <x:f>IF(WEEKDAY(A114,2)&gt;5,$B$7,IF(A114&lt;$B$8,$H$4,$B$6))</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E114" s="6" t="str">
         <x:f>IF(A114&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A114,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
@@ -4060,568 +4102,8 @@
         <x:v>Future</x:v>
       </x:c>
     </x:row>
-    <x:row r="115" ht="22" customHeight="1">
-      <x:c r="A115" s="7" t="n">
-        <x:v>46410</x:v>
-      </x:c>
-      <x:c r="B115" s="1" t="str">
-        <x:v>Sat</x:v>
-      </x:c>
-      <x:c r="C115" s="7" t="n">
-        <x:f>A115-WEEKDAY(A115,2)+1</x:f>
-        <x:v>46405</x:v>
-      </x:c>
-      <x:c r="D115" s="6" t="n">
-        <x:f>IF(WEEKDAY(A115,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="E115" s="6" t="str">
-        <x:f>IF(A115&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A115,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F115" s="6" t="str">
-        <x:f>IF(A115&gt;=$B$4,"",MAX(D115-E115,0))</x:f>
-      </x:c>
-      <x:c r="G115" s="6" t="str">
-        <x:f>IF(A115&gt;=$B$4,"",MAX(E115-D115,0))</x:f>
-      </x:c>
-      <x:c r="H115" s="6" t="str">
-        <x:f>IF(A115&gt;=$B$4,"",SUM($D$15:D115))</x:f>
-      </x:c>
-      <x:c r="I115" s="6" t="str">
-        <x:f>IF(A115&gt;$B$4,"",SUM($E$15:E115))</x:f>
-      </x:c>
-      <x:c r="J115" s="1" t="str">
-        <x:f>IF(A115&gt;$B$4,"Future",IF(A115=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A115,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E115=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="116" ht="22" customHeight="1">
-      <x:c r="A116" s="7" t="n">
-        <x:v>46411</x:v>
-      </x:c>
-      <x:c r="B116" s="1" t="str">
-        <x:v>Sun</x:v>
-      </x:c>
-      <x:c r="C116" s="7" t="n">
-        <x:f>A116-WEEKDAY(A116,2)+1</x:f>
-        <x:v>46405</x:v>
-      </x:c>
-      <x:c r="D116" s="6" t="n">
-        <x:f>IF(WEEKDAY(A116,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="E116" s="6" t="str">
-        <x:f>IF(A116&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A116,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F116" s="6" t="str">
-        <x:f>IF(A116&gt;=$B$4,"",MAX(D116-E116,0))</x:f>
-      </x:c>
-      <x:c r="G116" s="6" t="str">
-        <x:f>IF(A116&gt;=$B$4,"",MAX(E116-D116,0))</x:f>
-      </x:c>
-      <x:c r="H116" s="6" t="str">
-        <x:f>IF(A116&gt;=$B$4,"",SUM($D$15:D116))</x:f>
-      </x:c>
-      <x:c r="I116" s="6" t="str">
-        <x:f>IF(A116&gt;$B$4,"",SUM($E$15:E116))</x:f>
-      </x:c>
-      <x:c r="J116" s="1" t="str">
-        <x:f>IF(A116&gt;$B$4,"Future",IF(A116=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A116,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E116=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="117" ht="22" customHeight="1">
-      <x:c r="A117" s="7" t="n">
-        <x:v>46412</x:v>
-      </x:c>
-      <x:c r="B117" s="1" t="str">
-        <x:v>Mon</x:v>
-      </x:c>
-      <x:c r="C117" s="7" t="n">
-        <x:f>A117-WEEKDAY(A117,2)+1</x:f>
-        <x:v>46412</x:v>
-      </x:c>
-      <x:c r="D117" s="6" t="n">
-        <x:f>IF(WEEKDAY(A117,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="E117" s="6" t="str">
-        <x:f>IF(A117&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A117,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F117" s="6" t="str">
-        <x:f>IF(A117&gt;=$B$4,"",MAX(D117-E117,0))</x:f>
-      </x:c>
-      <x:c r="G117" s="6" t="str">
-        <x:f>IF(A117&gt;=$B$4,"",MAX(E117-D117,0))</x:f>
-      </x:c>
-      <x:c r="H117" s="6" t="str">
-        <x:f>IF(A117&gt;=$B$4,"",SUM($D$15:D117))</x:f>
-      </x:c>
-      <x:c r="I117" s="6" t="str">
-        <x:f>IF(A117&gt;$B$4,"",SUM($E$15:E117))</x:f>
-      </x:c>
-      <x:c r="J117" s="1" t="str">
-        <x:f>IF(A117&gt;$B$4,"Future",IF(A117=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A117,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E117=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="118" ht="22" customHeight="1">
-      <x:c r="A118" s="7" t="n">
-        <x:v>46413</x:v>
-      </x:c>
-      <x:c r="B118" s="1" t="str">
-        <x:v>Tue</x:v>
-      </x:c>
-      <x:c r="C118" s="7" t="n">
-        <x:f>A118-WEEKDAY(A118,2)+1</x:f>
-        <x:v>46412</x:v>
-      </x:c>
-      <x:c r="D118" s="6" t="n">
-        <x:f>IF(WEEKDAY(A118,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="E118" s="6" t="str">
-        <x:f>IF(A118&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A118,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F118" s="6" t="str">
-        <x:f>IF(A118&gt;=$B$4,"",MAX(D118-E118,0))</x:f>
-      </x:c>
-      <x:c r="G118" s="6" t="str">
-        <x:f>IF(A118&gt;=$B$4,"",MAX(E118-D118,0))</x:f>
-      </x:c>
-      <x:c r="H118" s="6" t="str">
-        <x:f>IF(A118&gt;=$B$4,"",SUM($D$15:D118))</x:f>
-      </x:c>
-      <x:c r="I118" s="6" t="str">
-        <x:f>IF(A118&gt;$B$4,"",SUM($E$15:E118))</x:f>
-      </x:c>
-      <x:c r="J118" s="1" t="str">
-        <x:f>IF(A118&gt;$B$4,"Future",IF(A118=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A118,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E118=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="119" ht="22" customHeight="1">
-      <x:c r="A119" s="7" t="n">
-        <x:v>46414</x:v>
-      </x:c>
-      <x:c r="B119" s="1" t="str">
-        <x:v>Wed</x:v>
-      </x:c>
-      <x:c r="C119" s="7" t="n">
-        <x:f>A119-WEEKDAY(A119,2)+1</x:f>
-        <x:v>46412</x:v>
-      </x:c>
-      <x:c r="D119" s="6" t="n">
-        <x:f>IF(WEEKDAY(A119,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="E119" s="6" t="str">
-        <x:f>IF(A119&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A119,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F119" s="6" t="str">
-        <x:f>IF(A119&gt;=$B$4,"",MAX(D119-E119,0))</x:f>
-      </x:c>
-      <x:c r="G119" s="6" t="str">
-        <x:f>IF(A119&gt;=$B$4,"",MAX(E119-D119,0))</x:f>
-      </x:c>
-      <x:c r="H119" s="6" t="str">
-        <x:f>IF(A119&gt;=$B$4,"",SUM($D$15:D119))</x:f>
-      </x:c>
-      <x:c r="I119" s="6" t="str">
-        <x:f>IF(A119&gt;$B$4,"",SUM($E$15:E119))</x:f>
-      </x:c>
-      <x:c r="J119" s="1" t="str">
-        <x:f>IF(A119&gt;$B$4,"Future",IF(A119=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A119,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E119=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="120" ht="22" customHeight="1">
-      <x:c r="A120" s="7" t="n">
-        <x:v>46415</x:v>
-      </x:c>
-      <x:c r="B120" s="1" t="str">
-        <x:v>Thu</x:v>
-      </x:c>
-      <x:c r="C120" s="7" t="n">
-        <x:f>A120-WEEKDAY(A120,2)+1</x:f>
-        <x:v>46412</x:v>
-      </x:c>
-      <x:c r="D120" s="6" t="n">
-        <x:f>IF(WEEKDAY(A120,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="E120" s="6" t="str">
-        <x:f>IF(A120&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A120,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F120" s="6" t="str">
-        <x:f>IF(A120&gt;=$B$4,"",MAX(D120-E120,0))</x:f>
-      </x:c>
-      <x:c r="G120" s="6" t="str">
-        <x:f>IF(A120&gt;=$B$4,"",MAX(E120-D120,0))</x:f>
-      </x:c>
-      <x:c r="H120" s="6" t="str">
-        <x:f>IF(A120&gt;=$B$4,"",SUM($D$15:D120))</x:f>
-      </x:c>
-      <x:c r="I120" s="6" t="str">
-        <x:f>IF(A120&gt;$B$4,"",SUM($E$15:E120))</x:f>
-      </x:c>
-      <x:c r="J120" s="1" t="str">
-        <x:f>IF(A120&gt;$B$4,"Future",IF(A120=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A120,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E120=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="121" ht="22" customHeight="1">
-      <x:c r="A121" s="7" t="n">
-        <x:v>46416</x:v>
-      </x:c>
-      <x:c r="B121" s="1" t="str">
-        <x:v>Fri</x:v>
-      </x:c>
-      <x:c r="C121" s="7" t="n">
-        <x:f>A121-WEEKDAY(A121,2)+1</x:f>
-        <x:v>46412</x:v>
-      </x:c>
-      <x:c r="D121" s="6" t="n">
-        <x:f>IF(WEEKDAY(A121,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="E121" s="6" t="str">
-        <x:f>IF(A121&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A121,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F121" s="6" t="str">
-        <x:f>IF(A121&gt;=$B$4,"",MAX(D121-E121,0))</x:f>
-      </x:c>
-      <x:c r="G121" s="6" t="str">
-        <x:f>IF(A121&gt;=$B$4,"",MAX(E121-D121,0))</x:f>
-      </x:c>
-      <x:c r="H121" s="6" t="str">
-        <x:f>IF(A121&gt;=$B$4,"",SUM($D$15:D121))</x:f>
-      </x:c>
-      <x:c r="I121" s="6" t="str">
-        <x:f>IF(A121&gt;$B$4,"",SUM($E$15:E121))</x:f>
-      </x:c>
-      <x:c r="J121" s="1" t="str">
-        <x:f>IF(A121&gt;$B$4,"Future",IF(A121=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A121,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E121=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="122" ht="22" customHeight="1">
-      <x:c r="A122" s="7" t="n">
-        <x:v>46417</x:v>
-      </x:c>
-      <x:c r="B122" s="1" t="str">
-        <x:v>Sat</x:v>
-      </x:c>
-      <x:c r="C122" s="7" t="n">
-        <x:f>A122-WEEKDAY(A122,2)+1</x:f>
-        <x:v>46412</x:v>
-      </x:c>
-      <x:c r="D122" s="6" t="n">
-        <x:f>IF(WEEKDAY(A122,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="E122" s="6" t="str">
-        <x:f>IF(A122&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A122,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F122" s="6" t="str">
-        <x:f>IF(A122&gt;=$B$4,"",MAX(D122-E122,0))</x:f>
-      </x:c>
-      <x:c r="G122" s="6" t="str">
-        <x:f>IF(A122&gt;=$B$4,"",MAX(E122-D122,0))</x:f>
-      </x:c>
-      <x:c r="H122" s="6" t="str">
-        <x:f>IF(A122&gt;=$B$4,"",SUM($D$15:D122))</x:f>
-      </x:c>
-      <x:c r="I122" s="6" t="str">
-        <x:f>IF(A122&gt;$B$4,"",SUM($E$15:E122))</x:f>
-      </x:c>
-      <x:c r="J122" s="1" t="str">
-        <x:f>IF(A122&gt;$B$4,"Future",IF(A122=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A122,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E122=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="123" ht="22" customHeight="1">
-      <x:c r="A123" s="7" t="n">
-        <x:v>46418</x:v>
-      </x:c>
-      <x:c r="B123" s="1" t="str">
-        <x:v>Sun</x:v>
-      </x:c>
-      <x:c r="C123" s="7" t="n">
-        <x:f>A123-WEEKDAY(A123,2)+1</x:f>
-        <x:v>46412</x:v>
-      </x:c>
-      <x:c r="D123" s="6" t="n">
-        <x:f>IF(WEEKDAY(A123,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="E123" s="6" t="str">
-        <x:f>IF(A123&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A123,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F123" s="6" t="str">
-        <x:f>IF(A123&gt;=$B$4,"",MAX(D123-E123,0))</x:f>
-      </x:c>
-      <x:c r="G123" s="6" t="str">
-        <x:f>IF(A123&gt;=$B$4,"",MAX(E123-D123,0))</x:f>
-      </x:c>
-      <x:c r="H123" s="6" t="str">
-        <x:f>IF(A123&gt;=$B$4,"",SUM($D$15:D123))</x:f>
-      </x:c>
-      <x:c r="I123" s="6" t="str">
-        <x:f>IF(A123&gt;$B$4,"",SUM($E$15:E123))</x:f>
-      </x:c>
-      <x:c r="J123" s="1" t="str">
-        <x:f>IF(A123&gt;$B$4,"Future",IF(A123=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A123,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E123=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="124" ht="22" customHeight="1">
-      <x:c r="A124" s="7" t="n">
-        <x:v>46419</x:v>
-      </x:c>
-      <x:c r="B124" s="1" t="str">
-        <x:v>Mon</x:v>
-      </x:c>
-      <x:c r="C124" s="7" t="n">
-        <x:f>A124-WEEKDAY(A124,2)+1</x:f>
-        <x:v>46419</x:v>
-      </x:c>
-      <x:c r="D124" s="6" t="n">
-        <x:f>IF(WEEKDAY(A124,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="E124" s="6" t="str">
-        <x:f>IF(A124&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A124,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F124" s="6" t="str">
-        <x:f>IF(A124&gt;=$B$4,"",MAX(D124-E124,0))</x:f>
-      </x:c>
-      <x:c r="G124" s="6" t="str">
-        <x:f>IF(A124&gt;=$B$4,"",MAX(E124-D124,0))</x:f>
-      </x:c>
-      <x:c r="H124" s="6" t="str">
-        <x:f>IF(A124&gt;=$B$4,"",SUM($D$15:D124))</x:f>
-      </x:c>
-      <x:c r="I124" s="6" t="str">
-        <x:f>IF(A124&gt;$B$4,"",SUM($E$15:E124))</x:f>
-      </x:c>
-      <x:c r="J124" s="1" t="str">
-        <x:f>IF(A124&gt;$B$4,"Future",IF(A124=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A124,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E124=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="125" ht="22" customHeight="1">
-      <x:c r="A125" s="7" t="n">
-        <x:v>46420</x:v>
-      </x:c>
-      <x:c r="B125" s="1" t="str">
-        <x:v>Tue</x:v>
-      </x:c>
-      <x:c r="C125" s="7" t="n">
-        <x:f>A125-WEEKDAY(A125,2)+1</x:f>
-        <x:v>46419</x:v>
-      </x:c>
-      <x:c r="D125" s="6" t="n">
-        <x:f>IF(WEEKDAY(A125,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="E125" s="6" t="str">
-        <x:f>IF(A125&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A125,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F125" s="6" t="str">
-        <x:f>IF(A125&gt;=$B$4,"",MAX(D125-E125,0))</x:f>
-      </x:c>
-      <x:c r="G125" s="6" t="str">
-        <x:f>IF(A125&gt;=$B$4,"",MAX(E125-D125,0))</x:f>
-      </x:c>
-      <x:c r="H125" s="6" t="str">
-        <x:f>IF(A125&gt;=$B$4,"",SUM($D$15:D125))</x:f>
-      </x:c>
-      <x:c r="I125" s="6" t="str">
-        <x:f>IF(A125&gt;$B$4,"",SUM($E$15:E125))</x:f>
-      </x:c>
-      <x:c r="J125" s="1" t="str">
-        <x:f>IF(A125&gt;$B$4,"Future",IF(A125=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A125,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E125=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="126" ht="22" customHeight="1">
-      <x:c r="A126" s="7" t="n">
-        <x:v>46421</x:v>
-      </x:c>
-      <x:c r="B126" s="1" t="str">
-        <x:v>Wed</x:v>
-      </x:c>
-      <x:c r="C126" s="7" t="n">
-        <x:f>A126-WEEKDAY(A126,2)+1</x:f>
-        <x:v>46419</x:v>
-      </x:c>
-      <x:c r="D126" s="6" t="n">
-        <x:f>IF(WEEKDAY(A126,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="E126" s="6" t="str">
-        <x:f>IF(A126&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A126,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F126" s="6" t="str">
-        <x:f>IF(A126&gt;=$B$4,"",MAX(D126-E126,0))</x:f>
-      </x:c>
-      <x:c r="G126" s="6" t="str">
-        <x:f>IF(A126&gt;=$B$4,"",MAX(E126-D126,0))</x:f>
-      </x:c>
-      <x:c r="H126" s="6" t="str">
-        <x:f>IF(A126&gt;=$B$4,"",SUM($D$15:D126))</x:f>
-      </x:c>
-      <x:c r="I126" s="6" t="str">
-        <x:f>IF(A126&gt;$B$4,"",SUM($E$15:E126))</x:f>
-      </x:c>
-      <x:c r="J126" s="1" t="str">
-        <x:f>IF(A126&gt;$B$4,"Future",IF(A126=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A126,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E126=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="127" ht="22" customHeight="1">
-      <x:c r="A127" s="7" t="n">
-        <x:v>46422</x:v>
-      </x:c>
-      <x:c r="B127" s="1" t="str">
-        <x:v>Thu</x:v>
-      </x:c>
-      <x:c r="C127" s="7" t="n">
-        <x:f>A127-WEEKDAY(A127,2)+1</x:f>
-        <x:v>46419</x:v>
-      </x:c>
-      <x:c r="D127" s="6" t="n">
-        <x:f>IF(WEEKDAY(A127,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="E127" s="6" t="str">
-        <x:f>IF(A127&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A127,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F127" s="6" t="str">
-        <x:f>IF(A127&gt;=$B$4,"",MAX(D127-E127,0))</x:f>
-      </x:c>
-      <x:c r="G127" s="6" t="str">
-        <x:f>IF(A127&gt;=$B$4,"",MAX(E127-D127,0))</x:f>
-      </x:c>
-      <x:c r="H127" s="6" t="str">
-        <x:f>IF(A127&gt;=$B$4,"",SUM($D$15:D127))</x:f>
-      </x:c>
-      <x:c r="I127" s="6" t="str">
-        <x:f>IF(A127&gt;$B$4,"",SUM($E$15:E127))</x:f>
-      </x:c>
-      <x:c r="J127" s="1" t="str">
-        <x:f>IF(A127&gt;$B$4,"Future",IF(A127=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A127,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E127=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="128" ht="22" customHeight="1">
-      <x:c r="A128" s="7" t="n">
-        <x:v>46423</x:v>
-      </x:c>
-      <x:c r="B128" s="1" t="str">
-        <x:v>Fri</x:v>
-      </x:c>
-      <x:c r="C128" s="7" t="n">
-        <x:f>A128-WEEKDAY(A128,2)+1</x:f>
-        <x:v>46419</x:v>
-      </x:c>
-      <x:c r="D128" s="6" t="n">
-        <x:f>IF(WEEKDAY(A128,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="E128" s="6" t="str">
-        <x:f>IF(A128&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A128,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F128" s="6" t="str">
-        <x:f>IF(A128&gt;=$B$4,"",MAX(D128-E128,0))</x:f>
-      </x:c>
-      <x:c r="G128" s="6" t="str">
-        <x:f>IF(A128&gt;=$B$4,"",MAX(E128-D128,0))</x:f>
-      </x:c>
-      <x:c r="H128" s="6" t="str">
-        <x:f>IF(A128&gt;=$B$4,"",SUM($D$15:D128))</x:f>
-      </x:c>
-      <x:c r="I128" s="6" t="str">
-        <x:f>IF(A128&gt;$B$4,"",SUM($E$15:E128))</x:f>
-      </x:c>
-      <x:c r="J128" s="1" t="str">
-        <x:f>IF(A128&gt;$B$4,"Future",IF(A128=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A128,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E128=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="129" ht="22" customHeight="1">
-      <x:c r="A129" s="7" t="n">
-        <x:v>46424</x:v>
-      </x:c>
-      <x:c r="B129" s="1" t="str">
-        <x:v>Sat</x:v>
-      </x:c>
-      <x:c r="C129" s="7" t="n">
-        <x:f>A129-WEEKDAY(A129,2)+1</x:f>
-        <x:v>46419</x:v>
-      </x:c>
-      <x:c r="D129" s="6" t="n">
-        <x:f>IF(WEEKDAY(A129,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="E129" s="6" t="str">
-        <x:f>IF(A129&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A129,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F129" s="6" t="str">
-        <x:f>IF(A129&gt;=$B$4,"",MAX(D129-E129,0))</x:f>
-      </x:c>
-      <x:c r="G129" s="6" t="str">
-        <x:f>IF(A129&gt;=$B$4,"",MAX(E129-D129,0))</x:f>
-      </x:c>
-      <x:c r="H129" s="6" t="str">
-        <x:f>IF(A129&gt;=$B$4,"",SUM($D$15:D129))</x:f>
-      </x:c>
-      <x:c r="I129" s="6" t="str">
-        <x:f>IF(A129&gt;$B$4,"",SUM($E$15:E129))</x:f>
-      </x:c>
-      <x:c r="J129" s="1" t="str">
-        <x:f>IF(A129&gt;$B$4,"Future",IF(A129=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A129,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E129=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="130" ht="22" customHeight="1">
-      <x:c r="A130" s="7" t="n">
-        <x:v>46425</x:v>
-      </x:c>
-      <x:c r="B130" s="1" t="str">
-        <x:v>Sun</x:v>
-      </x:c>
-      <x:c r="C130" s="7" t="n">
-        <x:f>A130-WEEKDAY(A130,2)+1</x:f>
-        <x:v>46419</x:v>
-      </x:c>
-      <x:c r="D130" s="6" t="n">
-        <x:f>IF(WEEKDAY(A130,2)&gt;5,$B$7,$B$6)</x:f>
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="E130" s="6" t="str">
-        <x:f>IF(A130&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A130,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F130" s="6" t="str">
-        <x:f>IF(A130&gt;=$B$4,"",MAX(D130-E130,0))</x:f>
-      </x:c>
-      <x:c r="G130" s="6" t="str">
-        <x:f>IF(A130&gt;=$B$4,"",MAX(E130-D130,0))</x:f>
-      </x:c>
-      <x:c r="H130" s="6" t="str">
-        <x:f>IF(A130&gt;=$B$4,"",SUM($D$15:D130))</x:f>
-      </x:c>
-      <x:c r="I130" s="6" t="str">
-        <x:f>IF(A130&gt;$B$4,"",SUM($E$15:E130))</x:f>
-      </x:c>
-      <x:c r="J130" s="1" t="str">
-        <x:f>IF(A130&gt;$B$4,"Future",IF(A130=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A130,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E130=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
-      </x:c>
-    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="F15:F130">
+  <x:conditionalFormatting sqref="F15:F114">
     <x:cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
       <x:formula>0</x:formula>
     </x:cfRule>
@@ -4668,7 +4150,7 @@
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="1" t="str">
-        <x:v>Monday–Sunday. First week starts tracking on 15 Oct: 32 h; full weeks: 50 h.</x:v>
+        <x:v>Monday–Sunday: first partial 32 h; transition 52 h; full new weeks 55 h; final preparation partial 35 h.</x:v>
       </x:c>
       <x:c r="B4" s="1"/>
       <x:c r="C4" s="1"/>
@@ -4731,23 +4213,23 @@
         <x:v>46307</x:v>
       </x:c>
       <x:c r="B8" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A8)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A8)</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="C8" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A8,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
-        <x:v>12</x:v>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A8,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D8" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A8)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A8)</x:f>
         <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="E8" s="6" t="n">
-        <x:f>MAX(C8-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A8,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
-        <x:v>7.500833333332778</x:v>
+        <x:f>MAX(C8-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A8,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:v>20.848611111110557</x:v>
       </x:c>
       <x:c r="F8" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A8,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C8,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A8,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C8,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G8" s="6" t="n">
@@ -4764,28 +4246,28 @@
         <x:v>46314</x:v>
       </x:c>
       <x:c r="B9" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A9)</x:f>
-        <x:v>50</x:v>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A9)</x:f>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C9" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A9,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
-        <x:v>0</x:v>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A9,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D9" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A9)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A9)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E9" s="6" t="n">
-        <x:f>MAX(C9-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A9,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
-        <x:v>0</x:v>
+        <x:f>MAX(C9-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A9,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="F9" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A9,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C9,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A9,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C9,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G9" s="6" t="n">
         <x:f>MAX(B9-D9,0)</x:f>
-        <x:v>50</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
         <x:f>IF(B9=0,0,D9/B9)</x:f>
@@ -4797,28 +4279,28 @@
         <x:v>46321</x:v>
       </x:c>
       <x:c r="B10" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A10)</x:f>
-        <x:v>50</x:v>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A10)</x:f>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C10" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A10,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A10,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D10" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A10)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A10)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E10" s="6" t="n">
-        <x:f>MAX(C10-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A10,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C10-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A10,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F10" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A10,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C10,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A10,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C10,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G10" s="6" t="n">
         <x:f>MAX(B10-D10,0)</x:f>
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
         <x:f>IF(B10=0,0,D10/B10)</x:f>
@@ -4830,28 +4312,28 @@
         <x:v>46328</x:v>
       </x:c>
       <x:c r="B11" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A11)</x:f>
-        <x:v>50</x:v>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A11)</x:f>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C11" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A11,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A11,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D11" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A11)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E11" s="6" t="n">
-        <x:f>MAX(C11-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A11,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C11-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A11,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F11" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A11,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C11,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A11,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C11,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G11" s="6" t="n">
         <x:f>MAX(B11-D11,0)</x:f>
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
         <x:f>IF(B11=0,0,D11/B11)</x:f>
@@ -4863,28 +4345,28 @@
         <x:v>46335</x:v>
       </x:c>
       <x:c r="B12" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A12)</x:f>
-        <x:v>50</x:v>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A12)</x:f>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C12" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A12,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A12,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D12" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A12)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A12)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E12" s="6" t="n">
-        <x:f>MAX(C12-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A12,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C12-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A12,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F12" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A12,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C12,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A12,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C12,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G12" s="6" t="n">
         <x:f>MAX(B12-D12,0)</x:f>
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H12" s="10" t="n">
         <x:f>IF(B12=0,0,D12/B12)</x:f>
@@ -4896,28 +4378,28 @@
         <x:v>46342</x:v>
       </x:c>
       <x:c r="B13" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A13)</x:f>
-        <x:v>50</x:v>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A13)</x:f>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C13" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A13,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A13,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D13" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A13)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A13)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E13" s="6" t="n">
-        <x:f>MAX(C13-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A13,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C13-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A13,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F13" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A13,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C13,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A13,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C13,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G13" s="6" t="n">
         <x:f>MAX(B13-D13,0)</x:f>
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H13" s="10" t="n">
         <x:f>IF(B13=0,0,D13/B13)</x:f>
@@ -4929,28 +4411,28 @@
         <x:v>46349</x:v>
       </x:c>
       <x:c r="B14" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A14)</x:f>
-        <x:v>50</x:v>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A14)</x:f>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C14" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A14,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A14,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D14" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A14)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A14)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E14" s="6" t="n">
-        <x:f>MAX(C14-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A14,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C14-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A14,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F14" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A14,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C14,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A14,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C14,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G14" s="6" t="n">
         <x:f>MAX(B14-D14,0)</x:f>
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H14" s="10" t="n">
         <x:f>IF(B14=0,0,D14/B14)</x:f>
@@ -4962,28 +4444,28 @@
         <x:v>46356</x:v>
       </x:c>
       <x:c r="B15" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A15)</x:f>
-        <x:v>50</x:v>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A15)</x:f>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C15" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A15,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A15,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D15" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A15)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A15)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E15" s="6" t="n">
-        <x:f>MAX(C15-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A15,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C15-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A15,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F15" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A15,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C15,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A15,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C15,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G15" s="6" t="n">
         <x:f>MAX(B15-D15,0)</x:f>
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H15" s="10" t="n">
         <x:f>IF(B15=0,0,D15/B15)</x:f>
@@ -4995,28 +4477,28 @@
         <x:v>46363</x:v>
       </x:c>
       <x:c r="B16" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A16)</x:f>
-        <x:v>50</x:v>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A16)</x:f>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C16" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A16,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A16,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D16" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A16)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A16)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E16" s="6" t="n">
-        <x:f>MAX(C16-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A16,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C16-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A16,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F16" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A16,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C16,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A16,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C16,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G16" s="6" t="n">
         <x:f>MAX(B16-D16,0)</x:f>
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H16" s="10" t="n">
         <x:f>IF(B16=0,0,D16/B16)</x:f>
@@ -5028,28 +4510,28 @@
         <x:v>46370</x:v>
       </x:c>
       <x:c r="B17" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A17)</x:f>
-        <x:v>50</x:v>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A17)</x:f>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C17" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A17,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A17,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D17" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A17)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A17)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E17" s="6" t="n">
-        <x:f>MAX(C17-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A17,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C17-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A17,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F17" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A17,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C17,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A17,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C17,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G17" s="6" t="n">
         <x:f>MAX(B17-D17,0)</x:f>
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H17" s="10" t="n">
         <x:f>IF(B17=0,0,D17/B17)</x:f>
@@ -5061,28 +4543,28 @@
         <x:v>46377</x:v>
       </x:c>
       <x:c r="B18" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A18)</x:f>
-        <x:v>50</x:v>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A18)</x:f>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C18" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A18,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A18,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D18" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A18)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A18)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E18" s="6" t="n">
-        <x:f>MAX(C18-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A18,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C18-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A18,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F18" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A18,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C18,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A18,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C18,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G18" s="6" t="n">
         <x:f>MAX(B18-D18,0)</x:f>
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H18" s="10" t="n">
         <x:f>IF(B18=0,0,D18/B18)</x:f>
@@ -5094,28 +4576,28 @@
         <x:v>46384</x:v>
       </x:c>
       <x:c r="B19" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A19)</x:f>
-        <x:v>50</x:v>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A19)</x:f>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C19" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A19,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A19,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D19" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A19)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A19)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E19" s="6" t="n">
-        <x:f>MAX(C19-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A19,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C19-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A19,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F19" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A19,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C19,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A19,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C19,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G19" s="6" t="n">
         <x:f>MAX(B19-D19,0)</x:f>
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H19" s="10" t="n">
         <x:f>IF(B19=0,0,D19/B19)</x:f>
@@ -5127,28 +4609,28 @@
         <x:v>46391</x:v>
       </x:c>
       <x:c r="B20" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A20)</x:f>
-        <x:v>50</x:v>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A20)</x:f>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C20" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A20,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A20,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D20" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A20)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A20)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E20" s="6" t="n">
-        <x:f>MAX(C20-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A20,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C20-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A20,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F20" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A20,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C20,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A20,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C20,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G20" s="6" t="n">
         <x:f>MAX(B20-D20,0)</x:f>
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H20" s="10" t="n">
         <x:f>IF(B20=0,0,D20/B20)</x:f>
@@ -5160,28 +4642,28 @@
         <x:v>46398</x:v>
       </x:c>
       <x:c r="B21" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A21)</x:f>
-        <x:v>50</x:v>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A21)</x:f>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C21" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A21,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A21,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D21" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A21)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A21)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E21" s="6" t="n">
-        <x:f>MAX(C21-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A21,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C21-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A21,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F21" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A21,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C21,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A21,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C21,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G21" s="6" t="n">
         <x:f>MAX(B21-D21,0)</x:f>
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H21" s="10" t="n">
         <x:f>IF(B21=0,0,D21/B21)</x:f>
@@ -5193,102 +4675,36 @@
         <x:v>46405</x:v>
       </x:c>
       <x:c r="B22" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A22)</x:f>
-        <x:v>50</x:v>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A22)</x:f>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C22" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A22,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A22,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D22" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A22)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A22)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E22" s="6" t="n">
-        <x:f>MAX(C22-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A22,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C22-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A22,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F22" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A22,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C22,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A22,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C22,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G22" s="6" t="n">
         <x:f>MAX(B22-D22,0)</x:f>
-        <x:v>50</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="H22" s="10" t="n">
         <x:f>IF(B22=0,0,D22/B22)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="22" customHeight="1">
-      <x:c r="A23" s="7" t="n">
-        <x:v>46412</x:v>
-      </x:c>
-      <x:c r="B23" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A23)</x:f>
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="C23" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A23,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D23" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A23)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E23" s="6" t="n">
-        <x:f>MAX(C23-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A23,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F23" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A23,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C23,0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G23" s="6" t="n">
-        <x:f>MAX(B23-D23,0)</x:f>
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="H23" s="10" t="n">
-        <x:f>IF(B23=0,0,D23/B23)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="22" customHeight="1">
-      <x:c r="A24" s="7" t="n">
-        <x:v>46419</x:v>
-      </x:c>
-      <x:c r="B24" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A24)</x:f>
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="C24" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$130,'Daily'!$C$15:$C$130,A24,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D24" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A24)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E24" s="6" t="n">
-        <x:f>MAX(C24-SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A24,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F24" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$130,'Daily'!$C$15:$C$130,A24,'Daily'!$A$15:$A$130,"&lt;"&amp;'Daily'!$B$4)-C24,0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G24" s="6" t="n">
-        <x:f>MAX(B24-D24,0)</x:f>
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="H24" s="10" t="n">
-        <x:f>IF(B24=0,0,D24/B24)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E8:E24">
+  <x:conditionalFormatting sqref="E8:E22">
     <x:cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
       <x:formula>0</x:formula>
     </x:cfRule>
@@ -5856,4 +5272,143 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="65" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>Confirmed time by source topic</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>Exact source labels. Mixed/setup time does not prove technology proficiency.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="28" customHeight="1">
+      <x:c r="A6" s="3" t="str">
+        <x:v>Source topic</x:v>
+      </x:c>
+      <x:c r="B6" s="3" t="str">
+        <x:v>Confirmed hours</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="1" t="str">
+        <x:v>Python / RRDAP: RDS-001 Product Catalogue</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="n">
+        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A7,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>0.5175</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="1" t="str">
+        <x:v>Python / RRDAP: setup and RDS-001</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="n">
+        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A8,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>2.225277777777778</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="1" t="str">
+        <x:v>Python / RetailFlow: setup and RF-001</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="n">
+        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A9,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>1.0919444444444444</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="1" t="str">
+        <x:v>Python: CSV reading and writing</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="n">
+        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A10,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>0.12722222222222224</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="1" t="str">
+        <x:v>Python: CSV writing and read-back</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="n">
+        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A11,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>2.8175000000000003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="1" t="str">
+        <x:v>Python: cleaner changed-input check</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="n">
+        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A12,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>0.4911111111111111</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="1" t="str">
+        <x:v>Python: dictionary foundations in Jupyter</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="n">
+        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A13,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>1.6424999999994445</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="1" t="str">
+        <x:v>Python: dictionary records baseline</x:v>
+      </x:c>
+      <x:c r="B14" s="6" t="n">
+        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A14,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>0.21111111111166667</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="1" t="str">
+        <x:v>Python: record cleaning</x:v>
+      </x:c>
+      <x:c r="B15" s="6" t="n">
+        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A15,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>0.22972222222166666</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="1" t="str">
+        <x:v>Python: valid and rejected record lists</x:v>
+      </x:c>
+      <x:c r="B16" s="6" t="n">
+        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A16,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>0.28194444444444444</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="1" t="str">
+        <x:v>SQL: LEFT JOIN and unmatched rows</x:v>
+      </x:c>
+      <x:c r="B17" s="6" t="n">
+        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A17,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>0.34055555555666667</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="1" t="str">
+        <x:v>SQL: joins counting grouping and SUM setup</x:v>
+      </x:c>
+      <x:c r="B18" s="6" t="n">
+        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A18,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>1.175</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Integrate Azure planning and interview evidence into RecallLab
</commit_message>
<xml_diff>
--- a/outputs/study-tracker/study-hours.xlsx
+++ b/outputs/study-tracker/study-hours.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="R645b99787c3941f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="R3a925f8c45464b2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="Reb46c3304c5a464d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topics" sheetId="4" r:id="Rfdc3a107eac445e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="Re7d9407a13c04fb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="Rc18eca6f7d664cc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="R2b7f1bf16c34408b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topics" sheetId="4" r:id="R9a41b58d40084752"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4213,23 +4213,23 @@
         <x:v>46307</x:v>
       </x:c>
       <x:c r="B8" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A8)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A8,'Daily'!$A$15:$A$114,"&lt;=46313")</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="C8" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A8,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A8,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46313")</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="D8" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A8)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A8,'Daily'!$A$15:$A$114,"&lt;=46313")</x:f>
         <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="E8" s="6" t="n">
-        <x:f>MAX(C8-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A8,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C8-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A8,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46313"),0)</x:f>
         <x:v>20.848611111110557</x:v>
       </x:c>
       <x:c r="F8" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A8,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C8,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A8,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46313")-C8,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G8" s="6" t="n">
@@ -4246,23 +4246,23 @@
         <x:v>46314</x:v>
       </x:c>
       <x:c r="B9" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A9)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A9,'Daily'!$A$15:$A$114,"&lt;=46320")</x:f>
         <x:v>52</x:v>
       </x:c>
       <x:c r="C9" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A9,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A9,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46320")</x:f>
         <x:v>18</x:v>
       </x:c>
       <x:c r="D9" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A9)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A9,'Daily'!$A$15:$A$114,"&lt;=46320")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E9" s="6" t="n">
-        <x:f>MAX(C9-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A9,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C9-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A9,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46320"),0)</x:f>
         <x:v>18</x:v>
       </x:c>
       <x:c r="F9" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A9,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C9,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A9,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46320")-C9,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G9" s="6" t="n">
@@ -4279,23 +4279,23 @@
         <x:v>46321</x:v>
       </x:c>
       <x:c r="B10" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A10)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A10,'Daily'!$A$15:$A$114,"&lt;=46327")</x:f>
         <x:v>55</x:v>
       </x:c>
       <x:c r="C10" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A10,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A10,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46327")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D10" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A10)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A10,'Daily'!$A$15:$A$114,"&lt;=46327")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E10" s="6" t="n">
-        <x:f>MAX(C10-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A10,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C10-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A10,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46327"),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F10" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A10,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C10,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A10,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46327")-C10,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G10" s="6" t="n">
@@ -4312,23 +4312,23 @@
         <x:v>46328</x:v>
       </x:c>
       <x:c r="B11" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A11)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A11,'Daily'!$A$15:$A$114,"&lt;=46334")</x:f>
         <x:v>55</x:v>
       </x:c>
       <x:c r="C11" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A11,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A11,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46334")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D11" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A11)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A11,'Daily'!$A$15:$A$114,"&lt;=46334")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E11" s="6" t="n">
-        <x:f>MAX(C11-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A11,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C11-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A11,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46334"),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F11" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A11,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C11,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A11,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46334")-C11,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G11" s="6" t="n">
@@ -4345,23 +4345,23 @@
         <x:v>46335</x:v>
       </x:c>
       <x:c r="B12" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A12)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A12,'Daily'!$A$15:$A$114,"&lt;=46341")</x:f>
         <x:v>55</x:v>
       </x:c>
       <x:c r="C12" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A12,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A12,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46341")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D12" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A12)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A12,'Daily'!$A$15:$A$114,"&lt;=46341")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E12" s="6" t="n">
-        <x:f>MAX(C12-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A12,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C12-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A12,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46341"),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F12" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A12,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C12,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A12,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46341")-C12,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G12" s="6" t="n">
@@ -4378,23 +4378,23 @@
         <x:v>46342</x:v>
       </x:c>
       <x:c r="B13" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A13)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A13,'Daily'!$A$15:$A$114,"&lt;=46348")</x:f>
         <x:v>55</x:v>
       </x:c>
       <x:c r="C13" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A13,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A13,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46348")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D13" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A13)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A13,'Daily'!$A$15:$A$114,"&lt;=46348")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E13" s="6" t="n">
-        <x:f>MAX(C13-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A13,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C13-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A13,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46348"),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F13" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A13,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C13,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A13,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46348")-C13,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G13" s="6" t="n">
@@ -4411,23 +4411,23 @@
         <x:v>46349</x:v>
       </x:c>
       <x:c r="B14" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A14)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A14,'Daily'!$A$15:$A$114,"&lt;=46355")</x:f>
         <x:v>55</x:v>
       </x:c>
       <x:c r="C14" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A14,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A14,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46355")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D14" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A14)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A14,'Daily'!$A$15:$A$114,"&lt;=46355")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E14" s="6" t="n">
-        <x:f>MAX(C14-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A14,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C14-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A14,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46355"),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F14" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A14,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C14,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A14,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46355")-C14,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G14" s="6" t="n">
@@ -4444,23 +4444,23 @@
         <x:v>46356</x:v>
       </x:c>
       <x:c r="B15" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A15)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A15,'Daily'!$A$15:$A$114,"&lt;=46362")</x:f>
         <x:v>55</x:v>
       </x:c>
       <x:c r="C15" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A15,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A15,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46362")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D15" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A15)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A15,'Daily'!$A$15:$A$114,"&lt;=46362")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E15" s="6" t="n">
-        <x:f>MAX(C15-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A15,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C15-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A15,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46362"),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F15" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A15,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C15,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A15,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46362")-C15,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G15" s="6" t="n">
@@ -4477,23 +4477,23 @@
         <x:v>46363</x:v>
       </x:c>
       <x:c r="B16" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A16)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A16,'Daily'!$A$15:$A$114,"&lt;=46369")</x:f>
         <x:v>55</x:v>
       </x:c>
       <x:c r="C16" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A16,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A16,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46369")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D16" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A16)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A16,'Daily'!$A$15:$A$114,"&lt;=46369")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E16" s="6" t="n">
-        <x:f>MAX(C16-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A16,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C16-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A16,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46369"),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F16" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A16,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C16,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A16,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46369")-C16,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G16" s="6" t="n">
@@ -4510,23 +4510,23 @@
         <x:v>46370</x:v>
       </x:c>
       <x:c r="B17" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A17)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A17,'Daily'!$A$15:$A$114,"&lt;=46376")</x:f>
         <x:v>55</x:v>
       </x:c>
       <x:c r="C17" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A17,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A17,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46376")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D17" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A17)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A17,'Daily'!$A$15:$A$114,"&lt;=46376")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E17" s="6" t="n">
-        <x:f>MAX(C17-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A17,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C17-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A17,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46376"),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F17" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A17,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C17,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A17,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46376")-C17,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G17" s="6" t="n">
@@ -4543,23 +4543,23 @@
         <x:v>46377</x:v>
       </x:c>
       <x:c r="B18" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A18)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A18,'Daily'!$A$15:$A$114,"&lt;=46383")</x:f>
         <x:v>55</x:v>
       </x:c>
       <x:c r="C18" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A18,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A18,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46383")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D18" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A18)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A18,'Daily'!$A$15:$A$114,"&lt;=46383")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E18" s="6" t="n">
-        <x:f>MAX(C18-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A18,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C18-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A18,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46383"),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F18" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A18,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C18,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A18,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46383")-C18,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G18" s="6" t="n">
@@ -4576,23 +4576,23 @@
         <x:v>46384</x:v>
       </x:c>
       <x:c r="B19" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A19)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A19,'Daily'!$A$15:$A$114,"&lt;=46390")</x:f>
         <x:v>55</x:v>
       </x:c>
       <x:c r="C19" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A19,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A19,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46390")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D19" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A19)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A19,'Daily'!$A$15:$A$114,"&lt;=46390")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E19" s="6" t="n">
-        <x:f>MAX(C19-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A19,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C19-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A19,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46390"),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F19" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A19,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C19,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A19,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46390")-C19,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G19" s="6" t="n">
@@ -4609,23 +4609,23 @@
         <x:v>46391</x:v>
       </x:c>
       <x:c r="B20" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A20)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A20,'Daily'!$A$15:$A$114,"&lt;=46397")</x:f>
         <x:v>55</x:v>
       </x:c>
       <x:c r="C20" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A20,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A20,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46397")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D20" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A20)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A20,'Daily'!$A$15:$A$114,"&lt;=46397")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E20" s="6" t="n">
-        <x:f>MAX(C20-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A20,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C20-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A20,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46397"),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F20" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A20,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C20,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A20,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46397")-C20,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G20" s="6" t="n">
@@ -4642,23 +4642,23 @@
         <x:v>46398</x:v>
       </x:c>
       <x:c r="B21" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A21)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A21,'Daily'!$A$15:$A$114,"&lt;=46404")</x:f>
         <x:v>55</x:v>
       </x:c>
       <x:c r="C21" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A21,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A21,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46404")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D21" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A21)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A21,'Daily'!$A$15:$A$114,"&lt;=46404")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E21" s="6" t="n">
-        <x:f>MAX(C21-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A21,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C21-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A21,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46404"),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F21" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A21,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C21,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A21,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46404")-C21,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G21" s="6" t="n">
@@ -4675,23 +4675,23 @@
         <x:v>46405</x:v>
       </x:c>
       <x:c r="B22" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A22)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A22,'Daily'!$A$15:$A$114,"&lt;=46409")</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="C22" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A22,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)</x:f>
+        <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A22,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46409")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D22" s="6" t="n">
-        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A22)</x:f>
+        <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A22,'Daily'!$A$15:$A$114,"&lt;=46409")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E22" s="6" t="n">
-        <x:f>MAX(C22-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A22,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4),0)</x:f>
+        <x:f>MAX(C22-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A22,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46409"),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F22" s="6" t="n">
-        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A22,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4)-C22,0)</x:f>
+        <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A22,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46409")-C22,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G22" s="6" t="n">

</xml_diff>

<commit_message>
Record Docker Pomodoro study handoff
</commit_message>
<xml_diff>
--- a/outputs/study-tracker/study-hours.xlsx
+++ b/outputs/study-tracker/study-hours.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="Re7d9407a13c04fb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="Rc18eca6f7d664cc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="R2b7f1bf16c34408b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topics" sheetId="4" r:id="R9a41b58d40084752"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="R35b5850a463f4db2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="Rbf4a57caa0a24116"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="Rdcc5475745e04ea2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topics" sheetId="4" r:id="R284dfcb8e72f4883"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -581,7 +581,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E15" s="6" t="n">
-        <x:f>IF(A15&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A15,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A15&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A15,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
         <x:v>2.8094444444449995</x:v>
       </x:c>
       <x:c r="F15" s="6" t="n">
@@ -601,7 +601,7 @@
         <x:v>2.8094444444449995</x:v>
       </x:c>
       <x:c r="J15" s="1" t="str">
-        <x:f>IF(A15&gt;$B$4,"Future",IF(A15=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A15,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E15=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A15&gt;$B$4,"Future",IF(A15=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A15,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E15=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Uncertain time</x:v>
       </x:c>
     </x:row>
@@ -621,7 +621,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E16" s="6" t="n">
-        <x:f>IF(A16&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A16,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A16&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A16,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
         <x:v>1.6897222222222223</x:v>
       </x:c>
       <x:c r="F16" s="6" t="n">
@@ -641,7 +641,7 @@
         <x:v>4.499166666667222</x:v>
       </x:c>
       <x:c r="J16" s="1" t="str">
-        <x:f>IF(A16&gt;$B$4,"Future",IF(A16=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A16,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E16=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A16&gt;$B$4,"Future",IF(A16=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A16,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E16=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Logged</x:v>
       </x:c>
     </x:row>
@@ -661,7 +661,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E17" s="6" t="n">
-        <x:f>IF(A17&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A17,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A17&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A17,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
         <x:v>6.652222222222223</x:v>
       </x:c>
       <x:c r="F17" s="6" t="n">
@@ -681,7 +681,7 @@
         <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J17" s="1" t="str">
-        <x:f>IF(A17&gt;$B$4,"Future",IF(A17=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A17,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E17=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A17&gt;$B$4,"Future",IF(A17=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A17,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E17=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Logged</x:v>
       </x:c>
     </x:row>
@@ -701,7 +701,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E18" s="6" t="n">
-        <x:f>IF(A18&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A18,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A18&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A18,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F18" s="6" t="n">
@@ -721,7 +721,7 @@
         <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J18" s="1" t="str">
-        <x:f>IF(A18&gt;$B$4,"Future",IF(A18=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A18,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E18=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A18&gt;$B$4,"Future",IF(A18=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A18,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E18=0,"No confirmed time","Logged"))))</x:f>
         <x:v>No confirmed time</x:v>
       </x:c>
     </x:row>
@@ -741,7 +741,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E19" s="6" t="n">
-        <x:f>IF(A19&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A19,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A19&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A19,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F19" s="6" t="n">
@@ -761,7 +761,7 @@
         <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J19" s="1" t="str">
-        <x:f>IF(A19&gt;$B$4,"Future",IF(A19=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A19,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E19=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A19&gt;$B$4,"Future",IF(A19=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A19,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E19=0,"No confirmed time","Logged"))))</x:f>
         <x:v>No confirmed time</x:v>
       </x:c>
     </x:row>
@@ -781,7 +781,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E20" s="6" t="n">
-        <x:f>IF(A20&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A20,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A20&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A20,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F20" s="6" t="n">
@@ -801,7 +801,7 @@
         <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J20" s="1" t="str">
-        <x:f>IF(A20&gt;$B$4,"Future",IF(A20=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A20,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E20=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A20&gt;$B$4,"Future",IF(A20=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A20,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E20=0,"No confirmed time","Logged"))))</x:f>
         <x:v>No confirmed time</x:v>
       </x:c>
     </x:row>
@@ -821,7 +821,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E21" s="6" t="n">
-        <x:f>IF(A21&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A21,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A21&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A21,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F21" s="6" t="n">
@@ -841,7 +841,7 @@
         <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J21" s="1" t="str">
-        <x:f>IF(A21&gt;$B$4,"Future",IF(A21=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A21,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E21=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A21&gt;$B$4,"Future",IF(A21=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A21,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E21=0,"No confirmed time","Logged"))))</x:f>
         <x:v>No confirmed time</x:v>
       </x:c>
     </x:row>
@@ -861,7 +861,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E22" s="6" t="n">
-        <x:f>IF(A22&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A22,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A22&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A22,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F22" s="6" t="str">
@@ -878,7 +878,7 @@
         <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J22" s="1" t="str">
-        <x:f>IF(A22&gt;$B$4,"Future",IF(A22=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A22,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E22=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A22&gt;$B$4,"Future",IF(A22=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A22,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E22=0,"No confirmed time","Logged"))))</x:f>
         <x:v>In progress</x:v>
       </x:c>
     </x:row>
@@ -898,7 +898,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E23" s="6" t="str">
-        <x:f>IF(A23&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A23,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A23&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A23,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F23" s="6" t="str">
         <x:f>IF(A23&gt;=$B$4,"",MAX(D23-E23,0))</x:f>
@@ -913,7 +913,7 @@
         <x:f>IF(A23&gt;$B$4,"",SUM($E$15:E23))</x:f>
       </x:c>
       <x:c r="J23" s="1" t="str">
-        <x:f>IF(A23&gt;$B$4,"Future",IF(A23=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A23,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E23=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A23&gt;$B$4,"Future",IF(A23=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A23,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E23=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -933,7 +933,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E24" s="6" t="str">
-        <x:f>IF(A24&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A24,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A24&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A24,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F24" s="6" t="str">
         <x:f>IF(A24&gt;=$B$4,"",MAX(D24-E24,0))</x:f>
@@ -948,7 +948,7 @@
         <x:f>IF(A24&gt;$B$4,"",SUM($E$15:E24))</x:f>
       </x:c>
       <x:c r="J24" s="1" t="str">
-        <x:f>IF(A24&gt;$B$4,"Future",IF(A24=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A24,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E24=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A24&gt;$B$4,"Future",IF(A24=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A24,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E24=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -968,7 +968,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E25" s="6" t="str">
-        <x:f>IF(A25&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A25,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A25&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A25,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F25" s="6" t="str">
         <x:f>IF(A25&gt;=$B$4,"",MAX(D25-E25,0))</x:f>
@@ -983,7 +983,7 @@
         <x:f>IF(A25&gt;$B$4,"",SUM($E$15:E25))</x:f>
       </x:c>
       <x:c r="J25" s="1" t="str">
-        <x:f>IF(A25&gt;$B$4,"Future",IF(A25=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A25,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E25=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A25&gt;$B$4,"Future",IF(A25=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A25,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E25=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1003,7 +1003,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E26" s="6" t="str">
-        <x:f>IF(A26&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A26,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A26&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A26,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F26" s="6" t="str">
         <x:f>IF(A26&gt;=$B$4,"",MAX(D26-E26,0))</x:f>
@@ -1018,7 +1018,7 @@
         <x:f>IF(A26&gt;$B$4,"",SUM($E$15:E26))</x:f>
       </x:c>
       <x:c r="J26" s="1" t="str">
-        <x:f>IF(A26&gt;$B$4,"Future",IF(A26=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A26,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E26=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A26&gt;$B$4,"Future",IF(A26=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A26,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E26=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1038,7 +1038,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E27" s="6" t="str">
-        <x:f>IF(A27&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A27,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A27&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A27,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F27" s="6" t="str">
         <x:f>IF(A27&gt;=$B$4,"",MAX(D27-E27,0))</x:f>
@@ -1053,7 +1053,7 @@
         <x:f>IF(A27&gt;$B$4,"",SUM($E$15:E27))</x:f>
       </x:c>
       <x:c r="J27" s="1" t="str">
-        <x:f>IF(A27&gt;$B$4,"Future",IF(A27=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A27,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E27=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A27&gt;$B$4,"Future",IF(A27=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A27,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E27=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1073,7 +1073,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E28" s="6" t="str">
-        <x:f>IF(A28&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A28,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A28&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A28,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F28" s="6" t="str">
         <x:f>IF(A28&gt;=$B$4,"",MAX(D28-E28,0))</x:f>
@@ -1088,7 +1088,7 @@
         <x:f>IF(A28&gt;$B$4,"",SUM($E$15:E28))</x:f>
       </x:c>
       <x:c r="J28" s="1" t="str">
-        <x:f>IF(A28&gt;$B$4,"Future",IF(A28=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A28,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E28=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A28&gt;$B$4,"Future",IF(A28=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A28,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E28=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1108,7 +1108,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E29" s="6" t="str">
-        <x:f>IF(A29&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A29,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A29&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A29,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F29" s="6" t="str">
         <x:f>IF(A29&gt;=$B$4,"",MAX(D29-E29,0))</x:f>
@@ -1123,7 +1123,7 @@
         <x:f>IF(A29&gt;$B$4,"",SUM($E$15:E29))</x:f>
       </x:c>
       <x:c r="J29" s="1" t="str">
-        <x:f>IF(A29&gt;$B$4,"Future",IF(A29=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A29,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E29=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A29&gt;$B$4,"Future",IF(A29=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A29,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E29=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1143,7 +1143,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E30" s="6" t="str">
-        <x:f>IF(A30&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A30,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A30&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A30,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F30" s="6" t="str">
         <x:f>IF(A30&gt;=$B$4,"",MAX(D30-E30,0))</x:f>
@@ -1158,7 +1158,7 @@
         <x:f>IF(A30&gt;$B$4,"",SUM($E$15:E30))</x:f>
       </x:c>
       <x:c r="J30" s="1" t="str">
-        <x:f>IF(A30&gt;$B$4,"Future",IF(A30=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A30,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E30=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A30&gt;$B$4,"Future",IF(A30=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A30,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E30=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1178,7 +1178,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E31" s="6" t="str">
-        <x:f>IF(A31&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A31,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A31&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A31,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F31" s="6" t="str">
         <x:f>IF(A31&gt;=$B$4,"",MAX(D31-E31,0))</x:f>
@@ -1193,7 +1193,7 @@
         <x:f>IF(A31&gt;$B$4,"",SUM($E$15:E31))</x:f>
       </x:c>
       <x:c r="J31" s="1" t="str">
-        <x:f>IF(A31&gt;$B$4,"Future",IF(A31=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A31,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E31=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A31&gt;$B$4,"Future",IF(A31=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A31,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E31=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1213,7 +1213,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E32" s="6" t="str">
-        <x:f>IF(A32&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A32,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A32&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A32,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F32" s="6" t="str">
         <x:f>IF(A32&gt;=$B$4,"",MAX(D32-E32,0))</x:f>
@@ -1228,7 +1228,7 @@
         <x:f>IF(A32&gt;$B$4,"",SUM($E$15:E32))</x:f>
       </x:c>
       <x:c r="J32" s="1" t="str">
-        <x:f>IF(A32&gt;$B$4,"Future",IF(A32=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A32,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E32=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A32&gt;$B$4,"Future",IF(A32=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A32,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E32=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1248,7 +1248,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E33" s="6" t="str">
-        <x:f>IF(A33&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A33,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A33&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A33,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F33" s="6" t="str">
         <x:f>IF(A33&gt;=$B$4,"",MAX(D33-E33,0))</x:f>
@@ -1263,7 +1263,7 @@
         <x:f>IF(A33&gt;$B$4,"",SUM($E$15:E33))</x:f>
       </x:c>
       <x:c r="J33" s="1" t="str">
-        <x:f>IF(A33&gt;$B$4,"Future",IF(A33=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A33,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E33=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A33&gt;$B$4,"Future",IF(A33=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A33,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E33=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1283,7 +1283,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E34" s="6" t="str">
-        <x:f>IF(A34&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A34,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A34&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A34,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F34" s="6" t="str">
         <x:f>IF(A34&gt;=$B$4,"",MAX(D34-E34,0))</x:f>
@@ -1298,7 +1298,7 @@
         <x:f>IF(A34&gt;$B$4,"",SUM($E$15:E34))</x:f>
       </x:c>
       <x:c r="J34" s="1" t="str">
-        <x:f>IF(A34&gt;$B$4,"Future",IF(A34=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A34,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E34=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A34&gt;$B$4,"Future",IF(A34=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A34,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E34=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1318,7 +1318,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E35" s="6" t="str">
-        <x:f>IF(A35&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A35,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A35&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A35,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F35" s="6" t="str">
         <x:f>IF(A35&gt;=$B$4,"",MAX(D35-E35,0))</x:f>
@@ -1333,7 +1333,7 @@
         <x:f>IF(A35&gt;$B$4,"",SUM($E$15:E35))</x:f>
       </x:c>
       <x:c r="J35" s="1" t="str">
-        <x:f>IF(A35&gt;$B$4,"Future",IF(A35=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A35,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E35=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A35&gt;$B$4,"Future",IF(A35=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A35,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E35=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1353,7 +1353,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E36" s="6" t="str">
-        <x:f>IF(A36&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A36,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A36&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A36,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F36" s="6" t="str">
         <x:f>IF(A36&gt;=$B$4,"",MAX(D36-E36,0))</x:f>
@@ -1368,7 +1368,7 @@
         <x:f>IF(A36&gt;$B$4,"",SUM($E$15:E36))</x:f>
       </x:c>
       <x:c r="J36" s="1" t="str">
-        <x:f>IF(A36&gt;$B$4,"Future",IF(A36=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A36,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E36=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A36&gt;$B$4,"Future",IF(A36=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A36,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E36=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1388,7 +1388,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E37" s="6" t="str">
-        <x:f>IF(A37&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A37,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A37&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A37,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F37" s="6" t="str">
         <x:f>IF(A37&gt;=$B$4,"",MAX(D37-E37,0))</x:f>
@@ -1403,7 +1403,7 @@
         <x:f>IF(A37&gt;$B$4,"",SUM($E$15:E37))</x:f>
       </x:c>
       <x:c r="J37" s="1" t="str">
-        <x:f>IF(A37&gt;$B$4,"Future",IF(A37=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A37,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E37=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A37&gt;$B$4,"Future",IF(A37=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A37,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E37=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1423,7 +1423,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E38" s="6" t="str">
-        <x:f>IF(A38&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A38,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A38&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A38,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F38" s="6" t="str">
         <x:f>IF(A38&gt;=$B$4,"",MAX(D38-E38,0))</x:f>
@@ -1438,7 +1438,7 @@
         <x:f>IF(A38&gt;$B$4,"",SUM($E$15:E38))</x:f>
       </x:c>
       <x:c r="J38" s="1" t="str">
-        <x:f>IF(A38&gt;$B$4,"Future",IF(A38=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A38,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E38=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A38&gt;$B$4,"Future",IF(A38=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A38,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E38=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1458,7 +1458,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E39" s="6" t="str">
-        <x:f>IF(A39&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A39,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A39&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A39,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F39" s="6" t="str">
         <x:f>IF(A39&gt;=$B$4,"",MAX(D39-E39,0))</x:f>
@@ -1473,7 +1473,7 @@
         <x:f>IF(A39&gt;$B$4,"",SUM($E$15:E39))</x:f>
       </x:c>
       <x:c r="J39" s="1" t="str">
-        <x:f>IF(A39&gt;$B$4,"Future",IF(A39=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A39,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E39=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A39&gt;$B$4,"Future",IF(A39=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A39,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E39=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1493,7 +1493,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E40" s="6" t="str">
-        <x:f>IF(A40&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A40,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A40&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A40,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F40" s="6" t="str">
         <x:f>IF(A40&gt;=$B$4,"",MAX(D40-E40,0))</x:f>
@@ -1508,7 +1508,7 @@
         <x:f>IF(A40&gt;$B$4,"",SUM($E$15:E40))</x:f>
       </x:c>
       <x:c r="J40" s="1" t="str">
-        <x:f>IF(A40&gt;$B$4,"Future",IF(A40=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A40,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E40=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A40&gt;$B$4,"Future",IF(A40=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A40,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E40=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1528,7 +1528,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E41" s="6" t="str">
-        <x:f>IF(A41&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A41,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A41&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A41,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F41" s="6" t="str">
         <x:f>IF(A41&gt;=$B$4,"",MAX(D41-E41,0))</x:f>
@@ -1543,7 +1543,7 @@
         <x:f>IF(A41&gt;$B$4,"",SUM($E$15:E41))</x:f>
       </x:c>
       <x:c r="J41" s="1" t="str">
-        <x:f>IF(A41&gt;$B$4,"Future",IF(A41=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A41,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E41=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A41&gt;$B$4,"Future",IF(A41=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A41,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E41=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1563,7 +1563,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E42" s="6" t="str">
-        <x:f>IF(A42&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A42,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A42&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A42,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F42" s="6" t="str">
         <x:f>IF(A42&gt;=$B$4,"",MAX(D42-E42,0))</x:f>
@@ -1578,7 +1578,7 @@
         <x:f>IF(A42&gt;$B$4,"",SUM($E$15:E42))</x:f>
       </x:c>
       <x:c r="J42" s="1" t="str">
-        <x:f>IF(A42&gt;$B$4,"Future",IF(A42=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A42,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E42=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A42&gt;$B$4,"Future",IF(A42=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A42,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E42=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1598,7 +1598,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E43" s="6" t="str">
-        <x:f>IF(A43&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A43,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A43&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A43,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F43" s="6" t="str">
         <x:f>IF(A43&gt;=$B$4,"",MAX(D43-E43,0))</x:f>
@@ -1613,7 +1613,7 @@
         <x:f>IF(A43&gt;$B$4,"",SUM($E$15:E43))</x:f>
       </x:c>
       <x:c r="J43" s="1" t="str">
-        <x:f>IF(A43&gt;$B$4,"Future",IF(A43=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A43,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E43=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A43&gt;$B$4,"Future",IF(A43=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A43,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E43=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1633,7 +1633,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E44" s="6" t="str">
-        <x:f>IF(A44&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A44,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A44&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A44,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F44" s="6" t="str">
         <x:f>IF(A44&gt;=$B$4,"",MAX(D44-E44,0))</x:f>
@@ -1648,7 +1648,7 @@
         <x:f>IF(A44&gt;$B$4,"",SUM($E$15:E44))</x:f>
       </x:c>
       <x:c r="J44" s="1" t="str">
-        <x:f>IF(A44&gt;$B$4,"Future",IF(A44=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A44,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E44=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A44&gt;$B$4,"Future",IF(A44=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A44,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E44=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1668,7 +1668,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E45" s="6" t="str">
-        <x:f>IF(A45&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A45,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A45&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A45,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F45" s="6" t="str">
         <x:f>IF(A45&gt;=$B$4,"",MAX(D45-E45,0))</x:f>
@@ -1683,7 +1683,7 @@
         <x:f>IF(A45&gt;$B$4,"",SUM($E$15:E45))</x:f>
       </x:c>
       <x:c r="J45" s="1" t="str">
-        <x:f>IF(A45&gt;$B$4,"Future",IF(A45=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A45,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E45=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A45&gt;$B$4,"Future",IF(A45=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A45,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E45=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1703,7 +1703,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E46" s="6" t="str">
-        <x:f>IF(A46&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A46,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A46&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A46,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F46" s="6" t="str">
         <x:f>IF(A46&gt;=$B$4,"",MAX(D46-E46,0))</x:f>
@@ -1718,7 +1718,7 @@
         <x:f>IF(A46&gt;$B$4,"",SUM($E$15:E46))</x:f>
       </x:c>
       <x:c r="J46" s="1" t="str">
-        <x:f>IF(A46&gt;$B$4,"Future",IF(A46=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A46,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E46=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A46&gt;$B$4,"Future",IF(A46=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A46,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E46=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1738,7 +1738,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E47" s="6" t="str">
-        <x:f>IF(A47&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A47,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A47&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A47,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F47" s="6" t="str">
         <x:f>IF(A47&gt;=$B$4,"",MAX(D47-E47,0))</x:f>
@@ -1753,7 +1753,7 @@
         <x:f>IF(A47&gt;$B$4,"",SUM($E$15:E47))</x:f>
       </x:c>
       <x:c r="J47" s="1" t="str">
-        <x:f>IF(A47&gt;$B$4,"Future",IF(A47=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A47,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E47=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A47&gt;$B$4,"Future",IF(A47=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A47,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E47=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1773,7 +1773,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E48" s="6" t="str">
-        <x:f>IF(A48&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A48,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A48&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A48,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F48" s="6" t="str">
         <x:f>IF(A48&gt;=$B$4,"",MAX(D48-E48,0))</x:f>
@@ -1788,7 +1788,7 @@
         <x:f>IF(A48&gt;$B$4,"",SUM($E$15:E48))</x:f>
       </x:c>
       <x:c r="J48" s="1" t="str">
-        <x:f>IF(A48&gt;$B$4,"Future",IF(A48=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A48,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E48=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A48&gt;$B$4,"Future",IF(A48=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A48,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E48=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1808,7 +1808,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E49" s="6" t="str">
-        <x:f>IF(A49&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A49,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A49&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A49,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F49" s="6" t="str">
         <x:f>IF(A49&gt;=$B$4,"",MAX(D49-E49,0))</x:f>
@@ -1823,7 +1823,7 @@
         <x:f>IF(A49&gt;$B$4,"",SUM($E$15:E49))</x:f>
       </x:c>
       <x:c r="J49" s="1" t="str">
-        <x:f>IF(A49&gt;$B$4,"Future",IF(A49=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A49,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E49=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A49&gt;$B$4,"Future",IF(A49=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A49,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E49=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1843,7 +1843,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E50" s="6" t="str">
-        <x:f>IF(A50&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A50,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A50&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A50,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F50" s="6" t="str">
         <x:f>IF(A50&gt;=$B$4,"",MAX(D50-E50,0))</x:f>
@@ -1858,7 +1858,7 @@
         <x:f>IF(A50&gt;$B$4,"",SUM($E$15:E50))</x:f>
       </x:c>
       <x:c r="J50" s="1" t="str">
-        <x:f>IF(A50&gt;$B$4,"Future",IF(A50=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A50,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E50=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A50&gt;$B$4,"Future",IF(A50=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A50,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E50=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1878,7 +1878,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E51" s="6" t="str">
-        <x:f>IF(A51&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A51,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A51&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A51,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F51" s="6" t="str">
         <x:f>IF(A51&gt;=$B$4,"",MAX(D51-E51,0))</x:f>
@@ -1893,7 +1893,7 @@
         <x:f>IF(A51&gt;$B$4,"",SUM($E$15:E51))</x:f>
       </x:c>
       <x:c r="J51" s="1" t="str">
-        <x:f>IF(A51&gt;$B$4,"Future",IF(A51=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A51,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E51=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A51&gt;$B$4,"Future",IF(A51=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A51,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E51=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1913,7 +1913,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E52" s="6" t="str">
-        <x:f>IF(A52&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A52,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A52&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A52,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F52" s="6" t="str">
         <x:f>IF(A52&gt;=$B$4,"",MAX(D52-E52,0))</x:f>
@@ -1928,7 +1928,7 @@
         <x:f>IF(A52&gt;$B$4,"",SUM($E$15:E52))</x:f>
       </x:c>
       <x:c r="J52" s="1" t="str">
-        <x:f>IF(A52&gt;$B$4,"Future",IF(A52=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A52,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E52=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A52&gt;$B$4,"Future",IF(A52=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A52,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E52=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1948,7 +1948,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E53" s="6" t="str">
-        <x:f>IF(A53&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A53,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A53&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A53,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F53" s="6" t="str">
         <x:f>IF(A53&gt;=$B$4,"",MAX(D53-E53,0))</x:f>
@@ -1963,7 +1963,7 @@
         <x:f>IF(A53&gt;$B$4,"",SUM($E$15:E53))</x:f>
       </x:c>
       <x:c r="J53" s="1" t="str">
-        <x:f>IF(A53&gt;$B$4,"Future",IF(A53=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A53,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E53=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A53&gt;$B$4,"Future",IF(A53=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A53,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E53=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1983,7 +1983,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E54" s="6" t="str">
-        <x:f>IF(A54&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A54,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A54&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A54,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F54" s="6" t="str">
         <x:f>IF(A54&gt;=$B$4,"",MAX(D54-E54,0))</x:f>
@@ -1998,7 +1998,7 @@
         <x:f>IF(A54&gt;$B$4,"",SUM($E$15:E54))</x:f>
       </x:c>
       <x:c r="J54" s="1" t="str">
-        <x:f>IF(A54&gt;$B$4,"Future",IF(A54=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A54,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E54=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A54&gt;$B$4,"Future",IF(A54=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A54,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E54=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2018,7 +2018,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E55" s="6" t="str">
-        <x:f>IF(A55&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A55,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A55&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A55,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F55" s="6" t="str">
         <x:f>IF(A55&gt;=$B$4,"",MAX(D55-E55,0))</x:f>
@@ -2033,7 +2033,7 @@
         <x:f>IF(A55&gt;$B$4,"",SUM($E$15:E55))</x:f>
       </x:c>
       <x:c r="J55" s="1" t="str">
-        <x:f>IF(A55&gt;$B$4,"Future",IF(A55=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A55,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E55=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A55&gt;$B$4,"Future",IF(A55=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A55,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E55=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2053,7 +2053,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E56" s="6" t="str">
-        <x:f>IF(A56&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A56,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A56&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A56,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F56" s="6" t="str">
         <x:f>IF(A56&gt;=$B$4,"",MAX(D56-E56,0))</x:f>
@@ -2068,7 +2068,7 @@
         <x:f>IF(A56&gt;$B$4,"",SUM($E$15:E56))</x:f>
       </x:c>
       <x:c r="J56" s="1" t="str">
-        <x:f>IF(A56&gt;$B$4,"Future",IF(A56=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A56,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E56=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A56&gt;$B$4,"Future",IF(A56=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A56,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E56=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2088,7 +2088,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E57" s="6" t="str">
-        <x:f>IF(A57&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A57,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A57&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A57,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F57" s="6" t="str">
         <x:f>IF(A57&gt;=$B$4,"",MAX(D57-E57,0))</x:f>
@@ -2103,7 +2103,7 @@
         <x:f>IF(A57&gt;$B$4,"",SUM($E$15:E57))</x:f>
       </x:c>
       <x:c r="J57" s="1" t="str">
-        <x:f>IF(A57&gt;$B$4,"Future",IF(A57=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A57,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E57=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A57&gt;$B$4,"Future",IF(A57=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A57,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E57=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2123,7 +2123,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E58" s="6" t="str">
-        <x:f>IF(A58&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A58,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A58&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A58,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F58" s="6" t="str">
         <x:f>IF(A58&gt;=$B$4,"",MAX(D58-E58,0))</x:f>
@@ -2138,7 +2138,7 @@
         <x:f>IF(A58&gt;$B$4,"",SUM($E$15:E58))</x:f>
       </x:c>
       <x:c r="J58" s="1" t="str">
-        <x:f>IF(A58&gt;$B$4,"Future",IF(A58=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A58,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E58=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A58&gt;$B$4,"Future",IF(A58=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A58,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E58=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2158,7 +2158,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E59" s="6" t="str">
-        <x:f>IF(A59&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A59,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A59&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A59,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F59" s="6" t="str">
         <x:f>IF(A59&gt;=$B$4,"",MAX(D59-E59,0))</x:f>
@@ -2173,7 +2173,7 @@
         <x:f>IF(A59&gt;$B$4,"",SUM($E$15:E59))</x:f>
       </x:c>
       <x:c r="J59" s="1" t="str">
-        <x:f>IF(A59&gt;$B$4,"Future",IF(A59=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A59,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E59=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A59&gt;$B$4,"Future",IF(A59=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A59,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E59=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2193,7 +2193,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E60" s="6" t="str">
-        <x:f>IF(A60&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A60,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A60&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A60,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F60" s="6" t="str">
         <x:f>IF(A60&gt;=$B$4,"",MAX(D60-E60,0))</x:f>
@@ -2208,7 +2208,7 @@
         <x:f>IF(A60&gt;$B$4,"",SUM($E$15:E60))</x:f>
       </x:c>
       <x:c r="J60" s="1" t="str">
-        <x:f>IF(A60&gt;$B$4,"Future",IF(A60=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A60,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E60=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A60&gt;$B$4,"Future",IF(A60=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A60,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E60=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2228,7 +2228,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E61" s="6" t="str">
-        <x:f>IF(A61&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A61,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A61&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A61,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F61" s="6" t="str">
         <x:f>IF(A61&gt;=$B$4,"",MAX(D61-E61,0))</x:f>
@@ -2243,7 +2243,7 @@
         <x:f>IF(A61&gt;$B$4,"",SUM($E$15:E61))</x:f>
       </x:c>
       <x:c r="J61" s="1" t="str">
-        <x:f>IF(A61&gt;$B$4,"Future",IF(A61=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A61,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E61=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A61&gt;$B$4,"Future",IF(A61=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A61,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E61=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2263,7 +2263,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E62" s="6" t="str">
-        <x:f>IF(A62&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A62,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A62&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A62,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F62" s="6" t="str">
         <x:f>IF(A62&gt;=$B$4,"",MAX(D62-E62,0))</x:f>
@@ -2278,7 +2278,7 @@
         <x:f>IF(A62&gt;$B$4,"",SUM($E$15:E62))</x:f>
       </x:c>
       <x:c r="J62" s="1" t="str">
-        <x:f>IF(A62&gt;$B$4,"Future",IF(A62=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A62,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E62=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A62&gt;$B$4,"Future",IF(A62=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A62,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E62=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2298,7 +2298,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E63" s="6" t="str">
-        <x:f>IF(A63&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A63,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A63&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A63,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F63" s="6" t="str">
         <x:f>IF(A63&gt;=$B$4,"",MAX(D63-E63,0))</x:f>
@@ -2313,7 +2313,7 @@
         <x:f>IF(A63&gt;$B$4,"",SUM($E$15:E63))</x:f>
       </x:c>
       <x:c r="J63" s="1" t="str">
-        <x:f>IF(A63&gt;$B$4,"Future",IF(A63=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A63,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E63=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A63&gt;$B$4,"Future",IF(A63=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A63,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E63=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2333,7 +2333,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E64" s="6" t="str">
-        <x:f>IF(A64&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A64,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A64&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A64,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F64" s="6" t="str">
         <x:f>IF(A64&gt;=$B$4,"",MAX(D64-E64,0))</x:f>
@@ -2348,7 +2348,7 @@
         <x:f>IF(A64&gt;$B$4,"",SUM($E$15:E64))</x:f>
       </x:c>
       <x:c r="J64" s="1" t="str">
-        <x:f>IF(A64&gt;$B$4,"Future",IF(A64=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A64,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E64=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A64&gt;$B$4,"Future",IF(A64=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A64,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E64=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2368,7 +2368,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E65" s="6" t="str">
-        <x:f>IF(A65&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A65,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A65&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A65,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F65" s="6" t="str">
         <x:f>IF(A65&gt;=$B$4,"",MAX(D65-E65,0))</x:f>
@@ -2383,7 +2383,7 @@
         <x:f>IF(A65&gt;$B$4,"",SUM($E$15:E65))</x:f>
       </x:c>
       <x:c r="J65" s="1" t="str">
-        <x:f>IF(A65&gt;$B$4,"Future",IF(A65=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A65,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E65=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A65&gt;$B$4,"Future",IF(A65=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A65,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E65=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2403,7 +2403,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E66" s="6" t="str">
-        <x:f>IF(A66&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A66,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A66&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A66,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F66" s="6" t="str">
         <x:f>IF(A66&gt;=$B$4,"",MAX(D66-E66,0))</x:f>
@@ -2418,7 +2418,7 @@
         <x:f>IF(A66&gt;$B$4,"",SUM($E$15:E66))</x:f>
       </x:c>
       <x:c r="J66" s="1" t="str">
-        <x:f>IF(A66&gt;$B$4,"Future",IF(A66=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A66,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E66=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A66&gt;$B$4,"Future",IF(A66=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A66,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E66=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2438,7 +2438,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E67" s="6" t="str">
-        <x:f>IF(A67&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A67,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A67&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A67,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F67" s="6" t="str">
         <x:f>IF(A67&gt;=$B$4,"",MAX(D67-E67,0))</x:f>
@@ -2453,7 +2453,7 @@
         <x:f>IF(A67&gt;$B$4,"",SUM($E$15:E67))</x:f>
       </x:c>
       <x:c r="J67" s="1" t="str">
-        <x:f>IF(A67&gt;$B$4,"Future",IF(A67=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A67,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E67=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A67&gt;$B$4,"Future",IF(A67=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A67,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E67=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2473,7 +2473,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E68" s="6" t="str">
-        <x:f>IF(A68&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A68,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A68&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A68,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F68" s="6" t="str">
         <x:f>IF(A68&gt;=$B$4,"",MAX(D68-E68,0))</x:f>
@@ -2488,7 +2488,7 @@
         <x:f>IF(A68&gt;$B$4,"",SUM($E$15:E68))</x:f>
       </x:c>
       <x:c r="J68" s="1" t="str">
-        <x:f>IF(A68&gt;$B$4,"Future",IF(A68=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A68,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E68=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A68&gt;$B$4,"Future",IF(A68=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A68,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E68=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2508,7 +2508,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E69" s="6" t="str">
-        <x:f>IF(A69&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A69,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A69&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A69,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F69" s="6" t="str">
         <x:f>IF(A69&gt;=$B$4,"",MAX(D69-E69,0))</x:f>
@@ -2523,7 +2523,7 @@
         <x:f>IF(A69&gt;$B$4,"",SUM($E$15:E69))</x:f>
       </x:c>
       <x:c r="J69" s="1" t="str">
-        <x:f>IF(A69&gt;$B$4,"Future",IF(A69=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A69,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E69=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A69&gt;$B$4,"Future",IF(A69=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A69,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E69=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2543,7 +2543,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E70" s="6" t="str">
-        <x:f>IF(A70&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A70,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A70&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A70,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F70" s="6" t="str">
         <x:f>IF(A70&gt;=$B$4,"",MAX(D70-E70,0))</x:f>
@@ -2558,7 +2558,7 @@
         <x:f>IF(A70&gt;$B$4,"",SUM($E$15:E70))</x:f>
       </x:c>
       <x:c r="J70" s="1" t="str">
-        <x:f>IF(A70&gt;$B$4,"Future",IF(A70=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A70,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E70=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A70&gt;$B$4,"Future",IF(A70=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A70,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E70=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2578,7 +2578,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E71" s="6" t="str">
-        <x:f>IF(A71&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A71,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A71&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A71,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F71" s="6" t="str">
         <x:f>IF(A71&gt;=$B$4,"",MAX(D71-E71,0))</x:f>
@@ -2593,7 +2593,7 @@
         <x:f>IF(A71&gt;$B$4,"",SUM($E$15:E71))</x:f>
       </x:c>
       <x:c r="J71" s="1" t="str">
-        <x:f>IF(A71&gt;$B$4,"Future",IF(A71=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A71,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E71=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A71&gt;$B$4,"Future",IF(A71=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A71,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E71=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2613,7 +2613,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E72" s="6" t="str">
-        <x:f>IF(A72&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A72,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A72&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A72,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F72" s="6" t="str">
         <x:f>IF(A72&gt;=$B$4,"",MAX(D72-E72,0))</x:f>
@@ -2628,7 +2628,7 @@
         <x:f>IF(A72&gt;$B$4,"",SUM($E$15:E72))</x:f>
       </x:c>
       <x:c r="J72" s="1" t="str">
-        <x:f>IF(A72&gt;$B$4,"Future",IF(A72=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A72,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E72=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A72&gt;$B$4,"Future",IF(A72=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A72,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E72=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2648,7 +2648,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E73" s="6" t="str">
-        <x:f>IF(A73&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A73,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A73&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A73,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F73" s="6" t="str">
         <x:f>IF(A73&gt;=$B$4,"",MAX(D73-E73,0))</x:f>
@@ -2663,7 +2663,7 @@
         <x:f>IF(A73&gt;$B$4,"",SUM($E$15:E73))</x:f>
       </x:c>
       <x:c r="J73" s="1" t="str">
-        <x:f>IF(A73&gt;$B$4,"Future",IF(A73=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A73,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E73=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A73&gt;$B$4,"Future",IF(A73=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A73,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E73=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2683,7 +2683,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E74" s="6" t="str">
-        <x:f>IF(A74&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A74,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A74&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A74,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F74" s="6" t="str">
         <x:f>IF(A74&gt;=$B$4,"",MAX(D74-E74,0))</x:f>
@@ -2698,7 +2698,7 @@
         <x:f>IF(A74&gt;$B$4,"",SUM($E$15:E74))</x:f>
       </x:c>
       <x:c r="J74" s="1" t="str">
-        <x:f>IF(A74&gt;$B$4,"Future",IF(A74=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A74,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E74=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A74&gt;$B$4,"Future",IF(A74=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A74,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E74=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2718,7 +2718,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E75" s="6" t="str">
-        <x:f>IF(A75&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A75,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A75&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A75,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F75" s="6" t="str">
         <x:f>IF(A75&gt;=$B$4,"",MAX(D75-E75,0))</x:f>
@@ -2733,7 +2733,7 @@
         <x:f>IF(A75&gt;$B$4,"",SUM($E$15:E75))</x:f>
       </x:c>
       <x:c r="J75" s="1" t="str">
-        <x:f>IF(A75&gt;$B$4,"Future",IF(A75=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A75,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E75=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A75&gt;$B$4,"Future",IF(A75=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A75,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E75=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2753,7 +2753,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E76" s="6" t="str">
-        <x:f>IF(A76&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A76,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A76&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A76,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F76" s="6" t="str">
         <x:f>IF(A76&gt;=$B$4,"",MAX(D76-E76,0))</x:f>
@@ -2768,7 +2768,7 @@
         <x:f>IF(A76&gt;$B$4,"",SUM($E$15:E76))</x:f>
       </x:c>
       <x:c r="J76" s="1" t="str">
-        <x:f>IF(A76&gt;$B$4,"Future",IF(A76=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A76,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E76=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A76&gt;$B$4,"Future",IF(A76=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A76,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E76=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2788,7 +2788,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E77" s="6" t="str">
-        <x:f>IF(A77&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A77,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A77&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A77,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F77" s="6" t="str">
         <x:f>IF(A77&gt;=$B$4,"",MAX(D77-E77,0))</x:f>
@@ -2803,7 +2803,7 @@
         <x:f>IF(A77&gt;$B$4,"",SUM($E$15:E77))</x:f>
       </x:c>
       <x:c r="J77" s="1" t="str">
-        <x:f>IF(A77&gt;$B$4,"Future",IF(A77=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A77,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E77=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A77&gt;$B$4,"Future",IF(A77=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A77,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E77=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2823,7 +2823,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E78" s="6" t="str">
-        <x:f>IF(A78&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A78,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A78&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A78,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F78" s="6" t="str">
         <x:f>IF(A78&gt;=$B$4,"",MAX(D78-E78,0))</x:f>
@@ -2838,7 +2838,7 @@
         <x:f>IF(A78&gt;$B$4,"",SUM($E$15:E78))</x:f>
       </x:c>
       <x:c r="J78" s="1" t="str">
-        <x:f>IF(A78&gt;$B$4,"Future",IF(A78=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A78,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E78=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A78&gt;$B$4,"Future",IF(A78=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A78,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E78=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2858,7 +2858,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E79" s="6" t="str">
-        <x:f>IF(A79&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A79,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A79&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A79,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F79" s="6" t="str">
         <x:f>IF(A79&gt;=$B$4,"",MAX(D79-E79,0))</x:f>
@@ -2873,7 +2873,7 @@
         <x:f>IF(A79&gt;$B$4,"",SUM($E$15:E79))</x:f>
       </x:c>
       <x:c r="J79" s="1" t="str">
-        <x:f>IF(A79&gt;$B$4,"Future",IF(A79=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A79,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E79=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A79&gt;$B$4,"Future",IF(A79=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A79,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E79=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2893,7 +2893,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E80" s="6" t="str">
-        <x:f>IF(A80&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A80,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A80&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A80,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F80" s="6" t="str">
         <x:f>IF(A80&gt;=$B$4,"",MAX(D80-E80,0))</x:f>
@@ -2908,7 +2908,7 @@
         <x:f>IF(A80&gt;$B$4,"",SUM($E$15:E80))</x:f>
       </x:c>
       <x:c r="J80" s="1" t="str">
-        <x:f>IF(A80&gt;$B$4,"Future",IF(A80=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A80,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E80=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A80&gt;$B$4,"Future",IF(A80=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A80,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E80=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2928,7 +2928,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E81" s="6" t="str">
-        <x:f>IF(A81&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A81,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A81&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A81,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F81" s="6" t="str">
         <x:f>IF(A81&gt;=$B$4,"",MAX(D81-E81,0))</x:f>
@@ -2943,7 +2943,7 @@
         <x:f>IF(A81&gt;$B$4,"",SUM($E$15:E81))</x:f>
       </x:c>
       <x:c r="J81" s="1" t="str">
-        <x:f>IF(A81&gt;$B$4,"Future",IF(A81=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A81,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E81=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A81&gt;$B$4,"Future",IF(A81=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A81,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E81=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2963,7 +2963,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E82" s="6" t="str">
-        <x:f>IF(A82&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A82,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A82&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A82,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F82" s="6" t="str">
         <x:f>IF(A82&gt;=$B$4,"",MAX(D82-E82,0))</x:f>
@@ -2978,7 +2978,7 @@
         <x:f>IF(A82&gt;$B$4,"",SUM($E$15:E82))</x:f>
       </x:c>
       <x:c r="J82" s="1" t="str">
-        <x:f>IF(A82&gt;$B$4,"Future",IF(A82=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A82,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E82=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A82&gt;$B$4,"Future",IF(A82=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A82,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E82=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2998,7 +2998,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E83" s="6" t="str">
-        <x:f>IF(A83&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A83,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A83&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A83,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F83" s="6" t="str">
         <x:f>IF(A83&gt;=$B$4,"",MAX(D83-E83,0))</x:f>
@@ -3013,7 +3013,7 @@
         <x:f>IF(A83&gt;$B$4,"",SUM($E$15:E83))</x:f>
       </x:c>
       <x:c r="J83" s="1" t="str">
-        <x:f>IF(A83&gt;$B$4,"Future",IF(A83=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A83,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E83=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A83&gt;$B$4,"Future",IF(A83=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A83,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E83=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3033,7 +3033,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E84" s="6" t="str">
-        <x:f>IF(A84&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A84,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A84&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A84,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F84" s="6" t="str">
         <x:f>IF(A84&gt;=$B$4,"",MAX(D84-E84,0))</x:f>
@@ -3048,7 +3048,7 @@
         <x:f>IF(A84&gt;$B$4,"",SUM($E$15:E84))</x:f>
       </x:c>
       <x:c r="J84" s="1" t="str">
-        <x:f>IF(A84&gt;$B$4,"Future",IF(A84=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A84,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E84=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A84&gt;$B$4,"Future",IF(A84=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A84,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E84=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3068,7 +3068,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E85" s="6" t="str">
-        <x:f>IF(A85&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A85,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A85&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A85,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F85" s="6" t="str">
         <x:f>IF(A85&gt;=$B$4,"",MAX(D85-E85,0))</x:f>
@@ -3083,7 +3083,7 @@
         <x:f>IF(A85&gt;$B$4,"",SUM($E$15:E85))</x:f>
       </x:c>
       <x:c r="J85" s="1" t="str">
-        <x:f>IF(A85&gt;$B$4,"Future",IF(A85=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A85,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E85=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A85&gt;$B$4,"Future",IF(A85=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A85,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E85=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3103,7 +3103,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E86" s="6" t="str">
-        <x:f>IF(A86&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A86,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A86&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A86,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F86" s="6" t="str">
         <x:f>IF(A86&gt;=$B$4,"",MAX(D86-E86,0))</x:f>
@@ -3118,7 +3118,7 @@
         <x:f>IF(A86&gt;$B$4,"",SUM($E$15:E86))</x:f>
       </x:c>
       <x:c r="J86" s="1" t="str">
-        <x:f>IF(A86&gt;$B$4,"Future",IF(A86=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A86,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E86=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A86&gt;$B$4,"Future",IF(A86=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A86,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E86=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3138,7 +3138,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E87" s="6" t="str">
-        <x:f>IF(A87&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A87,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A87&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A87,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F87" s="6" t="str">
         <x:f>IF(A87&gt;=$B$4,"",MAX(D87-E87,0))</x:f>
@@ -3153,7 +3153,7 @@
         <x:f>IF(A87&gt;$B$4,"",SUM($E$15:E87))</x:f>
       </x:c>
       <x:c r="J87" s="1" t="str">
-        <x:f>IF(A87&gt;$B$4,"Future",IF(A87=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A87,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E87=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A87&gt;$B$4,"Future",IF(A87=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A87,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E87=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3173,7 +3173,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E88" s="6" t="str">
-        <x:f>IF(A88&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A88,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A88&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A88,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F88" s="6" t="str">
         <x:f>IF(A88&gt;=$B$4,"",MAX(D88-E88,0))</x:f>
@@ -3188,7 +3188,7 @@
         <x:f>IF(A88&gt;$B$4,"",SUM($E$15:E88))</x:f>
       </x:c>
       <x:c r="J88" s="1" t="str">
-        <x:f>IF(A88&gt;$B$4,"Future",IF(A88=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A88,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E88=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A88&gt;$B$4,"Future",IF(A88=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A88,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E88=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3208,7 +3208,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E89" s="6" t="str">
-        <x:f>IF(A89&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A89,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A89&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A89,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F89" s="6" t="str">
         <x:f>IF(A89&gt;=$B$4,"",MAX(D89-E89,0))</x:f>
@@ -3223,7 +3223,7 @@
         <x:f>IF(A89&gt;$B$4,"",SUM($E$15:E89))</x:f>
       </x:c>
       <x:c r="J89" s="1" t="str">
-        <x:f>IF(A89&gt;$B$4,"Future",IF(A89=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A89,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E89=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A89&gt;$B$4,"Future",IF(A89=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A89,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E89=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3243,7 +3243,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E90" s="6" t="str">
-        <x:f>IF(A90&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A90,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A90&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A90,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F90" s="6" t="str">
         <x:f>IF(A90&gt;=$B$4,"",MAX(D90-E90,0))</x:f>
@@ -3258,7 +3258,7 @@
         <x:f>IF(A90&gt;$B$4,"",SUM($E$15:E90))</x:f>
       </x:c>
       <x:c r="J90" s="1" t="str">
-        <x:f>IF(A90&gt;$B$4,"Future",IF(A90=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A90,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E90=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A90&gt;$B$4,"Future",IF(A90=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A90,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E90=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3278,7 +3278,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E91" s="6" t="str">
-        <x:f>IF(A91&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A91,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A91&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A91,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F91" s="6" t="str">
         <x:f>IF(A91&gt;=$B$4,"",MAX(D91-E91,0))</x:f>
@@ -3293,7 +3293,7 @@
         <x:f>IF(A91&gt;$B$4,"",SUM($E$15:E91))</x:f>
       </x:c>
       <x:c r="J91" s="1" t="str">
-        <x:f>IF(A91&gt;$B$4,"Future",IF(A91=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A91,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E91=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A91&gt;$B$4,"Future",IF(A91=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A91,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E91=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3313,7 +3313,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E92" s="6" t="str">
-        <x:f>IF(A92&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A92,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A92&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A92,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F92" s="6" t="str">
         <x:f>IF(A92&gt;=$B$4,"",MAX(D92-E92,0))</x:f>
@@ -3328,7 +3328,7 @@
         <x:f>IF(A92&gt;$B$4,"",SUM($E$15:E92))</x:f>
       </x:c>
       <x:c r="J92" s="1" t="str">
-        <x:f>IF(A92&gt;$B$4,"Future",IF(A92=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A92,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E92=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A92&gt;$B$4,"Future",IF(A92=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A92,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E92=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3348,7 +3348,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E93" s="6" t="str">
-        <x:f>IF(A93&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A93,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A93&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A93,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F93" s="6" t="str">
         <x:f>IF(A93&gt;=$B$4,"",MAX(D93-E93,0))</x:f>
@@ -3363,7 +3363,7 @@
         <x:f>IF(A93&gt;$B$4,"",SUM($E$15:E93))</x:f>
       </x:c>
       <x:c r="J93" s="1" t="str">
-        <x:f>IF(A93&gt;$B$4,"Future",IF(A93=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A93,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E93=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A93&gt;$B$4,"Future",IF(A93=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A93,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E93=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3383,7 +3383,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E94" s="6" t="str">
-        <x:f>IF(A94&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A94,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A94&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A94,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F94" s="6" t="str">
         <x:f>IF(A94&gt;=$B$4,"",MAX(D94-E94,0))</x:f>
@@ -3398,7 +3398,7 @@
         <x:f>IF(A94&gt;$B$4,"",SUM($E$15:E94))</x:f>
       </x:c>
       <x:c r="J94" s="1" t="str">
-        <x:f>IF(A94&gt;$B$4,"Future",IF(A94=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A94,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E94=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A94&gt;$B$4,"Future",IF(A94=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A94,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E94=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3418,7 +3418,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E95" s="6" t="str">
-        <x:f>IF(A95&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A95,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A95&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A95,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F95" s="6" t="str">
         <x:f>IF(A95&gt;=$B$4,"",MAX(D95-E95,0))</x:f>
@@ -3433,7 +3433,7 @@
         <x:f>IF(A95&gt;$B$4,"",SUM($E$15:E95))</x:f>
       </x:c>
       <x:c r="J95" s="1" t="str">
-        <x:f>IF(A95&gt;$B$4,"Future",IF(A95=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A95,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E95=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A95&gt;$B$4,"Future",IF(A95=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A95,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E95=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3453,7 +3453,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E96" s="6" t="str">
-        <x:f>IF(A96&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A96,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A96&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A96,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F96" s="6" t="str">
         <x:f>IF(A96&gt;=$B$4,"",MAX(D96-E96,0))</x:f>
@@ -3468,7 +3468,7 @@
         <x:f>IF(A96&gt;$B$4,"",SUM($E$15:E96))</x:f>
       </x:c>
       <x:c r="J96" s="1" t="str">
-        <x:f>IF(A96&gt;$B$4,"Future",IF(A96=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A96,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E96=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A96&gt;$B$4,"Future",IF(A96=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A96,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E96=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3488,7 +3488,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E97" s="6" t="str">
-        <x:f>IF(A97&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A97,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A97&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A97,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F97" s="6" t="str">
         <x:f>IF(A97&gt;=$B$4,"",MAX(D97-E97,0))</x:f>
@@ -3503,7 +3503,7 @@
         <x:f>IF(A97&gt;$B$4,"",SUM($E$15:E97))</x:f>
       </x:c>
       <x:c r="J97" s="1" t="str">
-        <x:f>IF(A97&gt;$B$4,"Future",IF(A97=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A97,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E97=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A97&gt;$B$4,"Future",IF(A97=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A97,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E97=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3523,7 +3523,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E98" s="6" t="str">
-        <x:f>IF(A98&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A98,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A98&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A98,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F98" s="6" t="str">
         <x:f>IF(A98&gt;=$B$4,"",MAX(D98-E98,0))</x:f>
@@ -3538,7 +3538,7 @@
         <x:f>IF(A98&gt;$B$4,"",SUM($E$15:E98))</x:f>
       </x:c>
       <x:c r="J98" s="1" t="str">
-        <x:f>IF(A98&gt;$B$4,"Future",IF(A98=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A98,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E98=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A98&gt;$B$4,"Future",IF(A98=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A98,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E98=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3558,7 +3558,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E99" s="6" t="str">
-        <x:f>IF(A99&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A99,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A99&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A99,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F99" s="6" t="str">
         <x:f>IF(A99&gt;=$B$4,"",MAX(D99-E99,0))</x:f>
@@ -3573,7 +3573,7 @@
         <x:f>IF(A99&gt;$B$4,"",SUM($E$15:E99))</x:f>
       </x:c>
       <x:c r="J99" s="1" t="str">
-        <x:f>IF(A99&gt;$B$4,"Future",IF(A99=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A99,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E99=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A99&gt;$B$4,"Future",IF(A99=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A99,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E99=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3593,7 +3593,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E100" s="6" t="str">
-        <x:f>IF(A100&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A100,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A100&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A100,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F100" s="6" t="str">
         <x:f>IF(A100&gt;=$B$4,"",MAX(D100-E100,0))</x:f>
@@ -3608,7 +3608,7 @@
         <x:f>IF(A100&gt;$B$4,"",SUM($E$15:E100))</x:f>
       </x:c>
       <x:c r="J100" s="1" t="str">
-        <x:f>IF(A100&gt;$B$4,"Future",IF(A100=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A100,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E100=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A100&gt;$B$4,"Future",IF(A100=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A100,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E100=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3628,7 +3628,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E101" s="6" t="str">
-        <x:f>IF(A101&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A101,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A101&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A101,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F101" s="6" t="str">
         <x:f>IF(A101&gt;=$B$4,"",MAX(D101-E101,0))</x:f>
@@ -3643,7 +3643,7 @@
         <x:f>IF(A101&gt;$B$4,"",SUM($E$15:E101))</x:f>
       </x:c>
       <x:c r="J101" s="1" t="str">
-        <x:f>IF(A101&gt;$B$4,"Future",IF(A101=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A101,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E101=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A101&gt;$B$4,"Future",IF(A101=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A101,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E101=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3663,7 +3663,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E102" s="6" t="str">
-        <x:f>IF(A102&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A102,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A102&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A102,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F102" s="6" t="str">
         <x:f>IF(A102&gt;=$B$4,"",MAX(D102-E102,0))</x:f>
@@ -3678,7 +3678,7 @@
         <x:f>IF(A102&gt;$B$4,"",SUM($E$15:E102))</x:f>
       </x:c>
       <x:c r="J102" s="1" t="str">
-        <x:f>IF(A102&gt;$B$4,"Future",IF(A102=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A102,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E102=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A102&gt;$B$4,"Future",IF(A102=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A102,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E102=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3698,7 +3698,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E103" s="6" t="str">
-        <x:f>IF(A103&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A103,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A103&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A103,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F103" s="6" t="str">
         <x:f>IF(A103&gt;=$B$4,"",MAX(D103-E103,0))</x:f>
@@ -3713,7 +3713,7 @@
         <x:f>IF(A103&gt;$B$4,"",SUM($E$15:E103))</x:f>
       </x:c>
       <x:c r="J103" s="1" t="str">
-        <x:f>IF(A103&gt;$B$4,"Future",IF(A103=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A103,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E103=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A103&gt;$B$4,"Future",IF(A103=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A103,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E103=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3733,7 +3733,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E104" s="6" t="str">
-        <x:f>IF(A104&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A104,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A104&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A104,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F104" s="6" t="str">
         <x:f>IF(A104&gt;=$B$4,"",MAX(D104-E104,0))</x:f>
@@ -3748,7 +3748,7 @@
         <x:f>IF(A104&gt;$B$4,"",SUM($E$15:E104))</x:f>
       </x:c>
       <x:c r="J104" s="1" t="str">
-        <x:f>IF(A104&gt;$B$4,"Future",IF(A104=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A104,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E104=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A104&gt;$B$4,"Future",IF(A104=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A104,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E104=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3768,7 +3768,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E105" s="6" t="str">
-        <x:f>IF(A105&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A105,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A105&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A105,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F105" s="6" t="str">
         <x:f>IF(A105&gt;=$B$4,"",MAX(D105-E105,0))</x:f>
@@ -3783,7 +3783,7 @@
         <x:f>IF(A105&gt;$B$4,"",SUM($E$15:E105))</x:f>
       </x:c>
       <x:c r="J105" s="1" t="str">
-        <x:f>IF(A105&gt;$B$4,"Future",IF(A105=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A105,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E105=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A105&gt;$B$4,"Future",IF(A105=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A105,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E105=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3803,7 +3803,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E106" s="6" t="str">
-        <x:f>IF(A106&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A106,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A106&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A106,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F106" s="6" t="str">
         <x:f>IF(A106&gt;=$B$4,"",MAX(D106-E106,0))</x:f>
@@ -3818,7 +3818,7 @@
         <x:f>IF(A106&gt;$B$4,"",SUM($E$15:E106))</x:f>
       </x:c>
       <x:c r="J106" s="1" t="str">
-        <x:f>IF(A106&gt;$B$4,"Future",IF(A106=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A106,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E106=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A106&gt;$B$4,"Future",IF(A106=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A106,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E106=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3838,7 +3838,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E107" s="6" t="str">
-        <x:f>IF(A107&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A107,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A107&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A107,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F107" s="6" t="str">
         <x:f>IF(A107&gt;=$B$4,"",MAX(D107-E107,0))</x:f>
@@ -3853,7 +3853,7 @@
         <x:f>IF(A107&gt;$B$4,"",SUM($E$15:E107))</x:f>
       </x:c>
       <x:c r="J107" s="1" t="str">
-        <x:f>IF(A107&gt;$B$4,"Future",IF(A107=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A107,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E107=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A107&gt;$B$4,"Future",IF(A107=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A107,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E107=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3873,7 +3873,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E108" s="6" t="str">
-        <x:f>IF(A108&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A108,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A108&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A108,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F108" s="6" t="str">
         <x:f>IF(A108&gt;=$B$4,"",MAX(D108-E108,0))</x:f>
@@ -3888,7 +3888,7 @@
         <x:f>IF(A108&gt;$B$4,"",SUM($E$15:E108))</x:f>
       </x:c>
       <x:c r="J108" s="1" t="str">
-        <x:f>IF(A108&gt;$B$4,"Future",IF(A108=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A108,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E108=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A108&gt;$B$4,"Future",IF(A108=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A108,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E108=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3908,7 +3908,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E109" s="6" t="str">
-        <x:f>IF(A109&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A109,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A109&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A109,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F109" s="6" t="str">
         <x:f>IF(A109&gt;=$B$4,"",MAX(D109-E109,0))</x:f>
@@ -3923,7 +3923,7 @@
         <x:f>IF(A109&gt;$B$4,"",SUM($E$15:E109))</x:f>
       </x:c>
       <x:c r="J109" s="1" t="str">
-        <x:f>IF(A109&gt;$B$4,"Future",IF(A109=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A109,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E109=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A109&gt;$B$4,"Future",IF(A109=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A109,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E109=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3943,7 +3943,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E110" s="6" t="str">
-        <x:f>IF(A110&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A110,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A110&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A110,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F110" s="6" t="str">
         <x:f>IF(A110&gt;=$B$4,"",MAX(D110-E110,0))</x:f>
@@ -3958,7 +3958,7 @@
         <x:f>IF(A110&gt;$B$4,"",SUM($E$15:E110))</x:f>
       </x:c>
       <x:c r="J110" s="1" t="str">
-        <x:f>IF(A110&gt;$B$4,"Future",IF(A110=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A110,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E110=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A110&gt;$B$4,"Future",IF(A110=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A110,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E110=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3978,7 +3978,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E111" s="6" t="str">
-        <x:f>IF(A111&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A111,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A111&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A111,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F111" s="6" t="str">
         <x:f>IF(A111&gt;=$B$4,"",MAX(D111-E111,0))</x:f>
@@ -3993,7 +3993,7 @@
         <x:f>IF(A111&gt;$B$4,"",SUM($E$15:E111))</x:f>
       </x:c>
       <x:c r="J111" s="1" t="str">
-        <x:f>IF(A111&gt;$B$4,"Future",IF(A111=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A111,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E111=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A111&gt;$B$4,"Future",IF(A111=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A111,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E111=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4013,7 +4013,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E112" s="6" t="str">
-        <x:f>IF(A112&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A112,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A112&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A112,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F112" s="6" t="str">
         <x:f>IF(A112&gt;=$B$4,"",MAX(D112-E112,0))</x:f>
@@ -4028,7 +4028,7 @@
         <x:f>IF(A112&gt;$B$4,"",SUM($E$15:E112))</x:f>
       </x:c>
       <x:c r="J112" s="1" t="str">
-        <x:f>IF(A112&gt;$B$4,"Future",IF(A112=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A112,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E112=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A112&gt;$B$4,"Future",IF(A112=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A112,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E112=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4048,7 +4048,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E113" s="6" t="str">
-        <x:f>IF(A113&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A113,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A113&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A113,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F113" s="6" t="str">
         <x:f>IF(A113&gt;=$B$4,"",MAX(D113-E113,0))</x:f>
@@ -4063,7 +4063,7 @@
         <x:f>IF(A113&gt;$B$4,"",SUM($E$15:E113))</x:f>
       </x:c>
       <x:c r="J113" s="1" t="str">
-        <x:f>IF(A113&gt;$B$4,"Future",IF(A113=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A113,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E113=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A113&gt;$B$4,"Future",IF(A113=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A113,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E113=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4083,7 +4083,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E114" s="6" t="str">
-        <x:f>IF(A114&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$B$2:$B$21,A114,'Sessions'!$G$2:$G$21,"completed")/60)</x:f>
+        <x:f>IF(A114&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A114,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
       </x:c>
       <x:c r="F114" s="6" t="str">
         <x:f>IF(A114&gt;=$B$4,"",MAX(D114-E114,0))</x:f>
@@ -4098,7 +4098,7 @@
         <x:f>IF(A114&gt;$B$4,"",SUM($E$15:E114))</x:f>
       </x:c>
       <x:c r="J114" s="1" t="str">
-        <x:f>IF(A114&gt;$B$4,"Future",IF(A114=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$21,A114,'Sessions'!$G$2:$G$21,"needs_confirmation")&gt;0,"Uncertain time",IF(E114=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A114&gt;$B$4,"Future",IF(A114=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A114,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E114=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -5269,6 +5269,72 @@
         <x:v>Explicit resume-timer; established RRDAP topic retained. Break 19:58:56-20:56:51 (57m55s) excluded. RDS-001 approach/implementation pending; no new assessed learning. Explicit pause at 21:27:54 IST; 31m03s. No new learner submission or assessed learning in this chat; RDS-001 pending.</x:v>
       </x:c>
     </x:row>
+    <x:row r="22" ht="22" customHeight="1">
+      <x:c r="A22" s="1" t="str">
+        <x:v>DOC-20261022-POM1</x:v>
+      </x:c>
+      <x:c r="B22" s="7" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="C22" s="1" t="str">
+        <x:v>Docker: self-reported Pomodoro</x:v>
+      </x:c>
+      <x:c r="D22" s="1" t="str"/>
+      <x:c r="E22" s="1" t="str"/>
+      <x:c r="F22" s="1" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="G22" s="1" t="str">
+        <x:v>needs_confirmation</x:v>
+      </x:c>
+      <x:c r="H22" s="1" t="str">
+        <x:v>Learner reported one completed 25-minute Docker study interval and a subsequent 5-minute break. Exact start/end times in IST not supplied; duration is pending timestamp confirmation and excluded from confirmed totals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="22" customHeight="1">
+      <x:c r="A23" s="1" t="str">
+        <x:v>DOC-20261022-POM2</x:v>
+      </x:c>
+      <x:c r="B23" s="7" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="C23" s="1" t="str">
+        <x:v>Docker: self-reported Pomodoro</x:v>
+      </x:c>
+      <x:c r="D23" s="1" t="str"/>
+      <x:c r="E23" s="1" t="str"/>
+      <x:c r="F23" s="1" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="G23" s="1" t="str">
+        <x:v>needs_confirmation</x:v>
+      </x:c>
+      <x:c r="H23" s="1" t="str">
+        <x:v>Learner reported another completed 25-minute Docker study interval and 5-minute break. Exact start/end times in IST not supplied; duration is pending timestamp confirmation and excluded from confirmed totals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="22" customHeight="1">
+      <x:c r="A24" s="1" t="str">
+        <x:v>DOC-20261022-POM3</x:v>
+      </x:c>
+      <x:c r="B24" s="7" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="C24" s="1" t="str">
+        <x:v>Docker: self-reported Pomodoro</x:v>
+      </x:c>
+      <x:c r="D24" s="1" t="str"/>
+      <x:c r="E24" s="1" t="str"/>
+      <x:c r="F24" s="1" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="G24" s="1" t="str">
+        <x:v>needs_confirmation</x:v>
+      </x:c>
+      <x:c r="H24" s="1" t="str">
+        <x:v>Learner reported a third completed 25-minute Docker study interval and 5-minute break. Exact start/end times in IST not supplied; duration is pending timestamp confirmation and excluded from confirmed totals.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5302,109 +5368,118 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="1" t="str">
-        <x:v>Python / RRDAP: RDS-001 Product Catalogue</x:v>
+        <x:v>Docker: self-reported Pomodoro</x:v>
       </x:c>
       <x:c r="B7" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A7,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
-        <x:v>0.5175</x:v>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A7,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="1" t="str">
-        <x:v>Python / RRDAP: setup and RDS-001</x:v>
+        <x:v>Python / RRDAP: RDS-001 Product Catalogue</x:v>
       </x:c>
       <x:c r="B8" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A8,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
-        <x:v>2.225277777777778</x:v>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A8,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>0.5175</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="1" t="str">
-        <x:v>Python / RetailFlow: setup and RF-001</x:v>
+        <x:v>Python / RRDAP: setup and RDS-001</x:v>
       </x:c>
       <x:c r="B9" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A9,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
-        <x:v>1.0919444444444444</x:v>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A9,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>2.225277777777778</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="1" t="str">
-        <x:v>Python: CSV reading and writing</x:v>
+        <x:v>Python / RetailFlow: setup and RF-001</x:v>
       </x:c>
       <x:c r="B10" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A10,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
-        <x:v>0.12722222222222224</x:v>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A10,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>1.0919444444444444</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="1" t="str">
-        <x:v>Python: CSV writing and read-back</x:v>
+        <x:v>Python: CSV reading and writing</x:v>
       </x:c>
       <x:c r="B11" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A11,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
-        <x:v>2.8175000000000003</x:v>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A11,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>0.12722222222222224</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="1" t="str">
-        <x:v>Python: cleaner changed-input check</x:v>
+        <x:v>Python: CSV writing and read-back</x:v>
       </x:c>
       <x:c r="B12" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A12,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
-        <x:v>0.4911111111111111</x:v>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A12,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>2.8175000000000003</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="1" t="str">
-        <x:v>Python: dictionary foundations in Jupyter</x:v>
+        <x:v>Python: cleaner changed-input check</x:v>
       </x:c>
       <x:c r="B13" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A13,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
-        <x:v>1.6424999999994445</x:v>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A13,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>0.4911111111111111</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="1" t="str">
-        <x:v>Python: dictionary records baseline</x:v>
+        <x:v>Python: dictionary foundations in Jupyter</x:v>
       </x:c>
       <x:c r="B14" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A14,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
-        <x:v>0.21111111111166667</x:v>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A14,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>1.6424999999994445</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="1" t="str">
-        <x:v>Python: record cleaning</x:v>
+        <x:v>Python: dictionary records baseline</x:v>
       </x:c>
       <x:c r="B15" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A15,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
-        <x:v>0.22972222222166666</x:v>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A15,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>0.21111111111166667</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="1" t="str">
-        <x:v>Python: valid and rejected record lists</x:v>
+        <x:v>Python: record cleaning</x:v>
       </x:c>
       <x:c r="B16" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A16,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
-        <x:v>0.28194444444444444</x:v>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A16,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>0.22972222222166666</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="1" t="str">
-        <x:v>SQL: LEFT JOIN and unmatched rows</x:v>
+        <x:v>Python: valid and rejected record lists</x:v>
       </x:c>
       <x:c r="B17" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A17,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
-        <x:v>0.34055555555666667</x:v>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A17,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>0.28194444444444444</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="1" t="str">
+        <x:v>SQL: LEFT JOIN and unmatched rows</x:v>
+      </x:c>
+      <x:c r="B18" s="6" t="n">
+        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A18,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>0.34055555555666667</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="1" t="str">
         <x:v>SQL: joins counting grouping and SUM setup</x:v>
       </x:c>
-      <x:c r="B18" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$21,'Sessions'!$C$2:$C$21,A18,'Sessions'!$G$2:$G$21,"completed",'Sessions'!$B$2:$B$21,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+      <x:c r="B19" s="6" t="n">
+        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A19,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
         <x:v>1.175</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Save dataclass practice, notes and latest study checkpoint
</commit_message>
<xml_diff>
--- a/outputs/study-tracker/study-hours.xlsx
+++ b/outputs/study-tracker/study-hours.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="R35b5850a463f4db2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="Rbf4a57caa0a24116"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="Rdcc5475745e04ea2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topics" sheetId="4" r:id="R284dfcb8e72f4883"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" r:id="Rbf4937cab9f44efd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" r:id="R31b21e6bd1134175"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="3" r:id="Rbccd438493d74534"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topics" sheetId="4" r:id="R4cf7aaf49072466e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -355,7 +355,7 @@
         <x:v>Reporting date (IST)</x:v>
       </x:c>
       <x:c r="B4" s="8" t="n">
-        <x:v>46317</x:v>
+        <x:v>46321</x:v>
       </x:c>
       <x:c r="C4" s="1"/>
       <x:c r="D4" s="1" t="str">
@@ -388,7 +388,7 @@
       </x:c>
       <x:c r="E5" s="6" t="n">
         <x:f>SUMIFS(D15:D114,A15:A114,"&lt;"&amp;B4)</x:f>
-        <x:v>50</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="F5" s="1"/>
       <x:c r="G5" s="1" t="str">
@@ -413,7 +413,7 @@
       </x:c>
       <x:c r="E6" s="6" t="n">
         <x:f>MAX(E5-SUMIFS(E15:E114,A15:A114,"&lt;"&amp;B4),0)</x:f>
-        <x:v>38.84861111111056</x:v>
+        <x:v>72.84861111111056</x:v>
       </x:c>
       <x:c r="F6" s="1"/>
       <x:c r="G6" s="1"/>
@@ -581,7 +581,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E15" s="6" t="n">
-        <x:f>IF(A15&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A15,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A15&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A15,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
         <x:v>2.8094444444449995</x:v>
       </x:c>
       <x:c r="F15" s="6" t="n">
@@ -601,7 +601,7 @@
         <x:v>2.8094444444449995</x:v>
       </x:c>
       <x:c r="J15" s="1" t="str">
-        <x:f>IF(A15&gt;$B$4,"Future",IF(A15=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A15,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E15=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A15&gt;$B$4,"Future",IF(A15=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A15,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E15=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Uncertain time</x:v>
       </x:c>
     </x:row>
@@ -621,7 +621,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E16" s="6" t="n">
-        <x:f>IF(A16&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A16,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A16&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A16,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
         <x:v>1.6897222222222223</x:v>
       </x:c>
       <x:c r="F16" s="6" t="n">
@@ -641,7 +641,7 @@
         <x:v>4.499166666667222</x:v>
       </x:c>
       <x:c r="J16" s="1" t="str">
-        <x:f>IF(A16&gt;$B$4,"Future",IF(A16=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A16,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E16=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A16&gt;$B$4,"Future",IF(A16=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A16,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E16=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Logged</x:v>
       </x:c>
     </x:row>
@@ -661,7 +661,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E17" s="6" t="n">
-        <x:f>IF(A17&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A17,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A17&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A17,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
         <x:v>6.652222222222223</x:v>
       </x:c>
       <x:c r="F17" s="6" t="n">
@@ -681,7 +681,7 @@
         <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J17" s="1" t="str">
-        <x:f>IF(A17&gt;$B$4,"Future",IF(A17=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A17,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E17=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A17&gt;$B$4,"Future",IF(A17=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A17,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E17=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Logged</x:v>
       </x:c>
     </x:row>
@@ -701,7 +701,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E18" s="6" t="n">
-        <x:f>IF(A18&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A18,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A18&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A18,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F18" s="6" t="n">
@@ -721,7 +721,7 @@
         <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J18" s="1" t="str">
-        <x:f>IF(A18&gt;$B$4,"Future",IF(A18=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A18,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E18=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A18&gt;$B$4,"Future",IF(A18=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A18,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E18=0,"No confirmed time","Logged"))))</x:f>
         <x:v>No confirmed time</x:v>
       </x:c>
     </x:row>
@@ -741,7 +741,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E19" s="6" t="n">
-        <x:f>IF(A19&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A19,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A19&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A19,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F19" s="6" t="n">
@@ -761,7 +761,7 @@
         <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J19" s="1" t="str">
-        <x:f>IF(A19&gt;$B$4,"Future",IF(A19=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A19,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E19=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A19&gt;$B$4,"Future",IF(A19=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A19,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E19=0,"No confirmed time","Logged"))))</x:f>
         <x:v>No confirmed time</x:v>
       </x:c>
     </x:row>
@@ -781,7 +781,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E20" s="6" t="n">
-        <x:f>IF(A20&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A20,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A20&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A20,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F20" s="6" t="n">
@@ -801,7 +801,7 @@
         <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J20" s="1" t="str">
-        <x:f>IF(A20&gt;$B$4,"Future",IF(A20=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A20,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E20=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A20&gt;$B$4,"Future",IF(A20=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A20,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E20=0,"No confirmed time","Logged"))))</x:f>
         <x:v>No confirmed time</x:v>
       </x:c>
     </x:row>
@@ -821,7 +821,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E21" s="6" t="n">
-        <x:f>IF(A21&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A21,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A21&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A21,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F21" s="6" t="n">
@@ -841,7 +841,7 @@
         <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J21" s="1" t="str">
-        <x:f>IF(A21&gt;$B$4,"Future",IF(A21=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A21,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E21=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A21&gt;$B$4,"Future",IF(A21=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A21,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E21=0,"No confirmed time","Logged"))))</x:f>
         <x:v>No confirmed time</x:v>
       </x:c>
     </x:row>
@@ -861,25 +861,28 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E22" s="6" t="n">
-        <x:f>IF(A22&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A22,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F22" s="6" t="str">
+        <x:f>IF(A22&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A22,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F22" s="6" t="n">
         <x:f>IF(A22&gt;=$B$4,"",MAX(D22-E22,0))</x:f>
-      </x:c>
-      <x:c r="G22" s="6" t="str">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G22" s="6" t="n">
         <x:f>IF(A22&gt;=$B$4,"",MAX(E22-D22,0))</x:f>
-      </x:c>
-      <x:c r="H22" s="6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H22" s="6" t="n">
         <x:f>IF(A22&gt;=$B$4,"",SUM($D$15:D22))</x:f>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="I22" s="6" t="n">
         <x:f>IF(A22&gt;$B$4,"",SUM($E$15:E22))</x:f>
         <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J22" s="1" t="str">
-        <x:f>IF(A22&gt;$B$4,"Future",IF(A22=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A22,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E22=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>In progress</x:v>
+        <x:f>IF(A22&gt;$B$4,"Future",IF(A22=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A22,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E22=0,"No confirmed time","Logged"))))</x:f>
+        <x:v>Uncertain time</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="22" customHeight="1">
@@ -897,24 +900,29 @@
         <x:f>IF(WEEKDAY(A23,2)&gt;5,$B$7,IF(A23&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="E23" s="6" t="str">
-        <x:f>IF(A23&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A23,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F23" s="6" t="str">
+      <x:c r="E23" s="6" t="n">
+        <x:f>IF(A23&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A23,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F23" s="6" t="n">
         <x:f>IF(A23&gt;=$B$4,"",MAX(D23-E23,0))</x:f>
-      </x:c>
-      <x:c r="G23" s="6" t="str">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G23" s="6" t="n">
         <x:f>IF(A23&gt;=$B$4,"",MAX(E23-D23,0))</x:f>
-      </x:c>
-      <x:c r="H23" s="6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H23" s="6" t="n">
         <x:f>IF(A23&gt;=$B$4,"",SUM($D$15:D23))</x:f>
-      </x:c>
-      <x:c r="I23" s="6" t="str">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="I23" s="6" t="n">
         <x:f>IF(A23&gt;$B$4,"",SUM($E$15:E23))</x:f>
+        <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J23" s="1" t="str">
-        <x:f>IF(A23&gt;$B$4,"Future",IF(A23=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A23,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E23=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
+        <x:f>IF(A23&gt;$B$4,"Future",IF(A23=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A23,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E23=0,"No confirmed time","Logged"))))</x:f>
+        <x:v>No confirmed time</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="22" customHeight="1">
@@ -932,24 +940,29 @@
         <x:f>IF(WEEKDAY(A24,2)&gt;5,$B$7,IF(A24&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="E24" s="6" t="str">
-        <x:f>IF(A24&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A24,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F24" s="6" t="str">
+      <x:c r="E24" s="6" t="n">
+        <x:f>IF(A24&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A24,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F24" s="6" t="n">
         <x:f>IF(A24&gt;=$B$4,"",MAX(D24-E24,0))</x:f>
-      </x:c>
-      <x:c r="G24" s="6" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G24" s="6" t="n">
         <x:f>IF(A24&gt;=$B$4,"",MAX(E24-D24,0))</x:f>
-      </x:c>
-      <x:c r="H24" s="6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H24" s="6" t="n">
         <x:f>IF(A24&gt;=$B$4,"",SUM($D$15:D24))</x:f>
-      </x:c>
-      <x:c r="I24" s="6" t="str">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="I24" s="6" t="n">
         <x:f>IF(A24&gt;$B$4,"",SUM($E$15:E24))</x:f>
+        <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J24" s="1" t="str">
-        <x:f>IF(A24&gt;$B$4,"Future",IF(A24=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A24,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E24=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
+        <x:f>IF(A24&gt;$B$4,"Future",IF(A24=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A24,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E24=0,"No confirmed time","Logged"))))</x:f>
+        <x:v>No confirmed time</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="22" customHeight="1">
@@ -967,24 +980,29 @@
         <x:f>IF(WEEKDAY(A25,2)&gt;5,$B$7,IF(A25&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="E25" s="6" t="str">
-        <x:f>IF(A25&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A25,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
-      </x:c>
-      <x:c r="F25" s="6" t="str">
+      <x:c r="E25" s="6" t="n">
+        <x:f>IF(A25&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A25,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F25" s="6" t="n">
         <x:f>IF(A25&gt;=$B$4,"",MAX(D25-E25,0))</x:f>
-      </x:c>
-      <x:c r="G25" s="6" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G25" s="6" t="n">
         <x:f>IF(A25&gt;=$B$4,"",MAX(E25-D25,0))</x:f>
-      </x:c>
-      <x:c r="H25" s="6" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H25" s="6" t="n">
         <x:f>IF(A25&gt;=$B$4,"",SUM($D$15:D25))</x:f>
-      </x:c>
-      <x:c r="I25" s="6" t="str">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="I25" s="6" t="n">
         <x:f>IF(A25&gt;$B$4,"",SUM($E$15:E25))</x:f>
+        <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J25" s="1" t="str">
-        <x:f>IF(A25&gt;$B$4,"Future",IF(A25=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A25,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E25=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
+        <x:f>IF(A25&gt;$B$4,"Future",IF(A25=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A25,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E25=0,"No confirmed time","Logged"))))</x:f>
+        <x:v>No confirmed time</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="22" customHeight="1">
@@ -1002,8 +1020,9 @@
         <x:f>IF(WEEKDAY(A26,2)&gt;5,$B$7,IF(A26&lt;$B$8,$H$4,$B$6))</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="E26" s="6" t="str">
-        <x:f>IF(A26&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A26,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+      <x:c r="E26" s="6" t="n">
+        <x:f>IF(A26&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A26,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F26" s="6" t="str">
         <x:f>IF(A26&gt;=$B$4,"",MAX(D26-E26,0))</x:f>
@@ -1014,12 +1033,13 @@
       <x:c r="H26" s="6" t="str">
         <x:f>IF(A26&gt;=$B$4,"",SUM($D$15:D26))</x:f>
       </x:c>
-      <x:c r="I26" s="6" t="str">
+      <x:c r="I26" s="6" t="n">
         <x:f>IF(A26&gt;$B$4,"",SUM($E$15:E26))</x:f>
+        <x:v>11.151388888889445</x:v>
       </x:c>
       <x:c r="J26" s="1" t="str">
-        <x:f>IF(A26&gt;$B$4,"Future",IF(A26=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A26,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E26=0,"No confirmed time","Logged"))))</x:f>
-        <x:v>Future</x:v>
+        <x:f>IF(A26&gt;$B$4,"Future",IF(A26=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A26,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E26=0,"No confirmed time","Logged"))))</x:f>
+        <x:v>In progress</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="22" customHeight="1">
@@ -1038,7 +1058,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E27" s="6" t="str">
-        <x:f>IF(A27&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A27,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A27&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A27,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F27" s="6" t="str">
         <x:f>IF(A27&gt;=$B$4,"",MAX(D27-E27,0))</x:f>
@@ -1053,7 +1073,7 @@
         <x:f>IF(A27&gt;$B$4,"",SUM($E$15:E27))</x:f>
       </x:c>
       <x:c r="J27" s="1" t="str">
-        <x:f>IF(A27&gt;$B$4,"Future",IF(A27=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A27,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E27=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A27&gt;$B$4,"Future",IF(A27=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A27,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E27=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1073,7 +1093,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E28" s="6" t="str">
-        <x:f>IF(A28&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A28,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A28&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A28,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F28" s="6" t="str">
         <x:f>IF(A28&gt;=$B$4,"",MAX(D28-E28,0))</x:f>
@@ -1088,7 +1108,7 @@
         <x:f>IF(A28&gt;$B$4,"",SUM($E$15:E28))</x:f>
       </x:c>
       <x:c r="J28" s="1" t="str">
-        <x:f>IF(A28&gt;$B$4,"Future",IF(A28=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A28,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E28=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A28&gt;$B$4,"Future",IF(A28=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A28,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E28=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1108,7 +1128,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E29" s="6" t="str">
-        <x:f>IF(A29&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A29,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A29&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A29,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F29" s="6" t="str">
         <x:f>IF(A29&gt;=$B$4,"",MAX(D29-E29,0))</x:f>
@@ -1123,7 +1143,7 @@
         <x:f>IF(A29&gt;$B$4,"",SUM($E$15:E29))</x:f>
       </x:c>
       <x:c r="J29" s="1" t="str">
-        <x:f>IF(A29&gt;$B$4,"Future",IF(A29=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A29,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E29=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A29&gt;$B$4,"Future",IF(A29=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A29,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E29=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1143,7 +1163,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E30" s="6" t="str">
-        <x:f>IF(A30&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A30,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A30&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A30,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F30" s="6" t="str">
         <x:f>IF(A30&gt;=$B$4,"",MAX(D30-E30,0))</x:f>
@@ -1158,7 +1178,7 @@
         <x:f>IF(A30&gt;$B$4,"",SUM($E$15:E30))</x:f>
       </x:c>
       <x:c r="J30" s="1" t="str">
-        <x:f>IF(A30&gt;$B$4,"Future",IF(A30=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A30,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E30=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A30&gt;$B$4,"Future",IF(A30=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A30,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E30=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1178,7 +1198,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E31" s="6" t="str">
-        <x:f>IF(A31&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A31,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A31&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A31,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F31" s="6" t="str">
         <x:f>IF(A31&gt;=$B$4,"",MAX(D31-E31,0))</x:f>
@@ -1193,7 +1213,7 @@
         <x:f>IF(A31&gt;$B$4,"",SUM($E$15:E31))</x:f>
       </x:c>
       <x:c r="J31" s="1" t="str">
-        <x:f>IF(A31&gt;$B$4,"Future",IF(A31=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A31,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E31=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A31&gt;$B$4,"Future",IF(A31=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A31,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E31=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1213,7 +1233,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E32" s="6" t="str">
-        <x:f>IF(A32&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A32,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A32&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A32,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F32" s="6" t="str">
         <x:f>IF(A32&gt;=$B$4,"",MAX(D32-E32,0))</x:f>
@@ -1228,7 +1248,7 @@
         <x:f>IF(A32&gt;$B$4,"",SUM($E$15:E32))</x:f>
       </x:c>
       <x:c r="J32" s="1" t="str">
-        <x:f>IF(A32&gt;$B$4,"Future",IF(A32=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A32,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E32=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A32&gt;$B$4,"Future",IF(A32=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A32,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E32=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1248,7 +1268,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E33" s="6" t="str">
-        <x:f>IF(A33&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A33,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A33&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A33,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F33" s="6" t="str">
         <x:f>IF(A33&gt;=$B$4,"",MAX(D33-E33,0))</x:f>
@@ -1263,7 +1283,7 @@
         <x:f>IF(A33&gt;$B$4,"",SUM($E$15:E33))</x:f>
       </x:c>
       <x:c r="J33" s="1" t="str">
-        <x:f>IF(A33&gt;$B$4,"Future",IF(A33=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A33,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E33=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A33&gt;$B$4,"Future",IF(A33=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A33,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E33=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1283,7 +1303,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E34" s="6" t="str">
-        <x:f>IF(A34&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A34,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A34&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A34,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F34" s="6" t="str">
         <x:f>IF(A34&gt;=$B$4,"",MAX(D34-E34,0))</x:f>
@@ -1298,7 +1318,7 @@
         <x:f>IF(A34&gt;$B$4,"",SUM($E$15:E34))</x:f>
       </x:c>
       <x:c r="J34" s="1" t="str">
-        <x:f>IF(A34&gt;$B$4,"Future",IF(A34=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A34,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E34=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A34&gt;$B$4,"Future",IF(A34=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A34,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E34=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1318,7 +1338,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E35" s="6" t="str">
-        <x:f>IF(A35&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A35,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A35&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A35,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F35" s="6" t="str">
         <x:f>IF(A35&gt;=$B$4,"",MAX(D35-E35,0))</x:f>
@@ -1333,7 +1353,7 @@
         <x:f>IF(A35&gt;$B$4,"",SUM($E$15:E35))</x:f>
       </x:c>
       <x:c r="J35" s="1" t="str">
-        <x:f>IF(A35&gt;$B$4,"Future",IF(A35=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A35,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E35=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A35&gt;$B$4,"Future",IF(A35=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A35,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E35=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1353,7 +1373,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E36" s="6" t="str">
-        <x:f>IF(A36&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A36,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A36&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A36,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F36" s="6" t="str">
         <x:f>IF(A36&gt;=$B$4,"",MAX(D36-E36,0))</x:f>
@@ -1368,7 +1388,7 @@
         <x:f>IF(A36&gt;$B$4,"",SUM($E$15:E36))</x:f>
       </x:c>
       <x:c r="J36" s="1" t="str">
-        <x:f>IF(A36&gt;$B$4,"Future",IF(A36=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A36,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E36=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A36&gt;$B$4,"Future",IF(A36=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A36,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E36=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1388,7 +1408,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E37" s="6" t="str">
-        <x:f>IF(A37&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A37,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A37&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A37,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F37" s="6" t="str">
         <x:f>IF(A37&gt;=$B$4,"",MAX(D37-E37,0))</x:f>
@@ -1403,7 +1423,7 @@
         <x:f>IF(A37&gt;$B$4,"",SUM($E$15:E37))</x:f>
       </x:c>
       <x:c r="J37" s="1" t="str">
-        <x:f>IF(A37&gt;$B$4,"Future",IF(A37=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A37,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E37=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A37&gt;$B$4,"Future",IF(A37=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A37,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E37=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1423,7 +1443,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E38" s="6" t="str">
-        <x:f>IF(A38&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A38,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A38&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A38,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F38" s="6" t="str">
         <x:f>IF(A38&gt;=$B$4,"",MAX(D38-E38,0))</x:f>
@@ -1438,7 +1458,7 @@
         <x:f>IF(A38&gt;$B$4,"",SUM($E$15:E38))</x:f>
       </x:c>
       <x:c r="J38" s="1" t="str">
-        <x:f>IF(A38&gt;$B$4,"Future",IF(A38=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A38,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E38=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A38&gt;$B$4,"Future",IF(A38=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A38,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E38=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1458,7 +1478,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E39" s="6" t="str">
-        <x:f>IF(A39&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A39,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A39&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A39,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F39" s="6" t="str">
         <x:f>IF(A39&gt;=$B$4,"",MAX(D39-E39,0))</x:f>
@@ -1473,7 +1493,7 @@
         <x:f>IF(A39&gt;$B$4,"",SUM($E$15:E39))</x:f>
       </x:c>
       <x:c r="J39" s="1" t="str">
-        <x:f>IF(A39&gt;$B$4,"Future",IF(A39=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A39,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E39=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A39&gt;$B$4,"Future",IF(A39=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A39,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E39=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1493,7 +1513,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E40" s="6" t="str">
-        <x:f>IF(A40&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A40,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A40&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A40,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F40" s="6" t="str">
         <x:f>IF(A40&gt;=$B$4,"",MAX(D40-E40,0))</x:f>
@@ -1508,7 +1528,7 @@
         <x:f>IF(A40&gt;$B$4,"",SUM($E$15:E40))</x:f>
       </x:c>
       <x:c r="J40" s="1" t="str">
-        <x:f>IF(A40&gt;$B$4,"Future",IF(A40=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A40,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E40=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A40&gt;$B$4,"Future",IF(A40=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A40,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E40=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1528,7 +1548,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E41" s="6" t="str">
-        <x:f>IF(A41&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A41,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A41&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A41,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F41" s="6" t="str">
         <x:f>IF(A41&gt;=$B$4,"",MAX(D41-E41,0))</x:f>
@@ -1543,7 +1563,7 @@
         <x:f>IF(A41&gt;$B$4,"",SUM($E$15:E41))</x:f>
       </x:c>
       <x:c r="J41" s="1" t="str">
-        <x:f>IF(A41&gt;$B$4,"Future",IF(A41=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A41,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E41=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A41&gt;$B$4,"Future",IF(A41=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A41,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E41=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1563,7 +1583,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E42" s="6" t="str">
-        <x:f>IF(A42&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A42,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A42&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A42,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F42" s="6" t="str">
         <x:f>IF(A42&gt;=$B$4,"",MAX(D42-E42,0))</x:f>
@@ -1578,7 +1598,7 @@
         <x:f>IF(A42&gt;$B$4,"",SUM($E$15:E42))</x:f>
       </x:c>
       <x:c r="J42" s="1" t="str">
-        <x:f>IF(A42&gt;$B$4,"Future",IF(A42=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A42,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E42=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A42&gt;$B$4,"Future",IF(A42=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A42,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E42=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1598,7 +1618,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E43" s="6" t="str">
-        <x:f>IF(A43&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A43,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A43&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A43,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F43" s="6" t="str">
         <x:f>IF(A43&gt;=$B$4,"",MAX(D43-E43,0))</x:f>
@@ -1613,7 +1633,7 @@
         <x:f>IF(A43&gt;$B$4,"",SUM($E$15:E43))</x:f>
       </x:c>
       <x:c r="J43" s="1" t="str">
-        <x:f>IF(A43&gt;$B$4,"Future",IF(A43=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A43,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E43=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A43&gt;$B$4,"Future",IF(A43=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A43,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E43=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1633,7 +1653,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E44" s="6" t="str">
-        <x:f>IF(A44&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A44,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A44&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A44,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F44" s="6" t="str">
         <x:f>IF(A44&gt;=$B$4,"",MAX(D44-E44,0))</x:f>
@@ -1648,7 +1668,7 @@
         <x:f>IF(A44&gt;$B$4,"",SUM($E$15:E44))</x:f>
       </x:c>
       <x:c r="J44" s="1" t="str">
-        <x:f>IF(A44&gt;$B$4,"Future",IF(A44=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A44,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E44=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A44&gt;$B$4,"Future",IF(A44=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A44,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E44=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1668,7 +1688,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E45" s="6" t="str">
-        <x:f>IF(A45&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A45,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A45&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A45,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F45" s="6" t="str">
         <x:f>IF(A45&gt;=$B$4,"",MAX(D45-E45,0))</x:f>
@@ -1683,7 +1703,7 @@
         <x:f>IF(A45&gt;$B$4,"",SUM($E$15:E45))</x:f>
       </x:c>
       <x:c r="J45" s="1" t="str">
-        <x:f>IF(A45&gt;$B$4,"Future",IF(A45=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A45,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E45=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A45&gt;$B$4,"Future",IF(A45=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A45,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E45=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1703,7 +1723,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E46" s="6" t="str">
-        <x:f>IF(A46&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A46,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A46&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A46,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F46" s="6" t="str">
         <x:f>IF(A46&gt;=$B$4,"",MAX(D46-E46,0))</x:f>
@@ -1718,7 +1738,7 @@
         <x:f>IF(A46&gt;$B$4,"",SUM($E$15:E46))</x:f>
       </x:c>
       <x:c r="J46" s="1" t="str">
-        <x:f>IF(A46&gt;$B$4,"Future",IF(A46=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A46,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E46=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A46&gt;$B$4,"Future",IF(A46=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A46,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E46=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1738,7 +1758,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E47" s="6" t="str">
-        <x:f>IF(A47&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A47,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A47&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A47,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F47" s="6" t="str">
         <x:f>IF(A47&gt;=$B$4,"",MAX(D47-E47,0))</x:f>
@@ -1753,7 +1773,7 @@
         <x:f>IF(A47&gt;$B$4,"",SUM($E$15:E47))</x:f>
       </x:c>
       <x:c r="J47" s="1" t="str">
-        <x:f>IF(A47&gt;$B$4,"Future",IF(A47=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A47,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E47=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A47&gt;$B$4,"Future",IF(A47=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A47,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E47=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1773,7 +1793,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E48" s="6" t="str">
-        <x:f>IF(A48&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A48,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A48&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A48,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F48" s="6" t="str">
         <x:f>IF(A48&gt;=$B$4,"",MAX(D48-E48,0))</x:f>
@@ -1788,7 +1808,7 @@
         <x:f>IF(A48&gt;$B$4,"",SUM($E$15:E48))</x:f>
       </x:c>
       <x:c r="J48" s="1" t="str">
-        <x:f>IF(A48&gt;$B$4,"Future",IF(A48=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A48,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E48=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A48&gt;$B$4,"Future",IF(A48=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A48,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E48=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1808,7 +1828,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E49" s="6" t="str">
-        <x:f>IF(A49&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A49,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A49&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A49,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F49" s="6" t="str">
         <x:f>IF(A49&gt;=$B$4,"",MAX(D49-E49,0))</x:f>
@@ -1823,7 +1843,7 @@
         <x:f>IF(A49&gt;$B$4,"",SUM($E$15:E49))</x:f>
       </x:c>
       <x:c r="J49" s="1" t="str">
-        <x:f>IF(A49&gt;$B$4,"Future",IF(A49=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A49,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E49=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A49&gt;$B$4,"Future",IF(A49=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A49,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E49=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1843,7 +1863,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E50" s="6" t="str">
-        <x:f>IF(A50&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A50,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A50&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A50,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F50" s="6" t="str">
         <x:f>IF(A50&gt;=$B$4,"",MAX(D50-E50,0))</x:f>
@@ -1858,7 +1878,7 @@
         <x:f>IF(A50&gt;$B$4,"",SUM($E$15:E50))</x:f>
       </x:c>
       <x:c r="J50" s="1" t="str">
-        <x:f>IF(A50&gt;$B$4,"Future",IF(A50=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A50,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E50=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A50&gt;$B$4,"Future",IF(A50=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A50,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E50=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1878,7 +1898,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E51" s="6" t="str">
-        <x:f>IF(A51&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A51,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A51&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A51,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F51" s="6" t="str">
         <x:f>IF(A51&gt;=$B$4,"",MAX(D51-E51,0))</x:f>
@@ -1893,7 +1913,7 @@
         <x:f>IF(A51&gt;$B$4,"",SUM($E$15:E51))</x:f>
       </x:c>
       <x:c r="J51" s="1" t="str">
-        <x:f>IF(A51&gt;$B$4,"Future",IF(A51=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A51,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E51=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A51&gt;$B$4,"Future",IF(A51=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A51,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E51=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1913,7 +1933,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E52" s="6" t="str">
-        <x:f>IF(A52&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A52,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A52&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A52,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F52" s="6" t="str">
         <x:f>IF(A52&gt;=$B$4,"",MAX(D52-E52,0))</x:f>
@@ -1928,7 +1948,7 @@
         <x:f>IF(A52&gt;$B$4,"",SUM($E$15:E52))</x:f>
       </x:c>
       <x:c r="J52" s="1" t="str">
-        <x:f>IF(A52&gt;$B$4,"Future",IF(A52=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A52,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E52=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A52&gt;$B$4,"Future",IF(A52=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A52,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E52=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1948,7 +1968,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E53" s="6" t="str">
-        <x:f>IF(A53&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A53,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A53&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A53,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F53" s="6" t="str">
         <x:f>IF(A53&gt;=$B$4,"",MAX(D53-E53,0))</x:f>
@@ -1963,7 +1983,7 @@
         <x:f>IF(A53&gt;$B$4,"",SUM($E$15:E53))</x:f>
       </x:c>
       <x:c r="J53" s="1" t="str">
-        <x:f>IF(A53&gt;$B$4,"Future",IF(A53=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A53,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E53=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A53&gt;$B$4,"Future",IF(A53=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A53,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E53=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -1983,7 +2003,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E54" s="6" t="str">
-        <x:f>IF(A54&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A54,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A54&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A54,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F54" s="6" t="str">
         <x:f>IF(A54&gt;=$B$4,"",MAX(D54-E54,0))</x:f>
@@ -1998,7 +2018,7 @@
         <x:f>IF(A54&gt;$B$4,"",SUM($E$15:E54))</x:f>
       </x:c>
       <x:c r="J54" s="1" t="str">
-        <x:f>IF(A54&gt;$B$4,"Future",IF(A54=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A54,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E54=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A54&gt;$B$4,"Future",IF(A54=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A54,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E54=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2018,7 +2038,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E55" s="6" t="str">
-        <x:f>IF(A55&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A55,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A55&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A55,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F55" s="6" t="str">
         <x:f>IF(A55&gt;=$B$4,"",MAX(D55-E55,0))</x:f>
@@ -2033,7 +2053,7 @@
         <x:f>IF(A55&gt;$B$4,"",SUM($E$15:E55))</x:f>
       </x:c>
       <x:c r="J55" s="1" t="str">
-        <x:f>IF(A55&gt;$B$4,"Future",IF(A55=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A55,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E55=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A55&gt;$B$4,"Future",IF(A55=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A55,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E55=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2053,7 +2073,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E56" s="6" t="str">
-        <x:f>IF(A56&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A56,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A56&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A56,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F56" s="6" t="str">
         <x:f>IF(A56&gt;=$B$4,"",MAX(D56-E56,0))</x:f>
@@ -2068,7 +2088,7 @@
         <x:f>IF(A56&gt;$B$4,"",SUM($E$15:E56))</x:f>
       </x:c>
       <x:c r="J56" s="1" t="str">
-        <x:f>IF(A56&gt;$B$4,"Future",IF(A56=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A56,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E56=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A56&gt;$B$4,"Future",IF(A56=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A56,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E56=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2088,7 +2108,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E57" s="6" t="str">
-        <x:f>IF(A57&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A57,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A57&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A57,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F57" s="6" t="str">
         <x:f>IF(A57&gt;=$B$4,"",MAX(D57-E57,0))</x:f>
@@ -2103,7 +2123,7 @@
         <x:f>IF(A57&gt;$B$4,"",SUM($E$15:E57))</x:f>
       </x:c>
       <x:c r="J57" s="1" t="str">
-        <x:f>IF(A57&gt;$B$4,"Future",IF(A57=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A57,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E57=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A57&gt;$B$4,"Future",IF(A57=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A57,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E57=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2123,7 +2143,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E58" s="6" t="str">
-        <x:f>IF(A58&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A58,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A58&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A58,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F58" s="6" t="str">
         <x:f>IF(A58&gt;=$B$4,"",MAX(D58-E58,0))</x:f>
@@ -2138,7 +2158,7 @@
         <x:f>IF(A58&gt;$B$4,"",SUM($E$15:E58))</x:f>
       </x:c>
       <x:c r="J58" s="1" t="str">
-        <x:f>IF(A58&gt;$B$4,"Future",IF(A58=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A58,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E58=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A58&gt;$B$4,"Future",IF(A58=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A58,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E58=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2158,7 +2178,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E59" s="6" t="str">
-        <x:f>IF(A59&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A59,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A59&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A59,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F59" s="6" t="str">
         <x:f>IF(A59&gt;=$B$4,"",MAX(D59-E59,0))</x:f>
@@ -2173,7 +2193,7 @@
         <x:f>IF(A59&gt;$B$4,"",SUM($E$15:E59))</x:f>
       </x:c>
       <x:c r="J59" s="1" t="str">
-        <x:f>IF(A59&gt;$B$4,"Future",IF(A59=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A59,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E59=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A59&gt;$B$4,"Future",IF(A59=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A59,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E59=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2193,7 +2213,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E60" s="6" t="str">
-        <x:f>IF(A60&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A60,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A60&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A60,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F60" s="6" t="str">
         <x:f>IF(A60&gt;=$B$4,"",MAX(D60-E60,0))</x:f>
@@ -2208,7 +2228,7 @@
         <x:f>IF(A60&gt;$B$4,"",SUM($E$15:E60))</x:f>
       </x:c>
       <x:c r="J60" s="1" t="str">
-        <x:f>IF(A60&gt;$B$4,"Future",IF(A60=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A60,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E60=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A60&gt;$B$4,"Future",IF(A60=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A60,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E60=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2228,7 +2248,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E61" s="6" t="str">
-        <x:f>IF(A61&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A61,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A61&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A61,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F61" s="6" t="str">
         <x:f>IF(A61&gt;=$B$4,"",MAX(D61-E61,0))</x:f>
@@ -2243,7 +2263,7 @@
         <x:f>IF(A61&gt;$B$4,"",SUM($E$15:E61))</x:f>
       </x:c>
       <x:c r="J61" s="1" t="str">
-        <x:f>IF(A61&gt;$B$4,"Future",IF(A61=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A61,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E61=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A61&gt;$B$4,"Future",IF(A61=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A61,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E61=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2263,7 +2283,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E62" s="6" t="str">
-        <x:f>IF(A62&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A62,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A62&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A62,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F62" s="6" t="str">
         <x:f>IF(A62&gt;=$B$4,"",MAX(D62-E62,0))</x:f>
@@ -2278,7 +2298,7 @@
         <x:f>IF(A62&gt;$B$4,"",SUM($E$15:E62))</x:f>
       </x:c>
       <x:c r="J62" s="1" t="str">
-        <x:f>IF(A62&gt;$B$4,"Future",IF(A62=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A62,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E62=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A62&gt;$B$4,"Future",IF(A62=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A62,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E62=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2298,7 +2318,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E63" s="6" t="str">
-        <x:f>IF(A63&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A63,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A63&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A63,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F63" s="6" t="str">
         <x:f>IF(A63&gt;=$B$4,"",MAX(D63-E63,0))</x:f>
@@ -2313,7 +2333,7 @@
         <x:f>IF(A63&gt;$B$4,"",SUM($E$15:E63))</x:f>
       </x:c>
       <x:c r="J63" s="1" t="str">
-        <x:f>IF(A63&gt;$B$4,"Future",IF(A63=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A63,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E63=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A63&gt;$B$4,"Future",IF(A63=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A63,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E63=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2333,7 +2353,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E64" s="6" t="str">
-        <x:f>IF(A64&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A64,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A64&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A64,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F64" s="6" t="str">
         <x:f>IF(A64&gt;=$B$4,"",MAX(D64-E64,0))</x:f>
@@ -2348,7 +2368,7 @@
         <x:f>IF(A64&gt;$B$4,"",SUM($E$15:E64))</x:f>
       </x:c>
       <x:c r="J64" s="1" t="str">
-        <x:f>IF(A64&gt;$B$4,"Future",IF(A64=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A64,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E64=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A64&gt;$B$4,"Future",IF(A64=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A64,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E64=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2368,7 +2388,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E65" s="6" t="str">
-        <x:f>IF(A65&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A65,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A65&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A65,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F65" s="6" t="str">
         <x:f>IF(A65&gt;=$B$4,"",MAX(D65-E65,0))</x:f>
@@ -2383,7 +2403,7 @@
         <x:f>IF(A65&gt;$B$4,"",SUM($E$15:E65))</x:f>
       </x:c>
       <x:c r="J65" s="1" t="str">
-        <x:f>IF(A65&gt;$B$4,"Future",IF(A65=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A65,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E65=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A65&gt;$B$4,"Future",IF(A65=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A65,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E65=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2403,7 +2423,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E66" s="6" t="str">
-        <x:f>IF(A66&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A66,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A66&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A66,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F66" s="6" t="str">
         <x:f>IF(A66&gt;=$B$4,"",MAX(D66-E66,0))</x:f>
@@ -2418,7 +2438,7 @@
         <x:f>IF(A66&gt;$B$4,"",SUM($E$15:E66))</x:f>
       </x:c>
       <x:c r="J66" s="1" t="str">
-        <x:f>IF(A66&gt;$B$4,"Future",IF(A66=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A66,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E66=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A66&gt;$B$4,"Future",IF(A66=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A66,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E66=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2438,7 +2458,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E67" s="6" t="str">
-        <x:f>IF(A67&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A67,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A67&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A67,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F67" s="6" t="str">
         <x:f>IF(A67&gt;=$B$4,"",MAX(D67-E67,0))</x:f>
@@ -2453,7 +2473,7 @@
         <x:f>IF(A67&gt;$B$4,"",SUM($E$15:E67))</x:f>
       </x:c>
       <x:c r="J67" s="1" t="str">
-        <x:f>IF(A67&gt;$B$4,"Future",IF(A67=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A67,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E67=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A67&gt;$B$4,"Future",IF(A67=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A67,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E67=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2473,7 +2493,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E68" s="6" t="str">
-        <x:f>IF(A68&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A68,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A68&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A68,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F68" s="6" t="str">
         <x:f>IF(A68&gt;=$B$4,"",MAX(D68-E68,0))</x:f>
@@ -2488,7 +2508,7 @@
         <x:f>IF(A68&gt;$B$4,"",SUM($E$15:E68))</x:f>
       </x:c>
       <x:c r="J68" s="1" t="str">
-        <x:f>IF(A68&gt;$B$4,"Future",IF(A68=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A68,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E68=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A68&gt;$B$4,"Future",IF(A68=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A68,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E68=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2508,7 +2528,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E69" s="6" t="str">
-        <x:f>IF(A69&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A69,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A69&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A69,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F69" s="6" t="str">
         <x:f>IF(A69&gt;=$B$4,"",MAX(D69-E69,0))</x:f>
@@ -2523,7 +2543,7 @@
         <x:f>IF(A69&gt;$B$4,"",SUM($E$15:E69))</x:f>
       </x:c>
       <x:c r="J69" s="1" t="str">
-        <x:f>IF(A69&gt;$B$4,"Future",IF(A69=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A69,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E69=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A69&gt;$B$4,"Future",IF(A69=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A69,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E69=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2543,7 +2563,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E70" s="6" t="str">
-        <x:f>IF(A70&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A70,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A70&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A70,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F70" s="6" t="str">
         <x:f>IF(A70&gt;=$B$4,"",MAX(D70-E70,0))</x:f>
@@ -2558,7 +2578,7 @@
         <x:f>IF(A70&gt;$B$4,"",SUM($E$15:E70))</x:f>
       </x:c>
       <x:c r="J70" s="1" t="str">
-        <x:f>IF(A70&gt;$B$4,"Future",IF(A70=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A70,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E70=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A70&gt;$B$4,"Future",IF(A70=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A70,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E70=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2578,7 +2598,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E71" s="6" t="str">
-        <x:f>IF(A71&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A71,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A71&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A71,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F71" s="6" t="str">
         <x:f>IF(A71&gt;=$B$4,"",MAX(D71-E71,0))</x:f>
@@ -2593,7 +2613,7 @@
         <x:f>IF(A71&gt;$B$4,"",SUM($E$15:E71))</x:f>
       </x:c>
       <x:c r="J71" s="1" t="str">
-        <x:f>IF(A71&gt;$B$4,"Future",IF(A71=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A71,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E71=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A71&gt;$B$4,"Future",IF(A71=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A71,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E71=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2613,7 +2633,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E72" s="6" t="str">
-        <x:f>IF(A72&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A72,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A72&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A72,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F72" s="6" t="str">
         <x:f>IF(A72&gt;=$B$4,"",MAX(D72-E72,0))</x:f>
@@ -2628,7 +2648,7 @@
         <x:f>IF(A72&gt;$B$4,"",SUM($E$15:E72))</x:f>
       </x:c>
       <x:c r="J72" s="1" t="str">
-        <x:f>IF(A72&gt;$B$4,"Future",IF(A72=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A72,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E72=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A72&gt;$B$4,"Future",IF(A72=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A72,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E72=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2648,7 +2668,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E73" s="6" t="str">
-        <x:f>IF(A73&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A73,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A73&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A73,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F73" s="6" t="str">
         <x:f>IF(A73&gt;=$B$4,"",MAX(D73-E73,0))</x:f>
@@ -2663,7 +2683,7 @@
         <x:f>IF(A73&gt;$B$4,"",SUM($E$15:E73))</x:f>
       </x:c>
       <x:c r="J73" s="1" t="str">
-        <x:f>IF(A73&gt;$B$4,"Future",IF(A73=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A73,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E73=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A73&gt;$B$4,"Future",IF(A73=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A73,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E73=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2683,7 +2703,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E74" s="6" t="str">
-        <x:f>IF(A74&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A74,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A74&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A74,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F74" s="6" t="str">
         <x:f>IF(A74&gt;=$B$4,"",MAX(D74-E74,0))</x:f>
@@ -2698,7 +2718,7 @@
         <x:f>IF(A74&gt;$B$4,"",SUM($E$15:E74))</x:f>
       </x:c>
       <x:c r="J74" s="1" t="str">
-        <x:f>IF(A74&gt;$B$4,"Future",IF(A74=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A74,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E74=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A74&gt;$B$4,"Future",IF(A74=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A74,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E74=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2718,7 +2738,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E75" s="6" t="str">
-        <x:f>IF(A75&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A75,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A75&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A75,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F75" s="6" t="str">
         <x:f>IF(A75&gt;=$B$4,"",MAX(D75-E75,0))</x:f>
@@ -2733,7 +2753,7 @@
         <x:f>IF(A75&gt;$B$4,"",SUM($E$15:E75))</x:f>
       </x:c>
       <x:c r="J75" s="1" t="str">
-        <x:f>IF(A75&gt;$B$4,"Future",IF(A75=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A75,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E75=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A75&gt;$B$4,"Future",IF(A75=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A75,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E75=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2753,7 +2773,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E76" s="6" t="str">
-        <x:f>IF(A76&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A76,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A76&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A76,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F76" s="6" t="str">
         <x:f>IF(A76&gt;=$B$4,"",MAX(D76-E76,0))</x:f>
@@ -2768,7 +2788,7 @@
         <x:f>IF(A76&gt;$B$4,"",SUM($E$15:E76))</x:f>
       </x:c>
       <x:c r="J76" s="1" t="str">
-        <x:f>IF(A76&gt;$B$4,"Future",IF(A76=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A76,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E76=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A76&gt;$B$4,"Future",IF(A76=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A76,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E76=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2788,7 +2808,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E77" s="6" t="str">
-        <x:f>IF(A77&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A77,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A77&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A77,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F77" s="6" t="str">
         <x:f>IF(A77&gt;=$B$4,"",MAX(D77-E77,0))</x:f>
@@ -2803,7 +2823,7 @@
         <x:f>IF(A77&gt;$B$4,"",SUM($E$15:E77))</x:f>
       </x:c>
       <x:c r="J77" s="1" t="str">
-        <x:f>IF(A77&gt;$B$4,"Future",IF(A77=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A77,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E77=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A77&gt;$B$4,"Future",IF(A77=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A77,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E77=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2823,7 +2843,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E78" s="6" t="str">
-        <x:f>IF(A78&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A78,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A78&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A78,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F78" s="6" t="str">
         <x:f>IF(A78&gt;=$B$4,"",MAX(D78-E78,0))</x:f>
@@ -2838,7 +2858,7 @@
         <x:f>IF(A78&gt;$B$4,"",SUM($E$15:E78))</x:f>
       </x:c>
       <x:c r="J78" s="1" t="str">
-        <x:f>IF(A78&gt;$B$4,"Future",IF(A78=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A78,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E78=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A78&gt;$B$4,"Future",IF(A78=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A78,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E78=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2858,7 +2878,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E79" s="6" t="str">
-        <x:f>IF(A79&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A79,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A79&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A79,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F79" s="6" t="str">
         <x:f>IF(A79&gt;=$B$4,"",MAX(D79-E79,0))</x:f>
@@ -2873,7 +2893,7 @@
         <x:f>IF(A79&gt;$B$4,"",SUM($E$15:E79))</x:f>
       </x:c>
       <x:c r="J79" s="1" t="str">
-        <x:f>IF(A79&gt;$B$4,"Future",IF(A79=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A79,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E79=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A79&gt;$B$4,"Future",IF(A79=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A79,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E79=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2893,7 +2913,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E80" s="6" t="str">
-        <x:f>IF(A80&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A80,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A80&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A80,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F80" s="6" t="str">
         <x:f>IF(A80&gt;=$B$4,"",MAX(D80-E80,0))</x:f>
@@ -2908,7 +2928,7 @@
         <x:f>IF(A80&gt;$B$4,"",SUM($E$15:E80))</x:f>
       </x:c>
       <x:c r="J80" s="1" t="str">
-        <x:f>IF(A80&gt;$B$4,"Future",IF(A80=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A80,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E80=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A80&gt;$B$4,"Future",IF(A80=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A80,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E80=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2928,7 +2948,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E81" s="6" t="str">
-        <x:f>IF(A81&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A81,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A81&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A81,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F81" s="6" t="str">
         <x:f>IF(A81&gt;=$B$4,"",MAX(D81-E81,0))</x:f>
@@ -2943,7 +2963,7 @@
         <x:f>IF(A81&gt;$B$4,"",SUM($E$15:E81))</x:f>
       </x:c>
       <x:c r="J81" s="1" t="str">
-        <x:f>IF(A81&gt;$B$4,"Future",IF(A81=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A81,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E81=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A81&gt;$B$4,"Future",IF(A81=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A81,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E81=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2963,7 +2983,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E82" s="6" t="str">
-        <x:f>IF(A82&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A82,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A82&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A82,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F82" s="6" t="str">
         <x:f>IF(A82&gt;=$B$4,"",MAX(D82-E82,0))</x:f>
@@ -2978,7 +2998,7 @@
         <x:f>IF(A82&gt;$B$4,"",SUM($E$15:E82))</x:f>
       </x:c>
       <x:c r="J82" s="1" t="str">
-        <x:f>IF(A82&gt;$B$4,"Future",IF(A82=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A82,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E82=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A82&gt;$B$4,"Future",IF(A82=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A82,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E82=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -2998,7 +3018,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E83" s="6" t="str">
-        <x:f>IF(A83&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A83,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A83&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A83,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F83" s="6" t="str">
         <x:f>IF(A83&gt;=$B$4,"",MAX(D83-E83,0))</x:f>
@@ -3013,7 +3033,7 @@
         <x:f>IF(A83&gt;$B$4,"",SUM($E$15:E83))</x:f>
       </x:c>
       <x:c r="J83" s="1" t="str">
-        <x:f>IF(A83&gt;$B$4,"Future",IF(A83=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A83,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E83=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A83&gt;$B$4,"Future",IF(A83=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A83,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E83=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3033,7 +3053,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E84" s="6" t="str">
-        <x:f>IF(A84&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A84,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A84&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A84,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F84" s="6" t="str">
         <x:f>IF(A84&gt;=$B$4,"",MAX(D84-E84,0))</x:f>
@@ -3048,7 +3068,7 @@
         <x:f>IF(A84&gt;$B$4,"",SUM($E$15:E84))</x:f>
       </x:c>
       <x:c r="J84" s="1" t="str">
-        <x:f>IF(A84&gt;$B$4,"Future",IF(A84=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A84,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E84=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A84&gt;$B$4,"Future",IF(A84=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A84,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E84=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3068,7 +3088,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E85" s="6" t="str">
-        <x:f>IF(A85&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A85,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A85&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A85,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F85" s="6" t="str">
         <x:f>IF(A85&gt;=$B$4,"",MAX(D85-E85,0))</x:f>
@@ -3083,7 +3103,7 @@
         <x:f>IF(A85&gt;$B$4,"",SUM($E$15:E85))</x:f>
       </x:c>
       <x:c r="J85" s="1" t="str">
-        <x:f>IF(A85&gt;$B$4,"Future",IF(A85=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A85,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E85=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A85&gt;$B$4,"Future",IF(A85=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A85,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E85=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3103,7 +3123,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E86" s="6" t="str">
-        <x:f>IF(A86&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A86,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A86&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A86,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F86" s="6" t="str">
         <x:f>IF(A86&gt;=$B$4,"",MAX(D86-E86,0))</x:f>
@@ -3118,7 +3138,7 @@
         <x:f>IF(A86&gt;$B$4,"",SUM($E$15:E86))</x:f>
       </x:c>
       <x:c r="J86" s="1" t="str">
-        <x:f>IF(A86&gt;$B$4,"Future",IF(A86=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A86,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E86=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A86&gt;$B$4,"Future",IF(A86=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A86,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E86=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3138,7 +3158,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E87" s="6" t="str">
-        <x:f>IF(A87&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A87,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A87&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A87,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F87" s="6" t="str">
         <x:f>IF(A87&gt;=$B$4,"",MAX(D87-E87,0))</x:f>
@@ -3153,7 +3173,7 @@
         <x:f>IF(A87&gt;$B$4,"",SUM($E$15:E87))</x:f>
       </x:c>
       <x:c r="J87" s="1" t="str">
-        <x:f>IF(A87&gt;$B$4,"Future",IF(A87=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A87,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E87=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A87&gt;$B$4,"Future",IF(A87=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A87,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E87=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3173,7 +3193,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E88" s="6" t="str">
-        <x:f>IF(A88&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A88,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A88&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A88,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F88" s="6" t="str">
         <x:f>IF(A88&gt;=$B$4,"",MAX(D88-E88,0))</x:f>
@@ -3188,7 +3208,7 @@
         <x:f>IF(A88&gt;$B$4,"",SUM($E$15:E88))</x:f>
       </x:c>
       <x:c r="J88" s="1" t="str">
-        <x:f>IF(A88&gt;$B$4,"Future",IF(A88=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A88,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E88=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A88&gt;$B$4,"Future",IF(A88=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A88,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E88=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3208,7 +3228,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E89" s="6" t="str">
-        <x:f>IF(A89&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A89,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A89&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A89,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F89" s="6" t="str">
         <x:f>IF(A89&gt;=$B$4,"",MAX(D89-E89,0))</x:f>
@@ -3223,7 +3243,7 @@
         <x:f>IF(A89&gt;$B$4,"",SUM($E$15:E89))</x:f>
       </x:c>
       <x:c r="J89" s="1" t="str">
-        <x:f>IF(A89&gt;$B$4,"Future",IF(A89=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A89,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E89=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A89&gt;$B$4,"Future",IF(A89=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A89,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E89=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3243,7 +3263,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E90" s="6" t="str">
-        <x:f>IF(A90&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A90,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A90&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A90,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F90" s="6" t="str">
         <x:f>IF(A90&gt;=$B$4,"",MAX(D90-E90,0))</x:f>
@@ -3258,7 +3278,7 @@
         <x:f>IF(A90&gt;$B$4,"",SUM($E$15:E90))</x:f>
       </x:c>
       <x:c r="J90" s="1" t="str">
-        <x:f>IF(A90&gt;$B$4,"Future",IF(A90=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A90,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E90=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A90&gt;$B$4,"Future",IF(A90=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A90,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E90=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3278,7 +3298,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E91" s="6" t="str">
-        <x:f>IF(A91&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A91,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A91&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A91,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F91" s="6" t="str">
         <x:f>IF(A91&gt;=$B$4,"",MAX(D91-E91,0))</x:f>
@@ -3293,7 +3313,7 @@
         <x:f>IF(A91&gt;$B$4,"",SUM($E$15:E91))</x:f>
       </x:c>
       <x:c r="J91" s="1" t="str">
-        <x:f>IF(A91&gt;$B$4,"Future",IF(A91=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A91,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E91=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A91&gt;$B$4,"Future",IF(A91=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A91,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E91=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3313,7 +3333,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E92" s="6" t="str">
-        <x:f>IF(A92&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A92,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A92&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A92,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F92" s="6" t="str">
         <x:f>IF(A92&gt;=$B$4,"",MAX(D92-E92,0))</x:f>
@@ -3328,7 +3348,7 @@
         <x:f>IF(A92&gt;$B$4,"",SUM($E$15:E92))</x:f>
       </x:c>
       <x:c r="J92" s="1" t="str">
-        <x:f>IF(A92&gt;$B$4,"Future",IF(A92=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A92,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E92=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A92&gt;$B$4,"Future",IF(A92=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A92,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E92=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3348,7 +3368,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E93" s="6" t="str">
-        <x:f>IF(A93&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A93,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A93&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A93,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F93" s="6" t="str">
         <x:f>IF(A93&gt;=$B$4,"",MAX(D93-E93,0))</x:f>
@@ -3363,7 +3383,7 @@
         <x:f>IF(A93&gt;$B$4,"",SUM($E$15:E93))</x:f>
       </x:c>
       <x:c r="J93" s="1" t="str">
-        <x:f>IF(A93&gt;$B$4,"Future",IF(A93=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A93,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E93=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A93&gt;$B$4,"Future",IF(A93=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A93,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E93=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3383,7 +3403,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E94" s="6" t="str">
-        <x:f>IF(A94&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A94,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A94&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A94,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F94" s="6" t="str">
         <x:f>IF(A94&gt;=$B$4,"",MAX(D94-E94,0))</x:f>
@@ -3398,7 +3418,7 @@
         <x:f>IF(A94&gt;$B$4,"",SUM($E$15:E94))</x:f>
       </x:c>
       <x:c r="J94" s="1" t="str">
-        <x:f>IF(A94&gt;$B$4,"Future",IF(A94=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A94,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E94=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A94&gt;$B$4,"Future",IF(A94=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A94,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E94=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3418,7 +3438,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E95" s="6" t="str">
-        <x:f>IF(A95&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A95,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A95&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A95,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F95" s="6" t="str">
         <x:f>IF(A95&gt;=$B$4,"",MAX(D95-E95,0))</x:f>
@@ -3433,7 +3453,7 @@
         <x:f>IF(A95&gt;$B$4,"",SUM($E$15:E95))</x:f>
       </x:c>
       <x:c r="J95" s="1" t="str">
-        <x:f>IF(A95&gt;$B$4,"Future",IF(A95=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A95,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E95=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A95&gt;$B$4,"Future",IF(A95=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A95,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E95=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3453,7 +3473,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E96" s="6" t="str">
-        <x:f>IF(A96&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A96,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A96&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A96,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F96" s="6" t="str">
         <x:f>IF(A96&gt;=$B$4,"",MAX(D96-E96,0))</x:f>
@@ -3468,7 +3488,7 @@
         <x:f>IF(A96&gt;$B$4,"",SUM($E$15:E96))</x:f>
       </x:c>
       <x:c r="J96" s="1" t="str">
-        <x:f>IF(A96&gt;$B$4,"Future",IF(A96=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A96,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E96=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A96&gt;$B$4,"Future",IF(A96=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A96,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E96=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3488,7 +3508,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E97" s="6" t="str">
-        <x:f>IF(A97&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A97,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A97&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A97,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F97" s="6" t="str">
         <x:f>IF(A97&gt;=$B$4,"",MAX(D97-E97,0))</x:f>
@@ -3503,7 +3523,7 @@
         <x:f>IF(A97&gt;$B$4,"",SUM($E$15:E97))</x:f>
       </x:c>
       <x:c r="J97" s="1" t="str">
-        <x:f>IF(A97&gt;$B$4,"Future",IF(A97=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A97,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E97=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A97&gt;$B$4,"Future",IF(A97=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A97,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E97=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3523,7 +3543,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E98" s="6" t="str">
-        <x:f>IF(A98&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A98,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A98&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A98,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F98" s="6" t="str">
         <x:f>IF(A98&gt;=$B$4,"",MAX(D98-E98,0))</x:f>
@@ -3538,7 +3558,7 @@
         <x:f>IF(A98&gt;$B$4,"",SUM($E$15:E98))</x:f>
       </x:c>
       <x:c r="J98" s="1" t="str">
-        <x:f>IF(A98&gt;$B$4,"Future",IF(A98=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A98,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E98=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A98&gt;$B$4,"Future",IF(A98=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A98,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E98=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3558,7 +3578,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E99" s="6" t="str">
-        <x:f>IF(A99&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A99,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A99&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A99,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F99" s="6" t="str">
         <x:f>IF(A99&gt;=$B$4,"",MAX(D99-E99,0))</x:f>
@@ -3573,7 +3593,7 @@
         <x:f>IF(A99&gt;$B$4,"",SUM($E$15:E99))</x:f>
       </x:c>
       <x:c r="J99" s="1" t="str">
-        <x:f>IF(A99&gt;$B$4,"Future",IF(A99=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A99,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E99=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A99&gt;$B$4,"Future",IF(A99=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A99,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E99=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3593,7 +3613,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E100" s="6" t="str">
-        <x:f>IF(A100&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A100,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A100&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A100,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F100" s="6" t="str">
         <x:f>IF(A100&gt;=$B$4,"",MAX(D100-E100,0))</x:f>
@@ -3608,7 +3628,7 @@
         <x:f>IF(A100&gt;$B$4,"",SUM($E$15:E100))</x:f>
       </x:c>
       <x:c r="J100" s="1" t="str">
-        <x:f>IF(A100&gt;$B$4,"Future",IF(A100=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A100,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E100=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A100&gt;$B$4,"Future",IF(A100=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A100,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E100=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3628,7 +3648,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E101" s="6" t="str">
-        <x:f>IF(A101&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A101,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A101&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A101,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F101" s="6" t="str">
         <x:f>IF(A101&gt;=$B$4,"",MAX(D101-E101,0))</x:f>
@@ -3643,7 +3663,7 @@
         <x:f>IF(A101&gt;$B$4,"",SUM($E$15:E101))</x:f>
       </x:c>
       <x:c r="J101" s="1" t="str">
-        <x:f>IF(A101&gt;$B$4,"Future",IF(A101=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A101,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E101=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A101&gt;$B$4,"Future",IF(A101=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A101,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E101=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3663,7 +3683,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E102" s="6" t="str">
-        <x:f>IF(A102&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A102,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A102&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A102,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F102" s="6" t="str">
         <x:f>IF(A102&gt;=$B$4,"",MAX(D102-E102,0))</x:f>
@@ -3678,7 +3698,7 @@
         <x:f>IF(A102&gt;$B$4,"",SUM($E$15:E102))</x:f>
       </x:c>
       <x:c r="J102" s="1" t="str">
-        <x:f>IF(A102&gt;$B$4,"Future",IF(A102=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A102,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E102=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A102&gt;$B$4,"Future",IF(A102=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A102,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E102=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3698,7 +3718,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E103" s="6" t="str">
-        <x:f>IF(A103&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A103,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A103&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A103,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F103" s="6" t="str">
         <x:f>IF(A103&gt;=$B$4,"",MAX(D103-E103,0))</x:f>
@@ -3713,7 +3733,7 @@
         <x:f>IF(A103&gt;$B$4,"",SUM($E$15:E103))</x:f>
       </x:c>
       <x:c r="J103" s="1" t="str">
-        <x:f>IF(A103&gt;$B$4,"Future",IF(A103=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A103,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E103=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A103&gt;$B$4,"Future",IF(A103=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A103,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E103=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3733,7 +3753,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E104" s="6" t="str">
-        <x:f>IF(A104&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A104,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A104&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A104,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F104" s="6" t="str">
         <x:f>IF(A104&gt;=$B$4,"",MAX(D104-E104,0))</x:f>
@@ -3748,7 +3768,7 @@
         <x:f>IF(A104&gt;$B$4,"",SUM($E$15:E104))</x:f>
       </x:c>
       <x:c r="J104" s="1" t="str">
-        <x:f>IF(A104&gt;$B$4,"Future",IF(A104=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A104,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E104=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A104&gt;$B$4,"Future",IF(A104=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A104,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E104=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3768,7 +3788,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E105" s="6" t="str">
-        <x:f>IF(A105&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A105,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A105&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A105,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F105" s="6" t="str">
         <x:f>IF(A105&gt;=$B$4,"",MAX(D105-E105,0))</x:f>
@@ -3783,7 +3803,7 @@
         <x:f>IF(A105&gt;$B$4,"",SUM($E$15:E105))</x:f>
       </x:c>
       <x:c r="J105" s="1" t="str">
-        <x:f>IF(A105&gt;$B$4,"Future",IF(A105=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A105,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E105=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A105&gt;$B$4,"Future",IF(A105=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A105,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E105=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3803,7 +3823,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E106" s="6" t="str">
-        <x:f>IF(A106&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A106,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A106&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A106,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F106" s="6" t="str">
         <x:f>IF(A106&gt;=$B$4,"",MAX(D106-E106,0))</x:f>
@@ -3818,7 +3838,7 @@
         <x:f>IF(A106&gt;$B$4,"",SUM($E$15:E106))</x:f>
       </x:c>
       <x:c r="J106" s="1" t="str">
-        <x:f>IF(A106&gt;$B$4,"Future",IF(A106=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A106,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E106=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A106&gt;$B$4,"Future",IF(A106=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A106,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E106=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3838,7 +3858,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E107" s="6" t="str">
-        <x:f>IF(A107&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A107,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A107&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A107,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F107" s="6" t="str">
         <x:f>IF(A107&gt;=$B$4,"",MAX(D107-E107,0))</x:f>
@@ -3853,7 +3873,7 @@
         <x:f>IF(A107&gt;$B$4,"",SUM($E$15:E107))</x:f>
       </x:c>
       <x:c r="J107" s="1" t="str">
-        <x:f>IF(A107&gt;$B$4,"Future",IF(A107=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A107,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E107=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A107&gt;$B$4,"Future",IF(A107=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A107,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E107=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3873,7 +3893,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E108" s="6" t="str">
-        <x:f>IF(A108&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A108,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A108&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A108,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F108" s="6" t="str">
         <x:f>IF(A108&gt;=$B$4,"",MAX(D108-E108,0))</x:f>
@@ -3888,7 +3908,7 @@
         <x:f>IF(A108&gt;$B$4,"",SUM($E$15:E108))</x:f>
       </x:c>
       <x:c r="J108" s="1" t="str">
-        <x:f>IF(A108&gt;$B$4,"Future",IF(A108=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A108,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E108=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A108&gt;$B$4,"Future",IF(A108=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A108,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E108=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3908,7 +3928,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E109" s="6" t="str">
-        <x:f>IF(A109&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A109,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A109&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A109,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F109" s="6" t="str">
         <x:f>IF(A109&gt;=$B$4,"",MAX(D109-E109,0))</x:f>
@@ -3923,7 +3943,7 @@
         <x:f>IF(A109&gt;$B$4,"",SUM($E$15:E109))</x:f>
       </x:c>
       <x:c r="J109" s="1" t="str">
-        <x:f>IF(A109&gt;$B$4,"Future",IF(A109=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A109,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E109=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A109&gt;$B$4,"Future",IF(A109=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A109,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E109=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3943,7 +3963,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E110" s="6" t="str">
-        <x:f>IF(A110&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A110,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A110&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A110,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F110" s="6" t="str">
         <x:f>IF(A110&gt;=$B$4,"",MAX(D110-E110,0))</x:f>
@@ -3958,7 +3978,7 @@
         <x:f>IF(A110&gt;$B$4,"",SUM($E$15:E110))</x:f>
       </x:c>
       <x:c r="J110" s="1" t="str">
-        <x:f>IF(A110&gt;$B$4,"Future",IF(A110=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A110,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E110=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A110&gt;$B$4,"Future",IF(A110=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A110,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E110=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -3978,7 +3998,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E111" s="6" t="str">
-        <x:f>IF(A111&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A111,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A111&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A111,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F111" s="6" t="str">
         <x:f>IF(A111&gt;=$B$4,"",MAX(D111-E111,0))</x:f>
@@ -3993,7 +4013,7 @@
         <x:f>IF(A111&gt;$B$4,"",SUM($E$15:E111))</x:f>
       </x:c>
       <x:c r="J111" s="1" t="str">
-        <x:f>IF(A111&gt;$B$4,"Future",IF(A111=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A111,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E111=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A111&gt;$B$4,"Future",IF(A111=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A111,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E111=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4013,7 +4033,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E112" s="6" t="str">
-        <x:f>IF(A112&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A112,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A112&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A112,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F112" s="6" t="str">
         <x:f>IF(A112&gt;=$B$4,"",MAX(D112-E112,0))</x:f>
@@ -4028,7 +4048,7 @@
         <x:f>IF(A112&gt;$B$4,"",SUM($E$15:E112))</x:f>
       </x:c>
       <x:c r="J112" s="1" t="str">
-        <x:f>IF(A112&gt;$B$4,"Future",IF(A112=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A112,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E112=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A112&gt;$B$4,"Future",IF(A112=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A112,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E112=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4048,7 +4068,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E113" s="6" t="str">
-        <x:f>IF(A113&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A113,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A113&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A113,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F113" s="6" t="str">
         <x:f>IF(A113&gt;=$B$4,"",MAX(D113-E113,0))</x:f>
@@ -4063,7 +4083,7 @@
         <x:f>IF(A113&gt;$B$4,"",SUM($E$15:E113))</x:f>
       </x:c>
       <x:c r="J113" s="1" t="str">
-        <x:f>IF(A113&gt;$B$4,"Future",IF(A113=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A113,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E113=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A113&gt;$B$4,"Future",IF(A113=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A113,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E113=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4083,7 +4103,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E114" s="6" t="str">
-        <x:f>IF(A114&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$B$2:$B$24,A114,'Sessions'!$G$2:$G$24,"completed")/60)</x:f>
+        <x:f>IF(A114&gt;$B$4,"",SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$B$2:$B$27,A114,'Sessions'!$G$2:$G$27,"completed")/60)</x:f>
       </x:c>
       <x:c r="F114" s="6" t="str">
         <x:f>IF(A114&gt;=$B$4,"",MAX(D114-E114,0))</x:f>
@@ -4098,7 +4118,7 @@
         <x:f>IF(A114&gt;$B$4,"",SUM($E$15:E114))</x:f>
       </x:c>
       <x:c r="J114" s="1" t="str">
-        <x:f>IF(A114&gt;$B$4,"Future",IF(A114=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$24,A114,'Sessions'!$G$2:$G$24,"needs_confirmation")&gt;0,"Uncertain time",IF(E114=0,"No confirmed time","Logged"))))</x:f>
+        <x:f>IF(A114&gt;$B$4,"Future",IF(A114=$B$4,"In progress",IF(COUNTIFS('Sessions'!$B$2:$B$27,A114,'Sessions'!$G$2:$G$27,"needs_confirmation")&gt;0,"Uncertain time",IF(E114=0,"No confirmed time","Logged"))))</x:f>
         <x:v>Future</x:v>
       </x:c>
     </x:row>
@@ -4251,7 +4271,7 @@
       </x:c>
       <x:c r="C9" s="6" t="n">
         <x:f>SUMIFS('Daily'!$D$15:$D$114,'Daily'!$C$15:$C$114,A9,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46320")</x:f>
-        <x:v>18</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D9" s="6" t="n">
         <x:f>SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A9,'Daily'!$A$15:$A$114,"&lt;=46320")</x:f>
@@ -4259,7 +4279,7 @@
       </x:c>
       <x:c r="E9" s="6" t="n">
         <x:f>MAX(C9-SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A9,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46320"),0)</x:f>
-        <x:v>18</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="F9" s="6" t="n">
         <x:f>MAX(SUMIFS('Daily'!$E$15:$E$114,'Daily'!$C$15:$C$114,A9,'Daily'!$A$15:$A$114,"&lt;"&amp;'Daily'!$B$4,'Daily'!$A$15:$A$114,"&lt;=46320")-C9,0)</x:f>
@@ -5335,6 +5355,66 @@
         <x:v>Learner reported a third completed 25-minute Docker study interval and 5-minute break. Exact start/end times in IST not supplied; duration is pending timestamp confirmation and excluded from confirmed totals.</x:v>
       </x:c>
     </x:row>
+    <x:row r="25" ht="22" customHeight="1">
+      <x:c r="A25" s="1" t="str">
+        <x:v>POM-20261026-OTHER-MORNING-1</x:v>
+      </x:c>
+      <x:c r="B25" s="7" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="C25" s="1" t="str">
+        <x:v>Study: other computer morning Pomodoro</x:v>
+      </x:c>
+      <x:c r="D25" s="1" t="str"/>
+      <x:c r="E25" s="1" t="str"/>
+      <x:c r="F25" s="1"/>
+      <x:c r="G25" s="1" t="str">
+        <x:v>needs_confirmation</x:v>
+      </x:c>
+      <x:c r="H25" s="1" t="str">
+        <x:v>Learner reported three completed morning Pomodoros on another computer. Session 1 of 3; topic duration and IST start/end times not supplied. Count recorded; excluded from confirmed hours. Do not duplicate as local timer completions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="22" customHeight="1">
+      <x:c r="A26" s="1" t="str">
+        <x:v>POM-20261026-OTHER-MORNING-2</x:v>
+      </x:c>
+      <x:c r="B26" s="7" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="C26" s="1" t="str">
+        <x:v>Study: other computer morning Pomodoro</x:v>
+      </x:c>
+      <x:c r="D26" s="1" t="str"/>
+      <x:c r="E26" s="1" t="str"/>
+      <x:c r="F26" s="1"/>
+      <x:c r="G26" s="1" t="str">
+        <x:v>needs_confirmation</x:v>
+      </x:c>
+      <x:c r="H26" s="1" t="str">
+        <x:v>Learner reported three completed morning Pomodoros on another computer. Session 2 of 3; topic duration and IST start/end times not supplied. Count recorded; excluded from confirmed hours. Do not duplicate as local timer completions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="22" customHeight="1">
+      <x:c r="A27" s="1" t="str">
+        <x:v>POM-20261026-OTHER-MORNING-3</x:v>
+      </x:c>
+      <x:c r="B27" s="7" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="C27" s="1" t="str">
+        <x:v>Study: other computer morning Pomodoro</x:v>
+      </x:c>
+      <x:c r="D27" s="1" t="str"/>
+      <x:c r="E27" s="1" t="str"/>
+      <x:c r="F27" s="1"/>
+      <x:c r="G27" s="1" t="str">
+        <x:v>needs_confirmation</x:v>
+      </x:c>
+      <x:c r="H27" s="1" t="str">
+        <x:v>Learner reported three completed morning Pomodoros on another computer. Session 3 of 3; topic duration and IST start/end times not supplied. Count recorded; excluded from confirmed hours. Do not duplicate as local timer completions.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5371,7 +5451,7 @@
         <x:v>Docker: self-reported Pomodoro</x:v>
       </x:c>
       <x:c r="B7" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A7,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$C$2:$C$27,A7,'Sessions'!$G$2:$G$27,"completed",'Sessions'!$B$2:$B$27,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -5380,7 +5460,7 @@
         <x:v>Python / RRDAP: RDS-001 Product Catalogue</x:v>
       </x:c>
       <x:c r="B8" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A8,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$C$2:$C$27,A8,'Sessions'!$G$2:$G$27,"completed",'Sessions'!$B$2:$B$27,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
         <x:v>0.5175</x:v>
       </x:c>
     </x:row>
@@ -5389,7 +5469,7 @@
         <x:v>Python / RRDAP: setup and RDS-001</x:v>
       </x:c>
       <x:c r="B9" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A9,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$C$2:$C$27,A9,'Sessions'!$G$2:$G$27,"completed",'Sessions'!$B$2:$B$27,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
         <x:v>2.225277777777778</x:v>
       </x:c>
     </x:row>
@@ -5398,7 +5478,7 @@
         <x:v>Python / RetailFlow: setup and RF-001</x:v>
       </x:c>
       <x:c r="B10" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A10,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$C$2:$C$27,A10,'Sessions'!$G$2:$G$27,"completed",'Sessions'!$B$2:$B$27,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
         <x:v>1.0919444444444444</x:v>
       </x:c>
     </x:row>
@@ -5407,7 +5487,7 @@
         <x:v>Python: CSV reading and writing</x:v>
       </x:c>
       <x:c r="B11" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A11,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$C$2:$C$27,A11,'Sessions'!$G$2:$G$27,"completed",'Sessions'!$B$2:$B$27,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
         <x:v>0.12722222222222224</x:v>
       </x:c>
     </x:row>
@@ -5416,7 +5496,7 @@
         <x:v>Python: CSV writing and read-back</x:v>
       </x:c>
       <x:c r="B12" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A12,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$C$2:$C$27,A12,'Sessions'!$G$2:$G$27,"completed",'Sessions'!$B$2:$B$27,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
         <x:v>2.8175000000000003</x:v>
       </x:c>
     </x:row>
@@ -5425,7 +5505,7 @@
         <x:v>Python: cleaner changed-input check</x:v>
       </x:c>
       <x:c r="B13" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A13,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$C$2:$C$27,A13,'Sessions'!$G$2:$G$27,"completed",'Sessions'!$B$2:$B$27,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
         <x:v>0.4911111111111111</x:v>
       </x:c>
     </x:row>
@@ -5434,7 +5514,7 @@
         <x:v>Python: dictionary foundations in Jupyter</x:v>
       </x:c>
       <x:c r="B14" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A14,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$C$2:$C$27,A14,'Sessions'!$G$2:$G$27,"completed",'Sessions'!$B$2:$B$27,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
         <x:v>1.6424999999994445</x:v>
       </x:c>
     </x:row>
@@ -5443,7 +5523,7 @@
         <x:v>Python: dictionary records baseline</x:v>
       </x:c>
       <x:c r="B15" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A15,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$C$2:$C$27,A15,'Sessions'!$G$2:$G$27,"completed",'Sessions'!$B$2:$B$27,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
         <x:v>0.21111111111166667</x:v>
       </x:c>
     </x:row>
@@ -5452,7 +5532,7 @@
         <x:v>Python: record cleaning</x:v>
       </x:c>
       <x:c r="B16" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A16,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$C$2:$C$27,A16,'Sessions'!$G$2:$G$27,"completed",'Sessions'!$B$2:$B$27,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
         <x:v>0.22972222222166666</x:v>
       </x:c>
     </x:row>
@@ -5461,7 +5541,7 @@
         <x:v>Python: valid and rejected record lists</x:v>
       </x:c>
       <x:c r="B17" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A17,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$C$2:$C$27,A17,'Sessions'!$G$2:$G$27,"completed",'Sessions'!$B$2:$B$27,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
         <x:v>0.28194444444444444</x:v>
       </x:c>
     </x:row>
@@ -5470,7 +5550,7 @@
         <x:v>SQL: LEFT JOIN and unmatched rows</x:v>
       </x:c>
       <x:c r="B18" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A18,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$C$2:$C$27,A18,'Sessions'!$G$2:$G$27,"completed",'Sessions'!$B$2:$B$27,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
         <x:v>0.34055555555666667</x:v>
       </x:c>
     </x:row>
@@ -5479,8 +5559,17 @@
         <x:v>SQL: joins counting grouping and SUM setup</x:v>
       </x:c>
       <x:c r="B19" s="6" t="n">
-        <x:f>SUMIFS('Sessions'!$F$2:$F$24,'Sessions'!$C$2:$C$24,A19,'Sessions'!$G$2:$G$24,"completed",'Sessions'!$B$2:$B$24,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:f>SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$C$2:$C$27,A19,'Sessions'!$G$2:$G$27,"completed",'Sessions'!$B$2:$B$27,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
         <x:v>1.175</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="1" t="str">
+        <x:v>Study: other computer morning Pomodoro</x:v>
+      </x:c>
+      <x:c r="B20" s="6" t="n">
+        <x:f>SUMIFS('Sessions'!$F$2:$F$27,'Sessions'!$C$2:$C$27,A20,'Sessions'!$G$2:$G$27,"completed",'Sessions'!$B$2:$B$27,"&lt;="&amp;'Daily'!$B$4)/60</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>